<commit_message>
chore: completed Batch 13 extraction
</commit_message>
<xml_diff>
--- a/BSMA_AI_Run_V2.xlsx
+++ b/BSMA_AI_Run_V2.xlsx
@@ -22701,6 +22701,16 @@
           <t>BSMA0436</t>
         </is>
       </c>
+      <c r="E439" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F439" t="inlineStr">
+        <is>
+          <t>Not Individual Level</t>
+        </is>
+      </c>
       <c r="G439" t="inlineStr">
         <is>
           <t>Purpose – Literature on small and medium enterprises (SMEs) has so far produced limited evidence on how these firms pursue their organizational flexibility with information and communication technology (ICT) and ad hoc work practices. The purpose of this paper is to contribute to the extant literature by focusing on how SMEs use flexible work practices that provide latitude with respect to when employees work, where they work and via which communication medium. Specifically, the authors analyze how such practices are related to the conditions that SMEs face in reference to their competitive environment and their patterns of ICT usage.</t>
@@ -22724,7 +22734,11 @@
       <c r="K439" t="n">
         <v>2017</v>
       </c>
-      <c r="P439" s="8" t="n"/>
+      <c r="P439" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures flexible work practices at the firm level (SMEs), not individual-level boundary spanning behaviors.. Verbatim Evidence: "A survey was conducted on 304 Italian SMEs, with the aim of identifying the contextual dimensions where flexible work is chosen and the different typologies of flexible work implemented by companies."</t>
+        </is>
+      </c>
     </row>
     <row r="440" ht="18" customHeight="1" s="10">
       <c r="A440" t="inlineStr">
@@ -22737,6 +22751,16 @@
           <t>BSMA0437</t>
         </is>
       </c>
+      <c r="E440" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F440" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G440" t="inlineStr">
         <is>
           <t>Business Process Reengineering (BPR) was developed as a new idea which, it was suggested, could revolutionise the corporation and give it a major competitive advantage by simplifying key business processes and utilising information technology to secure cross-functional communication and focus on customer requirements. Rather than continue the debate about whether BPR is ‘good’ or ‘bad’, ‘old’ or ‘new’ (e.g. Earl, M.J., 1994. The new and the old of business process redesign. Journal of Strategic Information Systems 3 (1), 5–22; Mumford, E., 1994. New treatments or old remedies: is business process reengineering really socio-technical design. Journal of Strategic Information Systems 3 (4), 313–326), the focus here is on understanding how the concept ‘BPR’, however deﬁned, has been diffused across European ﬁrms. The results from a survey of ﬁrms in four countries support previous research on the diffusion process with the rate of adoption of BPR related to microorganisational level variables—characteristics of the ﬁrm and the boundary spanning activities of individual members. In addition there were differences across industry sectors and across countries in the extent of adoption of BPR. It is argued that attention to these meso-industry level and macro-national level factors, as well as the micro-organisational level dynamics, will improve our understanding of the relationship between networking and innovation processes. In particular, the paper focuses on how networking activity can be restrictive and lead to the creation of fashions which limit the extent of organisational learning during BPR adoption. q 1999 Elsevier Science B.V. All rights reserved.</t>
@@ -22760,7 +22784,11 @@
       <c r="K440" t="n">
         <v>1998</v>
       </c>
-      <c r="P440" s="8" t="n"/>
+      <c r="P440" s="8" t="inlineStr">
+        <is>
+          <t>The paper does not report a correlation matrix with Pearson r values; it is an empirical study but does not provide zero-order correlations.. Verbatim Evidence: "Table 1 Mean networking score for adopters and non-adopters... Table 2 Mean score for adopters and non-adopters... Table 6 Regression analysis with length of BPR adoption as the dependent variable"</t>
+        </is>
+      </c>
     </row>
     <row r="441" ht="18" customHeight="1" s="10">
       <c r="A441" t="inlineStr">
@@ -22773,6 +22801,16 @@
           <t>BSMA0438</t>
         </is>
       </c>
+      <c r="E441" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F441" t="inlineStr">
+        <is>
+          <t>No Correlation Matrix</t>
+        </is>
+      </c>
       <c r="G441" t="inlineStr">
         <is>
           <t>This exploratory study examined the practice of public relations in Zimbabwe by surveying and understanding public relations roles typically practiced by Zimbabwean PR practitioners. Through the lens of systems theory, the research investigated whether the practiced public relations roles allow organizations to perform all three boundary spanning functions such as output, throughput, and input. The results confirmed prior theoretically and empirically derived typology of roles (technician, manager, strategist) from the African continent. However, the observed structures of public relations roles deviate from previous findings, indicating that Zimbabwean PR practitioners’ professional roles may differ from those in neighboring countries.</t>
@@ -22796,7 +22834,11 @@
       <c r="K441" t="n">
         <v>2020</v>
       </c>
-      <c r="P441" s="8" t="n"/>
+      <c r="P441" s="8" t="inlineStr">
+        <is>
+          <t>The paper does not provide a zero-order correlation matrix of the study variables. It only reports three individual correlations between PR roles and a single 'Understanding of PR' variable in a non-square format (Table 3), which violates the square matrix extraction rule.. Verbatim Evidence: "Table 3... Pearson Product-Moment Correlations Between Public Relations Roles and Understanding of PR."</t>
+        </is>
+      </c>
     </row>
     <row r="442" ht="18" customHeight="1" s="10">
       <c r="A442" t="inlineStr">
@@ -22809,6 +22851,16 @@
           <t>BSMA0439</t>
         </is>
       </c>
+      <c r="E442" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F442" t="inlineStr">
+        <is>
+          <t>Qualitative/Historical</t>
+        </is>
+      </c>
       <c r="G442" t="inlineStr">
         <is>
           <t>This dissertation presents a critical perspective on the development of American journalism education by combining historical methods and a sociological framework. That framework is boundary work, and it serves as the organizing principle of this project. As such, this study privileges boundary work paradigms–participation, practices, and professionalism–over a chronological narrative. It uncovers the interrelationships and power dynamics that structured the development of journalism instruction in higher education. Moreover, it heeds the call for journalism historians to engage with other disciplines and develop more theoretical approaches to understanding the past.</t>
@@ -22832,7 +22884,11 @@
       <c r="K442" t="n">
         <v>2020</v>
       </c>
-      <c r="P442" s="8" t="n"/>
+      <c r="P442" s="8" t="inlineStr">
+        <is>
+          <t>The document is a historical dissertation examining the development of American journalism education. It does not measure individual-level boundary spanning behaviors, nor does it contain any quantitative empirical data or correlation matrices.. Verbatim Evidence: "This dissertation presents a critical perspective on the development of American journalism education by combining historical methods and a sociological framework."</t>
+        </is>
+      </c>
     </row>
     <row r="443" ht="18" customHeight="1" s="10">
       <c r="A443" t="inlineStr">
@@ -22845,6 +22901,16 @@
           <t>BSMA0440</t>
         </is>
       </c>
+      <c r="E443" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F443" t="inlineStr">
+        <is>
+          <t>EXCL_NON_INDIVIDUAL_LEVEL</t>
+        </is>
+      </c>
       <c r="G443" t="inlineStr">
         <is>
           <t>Research Summary:                              We study antecedents of innovation performance for the subsidiaries of multinational enterprises (MNEs) using the microfoundations approach. Based on the upper echelon perspective, we argue that managers’ characteristics, such as prior MNE work experience and industry experience, affect subsidiary innovation. We tested our hypotheses on a sample of 228 MNE subsidiaries from 11 countries. Results indicate that managers’ industry experience serves as an external boundary‐spanning capability and, therefore, it has a greater effect on autonomous subsidiaries. In contrast, managers’ prior MNE work experience functions as an internal boundary‐spanning capability and, therefore, it has a smaller effect on subsidiaries that are less autonomous or engage in R&amp;D.                                                          Managerial Summary:                              The success of an MNE now increasingly depends on its ability to generate knowledge anywhere in the world. Thus, the ability of foreign subsidiaries to generate innovation plays an increasingly important role in enhancing the performance of MNEs. In this regard, what factors determine the innovativeness of foreign subsidiaries is an important question for managers. Our study suggests that the international experience of the top management team (TMT) of a subsidiary and its CEO’s industry experience positively affect subsidiary innovation. Furthermore, the TMT’s international experience has a greater effect on the innovativeness of subsidiaries that remain dependent on their headquarters for knowledge transfer. In contrast, the CEO’s industry experience has a greater effect on the innovativeness of autonomous subsidiaries.</t>
@@ -22868,7 +22934,11 @@
       <c r="K443" t="n">
         <v>2019</v>
       </c>
-      <c r="P443" s="8" t="n"/>
+      <c r="P443" s="8" t="inlineStr">
+        <is>
+          <t>The unit of analysis is the subsidiary (firm level), not the individual. The study measures subsidiary innovation and aggregates managerial experience at the subsidiary level.. Verbatim Evidence: "With these criteria, we have 228 subsidiaries from 11 countries in our dataset."</t>
+        </is>
+      </c>
     </row>
     <row r="444" ht="18" customHeight="1" s="10">
       <c r="A444" t="inlineStr">
@@ -22881,6 +22951,16 @@
           <t>BSMA0441</t>
         </is>
       </c>
+      <c r="E444" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F444" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G444" t="inlineStr">
         <is>
           <t>Horizontal arrangements are increasingly deployed in organizational networks, yet research has rarely examined the effectiveness of these alliances. The coalition of disparate corporate cultures yields appreciable levels of role stress for people in boundary-spanning positions. Dedicated assets and communication modality are factors that influence the level of role ambiguity and conflict. The authors implicate these facets of role stress as antecedents to four forms of effectiveness drawn from the competing values framework. The authors present alternative perspectives that examine the relationship between stress and performance. The received view frames role stressors as linear, negative antecedents to organizational outcomes. The authors contrast this perspective with theories that espouse triphasic, parabolic, and interactive influences of stressors on organizational outcomes. Data gathered with 218 managers of dual-branded retail oil outlets indicate that the relevance of these alternative perspectives is mitigated by the form of effectiveness pursued by the organization. The results support a linear relationship between role conflict and bargaining efforts, yet they also offer evidence of nonlinear influences of role ambiguity on contributions to sales, customer satisfaction, and competence. The study concludes with a discussion of relevance of the findings to the management of horizontal alliances and to interorganizational theory.</t>
@@ -22904,7 +22984,11 @@
       <c r="K444" t="n">
         <v>2002</v>
       </c>
-      <c r="P444" s="8" t="n"/>
+      <c r="P444" s="8" t="inlineStr">
+        <is>
+          <t>The study measures role ambiguity and conflict for retail managers, who occupy boundary-spanning positions. Table 3 reports a raw correlation matrix with descriptive statistics.. Verbatim Evidence: "Inherent to the nature of boundary-spanning positions is the likelihood that people occupying these roles will experi-ence ambiguity and conflict. ... Table 3 provides correlations and descriptive statistics for the constructs."</t>
+        </is>
+      </c>
     </row>
     <row r="445" ht="18" customHeight="1" s="10">
       <c r="A445" t="inlineStr">
@@ -22915,6 +22999,16 @@
       <c r="B445" t="inlineStr">
         <is>
           <t>BSMA0442</t>
+        </is>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F445" t="inlineStr">
+        <is>
+          <t>Non-Individual Level</t>
         </is>
       </c>
       <c r="G445" t="inlineStr">
@@ -22959,7 +23053,11 @@
       <c r="K445" t="n">
         <v>2013</v>
       </c>
-      <c r="P445" s="8" t="n"/>
+      <c r="P445" s="8" t="inlineStr">
+        <is>
+          <t>The paper focuses on firm-level capabilities (alliance and network opportunity-sensing/seizing) rather than individual-level boundary spanning behaviors.. Verbatim Evidence: "By “inter-organizational relationships” I am referring to both alliance and network relationships collectively. One critical assumption underlying formation of inter-organizational relationships is that “organizations are assumed to make conscious, intentional decisions to establish an IOR [inter-organizational relationship] for explicitly formulated purposes” (Oliver, 1990: 242)."</t>
+        </is>
+      </c>
     </row>
     <row r="446" ht="18" customHeight="1" s="10">
       <c r="A446" t="inlineStr">
@@ -22972,6 +23070,16 @@
           <t>BSMA0443</t>
         </is>
       </c>
+      <c r="E446" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F446" t="inlineStr">
+        <is>
+          <t>3 = No individual-level boundary spanning behaviors</t>
+        </is>
+      </c>
       <c r="G446" t="inlineStr">
         <is>
           <t>Purpose – This study recognizes service as the majority contributor to global and US gross domestic product and the importance of innovation speed to service innovation. Generating innovative products and services at a faster rate generates advantages for business-to-business (B2B) service organizations in keeping up with and moving ahead of rivals. This study aims to introduce the concept of capacity for social exchange (CSE) in buyer–supplier relationships, which reflects the degree to which individuals possess competencies that enable the exchange of information, and this study also explores how CSE affects knowledge sharing and innovation speed within a supply chain organization.</t>
@@ -22995,7 +23103,11 @@
       <c r="K446" t="n">
         <v>2023</v>
       </c>
-      <c r="P446" s="8" t="n"/>
+      <c r="P446" s="8" t="inlineStr">
+        <is>
+          <t>The study measures variables at the business unit or firm level, not the individual employee level. Additionally, the boundary-spanning variable (Knowledge channels) is absent from the correlation matrix.. Verbatim Evidence: "Please respond to Items 14-16 related to knowledge management practices of your business unit. 14. Our employees regularly visit supply chain partners to enable two-way sharing of expertise."</t>
+        </is>
+      </c>
     </row>
     <row r="447" ht="18" customHeight="1" s="10">
       <c r="A447" t="inlineStr">
@@ -23008,6 +23120,16 @@
           <t>BSMA0444</t>
         </is>
       </c>
+      <c r="E447" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F447" t="inlineStr">
+        <is>
+          <t>Non-Individual Level</t>
+        </is>
+      </c>
       <c r="G447" t="inlineStr">
         <is>
           <t>Purpose – The authors aim to develop and test hypotheses that link outsourcing and subcontracting-in activities of small high-tech ﬁrms to their radical innovativeness. In addition, they seek to investigate how a ﬁrm’s strategy moderates the associations between their outsourcing and subcontracting-in activities and radical innovativeness.</t>
@@ -23031,7 +23153,11 @@
       <c r="K447" t="n">
         <v>2013</v>
       </c>
-      <c r="P447" s="8" t="n"/>
+      <c r="P447" s="8" t="inlineStr">
+        <is>
+          <t>The study measures boundary spanning activities (outsourcing and subcontracting-in) at the firm level rather than the individual level.. Verbatim Evidence: "The authors aim to develop and test hypotheses that link outsourcing and subcontracting-in activities of small high-tech firms to their radical innovativeness."</t>
+        </is>
+      </c>
     </row>
     <row r="448" ht="18" customHeight="1" s="10">
       <c r="A448" t="inlineStr">
@@ -23044,6 +23170,16 @@
           <t>BSMA0445</t>
         </is>
       </c>
+      <c r="E448" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F448" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G448" t="inlineStr">
         <is>
           <t>Purpose – This paper proposes a research model in which work engagement (WE) mediates the effects of corporate social responsibility (CSR) and internal marketing (IM) simultaneously on customer-oriented boundary-spanning behavior (COBSB).</t>
@@ -23067,7 +23203,11 @@
       <c r="K448" t="n">
         <v>2022</v>
       </c>
-      <c r="P448" s="8" t="n"/>
+      <c r="P448" s="8" t="inlineStr">
+        <is>
+          <t>The paper does not provide a valid raw zero-order correlation matrix. The correlation tables (Table 2 and Table 4) are discriminant validity matrices with square roots of AVEs on the diagonal and nonsensical/squared correlations off-diagonal.. Verbatim Evidence: "Note(s): Square roots of AVEs are in italics on the diagonals"</t>
+        </is>
+      </c>
     </row>
     <row r="449" ht="18" customHeight="1" s="10">
       <c r="A449" t="inlineStr">
@@ -23080,6 +23220,16 @@
           <t>BSMA0446</t>
         </is>
       </c>
+      <c r="E449" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F449" t="inlineStr">
+        <is>
+          <t>Code 1</t>
+        </is>
+      </c>
       <c r="G449" t="inlineStr">
         <is>
           <t>Background The health-care environment requires hospital units to coordinate efforts autonomously across their boundaries and to manage relationships with other professionals, units and departments. Boundary spanning has become increasingly important for ﬁrst-line nurse managers as unit gatekeepers; however, the available measures are limited. Method The 30-item instrument was developed from a literature review. Survey participants were 4918 nurses at 231 hospital units. Statistical analyses of construct validity and internal consistency were performed. Furthermore, the correlation between nurses’ scores on the Nurse Managers Boundary Spanning Scale and nurses’ evaluations of their managers were examined. Results Three factors and 26 items were derived from factor analyses: connecting and mediating, informing and feedback utilisation, and resource acquisition. Cronbach’s subscales’ alpha coefﬁcients were above 0.9. Correlation analysis indicated that the Nurse Managers Boundary Spanning Scale score correlated with nurses’ positive perceptions of their managers. Conclusion This study demonstrates tentative support for the validity and reliability of the Nurse Managers Boundary Spanning Scale. Although further study is needed, the Nurse Managers Boundary Spanning Scale shows possibilities as a new measurement of nursing leadership. Implications This study underscores measures to build on nurse managers’ roles by building on the limited research available.</t>
@@ -23103,7 +23253,11 @@
       <c r="K449" t="n">
         <v>2016</v>
       </c>
-      <c r="P449" s="8" t="n"/>
+      <c r="P449" s="8" t="inlineStr">
+        <is>
+          <t>The paper does not provide a full zero-order Pearson correlation matrix containing Means, Standard Deviations, and intercorrelations among the study variables. It only reports a single column of correlations in Table 3.. Verbatim Evidence: "Correlation coefﬁcients between the NMBS subscales and nurses’ evaluations for nurse managers are presented in Table 3. All three subscales demonstrated signiﬁcant positive correlation coefﬁcients."</t>
+        </is>
+      </c>
     </row>
     <row r="450" ht="18" customHeight="1" s="10">
       <c r="A450" t="inlineStr">
@@ -23116,6 +23270,16 @@
           <t>BSMA0447</t>
         </is>
       </c>
+      <c r="E450" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F450" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G450" t="inlineStr">
         <is>
           <t>This study examines how cultural performance orientation moderates the influence of human resource management (HRM) controls on boundary-spanning employees' behavioural strategies and satisfaction. Based on primary data obtained from 1049 salespeople in six countries (France, Ireland, Italy, Spain, United Kingdom, and the United States of America) and secondary data on cultural performance orientation, multilevel regression analyses show that national culture has a strong effect on the way boundary-spanning employees allocate their effort in response to HRM control. In particular, our results suggest that the more behaviour controls are used with boundary-spanning employees, the less attention they pay to customers and the more emphasis they place on their supervisors and non-selling tasks. Specifically, cultural performance orientation is shown to moderate significantly those relationships. Furthermore, results indicate that cultural performance orientation heightens boundary-spanning employees' job satisfaction resulting from behaviour control. Preliminary explanations for the differing impact of HRM control efficiency across cultures can be proposed.</t>
@@ -23139,7 +23303,11 @@
       <c r="K450" t="n">
         <v>2010</v>
       </c>
-      <c r="P450" s="8" t="n"/>
+      <c r="P450" s="8" t="inlineStr">
+        <is>
+          <t>The paper empirically examines individual-level boundary-spanning employees (salespeople) and measures their boundary-spanning behavior (focus on customer). It also provides a zero-order correlation matrix that is not labeled as latent.. Verbatim Evidence: "The means, standard deviations and bivariate correlations of all the variables used in this research are presented in Table 2."</t>
+        </is>
+      </c>
     </row>
     <row r="451" ht="18" customHeight="1" s="10">
       <c r="A451" t="inlineStr">
@@ -23150,6 +23318,16 @@
       <c r="B451" t="inlineStr">
         <is>
           <t>BSMA0448</t>
+        </is>
+      </c>
+      <c r="E451" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F451" t="inlineStr">
+        <is>
+          <t>NA</t>
         </is>
       </c>
       <c r="G451" t="inlineStr">
@@ -23209,7 +23387,11 @@
       <c r="K451" t="n">
         <v>2013</v>
       </c>
-      <c r="P451" s="8" t="n"/>
+      <c r="P451" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures individual-level boundary management (segmentation) behaviors and provides a valid zero-order Pearson correlation matrix.. Verbatim Evidence: "The primary purpose of this study was to examine the role of segmentation behaviors within the work-nonwork interface... Table J1 Primary Study Correlations"</t>
+        </is>
+      </c>
     </row>
     <row r="452" ht="18" customHeight="1" s="10">
       <c r="A452" t="inlineStr">
@@ -23222,6 +23404,16 @@
           <t>BSMA0449</t>
         </is>
       </c>
+      <c r="E452" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F452" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G452" t="inlineStr">
         <is>
           <t>The involvement of customer contact personnel in the strategy process is a largely unexplored area in both marketing and strategic management. Based on social exchange theory, and in particular, the notion of trust within this context, we examine the nature and extent of strategy participation exhibited by customer contact personnel. Exploring dyadic relationships we found that the extent to which contact personnel trust their supervisors positively influence their willingness to participate in strategic activities. Furthermore, we found that communication and information sharing moderate the relationship between trust and strategic activities. Thus, the more contact personnel are involved in the strategic process, the more likely supervisors are to rate the contact person's selling performance as high.</t>
@@ -23245,7 +23437,11 @@
       <c r="K452" t="n">
         <v>2008</v>
       </c>
-      <c r="P452" s="8" t="n"/>
+      <c r="P452" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures individual-level boundary spanning behaviors (strategic activities of customer contact personnel) and contains a raw zero-order correlation matrix (Table 1) without being labeled as latent construct intercorrelations.. Verbatim Evidence: "As boundary spanners, customer contact personnel provide an important link between the organization and its customers and provide a potentially valuable source of strategic information to managers."</t>
+        </is>
+      </c>
     </row>
     <row r="453" ht="18" customHeight="1" s="10">
       <c r="A453" t="inlineStr">
@@ -23258,6 +23454,16 @@
           <t>BSMA0450</t>
         </is>
       </c>
+      <c r="E453" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F453" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G453" t="inlineStr">
         <is>
           <t>Using a sample of 89 mid-level managers in a US based urban hospital, this study investigates relationships among three measures of network centrality and managers’ divergent strategic activity. While prior work has demonstrated a relationship between managers’ boundary-spanning responsibilities and strategic activity, inadequate attention has been paid to managers’ internal network position. Drawing from established theory, we consider expected network ﬂows associated with three elements of the strategic renewal process. From this, we hypothesize and test relationships among managers’ divergent activity and three measures of network centrality. Our ﬁndings suggest speciﬁc relationships between alternative forms of network centrality and particular elements of the strategic renewal process. Consistent with existing research, the ﬁndings also show boundary-spanning managers to be more strategically active than their non-boundary-spanning counterparts.</t>
@@ -23281,7 +23487,11 @@
       <c r="K453" t="n">
         <v>2007</v>
       </c>
-      <c r="P453" s="8" t="n"/>
+      <c r="P453" s="8" t="inlineStr">
+        <is>
+          <t>The study treats boundary spanning as a nominal job role/departmental proxy (e.g., marketing vs finance) rather than a measured behavioral construct.. Verbatim Evidence: "Thus, our measure of boundary-spanning was based on functional descriptions of sub-units and formal organizational roles. ... First, consistent with Thompson (1967), the following functions were classified as boundary-spanning: direct patient care, marketing, human resource management, purchasing. Non-boundary-spanning positions included MIS, accounting, finance, and utilization review."</t>
+        </is>
+      </c>
     </row>
     <row r="454" ht="18" customHeight="1" s="10">
       <c r="A454" t="inlineStr">
@@ -23294,6 +23504,16 @@
           <t>BSMA0451</t>
         </is>
       </c>
+      <c r="E454" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F454" t="inlineStr">
+        <is>
+          <t>No Quantitative Data / Not Empirical</t>
+        </is>
+      </c>
       <c r="G454" t="inlineStr">
         <is>
           <t>Committed customers are proﬁtable to an organization for the long term. Customer commitment forms when a customer’s expectation is satisﬁed and the customer realizes fair value from his/her relationship with the organization. From an organization’s perspective, this value reﬂects customer equity, but from a customer’s perspective, it represents the customer’s perceived value of the relationship. In order to manage such a relationship successfully, it is necessary to support diverse customer information – such as of-the-customer, for-the-customer, and by-the-customer information. A customer information system (CIS) plays the role of boundary spanning that manages and distributes customer information. But the gap between marketing and IT strategy is a barrier in implementing a successful CIS. The CIS, which includes the database, communication channel, and decision model for relationship management, should be designed to facilitate the two-way customer relationship exchanges. This paper develops a framework of dynamic customer relationship management, suggests the information technology strategy to support the framework, and illustrates the applicability of such framework and strategy through a real business case.</t>
@@ -23317,7 +23537,11 @@
       <c r="K454" t="n">
         <v>2003</v>
       </c>
-      <c r="P454" s="8" t="n"/>
+      <c r="P454" s="8" t="inlineStr">
+        <is>
+          <t>The paper presents a conceptual framework and a qualitative case study of Maeil Dairy Corporation. It does not quantitatively measure individual-level boundary spanning behaviors and does not contain a correlation matrix.. Verbatim Evidence: "We can analyze the relationship value of the two different customer relationships only qualitatively since Maeil Corp. lacks transactional data about customers and there are no formal channels for monitoring their customer value"</t>
+        </is>
+      </c>
     </row>
     <row r="455" ht="18" customHeight="1" s="10">
       <c r="A455" t="inlineStr">
@@ -23330,6 +23554,16 @@
           <t>BSMA0452</t>
         </is>
       </c>
+      <c r="E455" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F455" t="inlineStr">
+        <is>
+          <t>No Correlation Matrix</t>
+        </is>
+      </c>
       <c r="G455" t="inlineStr">
         <is>
           <t>Abstract             How do boundary spanners, through processes of temporal sensemaking, use established and newly forming relationships to create value in science‐based SMEs? In addressing this question, we examine the creation of social capital arising from the activities that boundary spanners use in establishing ‘ties that bind’ people together. We show how effective boundary‐spanning activities are able to promote collaborations across scientific and related disciplines, supporting knowledge generation and innovation. Sensemaking is central to this process. We illustrate how retrospective sensemaking draws on knowledge, skills and experiences, often triggered through historical connections and personal contacts, whilst prospective sensemaking often arose in the search for new customers and in the ongoing assessment of future potential markets. We reveal how combining individual and collective boundary spanning with a continual movement between the backward glance (retrospective) and more future‐oriented (prospective) sensemaking was particularly effective in generating new understandings and opportunities. We use our findings to present an inductive model of value creation that frames the dynamic interplay between individual and collective boundary‐spanning activities and temporal sensemaking in the generation of social capital that acts as a knowledge resource for identifying and evaluating ideas for innovation and future pathways to value creation.</t>
@@ -23353,7 +23587,11 @@
       <c r="K455" t="n">
         <v>2024</v>
       </c>
-      <c r="P455" s="8" t="n"/>
+      <c r="P455" s="8" t="inlineStr">
+        <is>
+          <t>The paper is a qualitative study utilizing a grounded theory approach and semi-structured interviews. It does not contain any quantitative measures or a correlation matrix.. Verbatim Evidence: "This study draws on data from qualitative fieldwork, allowing an in-depth exploration of the phenomenon of interest. Semi-structured interviews provided the flexibility to gather rich data essential to answering our research question."</t>
+        </is>
+      </c>
     </row>
     <row r="456" ht="18" customHeight="1" s="10">
       <c r="A456" t="inlineStr">
@@ -23366,6 +23604,16 @@
           <t>BSMA0453</t>
         </is>
       </c>
+      <c r="E456" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F456" t="inlineStr">
+        <is>
+          <t>Editorial/Not Empirical</t>
+        </is>
+      </c>
       <c r="G456" t="inlineStr">
         <is>
           <t>In this editorial for our special issue on interorganizational collaboration (IOC), we position collaborative action in the context of the concurrent global crises that necessitate the bridging of interests, positions, competencies, and resources. We unpack the notion of IOC in terms of its conditions, phases, practices, and dynamics, and provide an overview of how the contributing authors support such understanding of cross-boundary collaboration. Through their action-oriented approaches to research and learning, they show a promising interplay of insight and impact. We underline their search for impact and aim to reinforce the potential of IOC not just to be successful, but also highly meaningful to address grand challenges. We therefore take a normative stance and describe how the intertwined notions of justice, resilience, and thriving can serve as a compass to legitimize, organize, facilitate, assess, and study IOC as an important pathway for the co-creation of a better world.</t>
@@ -23389,7 +23637,11 @@
       <c r="K456" t="n">
         <v>2022</v>
       </c>
-      <c r="P456" s="8" t="n"/>
+      <c r="P456" s="8" t="inlineStr">
+        <is>
+          <t>The paper is an editorial for a special issue and does not contain any empirical quantitative data or measure individual-level boundary spanning behaviors.. Verbatim Evidence: "In this editorial for our special issue on interorganizational collaboration (IOC), we position collaborative action in the context of the concurrent global crises..."</t>
+        </is>
+      </c>
     </row>
     <row r="457" ht="18" customHeight="1" s="10">
       <c r="A457" t="inlineStr">
@@ -23402,6 +23654,16 @@
           <t>BSMA0454</t>
         </is>
       </c>
+      <c r="E457" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F457" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G457" t="inlineStr">
         <is>
           <t>Multinational corporations (MNCs) need to sense, source, and mobilize knowledge when and where it arises, whether at home, or elsewhere in the world. For this reason, MNCs beneﬁt from employee networks of relationships that span across intraorganizational barriers, allowing for the eﬃcient mobilization of knowledge across boundaries. Yet, which organizational members are more likely to be able to develop these boundary spanning networks? We leverage a unique data set from a large multinational corporation to empirically test a comprehensive model that captures the eﬀect of an employee’s mandate, expertise, and behavioral orientations on her likelihood to span intraorganizational boundaries that manifest themselves in the form of hierarchies, intra-functional domains, and geographic territories. We ﬁnd that the employees that are more likely to be boundary spanners are those having mandates with a global impact, high levels of expertise, and a collaborative orientation in their networking behaviors. In addition, we ﬁnd that these eﬀects are stronger for those employees that have large formal workﬂow networks.</t>
@@ -23425,7 +23687,11 @@
       <c r="K457" t="n">
         <v>2019</v>
       </c>
-      <c r="P457" s="8" t="n"/>
+      <c r="P457" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures individual-level boundary spanning behaviors (intraorganizational boundary spanning networks) and provides a raw, zero-order correlation matrix with means and standard deviations.. Verbatim Evidence: "The correlation matrix for all variables including mean values, standard deviation, minimum and maximum values are shown in Table 1. It is noticeable that all three hypothesized variables (global impact, expert and collaborative networking orientation) have significant and positive bivariate correlations with the boundary spanning index"</t>
+        </is>
+      </c>
     </row>
     <row r="458" ht="18" customHeight="1" s="10">
       <c r="A458" t="inlineStr">
@@ -23438,6 +23704,16 @@
           <t>BSMA0455</t>
         </is>
       </c>
+      <c r="E458" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F458" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
       <c r="G458" t="inlineStr">
         <is>
           <t>Abstract: Rural journalists are news professionals, but also citizens engaged in their communities. The function and purpose of local journalism and public relations have become interdependent as media and communication has become more digital. These relationships create some tensions and it is in this environment that rural journalists make daily choices to cover a story or run prepared content provided by an outside source. Through the lens of boundary work, this study explores how (n=33) self-identifying rural journalists navigated this gray area and walked the line between creating authentic journalistic content and publishing public relations content. We found that in principle they identi ed stark boundaries between public relations and rural journalism based on journalistic norms, but in practice these journalists were often put in a position to engage in public relations work to support their communities.</t>
@@ -23461,7 +23737,11 @@
       <c r="K458" t="n">
         <v>2024</v>
       </c>
-      <c r="P458" s="8" t="n"/>
+      <c r="P458" s="8" t="inlineStr">
+        <is>
+          <t>The study is qualitative, relying on semi-structured interviews (n=33) to explore how rural journalists navigate the boundary between journalism and public relations. It contains no quantitative data or correlation matrix.. Verbatim Evidence: "Researchers analyzed data from long-form interviews (n=33) conducted in late 2020 and early 2021... Researchers transcribed the interviews and used textual analysis on the transcripts."</t>
+        </is>
+      </c>
     </row>
     <row r="459" ht="18" customHeight="1" s="10">
       <c r="A459" t="inlineStr">
@@ -23474,6 +23754,16 @@
           <t>BSMA0456</t>
         </is>
       </c>
+      <c r="E459" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F459" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G459" t="inlineStr">
         <is>
           <t>We present a view of trust in boundary spanners as explained by the extent of role autonomy, a multidimensional concept that reflects the discretion that agents have in interpreting and enacting their roles. We argue that, in a buyer-supplier context, purchasing managers will be trusted to a greater extent by supplier representatives when they are free from constraints that limit their ability to interpret their boundary-spanning roles. We conceptualize and measure three key components of role autonomy: Functional influence, tenure, and clan culture. Taken together, these components of role autonomy shape and define the purchasing manager's willingness and capacity to make and uphold commitments to supplier representatives. Role autonomy permits purchasing managers to engage in discretionary behaviors that allow supplier representatives to leam about their underlying motives and intentions. We test hypotheses linking the components of role autonomy to trust on a sample of 119 buyer-supplier relationships. We use a dyadic research design that combines data from purchasing managers and supplier representatives. The results suggest that granting purchasing managers greater autonomy enhances supplier representative trust in purchasing managers. By drawing attention to role autonomy as a feature of organizations that influences trust we highlight the importance of organizational context in contributing to a deeper understanding of trust.</t>
@@ -23497,7 +23787,11 @@
       <c r="K459" t="n">
         <v>2003</v>
       </c>
-      <c r="P459" s="8" t="n"/>
+      <c r="P459" s="8" t="inlineStr">
+        <is>
+          <t>[No measure of boundary spanning behavior] The study examines trust in boundary spanners and their role autonomy, but does not measure or report effect sizes for boundary spanning behavior itself.. Verbatim Evidence: "We are interested in understanding how the definition of the boundary-spanning role affects the degree of discretion available to the organizational agents performing those roles and the trust reposed in them."</t>
+        </is>
+      </c>
     </row>
     <row r="460" ht="18" customHeight="1" s="10">
       <c r="A460" t="inlineStr">
@@ -23510,6 +23804,16 @@
           <t>BSMA0457</t>
         </is>
       </c>
+      <c r="E460" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F460" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G460" t="inlineStr">
         <is>
           <t>Opportunism is a common issue in inter – firm relationships, which increases transaction costs, impairs firm performance and supply chain efficiency, and deteriorates relationship quality. Previous studies have intensively investigated factors influencing opportunism but overfocusing on the organisational level. Recently, supply chain researchers have called for identifying factors influencing opportunism at the individual level to gain a more comprehensive understanding of opportunism. Based on transaction cost theory, resource dependence theory, and boundary spanning theory, this study seeks to advance the emerging research stream on opportunism at the individual level by investigating how buyer agents’ boundary spanning capabilities and firms’ long – term relationship orientation can help manage supplier agents’ opportunism. Using a cross – sectional data set of 406 buyer agents from manufacturing companies collected from February to April 2021 in Japan, we tested a set of hypotheses through regression and conditional process analyses. Our findings suggest that buyer agents’ strategic communication and firms’ long – term relationship orientation are critical factors that reduce supplier agents’ opportunism.</t>
@@ -23533,7 +23837,11 @@
       <c r="K460" t="n">
         <v>2024</v>
       </c>
-      <c r="P460" s="8" t="n"/>
+      <c r="P460" s="8" t="inlineStr">
+        <is>
+          <t>The study measures individual-level boundary spanning behaviors (strategic communication capability, professional knowledge, and compromise ability) of purchasing agents. The correlation matrix is not explicitly labeled as latent construct intercorrelations and provides a standard correlation matrix with 1s on the diagonal.. Verbatim Evidence: "Table 2 presents the correlation matrix, CR, Cronbach’s α, and KMO values."</t>
+        </is>
+      </c>
     </row>
     <row r="461" ht="18" customHeight="1" s="10">
       <c r="A461" t="inlineStr">
@@ -23546,6 +23854,16 @@
           <t>BSMA0458</t>
         </is>
       </c>
+      <c r="E461" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F461" t="inlineStr">
+        <is>
+          <t>EXCL-QUAL</t>
+        </is>
+      </c>
       <c r="G461" t="inlineStr">
         <is>
           <t>This study contributes to a body of scholarship that demonstrates the benefits and need of employee-driven and defined wellness at work processes. This participatory action research study brought together a team of employees within a remote-work, start-up organization to define and design a process for implementing wellness at work for their organization. Through a participatory process that allowed outcomes to emerge from the group, employees identified opportunities to foster embodied wellness in their organization in three core areas: organizational, personal, and cross-boundary initiatives. Through a reflective collaboration, employees generated ideas and developed a plan to address employee-identified priorities that will foster wellness in their organization. What emerged from the process is a model for participatory health meaning-making called the Landscaping Wellness model that future practitioners and scholars may utilize to facilitate storytelling, idea generation, and planning processes for worker-defined wellness, thus honoring the nuanced and complex nature of wellness itself.</t>
@@ -23569,7 +23887,11 @@
       <c r="K461" t="n">
         <v>2023</v>
       </c>
-      <c r="P461" s="8" t="n"/>
+      <c r="P461" s="8" t="inlineStr">
+        <is>
+          <t>The paper is a qualitative participatory action research dissertation and does not contain quantitative zero-order correlations or measure individual-level boundary spanning behaviors.. Verbatim Evidence: "This participatory action research study brought together a team of employees within a remote-work, start-up organization to define and design a process for implementing wellness at work for their organization."</t>
+        </is>
+      </c>
     </row>
     <row r="462" ht="18" customHeight="1" s="10">
       <c r="A462" t="inlineStr">
@@ -23582,6 +23904,16 @@
           <t>BSMA0459</t>
         </is>
       </c>
+      <c r="E462" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F462" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G462" t="inlineStr">
         <is>
           <t>While behavior is influenced to a large extent by the situation in which it occurs, it is argued that consequences of engaging in boundary-spanning activity are likely to diminish the impact of the internal work setting on boundary spanners' work behavior. To assess this premise, four hypotheses are proposed regarding the mitigating effects of boundary-spanning activity on the relationship between three work setting features and a set of behaviors. Findings indicate that this relationship is weaker among spanners than among other organizational members for one of the three work-setting variables. In addition, the mitigating effects increase as the amount of boundary activity increases. These results appear limited to in-person boundary activity, as opposed to boundary interactions over the phone, and the location of the boundary activity does not appear to be a relevant factor. Implications for managers and for scholars are discussed.</t>
@@ -23605,7 +23937,11 @@
       <c r="K462" t="n">
         <v>1995</v>
       </c>
-      <c r="P462" s="8" t="n"/>
+      <c r="P462" s="8" t="inlineStr">
+        <is>
+          <t>The paper does not provide a zero-order correlation matrix (no Means, SD, and Correlations matrix). Only regression results (Exhibit 2) and select correlations are reported in the text.. Verbatim Evidence: "Results for the two regressions in the first analysis are provided in exhibit 2. Looking first at the multiple R2s from the two regressions..."</t>
+        </is>
+      </c>
     </row>
     <row r="463" ht="18" customHeight="1" s="10">
       <c r="A463" t="inlineStr">
@@ -23618,6 +23954,16 @@
           <t>BSMA0460</t>
         </is>
       </c>
+      <c r="E463" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F463" t="inlineStr">
+        <is>
+          <t>Code 99: Other - No Zero-Order Correlation Matrix</t>
+        </is>
+      </c>
       <c r="G463" t="inlineStr">
         <is>
           <t>This dissertation examined the relationships between three work setting characteristics, namely work group goals, managerial behavior, and job design, and six categories of specific job behaviors. Furthermore, the moderating effects of involvement in boundary spanning activity on the above relationship were also explored. It was hypothesized that involvement in boundary activity weakens the relationships between the work setting characteristics and behavior. A survey of 107 non-supervisory employees in two organizations provided the data for the study. Regression analysis was the primary method used to evaluate ten specific hypotheses. Major conclusions from the study include the following. First, goal characteristics are strongly related to the frequency of this set of behaviors only among boundary spanners. Second, the managerial behaviors assessed are strongly related to the frequency of these employee behaviors only among non-spanners. Third, job design is not related to the frequency of these behaviors among either group. Finally, among boundary spanners only, the degree to which their behavior can be accurately predicted from these three work setting characteristics, separately and combined, is negatively related to how much they engage in one type of boundary interaction. This final conclusion provides support for the major premise of this thesis, that involvement in boundary activity reduces the impact of an individual's work setting on his or her behavior.</t>
@@ -23641,7 +23987,11 @@
       <c r="K463" t="n">
         <v>1989</v>
       </c>
-      <c r="P463" s="8" t="n"/>
+      <c r="P463" s="8" t="inlineStr">
+        <is>
+          <t>The paper does not report a zero-order correlation matrix for Boundary Spanning. The boundary spanning measure is only correlated with regression residuals and behavioral variance scores.. Verbatim Evidence: "The correlations between the regression residuals and the amount of boundary activity are presented in Table 15. [...] The measures of amount of boundary activity were also correlated with the index of Behavioral Consistency to examine whether greater variance in behavior was associated with greater amounts of boundary activity. These correlations are presented in Table 20."</t>
+        </is>
+      </c>
     </row>
     <row r="464" ht="18" customHeight="1" s="10">
       <c r="A464" t="inlineStr">
@@ -23654,6 +24004,16 @@
           <t>BSMA0461</t>
         </is>
       </c>
+      <c r="E464" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F464" t="inlineStr">
+        <is>
+          <t>Non-Individual Anchor</t>
+        </is>
+      </c>
       <c r="G464" t="inlineStr">
         <is>
           <t>We argue in this paper that when the knowledge base of an industry is both complex and expanding and the sources of expertise are widely dispersed, the locus of innovation will be found in networks of learning, rather than in individual firms. The large-scale reliance on interorganizational collaborations in the biotechnology industry reflects a fundamental and pervasive concern with access to knowledge. We develop a network approach to organizational learning and derive firm-level, longitudinal hypotheses that link research and development alliances, experience with managing interfirm relationships, network position, rates of growth, and portfolios of collaborative activities. We test these hypotheses on a sample of dedicated biotechnology firms in the years 1990-1994. Results from pooled, within-firm, time series analyses support a learning view and have broad implications for future theoretical and empirical research on organizational networks and strategic alliances.</t>
@@ -23677,7 +24037,11 @@
       <c r="K464" t="n">
         <v>1996</v>
       </c>
-      <c r="P464" s="8" t="n"/>
+      <c r="P464" s="8" t="inlineStr">
+        <is>
+          <t>The unit of analysis is at the firm level, examining interorganizational collaborations and R&amp;D alliances among biotechnology firms, rather than individual-level boundary spanning behaviors.. Verbatim Evidence: "We test these hypotheses on a sample of dedicated biotechnology firms in the years 1990-1994."</t>
+        </is>
+      </c>
     </row>
     <row r="465" ht="18" customHeight="1" s="10">
       <c r="A465" t="inlineStr">
@@ -23690,6 +24054,16 @@
           <t>BSMA0462</t>
         </is>
       </c>
+      <c r="E465" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F465" t="inlineStr">
+        <is>
+          <t>No Correlational Data</t>
+        </is>
+      </c>
       <c r="G465" t="inlineStr">
         <is>
           <t>Purpose – Twenty-first century crises reaffirm the need of faster mobilization of resources during crises. Without interorganizational collaboration and resource mobilization, organizing efficient response is not possible. Resource mobilization is an essential aspect of response. It ensures a faster and better response. Collaboration between teams of emergency responders may include commonly known boundary spanning activities such as resource sharing, information sharing and communication. The purpose of this paper is to contribute our knowledge of how to organize a better crisis response through collaboration. More precisely, what strategies work as drivers for emergency responder teams during collaboration in crisis scenarios.</t>
@@ -23713,7 +24087,11 @@
       <c r="K465" t="n">
         <v>2021</v>
       </c>
-      <c r="P465" s="8" t="n"/>
+      <c r="P465" s="8" t="inlineStr">
+        <is>
+          <t>The paper uses an experimental design with tabletop exercises and reports Wilcoxon signed-rank tests, lacking a zero-order correlation matrix.. Verbatim Evidence: "Through design of experiments, using tabletop exercises and online surveys, this study investigates the drivers of collaboration during a crisis scenario."</t>
+        </is>
+      </c>
     </row>
     <row r="466" ht="18" customHeight="1" s="10">
       <c r="A466" t="inlineStr">
@@ -23726,6 +24104,16 @@
           <t>BSMA0463</t>
         </is>
       </c>
+      <c r="E466" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F466" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G466" t="inlineStr">
         <is>
           <t>Interpersonal interactions between boundary spanning individuals have a fundamental role in how interorganizational interactions develop. This study examines interpersonal interaction and the eﬀects of likeability on two attributes that are central to many organizations: commodity prices as negotiation outcomes and a partner's willingness to engage in collaboration. Speciﬁcally, we aim to answer: how does interpersonal likeability impact negotiation outcomes in terms of commodity prices and how does it aﬀect a partner's willingness to engage in collaboration? Based on social exchange theory we draw hypotheses that are tested using data gathered from experiments with 220 participants. The ﬁndings indicate that likeability signiﬁcantly inﬂuences a partner's willingness to engage in collaboration but does not signiﬁcantly inﬂuence negotiation proﬁts. The implications of these ﬁndings for research and practice are discussed.</t>
@@ -23749,7 +24137,11 @@
       <c r="K466" t="n">
         <v>2017</v>
       </c>
-      <c r="P466" s="8" t="n"/>
+      <c r="P466" s="8" t="inlineStr">
+        <is>
+          <t>The study measures boundary spanning behaviors (bargaining strategy) at the individual level and provides a valid matrix of raw, zero-order Pearson correlations.. Verbatim Evidence: "Table 3: Means, standard deviations, correlations and quality criteria of constructs... Pearson correlations significant at the p &lt; 0.05 level."</t>
+        </is>
+      </c>
     </row>
     <row r="467" ht="18" customHeight="1" s="10">
       <c r="A467" t="inlineStr">
@@ -23762,6 +24154,16 @@
           <t>BSMA0464</t>
         </is>
       </c>
+      <c r="E467" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F467" t="inlineStr">
+        <is>
+          <t>NOT_EMPIRICAL</t>
+        </is>
+      </c>
       <c r="G467" t="inlineStr">
         <is>
           <t>The disciplinary backgrounds of leadership studies educators have considerable influence on the future of the field; however, disciplinary expertise and credentialing have yet to be examined thoroughly in the literature. Decisions pertaining to the preparation and credentialing of leadership educators, particularly among faculty, are a necessary supplement to existing discourse on the standardization of academic programs and the aim and scope of scholarship privileged within the field. While disciplinary boundaries are permeable and fluid, the organizational boundaries defined within institutions based on disciplinary affiliation impose specific expectations and limitations that may artificially constrain interdisciplinary pursuits, including those within leadership studies. The current article presents a conceptualization of how disciplinary expertise and faculty credentialing may shape the future of leadership studies. It is recommended that leadership studies faculty cultivate program‐level consensus, demonstrate the integrity of leadership studies curricula, enhance interdisciplinary legitimacy through boundary spanning, determine the future trajectory of leadership studies, and set the course accordingly.</t>
@@ -23785,7 +24187,11 @@
       <c r="K467" t="n">
         <v>2023</v>
       </c>
-      <c r="P467" s="8" t="n"/>
+      <c r="P467" s="8" t="inlineStr">
+        <is>
+          <t>The paper is a conceptual article discussing disciplinary expertise and faculty credentialing in leadership studies. It does not measure individual-level boundary spanning behaviors, nor does it contain a quantitative correlation matrix.. Verbatim Evidence: "The current article presents a conceptualization of how disciplinary expertise and faculty credentialing may shape the future of leadership studies."</t>
+        </is>
+      </c>
     </row>
     <row r="468" ht="18" customHeight="1" s="10">
       <c r="A468" t="inlineStr">
@@ -23798,6 +24204,16 @@
           <t>BSMA0465</t>
         </is>
       </c>
+      <c r="E468" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F468" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G468" t="inlineStr">
         <is>
           <t>The purpose of this paper is to advance and empirically investigate how perceived organisational support inﬂuences marketing managers’ boundary-spanning marketing activities (cross-functional communication and customer connections), and how these activities subsequently impact supply-chain efﬁciency. By analysing survey responses from 348 marketing managers, we demonstrate that a supportive organisational climate provides managerial incentives not only to develop strong allegiance to the welfare of multi-foci groups within the organisation but also to engage in active cross-functional market intelligence exchange and customer servicing, which in turn leads to superior supply-chain efﬁciencies. The paper offers strategic guides to both academicians and practitioners on how to promote marketing managers’ role in strengthening dependencies among various functional departments for cohesive product, service, and ﬁnancial offerings.</t>
@@ -23821,7 +24237,11 @@
       <c r="K468" t="n">
         <v>2012</v>
       </c>
-      <c r="P468" s="8" t="n"/>
+      <c r="P468" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures individual-level boundary spanning behaviors (marketing managers' cross-functional market intelligence exchange and customer accommodation) and provides a zero-order correlation matrix of summated indices.. Verbatim Evidence: "The items corresponding to each construct/dimension were summed and averaged in order to obtain a summated index. The summary statistics are reported for this index."</t>
+        </is>
+      </c>
     </row>
     <row r="469" ht="18" customHeight="1" s="10">
       <c r="A469" t="inlineStr">
@@ -23834,6 +24254,16 @@
           <t>BSMA0466</t>
         </is>
       </c>
+      <c r="E469" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F469" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G469" t="inlineStr">
         <is>
           <t>Creative idea generation does not necessarily lead to the implementation of these ideas. Although the conditional relationship between creative idea generation and implementation has frequently been recognized, there have been few studies of the moderating factors that facilitate converting creative ideas into tangible innovations. To fill this research gap, we explore whether leader performance-prove goal orientation facilitates the implementation of creative ideas at the team level. Furthermore, we investigate the mediating role of leader comprehensive boundary-spanning strategy in the moderating effect of leader performance-prove goal orientation. From an analysis of data from 83 new product development (NPD) teams, we find the following: (1) Leader performance-prove goal orientation positively moderates the relationship between idea generation and implementation. (2) Leader ambassadorial activities and task coordination both positively moderate the relationship between idea generation and implementation. (3) The moderating role of leader performance-prove goal orientation is mediated by leader ambassadorial activities. Our findings have theoretical and practical implications for innovation management in NPD teams.</t>
@@ -23857,7 +24287,11 @@
       <c r="K469" t="n">
         <v>2021</v>
       </c>
-      <c r="P469" s="8" t="n"/>
+      <c r="P469" s="8" t="inlineStr">
+        <is>
+          <t>Paper measures individual leader boundary-spanning behaviors and provides a valid zero-order correlation matrix.. Verbatim Evidence: "Following Ancona and Caldwell (1992), we used the self-evaluation method to ask team leaders to evaluate their level of boundary-spanning behaviors."</t>
+        </is>
+      </c>
     </row>
     <row r="470" ht="18" customHeight="1" s="10">
       <c r="A470" t="inlineStr">
@@ -23870,6 +24304,16 @@
           <t>BSMA0467</t>
         </is>
       </c>
+      <c r="E470" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F470" t="inlineStr">
+        <is>
+          <t>Wrong level of analysis</t>
+        </is>
+      </c>
       <c r="G470" t="inlineStr">
         <is>
           <t>This study constructs a theoretical model to test and prove that organizational forgetting influences cross-boundary innovation and testifies to the moderating role of Institutionalized organizational mission in the said relationship. Data was collected through a convenient sampling technique from 353 middle and senior managers of entrepreneurial enterprises in China through online and offline modes. Additionally, we used confirmatory factor analysis, multiple regression, and bootstrap analysis to verify hypotheses using Analysis of a moment structures and Statistical Package for the Social Sciences latest versions. The results show that organizational forgetting has a significantly positive impact on cross-boundary innovation and binary knowledge sharing plays a mediating role in the relationship between organizational forgetting and cross-boundary innovation. Moreover, the mediating effect of exploitative knowledge sharing on the relationship between organizational forgetting and cross-boundary innovation is more substantial than exploratory knowledge sharing. This study separates the impact mechanism of exploitative and exploratory knowledge sharing as a mediator unanimously and proves that Institutionalized organizational mission has a significant moderating role in the relationship between organizational forgetting and cross-boundary innovation. This research offers significant implications for Chinese enterprises to bolster cross-boundary innovation to achieve growth.</t>
@@ -23893,7 +24337,11 @@
       <c r="K470" t="n">
         <v>2022</v>
       </c>
-      <c r="P470" s="8" t="n"/>
+      <c r="P470" s="8" t="inlineStr">
+        <is>
+          <t>The boundary spanning construct (cross-boundary innovation) is measured at the organizational/firm level rather than the individual level. Furthermore, the reported correlation matrix uses latent construct intercorrelations for discriminant validity (Fornell-Larcker criterion) rather than raw zero-order correlations.. Verbatim Evidence: "This research is about learning and innovation at the enterprise level... CBI1. The firm often introduces elements from different fields to improve the operating conditions of related businesses"</t>
+        </is>
+      </c>
     </row>
     <row r="471" ht="18" customHeight="1" s="10">
       <c r="A471" t="inlineStr">
@@ -23906,6 +24354,16 @@
           <t>BSMA0468</t>
         </is>
       </c>
+      <c r="E471" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F471" t="inlineStr">
+        <is>
+          <t>No Correlation Matrix</t>
+        </is>
+      </c>
       <c r="G471" t="inlineStr">
         <is>
           <t>Changing workforce demographics and advanced information communication technologies (ICT) have created new challenges for employers striving to remain competitive. To address these challenges, employers have focused efforts on attracting and retaining quality employees by offering flexible work arrangements. Boundary management strategy (BMS) has emerged as a theoretical framework for understanding work-arrangement preferences and achieving a more effective person-organization fit.</t>
@@ -23929,7 +24387,11 @@
       <c r="K471" t="n">
         <v>2018</v>
       </c>
-      <c r="P471" s="8" t="n"/>
+      <c r="P471" s="8" t="inlineStr">
+        <is>
+          <t>The study employs a 2x2 factorial quasi-experimental ANOVA design and does not report a zero-order correlation matrix.. Verbatim Evidence: "This quasi-experimental study consisted of a 2 X 2 factorial design... A two-way ANOVA was conducted to determine whether there was a statistically significant difference in applicant attraction to a job that offers a TelWA or a StdWA, depending on whether participants prefer an integration or segmentation boundary management strategy."</t>
+        </is>
+      </c>
     </row>
     <row r="472" ht="18" customHeight="1" s="10">
       <c r="A472" t="inlineStr">
@@ -23942,6 +24404,16 @@
           <t>BSMA0469</t>
         </is>
       </c>
+      <c r="E472" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F472" t="inlineStr">
+        <is>
+          <t>Wrong Level of Analysis</t>
+        </is>
+      </c>
       <c r="G472" t="inlineStr">
         <is>
           <t>How do leaders of established organizations effectively manage intrafirm entrepreneurial groups so that they can be successful? Focusing on drivers of breakthrough groups’ performance and radical innovation, this research identifies drivers and proposes a multifaceted model providing a pathway for breakthrough business growth in an organically driven mode. The corporate entrepreneurship (CE) and innovation management literature, while helpful in describing the difficulty associated with leading CE and ambidextrous organizations, are focused on wider structural or behavioral solutions to address ambidexterity challenges and product innovation, omitting the unit of analysis—the group/team—and the drivers that influence groups’ breakthrough innovation and performance aims in a contemporary context in which organizations’ business models can change in the blink of an eye. Using a QUAN→ qual design, the research follows aninside-out logic’to account for the position of each introduced construct in the nomological network, which include (1) intragroup mechanisms;(2) team boundary mechanisms (boundary buffering and spanning);(3) environmental mechanisms including senior management communication, incentives, proactive IT stance; and,(4) contextual influences. The prevalence of a mismatch between conventional incentives vis-a-vis team members’ breakthrough pursuits is also investigated. Findings reveal a paradox around top management communication, as well as the mediating roles of team buffering and spanning on the relationship between relational climate and outcome variables, radical innovation, and team performance. Overall, results suggest that that just having a top team (ie, good relational climate) is not enough for breakthrough performance, and could be for naught should the team’s boundaries not be managed by leaders as to create buffering (from extra-team interference) and spanning (or access to resources) beyond the team. Environmental mechanisms, and particularly proactive IT capabilities and nuanced senior management communication, also matter when it comes to teams’ success. It is hoped that this work, comprising novel constructs and a unique team focus in the context of breakthrough innovation and corporate entrepreneurship, will help drive the two streams of research into new directions.</t>
@@ -23965,7 +24437,11 @@
       <c r="K472" t="n">
         <v>2021</v>
       </c>
-      <c r="P472" s="8" t="n"/>
+      <c r="P472" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures boundary spanning at the team/group level, not the individual level.. Verbatim Evidence: "My unit of analysis is the entrepreneurial group pursuing radical innovation initiatives... Therefore, the unit of analysis is the cross-functional group."</t>
+        </is>
+      </c>
     </row>
     <row r="473" ht="18" customHeight="1" s="10">
       <c r="A473" t="inlineStr">
@@ -23978,6 +24454,16 @@
           <t>BSMA0470</t>
         </is>
       </c>
+      <c r="E473" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F473" t="inlineStr">
+        <is>
+          <t>Non-Individual Anchors</t>
+        </is>
+      </c>
       <c r="G473" t="inlineStr">
         <is>
           <t>This study investigated the communication behaviors and performances of 50 R&amp;D project groups that varied in terms of group longevity, as measured by the average length of time project members had worked together. Analyses revealed that project groups became increasingly isolated from key information sources both within and outside their organizations with increasing stability in project membership. Such reductions in project communication were also shown to affect adversely the technical performance of project groups. Furthermore, variations in communication activities were more associated with the tenure composition of project groups than with the project tenures of individual engineers. These findings are presented and discussed in the more general terms of what happens in project groups with increasing group longevity.</t>
@@ -24001,7 +24487,11 @@
       <c r="K473" t="n">
         <v>1982</v>
       </c>
-      <c r="P473" s="8" t="n"/>
+      <c r="P473" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures project communication at the group level (N=50 project groups) rather than the individual level.. Verbatim Evidence: "This study investigated the communication behaviors and performances of 50 R&amp;D project groups that varied in terms of group longevity..."</t>
+        </is>
+      </c>
     </row>
     <row r="474" ht="18" customHeight="1" s="10">
       <c r="A474" t="inlineStr">
@@ -24014,6 +24504,16 @@
           <t>BSMA0471</t>
         </is>
       </c>
+      <c r="E474" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F474" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G474" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this research is to explore how ﬁrm market orientation, as a culture, affects the service climate that develops in the ﬁrm. Design/methodology/approach – Empirical testing is performed at the managerial level and boundary-spanning employee level as part of this multilevel study. The sample includes participants from a US-based ﬁrm operating in the hospitality industry.</t>
@@ -24037,7 +24537,11 @@
       <c r="K474" t="n">
         <v>2014</v>
       </c>
-      <c r="P474" s="8" t="n"/>
+      <c r="P474" s="8" t="inlineStr">
+        <is>
+          <t>Paper measures individual-level boundary spanning flexibility (adaptive selling) and provides a raw, zero-order correlation matrix (Means, SD, and Correlations).. Verbatim Evidence: "Table I Descriptive statistics, reliabilities and correlations of study variables"</t>
+        </is>
+      </c>
     </row>
     <row r="475" ht="18" customHeight="1" s="10">
       <c r="A475" t="inlineStr">
@@ -24050,6 +24554,16 @@
           <t>BSMA0472</t>
         </is>
       </c>
+      <c r="E475" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F475" t="inlineStr">
+        <is>
+          <t>No Boundary Spanning Measure</t>
+        </is>
+      </c>
       <c r="G475" t="inlineStr">
         <is>
           <t>Software professionals perform boundary-spanning activities, and thus need strong interpersonal, technical, and organizational knowledge to be professionally competent. They have to perform in a demanding work environment characterized by strict deadlines, differing time zones, interdependency in teams, increased interaction with clients, and extended work hours. These characteristics lead to occupational stress and work exhaustion. Yet, the impact of stress is felt in different ways by different people, even if they perform the same functions. These differences in the perception of stress can be caused by varying confidence in their technical capabilities. People possess varying technical capabilities, based on their acquisition of technical skills, comfort level in using the technology, and intrinsic motivation. These attributes represent the human-computer interaction (HCI) personality of software professionals. This article examines whether these HCI factors moderate the relationship between occupational stress and work exhaustion. Data were collected from software professionals located in Chennai and Bangalore in India. The data revealed that HCI factors had a main effect but no significant moderating effects on work exhaustion. The control over the technology variable emerged as the key variable among the HCI factors that affected software professionals' ability to cope with stress and work exhaustion.</t>
@@ -24073,7 +24587,11 @@
       <c r="K475" t="n">
         <v>2005</v>
       </c>
-      <c r="P475" s="8" t="n"/>
+      <c r="P475" s="8" t="inlineStr">
+        <is>
+          <t>The paper does not measure any individual-level boundary spanning behaviors. The variables measured focus on human-computer interaction factors, occupational stress, and work exhaustion.. Verbatim Evidence: "The main objective of this article is to explore the concomitant role of the HCI variables such as CSE, technology-training efficacy, perceived control over technology, and intrinsic motivation as moderators in the relationship between occupational stress and work exhaustion among software professionals."</t>
+        </is>
+      </c>
     </row>
     <row r="476" ht="18" customHeight="1" s="10">
       <c r="A476" t="inlineStr">
@@ -24086,6 +24604,16 @@
           <t>BSMA0473</t>
         </is>
       </c>
+      <c r="E476" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F476" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G476" t="inlineStr">
         <is>
           <t>Contrary to much boundary spanning research, we examined the negative consequences of boundary spanning contact in multi-organizational contexts. Results from a sample of 833 Dutch peacekeepers show that employees’ boundary spanning contact with members of other organizations was associated with reports of negative relationships with external parties (e.g., work-speciﬁc problems, culture-speciﬁc problems). These negative relationships also had a spillover effect such that they mediated the effect of boundary spanning contact on boundary spanners’ negative attitudes toward their own jobs and organization (e.g., job attractiveness and conﬁdence in the organization). Copyright # 2010 John Wiley &amp; Sons, Ltd.</t>
@@ -24109,7 +24637,11 @@
       <c r="K476" t="n">
         <v>2011</v>
       </c>
-      <c r="P476" s="8" t="n"/>
+      <c r="P476" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures individual-level boundary spanning behaviors (frequency of boundary-spanning contact with members of other organizations) and provides a clear zero-order correlation matrix (Table 1) containing means, standard deviations, and raw correlations without any indication of latent construct intercorrelations.. Verbatim Evidence: "Since we were interested in all instances of employees' inter-organizational contact, we operationalized this variable as frequency of boundary-spanning contact between peacekeepers and members of other organizations such as NGOs, inter-governmental organizations, and local authorities... Table 1. Means, standard deviations, and correlations between variables"</t>
+        </is>
+      </c>
     </row>
     <row r="477" ht="18" customHeight="1" s="10">
       <c r="A477" t="inlineStr">
@@ -24122,6 +24654,16 @@
           <t>BSMA0474</t>
         </is>
       </c>
+      <c r="E477" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F477" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G477" t="inlineStr">
         <is>
           <t>Boundary-spanning activities were studied in 15 organizations engaged in basic and applied research. Included in the study were 281 scientists and engineers. Contrary to prior theory and research, this study found bound-ary-spanning activities to be unrelated to job satisfaction. It was strongly related to perceptions of research and development team collaboration, job motivation, task uncertainty, locus of control, team cohesiveness, and individualproductivity. The research reported here makes a strong case for including group processes and characteristics in future studies involving boundary-spanning activities. The results also give increased impetus to re-search which examines the relationships between boundary-spanning activi-ties and individual productivity.</t>
@@ -24145,7 +24687,11 @@
       <c r="K477" t="n">
         <v>1979</v>
       </c>
-      <c r="P477" s="8" t="n"/>
+      <c r="P477" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures individual-level boundary spanning activities and provides zero-order Pearson correlations between BSA and other variables in Table I.. Verbatim Evidence: "Boundary-Spanning Activities (BSA). A four-item BSA scale based on the work of Keller et al. (1976) was used to assess boundary spanning in this study. [...] Table I. Pearson Product Moment Correlations Between Predictor and Boundary-Spanning Activity (BSA)"</t>
+        </is>
+      </c>
     </row>
     <row r="478" ht="18" customHeight="1" s="10">
       <c r="A478" t="inlineStr">
@@ -24158,6 +24704,16 @@
           <t>BSMA0475</t>
         </is>
       </c>
+      <c r="E478" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F478" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G478" t="inlineStr">
         <is>
           <t>A review of previous studies on the relationship between boundary spanning activity and environment indicates that the full effects of environment have not been investigated due to the restricted representation of environmental effects. In addition, we argue that the boundary spanning-environment relationship may be moderated by function, hierarchical level, perceived influence, size, and industry. Accordingly, an enlarged model of the boundary spanning-environment relationship is tested in both the high-technology electronics industry and the wood products industry. Results indicate that boundary spanning activity is related to environment, but this relationship appears to vary along dimensions of environment as well as by industry. In addition, size, perceived influence, and function are found to moderate the boundary spanning-environment relationship. Implications for further studies include a reconceptualization of the boundary spanning-environment relationship based on the findings.</t>
@@ -24181,7 +24737,11 @@
       <c r="K478" t="n">
         <v>1985</v>
       </c>
-      <c r="P478" s="8" t="n"/>
+      <c r="P478" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures individual-level boundary spanning behaviors and provides a valid zero-order correlation matrix.. Verbatim Evidence: "Boundary spanning was measured using Miles' (1980) set of eight boundary spanning activities... The upper right-hand matrix consists of zero-order correlations for the wood products sample (n = 92); the lower left-hand matrix consists of zero-order correlations for the high-technology electronics sample (n = 278)."</t>
+        </is>
+      </c>
     </row>
     <row r="479" ht="18" customHeight="1" s="10">
       <c r="A479" t="inlineStr">
@@ -24194,6 +24754,16 @@
           <t>BSMA0476</t>
         </is>
       </c>
+      <c r="E479" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F479" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G479" t="inlineStr">
         <is>
           <t>Viewing knowledge as rooted in individuals, this study investigates knowledge transfer in multinational corporations (MNCs) from an individual-level perspective. Speciﬁcally, the author focuses on inpatriates as a particular group of knowledge actors in MNCs and examines the role of inpatriates’ boundary spanning between their home unit and the headquarters for transferring their knowledge to headquarters staff. Based on a sample of 269 inpatriates in 10 German MNCs, the author found that inpatriates’ boundary spanning is positively related to inpatriates’ individual efforts to transfer knowledge and inpatriates’ perceptions of HQ staff efforts to acquire subsidiary-speciﬁc knowledge. Both perceived HQ absorptive capacity and mentoring by HQ staff moderate these relationships.This study’s ﬁndings contribute to our understanding of the theoretical mechanisms through which MNC knowledge ﬂows occur and highlight key requirements for the design of international stafﬁng practices. © 2011 Wiley Periodicals, Inc.</t>
@@ -24217,7 +24787,11 @@
       <c r="K479" t="n">
         <v>2011</v>
       </c>
-      <c r="P479" s="8" t="n"/>
+      <c r="P479" s="8" t="inlineStr">
+        <is>
+          <t>The study measures individual-level boundary spanning ('Inpatriates' boundary spanning') and provides a raw, zero-order correlation matrix (Table II).. Verbatim Evidence: "Table II Means, Standard Deviations, and Correlations"</t>
+        </is>
+      </c>
     </row>
     <row r="480" ht="18" customHeight="1" s="10">
       <c r="A480" t="inlineStr">
@@ -24230,6 +24804,16 @@
           <t>BSMA0477</t>
         </is>
       </c>
+      <c r="E480" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F480" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G480" t="inlineStr">
         <is>
           <t>Examined relationships between major role requirements and experienced role stress, using data from 202 research and development professionals. Measures (including those of JR Rizzo et al, 1970) of role stress included various types of role conflict and ambiguity. Role requirements included integration and boundary-spanning activities, personnel supervision, and scientific research. Role conflict was more sensitive than role ambiguity to differences in research and development role requirements; and integration and boundary-spanning activities were the best predictors of experienced role conflict, especially of the intersender variety.</t>
@@ -24253,7 +24837,11 @@
       <c r="K480" t="n">
         <v>1976</v>
       </c>
-      <c r="P480" s="8" t="n"/>
+      <c r="P480" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures individual-level boundary-spanning activities and provides raw, zero-order correlations with role stress variables.. Verbatim Evidence: "A correlational analysis of relationships between the role stress and role requirement variables provides support for the hypotheses (see Table 4)."</t>
+        </is>
+      </c>
     </row>
     <row r="481" ht="18" customHeight="1" s="10">
       <c r="A481" t="inlineStr">
@@ -24266,6 +24854,16 @@
           <t>BSMA0478</t>
         </is>
       </c>
+      <c r="E481" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F481" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G481" t="inlineStr">
         <is>
           <t>We examined the relationship between group boundary spanners' work group identification and effective (i. E., harmonious and productive) intergroup relations in 53 work groups in five health care organizations. The data suggest this relationship was moderated by boundary spanners' levels of organizational identification, thus supporting a dual identity model. Limited support was found for the moderating effect of intergroup contact. Finally, if boundary spanners displayed frequent intergroup contact and identified highly with their organization, group identification was most strongly related to effective intergroup relations.</t>
@@ -24289,7 +24887,11 @@
       <c r="K481" t="n">
         <v>2006</v>
       </c>
-      <c r="P481" s="8" t="n"/>
+      <c r="P481" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures boundary spanning behaviors at the individual level (intergroup contact) and reports raw, zero-order correlations in a standard matrix.. Verbatim Evidence: "As both identification constructs and intergroup-contact were individual-level, responses were not aggregated."</t>
+        </is>
+      </c>
     </row>
     <row r="482" ht="18" customHeight="1" s="10">
       <c r="A482" t="inlineStr">
@@ -24302,6 +24904,16 @@
           <t>BSMA0479</t>
         </is>
       </c>
+      <c r="E482" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F482" t="inlineStr">
+        <is>
+          <t>Team-Level Boundary Spanning</t>
+        </is>
+      </c>
       <c r="G482" t="inlineStr">
         <is>
           <t>Claims have been recently made for a seven‐factor model that ndifferentiated performance levels in project teams. We have tested the model with results from a self‐report inventory. Forty‐four opportunities for data collection were taken and a total of 1103 useable inventories collected from participants across European, Asian and African locations. Teams reported on were predominantly work‐related. All seven factors correlate as predicted with leadership and team‐performance criteria. We report results supporting the original proposition that team effectiveness, including its creativity, can be interpreted as arising through leadership interventions of a transformational kind, which impact on a set of theoretically‐derived team factors.</t>
@@ -24325,7 +24937,11 @@
       <c r="K482" t="n">
         <v>2001</v>
       </c>
-      <c r="P482" s="8" t="n"/>
+      <c r="P482" s="8" t="inlineStr">
+        <is>
+          <t>The boundary spanning measure (Network activators) is a team-level construct, not an individual-level construct.. Verbatim Evidence: "In its current format, the inventory collects self-reports on seven sets of three items for the seven team factors."</t>
+        </is>
+      </c>
     </row>
     <row r="483" ht="18" customHeight="1" s="10">
       <c r="A483" t="inlineStr">
@@ -24338,6 +24954,16 @@
           <t>BSMA0480</t>
         </is>
       </c>
+      <c r="E483" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F483" t="inlineStr">
+        <is>
+          <t>No Correlation Matrix</t>
+        </is>
+      </c>
       <c r="G483" t="inlineStr">
         <is>
           <t>This study examined the transdisciplinary area of cognitive science, and was framed around the sociological notion of the boundary object. Harmonizing theoretical and technical approaches, methods introduced in this work moved beyond qualitative study practices traditional to boundary object theory work to a mixed-methods data-driven approach. Bibliometric Web of Science data, enriched with National Science Foundation (NSF) journal classifications, formed the foundation from which a seed-and-expand dataset were created from journals containing the string cogni* and their cited articles for the years 2006–2016. This two-tiered dataset allowed for the analysis of boundary-spanning interdisciplinary concepts, as identified by noun phrases, and their inhabitance within the intellectual space of the NSF taxonomy. The most interdisciplinary concepts were analyzed for their conceptual periphera using term co-occurrences, and the underlying sociological structures of co-authorship. Two concepts met the criterion of publication in all six core-level NSF disciplines resulted in two for this analysis:" children's," and" case study." Clearer clusters of term co-occurrences were present for" children's" than were for" case study," demonstrating the conceptual periphera. The underlying social structures for" children's" were more interconnected than those for" case study." The findings of this study suggest that different types of research problems, in conjunction with the methodology used to explore them, may be more useful to pinpoint boundary-inhabiting interdisciplinary epistemologies and other conceptual phenomena than the examination of broadly defined boundary-spanning concepts alone.</t>
@@ -24361,7 +24987,11 @@
       <c r="K483" t="n">
         <v>2020</v>
       </c>
-      <c r="P483" s="8" t="n"/>
+      <c r="P483" s="8" t="inlineStr">
+        <is>
+          <t>The paper is a bibliometric dissertation analyzing interdisciplinary concepts and co-authorship networks. It does not contain an empirical, quantitative study with a zero-order correlation matrix.. Verbatim Evidence: "This study examined the transdisciplinary area of cognitive science, and was framed around the sociological notion of the boundary object... Bibliometric Web of Science data, enriched with National Science Foundation (NSF) journal classifications, formed the foundation from which a seed-and-expand dataset were created"</t>
+        </is>
+      </c>
     </row>
     <row r="484" ht="18" customHeight="1" s="10">
       <c r="A484" t="inlineStr">
@@ -24374,6 +25004,16 @@
           <t>BSMA0481</t>
         </is>
       </c>
+      <c r="E484" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F484" t="inlineStr">
+        <is>
+          <t>No Quantitative Data</t>
+        </is>
+      </c>
       <c r="G484" t="inlineStr">
         <is>
           <t>Qualitative evidence from an action research study is used to address the research question ‘how can institutional context help explain frustrations within local collaborations?’ This study of multi-agency collaboration for local economic strategy in Ireland ﬁnds that individual and organization actions at a local level are substantially shaped along paths structured by funding and performance management arrangements of multiple central government departments. The article concludes that any calls for greater collaboration at a local level will produce limited effects without a simultaneous scrutiny of crossboundary working at the centre.</t>
@@ -24397,7 +25037,11 @@
       <c r="K484" t="n">
         <v>2013</v>
       </c>
-      <c r="P484" s="8" t="n"/>
+      <c r="P484" s="8" t="inlineStr">
+        <is>
+          <t>The paper is a qualitative action research study using an ethnographic approach and does not provide quantitative data or a correlation matrix.. Verbatim Evidence: "An ethnographic approach dominated (Gray, 2009), in which much of the research material collected consisted of extensive observational notes and quotes recorded verbatim in the course of regular ESP and sub-group meetings"</t>
+        </is>
+      </c>
     </row>
     <row r="485" ht="18" customHeight="1" s="10">
       <c r="A485" t="inlineStr">
@@ -24410,6 +25054,16 @@
           <t>BSMA0482</t>
         </is>
       </c>
+      <c r="E485" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F485" t="inlineStr">
+        <is>
+          <t>NO_BS_MEASURE</t>
+        </is>
+      </c>
       <c r="G485" t="inlineStr">
         <is>
           <t>Previous research demonstrates the destructive consequences of role stress for the work outcomes of employees occupying boundary-spanning positions. Most studies examine the behavior and performance of industrial salespeople. In contrast, limited evidence exists regarding the antecedents and consequences of role stress in service organizations. This article helps fill this notable gap by investigating the correlates of role ambiguity in the context of frontline managers in banking institutions. The article offers a conceptual model and an empirical test using data gathered from 316 bank branch managers. The study findings reveal that information control is an effective mechanism for reducing role ambiguity. The results also indicate that role ambiguity negatively affects job performance and job satisfaction, intrinsic motivation positively relates to job satisfaction, and bank managers' job performance enhances branch effectiveness. The article concludes with a discussion of study implications and suggestions for future research in the field.</t>
@@ -24433,7 +25087,11 @@
       <c r="K485" t="n">
         <v>2012</v>
       </c>
-      <c r="P485" s="8" t="n"/>
+      <c r="P485" s="8" t="inlineStr">
+        <is>
+          <t>The paper surveys employees in boundary-spanning positions (bank branch managers) but does not actually measure any individual-level boundary spanning behaviors. The variables measured are information control, role ambiguity, intrinsic motivation, job satisfaction, and performance.. Verbatim Evidence: "This study develops a broad conceptual framework that examines interrelationships among information control, role ambiguity, intrinsic motivation, job outcomes, and organizational effectiveness and offers an empirical test for a structural model using data collected from bank branch managers."</t>
+        </is>
+      </c>
     </row>
     <row r="486" ht="18" customHeight="1" s="10">
       <c r="A486" t="inlineStr">
@@ -24446,6 +25104,16 @@
           <t>BSMA0483</t>
         </is>
       </c>
+      <c r="E486" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F486" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G486" t="inlineStr">
         <is>
           <t>As firms experience relentless pressure to innovate and improve, many are responding by creating organizational structures that promote cross‐functional and cross‐boundary communication, coordination, and collaboration. Because most firms studied expect to use teams to support future procurement and sourcing decision making, it is important to understand how to best manage the cross‐functional sourcing team process. Unfortunately, researchers who study teams rarely reach the same conclusions about the factors affecting team success. There is one variable, however, that most researchers agree consistently affects team success — the effectiveness of the formal team leader.
@@ -24470,7 +25138,11 @@
       <c r="K486" t="n">
         <v>1996</v>
       </c>
-      <c r="P486" s="8" t="n"/>
+      <c r="P486" s="8" t="inlineStr">
+        <is>
+          <t>The paper is a conceptual piece describing team leadership requirements and presents assessment scales without providing a correlation matrix or quantitative results.. Verbatim Evidence: "The purpose of this article is to examine the critical role that team leaders play and the challenges they face in a cross-functional sourcing team environment."</t>
+        </is>
+      </c>
     </row>
     <row r="487" ht="18" customHeight="1" s="10">
       <c r="A487" t="inlineStr">
@@ -24483,6 +25155,16 @@
           <t>BSMA0484</t>
         </is>
       </c>
+      <c r="E487" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F487" t="inlineStr">
+        <is>
+          <t>No Correlation Matrix</t>
+        </is>
+      </c>
       <c r="G487" t="inlineStr">
         <is>
           <t>For years many researchers and practitioners have been calling for a more boundary-spanning or cross-functional view of the management of businesses. As any student of optimization will note, the combination of several optimized sub-systems will rarely, if ever, result in a globally optimized system. It is much the same with a business. Decisions that may appear extremely good within the confines of a single organizational area are often clearly dysfunctional when viewed from other areas of the organization. To effectively compete in today's marketplace, firms need to effectively link their diverse functional areas. This article provides an example of how the marketing, operations, and purchasing areas can be effectively linked to accomplish the common goal of effectively competing in the value market segment of consumer goods and services.</t>
@@ -24506,7 +25188,11 @@
       <c r="K487" t="n">
         <v>1995</v>
       </c>
-      <c r="P487" s="8" t="n"/>
+      <c r="P487" s="8" t="inlineStr">
+        <is>
+          <t>The paper is a conceptual and mathematical modeling study on the integration of marketing, operations, and purchasing at the organizational level. It does not measure individual-level boundary spanning behaviors and does not contain an empirical correlation matrix.. Verbatim Evidence: "The purpose of this paper is to identify and demonstrate how an integrated approach to marketing, operations, and purchasing can provide opportunities for a firm to lower costs and increase sales of products and services in the value market segment."</t>
+        </is>
+      </c>
     </row>
     <row r="488" ht="18" customHeight="1" s="10">
       <c r="A488" t="inlineStr">
@@ -24519,6 +25205,16 @@
           <t>BSMA0485</t>
         </is>
       </c>
+      <c r="E488" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F488" t="inlineStr">
+        <is>
+          <t>Non-Individual Level</t>
+        </is>
+      </c>
       <c r="G488" t="inlineStr">
         <is>
           <t>In spite of increasing research attention given to individual creativity and organizational innovation, there are comparatively few studies investigating innovation in work groups. This is unfortunate given the increased use of groups to perform work in organizations. This dissertation addresses some of the inadequacies in the current literature by developing and testing a model of innovation in ongoing, task-performing work groups. The theoretical model uses an input-process-output framework common to group research. The input portion of the model is individual innovativeness. The group process portion of the model is group support for innovation. The output portion of the model is group innovation. Group support for innovation was expected to mediate the influence of individual innovativeness on group innovation. Expectancy theory is used to explain the hypothesized relationships of group support for innovation with group innovative potency, group scouting, group psychological safety, and group innovation encouragement norms. This dissertation used a cross-sectional design in a field setting. Surveys were given to group members and their supervisors in two organizations. Thirty-three work groups were used in the study. Hierarchical regression was used to test the hypotheses. Among the main findings was that group support for innovation was positively associated with group innovation quantity and quality. Group innovative potency and supervisor support were both positively associated with group support for innovation. Constructive controversy moderated the relationship between group support for innovation and group innovation quantity. Contrary to expectations, the relationship between group support for innovation and innovation was stronger when constructive controversy was low than when it was high. The findings, directions for future research, and implications for managers are discussed.</t>
@@ -24542,7 +25238,11 @@
       <c r="K488" t="n">
         <v>2002</v>
       </c>
-      <c r="P488" s="8" t="n"/>
+      <c r="P488" s="8" t="inlineStr">
+        <is>
+          <t>The boundary spanning behavior (Group Scouting) is measured and reported at the group level (N=33 groups), rather than the individual level.. Verbatim Evidence: "Table 2 shows the means, standard deviations, and zero-order correlations for each of the measures of interest at the group level."</t>
+        </is>
+      </c>
     </row>
     <row r="489" ht="18" customHeight="1" s="10">
       <c r="A489" t="inlineStr">
@@ -24555,6 +25255,16 @@
           <t>BSMA0486</t>
         </is>
       </c>
+      <c r="E489" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F489" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G489" t="inlineStr">
         <is>
           <t>Employee contextual performance is a crucial determinant of organizational effectiveness, growth, and performance. Therefore, this research focuses on employees’ contextual performance issues seen from the perspective of boundary-spanning leaders (BSL), creativity, and proactive work behavior (PWB). The aim is to reveal the effect of BSL, creativity, and PWB on employees’ contextual performance and find new models of the role of creativity and PWB in mediating the effect of BSL on employees’ contextual performance. The research involved 420 employees from companies in the finance, trade, services, and investment industry sectors in Indonesia. A Likert scale questionnaire designed in Google Forms was used to conduct a survey via the WhatsApp application. Data analysis using structural equation modelling (SEM) shows that BSL, creativity, and PWB significantly direct affect employees' contextual performance; BSL and creativity significantly direct affect employees' PWB; and BSL significantly indirectly affect employees' contextual performance mediated by creativity and PWB. Accordingly, this study proves a new empirical model regarding the effect of BSL on employee contextual performance mediated by creativity and PWB. Based on these findings, this study suggests that researchers and practitioners utilize the empirical model from this study as a strategy to improve employee contextual performance through BSL with a mediation mechanism of creativity and PWB in the future.</t>
@@ -24578,7 +25288,11 @@
       <c r="K489" t="n">
         <v>2023</v>
       </c>
-      <c r="P489" s="8" t="n"/>
+      <c r="P489" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures Boundary-Spanning Leadership (BSL) and its dimensions at the individual level, and provides a raw, zero-order correlation matrix with Means and SDs.. Verbatim Evidence: "Table 2. Descriptive Statistics and Correlation Analysis"</t>
+        </is>
+      </c>
     </row>
     <row r="490" ht="18" customHeight="1" s="10">
       <c r="A490" t="inlineStr">
@@ -24591,6 +25305,16 @@
           <t>BSMA0487</t>
         </is>
       </c>
+      <c r="E490" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F490" t="inlineStr">
+        <is>
+          <t>NON_INDIVIDUAL_LEVEL</t>
+        </is>
+      </c>
       <c r="G490" t="inlineStr">
         <is>
           <t>Purpose – This study seeks to address a gap in the literature by investigating product management (PM) as a set of ﬁrm-level activities, distinct from the behaviours embedded within the market orientation (MO) construct. This research establishes PM as a set of organizational activities, which lie at the boundary between the traditional functions of the ﬁrm.</t>
@@ -24614,7 +25338,11 @@
       <c r="K490" t="n">
         <v>2011</v>
       </c>
-      <c r="P490" s="8" t="n"/>
+      <c r="P490" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures product management as a firm-level organizational boundary spanning capability rather than an individual-level behavior, and it does not contain a zero-order correlation matrix.. Verbatim Evidence: "This study adds to the literature by taking an unconventional approach, whereby it examines product management as a set of boundary spanning organizational capabilities."</t>
+        </is>
+      </c>
     </row>
     <row r="491" ht="18" customHeight="1" s="10">
       <c r="A491" t="inlineStr">
@@ -24627,6 +25355,16 @@
           <t>BSMA0488</t>
         </is>
       </c>
+      <c r="E491" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F491" t="inlineStr">
+        <is>
+          <t>LoA_VIOLATION</t>
+        </is>
+      </c>
       <c r="G491" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this paper is to examine the impact of product management as a set of organizational capabilities. It aims to investigate product management as a set of boundary spanning capabilities, by empirically relating these to ﬁrm performance.</t>
@@ -24650,7 +25388,11 @@
       <c r="K491" t="n">
         <v>2011</v>
       </c>
-      <c r="P491" s="8" t="n"/>
+      <c r="P491" s="8" t="inlineStr">
+        <is>
+          <t>The study analyzes boundary spanning activities at the firm level rather than the individual level.. Verbatim Evidence: "This research establishes PM as a set of organizational activities, which lie at the boundary between the traditional functions of the firm."</t>
+        </is>
+      </c>
     </row>
     <row r="492" ht="18" customHeight="1" s="10">
       <c r="A492" t="inlineStr">
@@ -24663,6 +25405,16 @@
           <t>BSMA0489</t>
         </is>
       </c>
+      <c r="E492" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F492" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G492" t="inlineStr">
         <is>
           <t>No Abstract</t>
@@ -24687,7 +25439,11 @@
       <c r="K492" t="n">
         <v>1984</v>
       </c>
-      <c r="P492" s="8" t="n"/>
+      <c r="P492" s="8" t="inlineStr">
+        <is>
+          <t>The study examines interorganizational linking mechanisms at the organizational level (Health Systems Agencies and hospitals), not at the individual level.. Verbatim Evidence: "The unit of analysis for this study was a request for project funding approval submitted by a health industry activity."</t>
+        </is>
+      </c>
     </row>
     <row r="493" ht="18" customHeight="1" s="10">
       <c r="A493" t="inlineStr">
@@ -24700,6 +25456,16 @@
           <t>BSMA0490</t>
         </is>
       </c>
+      <c r="E493" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F493" t="inlineStr">
+        <is>
+          <t>NO_BOUNDARY_SPANNING</t>
+        </is>
+      </c>
       <c r="G493" t="inlineStr">
         <is>
           <t>In this paper, we present an empirical study of 1,156 open source virtual reality (VR) projects from Unity List. Our study shows that the number of open source VR software projects are steadily growing, and some large projects attracting many developers are emerging. The most popular topic of VR software is still games. We also found that VR developers often face misscommit of automatically generated ﬁles.</t>
@@ -24723,7 +25489,11 @@
       <c r="K493" t="n">
         <v>2017</v>
       </c>
-      <c r="P493" s="8" t="n"/>
+      <c r="P493" s="8" t="inlineStr">
+        <is>
+          <t>The paper is a software engineering empirical study analyzing metadata of open-source VR projects (e.g., number of projects, commits, developers). It does not measure individual-level boundary spanning behaviors or provide a correlation matrix.. Verbatim Evidence: "In this paper, we present an empirical study on all 1,156 open source virtual-reality software projects collected from Unity List"</t>
+        </is>
+      </c>
     </row>
     <row r="494" ht="18" customHeight="1" s="10">
       <c r="A494" t="inlineStr">
@@ -24736,6 +25506,16 @@
           <t>BSMA0491</t>
         </is>
       </c>
+      <c r="E494" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F494" t="inlineStr">
+        <is>
+          <t>Non-Individual Anchors</t>
+        </is>
+      </c>
       <c r="G494" t="inlineStr">
         <is>
           <t>In today’s rapidly evolving business landscape, the capacity of new product development (NPD) teams to innovate hinges significantly on their ability to leverage external networks, known as ‘team boundary spanning’. While this activity is traditionally viewed as beneficial, its potential to exacerbate job stress and consequently diminish team satisfaction and NPD performance demands closer examination. Our research extends this area of inquiry by exploring the impact of team boundary spanning on job stress within NPD teams. Drawing on the conservation of resources theory, we hypothesize that team boundary spanning increases job stress which, in turn, decreases job satisfaction and NPD performance. This study also investigates the role of team boundary buffering as both a proactive and reactive intervention to mitigate the stress experienced by teams. Data were collected from 140 NPD projects in high and medium-high technology firms. Results reveal that team boundary spanning indeed elevates job stress and that high levels of stress correlate with declines in product quality and job satisfaction. Additionally, our results indicate that while team boundary buffering is not an effective proactive stress intervention, it is beneficial as a reactive intervention to the stress precipitated by boundary spanning activities.</t>
@@ -24759,7 +25539,11 @@
       <c r="K494" t="n">
         <v>2025</v>
       </c>
-      <c r="P494" s="8" t="n"/>
+      <c r="P494" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures boundary spanning at the team level, explicitly excluding it from this individual-level meta-analysis.. Verbatim Evidence: "In contrast, our study measures both boundary spanning and its negative effects at the team level, offering a novel perspective by examining how team boundary spanning leads to job stress"</t>
+        </is>
+      </c>
     </row>
     <row r="495" ht="18" customHeight="1" s="10">
       <c r="A495" t="inlineStr">
@@ -24772,6 +25556,16 @@
           <t>BSMA0492</t>
         </is>
       </c>
+      <c r="E495" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F495" t="inlineStr">
+        <is>
+          <t>Qualitative Study</t>
+        </is>
+      </c>
       <c r="G495" t="inlineStr">
         <is>
           <t>Abstract             In this study, we analyse the discursive strategies of professionalization used by psychology in Spain during its professionalization phase in the health sector in the early twenty-first century. Our primary focus is the conflict with political regulators and other healthcare professions after the Ley de Ordenación de Profesiones Sanitarias (Healthcare Professions Act) came into effect, since this Act calls into question the extent to which psychology can be viewed as health care. We use discourse analysis to determine the discursive structure of the conflict, which has an interprofessional dimension, as well as the professionalization and social closure strategies of psychology within the framework of professional relationships (boundary work). We argue that understanding this conflict requires viewing it as part of the European and international regulation context of healthcare professions. Highlighted in the analysis is the emergence of two psychology discourses divided into four modes of enunciation (professionalizing, cultural, scientific, and political–economic). Among other aspects, the conclusions focus on the dual interprofessional and intraprofessional nature of the conflict and evidence of a dual closure in psychology. The latter’s professionalization strategies in the sector occasionally resemble those employed by nursing, although at other times they are similar to those followed by some paramedical professions.</t>
@@ -24795,7 +25589,11 @@
       <c r="K495" t="n">
         <v>2025</v>
       </c>
-      <c r="P495" s="8" t="n"/>
+      <c r="P495" s="8" t="inlineStr">
+        <is>
+          <t>The paper relies on qualitative discourse analysis. It does not measure individual-level boundary spanning behaviors, and does not contain a quantitative correlation matrix.. Verbatim Evidence: "We studied the discourse concerning the LOPS to analyse the conflict and the mobilizations generated in psychology after the Act was published. For the analysis, we collated a total of thirty-six public documents in both paper and digital formats."</t>
+        </is>
+      </c>
     </row>
     <row r="496" ht="18" customHeight="1" s="10">
       <c r="A496" t="inlineStr">
@@ -24808,6 +25606,16 @@
           <t>BSMA0493</t>
         </is>
       </c>
+      <c r="E496" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F496" t="inlineStr">
+        <is>
+          <t>EX_NOT_EMPIRICAL</t>
+        </is>
+      </c>
       <c r="G496" t="inlineStr">
         <is>
           <t>No Abstract</t>
@@ -24831,7 +25639,11 @@
       <c r="K496" t="n">
         <v>2020</v>
       </c>
-      <c r="P496" s="8" t="n"/>
+      <c r="P496" s="8" t="inlineStr">
+        <is>
+          <t>The paper is an introduction to a virtual special issue on flexible work practices, summarizing other papers. It does not present original empirical data, measure individual-level boundary spanning behaviors, or contain a zero-order correlation matrix.. Verbatim Evidence: "Human Relations virtual special issues bring together and highlight related research on a particular topic. Each collection is compiled and introduced by two of the journal's editors"</t>
+        </is>
+      </c>
     </row>
     <row r="497" ht="18" customHeight="1" s="10">
       <c r="A497" t="inlineStr">
@@ -24844,6 +25656,16 @@
           <t>BSMA0494</t>
         </is>
       </c>
+      <c r="E497" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F497" t="inlineStr">
+        <is>
+          <t>Not Empirical</t>
+        </is>
+      </c>
       <c r="G497" t="inlineStr">
         <is>
           <t>Projects fail, and project managers are held responsible for these failures. This conceptual paper contends the cause of the success or failure of a project rests with the individuals who, in theory, comprise the project team. Research into project success or failure assumes a project team exists. This assumption deflects the need to look at the individuals who make up the team on which project managers depend for success. The lack of focus on these individuals undermines a project manager’s need and desire of a cohesive team to perform the work for a project. This study exposes the gap in the project management literature about the impact on the success of a project of the individuals who comprise the project team. A series of questions give direction for future research on this topic.</t>
@@ -24867,7 +25689,11 @@
       <c r="K497" t="n">
         <v>2019</v>
       </c>
-      <c r="P497" s="8" t="n"/>
+      <c r="P497" s="8" t="inlineStr">
+        <is>
+          <t>The paper is a conceptual piece and does not contain empirical data or a correlation matrix.. Verbatim Evidence: "This conceptual paper contends the cause of the success or failure of a project rests with the individuals who, in theory, comprise the project team."</t>
+        </is>
+      </c>
     </row>
     <row r="498" ht="18" customHeight="1" s="10">
       <c r="A498" t="inlineStr">
@@ -24880,6 +25706,16 @@
           <t>BSMA0495</t>
         </is>
       </c>
+      <c r="E498" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F498" t="inlineStr">
+        <is>
+          <t>Latent correlations only</t>
+        </is>
+      </c>
       <c r="G498" t="inlineStr">
         <is>
           <t>Process Management Programs (PMPs) rely heavily on the standardization of activities to improve organizational efficiency and reliability. Standardization, however, can lead to rigidity and inertia, which may eventually inhibit exploration and innovation. While scholars have provided cognitive and routine-based arguments to cope with this dilemma, the fact that standardization is a social process that requires collaboration between individuals has been overlooked. In this paper, we propose that standardization can improve a team’s social capital and thereby facilitate the activities that enable exploration. Specifically, we hypothesize that standardization relates positively to external communication, psychological safety, and the perception of support for innovation in operational teams. These three social capital attributes mediate the relationship between standardization and exploration. We tested this multilevel mediation model by analysing 431 members of 62 operational teams in a large multinational mining company that had recently implemented a Process Management Program (Lean Management). Our multilevel mediation results confirmed that standardisation promoted exploration by enhancing the teams’ social capital. For robustness we tested our model with a second survey of 450 workers of different companies and obtained similar results. Therefore, we propose that the productivity dilemma can be balanced by improving operational teams’ social capital.</t>
@@ -24903,7 +25739,11 @@
       <c r="K498" t="n">
         <v>2023</v>
       </c>
-      <c r="P498" s="8" t="n"/>
+      <c r="P498" s="8" t="inlineStr">
+        <is>
+          <t>The paper provides a correlation matrix used for discriminant validity containing the squared root of AVE on the diagonal and latent construct intercorrelations, instead of raw zero-order correlations.. Verbatim Evidence: "Second, the values in parentheses in Table 1 (a) indicate the squared root of AVE. These values are higher than the inter-correlation coefficient among constructs used in the model, indicating that discriminant validity has been achieved"</t>
+        </is>
+      </c>
     </row>
     <row r="499" ht="18" customHeight="1" s="10">
       <c r="A499" t="inlineStr">
@@ -24916,6 +25756,16 @@
           <t>BSMA0496</t>
         </is>
       </c>
+      <c r="E499" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F499" t="inlineStr">
+        <is>
+          <t>Code 99: Other - Firm-level</t>
+        </is>
+      </c>
       <c r="G499" t="inlineStr">
         <is>
           <t>Abstract             Recognition of the firm's tendency toward local search has given rise to concepts celebrating exploration that overcomes this tendency. To move beyond local search requires that exploration span some boundary, be it organizational or technological. While several studies have encouraged boundary‐spanning exploration, few have considered both types of boundaries systematically. In doing so, we create a typology of exploration behaviors: local exploration spans neither boundary, external boundary‐spanning exploration spans the firm boundary only, internal boundary‐spanning exploration spans the technological boundary only, and radical exploration spans both boundaries. Using this typology, we analyze the impact of knowledge generated by these different types of exploration on subsequent technological evolution.                            In our study of patenting activity in optical disk technology, we find that exploration that does not span organizational boundaries consistently generates lower impact on subsequent technological evolution. In addition, we find that the impact of exploration on subsequent technological evolution               within               the optical disk domain is highest when the exploration spans organizational boundaries but not technological boundaries. At the same time, we find that the impact of exploration on subsequent technological development               beyond               the optical disk domain is greatest when exploration spans both organizational and technological boundaries. Copyright © 2001 John Wiley &amp; Sons, Ltd.</t>
@@ -24939,7 +25789,11 @@
       <c r="K499" t="n">
         <v>2001</v>
       </c>
-      <c r="P499" s="8" t="n"/>
+      <c r="P499" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures boundary spanning at the firm level rather than the individual level. Additionally, the reported correlation matrix contains partial correlations rather than zero-order Pearson correlations.. Verbatim Evidence: "The basic unit of analysis is the individual patent and its associated content, and the level of the analysis is the firm."</t>
+        </is>
+      </c>
     </row>
     <row r="500" ht="18" customHeight="1" s="10">
       <c r="A500" t="inlineStr">
@@ -24952,6 +25806,16 @@
           <t>BSMA0497</t>
         </is>
       </c>
+      <c r="E500" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F500" t="inlineStr">
+        <is>
+          <t>No_Boundary_Spanning</t>
+        </is>
+      </c>
       <c r="G500" t="inlineStr">
         <is>
           <t>We propose and test a relational boundary-blurring framework, examining how employees’ evaluations of colleagues’ characteristics drive their decisions to connect with colleagues as friends online. We use a multi-method approach across four studies to investigate how self-disclosure of personal information, gender, and rank shape warmth evaluations of colleagues and subsequent boundary blurring decisions on online social networks such as Facebook. Study 1, a large archival study using a nationally representative sample, finds that connecting as friends with colleagues online is prevalent. Study 2, examining employees across several industries, shows that people experience connecting as friends with colleagues online as boundary blurring. Two experimental studies (Studies 3 and 4) ascertain that employees are more likely to connect as friends online with colleagues who engage in more (vs. less) self-disclosure and are less likely to connect with bosses (vs. peers). Further, self-disclosure, gender, and rank interact, such that employees are more likely to connect with female bosses who disclose more, compared to those who disclose less, and compared to male bosses, regardless of self-disclosure. Our work contributes to boundary management research by demonstrating that employees’ decisions to blur the personal/professional boundary online crucially depends on whom they are blurring the boundary with.</t>
@@ -24975,7 +25839,11 @@
       <c r="K500" t="n">
         <v>2022</v>
       </c>
-      <c r="P500" s="8" t="n"/>
+      <c r="P500" s="8" t="inlineStr">
+        <is>
+          <t>The paper focuses on work-personal boundary blurring (e.g., connecting with colleagues on Facebook) and boundary management (segmentation/integration), rather than individual-level boundary spanning behaviors across organizational or team boundaries.. Verbatim Evidence: "We depart from past work to examine a novel aspect of boundary management: with whom we blur the boundary."</t>
+        </is>
+      </c>
     </row>
     <row r="501" ht="18" customHeight="1" s="10">
       <c r="A501" t="inlineStr">
@@ -24988,6 +25856,16 @@
           <t>BSMA0498</t>
         </is>
       </c>
+      <c r="E501" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F501" t="inlineStr">
+        <is>
+          <t>Non-Individual Level of Analysis</t>
+        </is>
+      </c>
       <c r="G501" t="inlineStr">
         <is>
           <t>A model of cross-functional project groups was developed and hypotheses were tested in a study of 93 research and new product development groups from four companies. The results showed that functional diversity had indirect effects through external communication on one-year-later measures. Technical quality and schedule and budget performance improved, but group cohesiveness diminished. Functional diversity also had an indirect effect through job stress on group cohesiveness, which was again reduced. Implications for the development of conceptual models of cross-functional groups and their effective management are discussed.</t>
@@ -25011,7 +25889,11 @@
       <c r="K501" t="n">
         <v>2001</v>
       </c>
-      <c r="P501" s="8" t="n"/>
+      <c r="P501" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures cross-functional project groups and external communication at the project-group level rather than at the individual level.. Verbatim Evidence: "Hence, all variables were aggregated to project group means because the model, research questions, and hypotheses were focused on this level of analysis."</t>
+        </is>
+      </c>
     </row>
     <row r="502" ht="18" customHeight="1" s="10">
       <c r="A502" t="inlineStr">
@@ -25024,6 +25906,16 @@
           <t>BSMA0499</t>
         </is>
       </c>
+      <c r="E502" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F502" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G502" t="inlineStr">
         <is>
           <t>Boundary-spanning activity was studied in a large manufacturing company through a sample of 192 managers, engineers, and supervisors. Contrary to prior theory and research, this study found boundary-spanning activity unrelated to role conflict or ambiguity and positively related to job satisfac-tion for the total sample. Boundary-spanning activity was also positively related to a number of job characteristics for the total sample. Marked dif-ferences in boundary-spanning activity and its relationships with other variables, however, were found across occupational levels. While managers and engineers generally had boundary-spanning activity related to high levels of job satisfaction and job characteristics, first-level supervisors had boundary-spanning activity related to higher role conflict and lower job satisfaction with opportunities for promotion.</t>
@@ -25047,7 +25939,11 @@
       <c r="K502" t="n">
         <v>1976</v>
       </c>
-      <c r="P502" s="8" t="n"/>
+      <c r="P502" s="8" t="inlineStr">
+        <is>
+          <t>The paper is an empirical study that measures individual-level boundary spanning and reports zero-order correlations.. Verbatim Evidence: "Table I. Zero-Order Correlations between Boundary-Spanning Activity and Role, Satisfaction, and Job Characteristic Variables (Total Sample, N=192)"</t>
+        </is>
+      </c>
     </row>
     <row r="503" ht="18" customHeight="1" s="10">
       <c r="A503" t="inlineStr">
@@ -25060,6 +25956,16 @@
           <t>BSMA0500</t>
         </is>
       </c>
+      <c r="E503" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F503" t="inlineStr">
+        <is>
+          <t>No Correlation Matrix</t>
+        </is>
+      </c>
       <c r="G503" t="inlineStr">
         <is>
           <t>A naturally occurring field experiment of job change was conducted over a one-year period in three applied research and development organizations. The experimental group (n = 42) were those employees who had been promoted or assigned to a different job. Employees who had maintained the same job made up the nonequivalent control group (n = 166). Standardized change score analysis showed the job change group to have greater increases in performance, innovativeness, and job satisfaction, as well as a greater reduction in role ambiguity when compared to the nonequivalent control group. In addition, the job change group reported greater increases in the job characteristics of variety and task autonomy, as well as in the role requirements of integration and boundary-spanning activities. The importance of the results and the role of field experimentation are discussed.</t>
@@ -25083,7 +25989,11 @@
       <c r="K503" t="n">
         <v>1981</v>
       </c>
-      <c r="P503" s="8" t="n"/>
+      <c r="P503" s="8" t="inlineStr">
+        <is>
+          <t>The paper does not report a zero-order correlation matrix for the variables measured.. Verbatim Evidence: "Significant changes were tested by the differences between the treatment-effect correlations (not reported since the magnitudes of the correlations do not have meaning) as explained in the prior section."</t>
+        </is>
+      </c>
     </row>
     <row r="504" ht="18" customHeight="1" s="10">
       <c r="A504" t="inlineStr">
@@ -25094,6 +26004,16 @@
       <c r="B504" t="inlineStr">
         <is>
           <t>BSMA0501</t>
+        </is>
+      </c>
+      <c r="E504" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F504" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
         </is>
       </c>
       <c r="G504" t="inlineStr">
@@ -25121,7 +26041,11 @@
       <c r="K504" t="n">
         <v>2025</v>
       </c>
-      <c r="P504" s="8" t="n"/>
+      <c r="P504" s="8" t="inlineStr">
+        <is>
+          <t>The focal spanner is the manager (BSL), but the only other variables in the correlation matrix are subordinate-level (nurses' ACAP and Job Embeddedness). Per Dyadic Data rules, variables about the subordinate must be excluded, leaving no valid effect sizes.. Verbatim Evidence: "We investigated the impact of BSL on nurses’ absorptive capacity... and its impact on job embeddedness"</t>
+        </is>
+      </c>
     </row>
     <row r="505" ht="18" customHeight="1" s="10">
       <c r="A505" t="inlineStr">
@@ -25134,6 +26058,16 @@
           <t>BSMA0502</t>
         </is>
       </c>
+      <c r="E505" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F505" t="inlineStr">
+        <is>
+          <t>No Empirical Data</t>
+        </is>
+      </c>
       <c r="G505" t="inlineStr">
         <is>
           <t>The human resource management (HRM) function has realized a considerable increase in power, influence, and reputation, but it has not been examined from the perspective of organizational boundary spanning. Because boundary spanning's function of information control provides a source of power, it is helpful in explaining HRM's growing influence in US organizations. However, our conceptualization of the boundary spanning role needs to be refined to incorporate developments after its initial creation. Hence, an evolutionary model is proposed that depicts two stages that the boundary spanning role subsequently undergoes when the conditions for its initial creation are no longer present to justify its existence. Despite what we have termed “phantom threats,” boundary spanners are able to maintain their influence through astute management of information that portrays their continued usefulness. This phase however cannot last forever, and boundary spanners need to discover new threats. A review of the development and evolution of HRM in the U.S. supports the proposed model. Because each of the three stages are reflected in the communication patterns of the boundary spanner, several propositions based on the notion of information richness and the nature of the language used in communicating with three critical groups (i.e., external contacts, management, and subordinate staff) are generated to test the model. Finally, suggestions for research are made.</t>
@@ -25157,7 +26091,11 @@
       <c r="K505" t="n">
         <v>1998</v>
       </c>
-      <c r="P505" s="8" t="n"/>
+      <c r="P505" s="8" t="inlineStr">
+        <is>
+          <t>The paper is a conceptual and theoretical piece proposing an evolutionary model of the boundary spanning role of the Human Resources function. It does not contain any empirical data or a correlation matrix.. Verbatim Evidence: "In summary, the HRM function over the last twenty years supplies some support for the proposed model. Obviously, more systematic testing of this model is needed, however. We next offer some suggestions for research based on several propositions that can be generated from our proposed model."</t>
+        </is>
+      </c>
     </row>
     <row r="506" ht="18" customHeight="1" s="10">
       <c r="A506" t="inlineStr">
@@ -25170,6 +26108,16 @@
           <t>BSMA0503</t>
         </is>
       </c>
+      <c r="E506" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F506" t="inlineStr">
+        <is>
+          <t>Not individual-level</t>
+        </is>
+      </c>
       <c r="G506" t="inlineStr">
         <is>
           <t>This paper presents a new perspective on the ambidexterity debate. Basing our work on the assumption that learning is a multilevel process, we develop and empirically test whether, how, and with what consequences firms can balance explorativeand exploitative technology-learning activities across their organizational boundaries. Hypotheses are tested through a longitudinal panel of data tracking the cross-boundary learning strategies of 153 companies involved with innovation in the worldwide fuel cell industry over the period 1999-2006. By juxtaposing intra- and interorganizationalexploration-exploitation, we find that the pursuit of cross-boundary ambidexterity is worthwhile. Firms that engage in internal exploitation tend to balance such learning orientation with explorative interorganizational agreements. Consistently, those firms engaged in external exploitation tend to balance it with an internal focus on exploration, at least in the case of exploitative alliances involving familiar partners. Moreover, results confirm that such complementary cross-boundary strategies improve a firm’s innovative performance.</t>
@@ -25193,7 +26141,11 @@
       <c r="K506" t="n">
         <v>2010</v>
       </c>
-      <c r="P506" s="8" t="n"/>
+      <c r="P506" s="8" t="inlineStr">
+        <is>
+          <t>The study analyzes firm-level cross-boundary learning strategies and ambidexterity, measuring patents and alliances at the organizational (firm-year) level rather than individual-level boundary spanning behaviors.. Verbatim Evidence: "Given our interest in testing the existence and performance consequences of cross-boundary ambidexterity, the firm-year represents the unit of analysis that captures firm-level tendencies."</t>
+        </is>
+      </c>
     </row>
     <row r="507" ht="18" customHeight="1" s="10">
       <c r="A507" t="inlineStr">
@@ -25206,6 +26158,16 @@
           <t>BSMA0504</t>
         </is>
       </c>
+      <c r="E507" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F507" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G507" t="inlineStr">
         <is>
           <t>This paper considers the mutual value co-creation that can occur when both parties in a cross sector partnership learn to innovate within the relationship. Despite suggestions that there are often asymmetrical returns to the business partner, nonproﬁt partners also accrue beneﬁts (Austin &amp; Seitanidi, 2012). In particular we consider how the relationship is inﬂuenced by the actors’ abilities to accommodate, adapt, learn and co-create solutions as they learn how to do things differently or better in response to the challenges they face. This is achieved using data from a longitudinal analysis of a crosssector partnership between a business and an arts organisation in Ireland. This offers a unique opportunity to trace the emergence of the partnership over time, and, speciﬁcally, to consider the impact of innovations co-created by the actors involved. Our analysis will demonstrate that innovation at the level of the relationship emerged from the incremental problem solving processes of the individuals involved. This foregrounds the impact of individual boundary spanners and the import of social capital in realising the potential of this partnership. In this regard we put forward three key boundary spanning roles, boundary spanner as network builder, as entrepreneur, as facilitator/mediator. The paper concludes with suggestions for further research and consideration of managerial implications arising from this study.</t>
@@ -25229,7 +26191,11 @@
       <c r="K507" t="n">
         <v>2016</v>
       </c>
-      <c r="P507" s="8" t="n"/>
+      <c r="P507" s="8" t="inlineStr">
+        <is>
+          <t>Qualitative case study lacking quantitative data and correlation matrix. Verbatim Evidence: "Real time data, in the form of in-depth interviews (9 in total), was collected between 2001 and 2005"</t>
+        </is>
+      </c>
     </row>
     <row r="508" ht="18" customHeight="1" s="10">
       <c r="A508" t="inlineStr">
@@ -25242,6 +26208,16 @@
           <t>BSMA0505</t>
         </is>
       </c>
+      <c r="E508" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F508" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G508" t="inlineStr">
         <is>
           <t>Retaining information technology (IT) professionals is important for organizations, given the challenges in sourcing for IT talent. Prior research has largely focused on understanding employee turnover from an intra-individual perspective. In this study we examine employee turnover from a structural perspective. We investigate the impact on IT turnover of organizations' Internal Labor Market (ILM) strategies. ILM strategies include human resource rules, practices, and policies including hiring and promotion criteria, job ladders, wage systems and training procedures. We collect data on ILM strategies and turnover rates for eight major IT jobs across forty-one organizations and analyze the data using confirmatory agglomerative hierarchical clustering techniques. Our results show that organizations adopt distinct ILM strategies for different IT jobs, and that these strategies relate to differential turnover rates. Specifically, technically-oriented IT jobs cluster in craft ILM strategies that are associated with higher turnover, whereas managerially-oriented IT jobs cluster in industrial ILM strategies that are associated with lower turnover. Further, depending on their contingencies of goal orientation (not-for-profit versus for-profit), IT focus (IT producer versus user), and information intensity (IT critical versus support), organizations adopt an industrial ILM strategy for their technically-oriented IT jobs to dampen turnover. Not-for-profit and IT user organizations where IT is critical adopt industrial ILM strategies for their technically-oriented IT jobs to attenuate turnover and improve the predictability of their IT workforce. IT producers and IT users where IT plays a supporting role adopt craft ILM strategies that engender higher turnover to remain timely and flexible in IT skills acquisition.</t>
@@ -25265,7 +26241,11 @@
       <c r="K508" t="n">
         <v>2004</v>
       </c>
-      <c r="P508" s="8" t="n"/>
+      <c r="P508" s="8" t="inlineStr">
+        <is>
+          <t>Paper examines structural Internal Labor Market (ILM) strategies (entry features, job attributes) and actual turnover rates at the job-level across organizations. It does not measure individual-level boundary spanning behaviors, and does not contain a zero-order correlation matrix.. Verbatim Evidence: "To elicit the ILM strategies for IT jobs in each organization, we identified eight major jobs in the IT profession... We developed a set of structured questions based on Osterman (1984) as shown in Appendix A to assess the different ILM attributes for each job."</t>
+        </is>
+      </c>
     </row>
     <row r="509" ht="18" customHeight="1" s="10">
       <c r="A509" t="inlineStr">
@@ -25278,6 +26258,16 @@
           <t>BSMA0506</t>
         </is>
       </c>
+      <c r="E509" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F509" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G509" t="inlineStr">
         <is>
           <t>While researchers have probed predictors of product managers' performance in consumer goods firms, few have looked at the performance of the industrial product manager. In this article, Steven Lysonski and Arch Woodside use path analysis to examine causal models of industrial product managers' performance during periods of rapid technological change. Key variables are analyzed, including the effects of environmental uncertainty, boundary spanning behavior, role pressures, role outcomes and two performance measures. A total of 69 industrial product managers from New Zealand Telecom completed a questionnaire that included both operational measures of the key variables and their overall job performance. The results suggest that most of the hypothesized relationships are supportable empirically. Performance was hindered by environmental uncertainty, role conflict, role ambiguity, tension and dissatisfaction. The authors discuss their study's implications for improving the effectiveness of product management practices.</t>
@@ -25301,7 +26291,11 @@
       <c r="K509" t="n">
         <v>1989</v>
       </c>
-      <c r="P509" s="8" t="n"/>
+      <c r="P509" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures individual-level boundary spanning behavior of industrial product managers and reports a full zero-order correlation matrix for all scale constructs. The path analysis was based on observed regression (not LISREL), so the correlations are not latent.. Verbatim Evidence: "Boundary spanning, defined as the frequency of verbal, written, formal and informal communication beyond the product manager's department, was measured using a modified instrument designed by Aiken and Hage"</t>
+        </is>
+      </c>
     </row>
     <row r="510" ht="18" customHeight="1" s="10">
       <c r="A510" t="inlineStr">
@@ -25314,6 +26308,16 @@
           <t>BSMA0507</t>
         </is>
       </c>
+      <c r="E510" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F510" t="inlineStr">
+        <is>
+          <t>Non-Individual Level</t>
+        </is>
+      </c>
       <c r="G510" t="inlineStr">
         <is>
           <t>Manufacturing ﬁrms are increasingly seeking cost and other competitive advantages by tightly coupling and managing their relationship with suppliers. Among other mechanisms, interorganizational systems (IOS) that facilitate boundary-spanning activities of a ﬁrm enable them to effectively manage different types of buyer–supplier relationships. This study integrates literature from the operations and information systems ﬁelds to create a joint perspective in understanding the linkages between the nature of the IOS, buyer–supplier relationships, and manufacturing performance at the dyadic level. External integration, breadth, and initiation are used to capture IOS functionality, and their effect on process efﬁciency and sourcing leverage is examined. The study also explores the differences in how manufacturing ﬁrms use IOS when operating under varying levels of competitive intensity and product standardization. In order to test the research models and related hypothesis, empirical data on buyer–supplier dyads is collected from manufacturing ﬁrms. The results show that only higher levels of external integration that go beyond simple procurement systems, as well as who initiates the IOS, allow manufacturing ﬁrms to enhance process efﬁciency. In contrast, IOS breadth and IOS initiation enable manufacturing ﬁrms to enhance sourcing leverage over their suppliers. In addition, ﬁrms making standardized products in highly competitive environments tend to achieve higher process efﬁciencies and have higher levels of external integration. The study shows how speciﬁc IOS decisions allow manufacturing ﬁrms to better manage their dependence on the supplier for resources and thereby select system functionalities that are consistent with their own operating environments and the desired supply chain design.</t>
@@ -25337,7 +26341,11 @@
       <c r="K510" t="n">
         <v>2005</v>
       </c>
-      <c r="P510" s="8" t="n"/>
+      <c r="P510" s="8" t="inlineStr">
+        <is>
+          <t>The study measures boundary spanning and interorganizational systems at the firm/organizational level rather than the individual level.. Verbatim Evidence: "Data were collected from manufacturing firms on organizational-level variables, as well as on the characteristics of the IOS that support their interaction with the suppliers."</t>
+        </is>
+      </c>
     </row>
     <row r="511" ht="18" customHeight="1" s="10">
       <c r="A511" t="inlineStr">
@@ -25350,6 +26358,16 @@
           <t>BSMA0508</t>
         </is>
       </c>
+      <c r="E511" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F511" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G511" t="inlineStr">
         <is>
           <t>Purpose – Drawing on the conservation of resources theory, this research examines the relationship between managers’ servant leadership and frontline employees’ customer-oriented boundary-spanning behaviors by considering career meaningfulness as an underlying mechanism. Furthermore, this study investigates a moderated mediation model by proposing work centrality as a boundary condition in the relationship between career meaningfulness and customer-oriented boundary-spanning behaviors.</t>
@@ -25373,7 +26391,11 @@
       <c r="K511" t="n">
         <v>2025</v>
       </c>
-      <c r="P511" s="8" t="n"/>
+      <c r="P511" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures individual-level customer-oriented boundary-spanning behaviors and provides a valid zero-order correlation matrix.. Verbatim Evidence: "Customer-oriented boundary-spanning behaviors were evaluated using a thirteen-item scale developed by Bettencourt et al. (2005)."</t>
+        </is>
+      </c>
     </row>
     <row r="512" ht="18" customHeight="1" s="10">
       <c r="A512" t="inlineStr">
@@ -25386,6 +26408,16 @@
           <t>BSMA0509</t>
         </is>
       </c>
+      <c r="E512" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F512" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G512" t="inlineStr">
         <is>
           <t>Many humanitarian aid workers receive training prior to being dispatched into the field, but they often encounter challenges that require additional learning and creativity. Consequently, aid organizations formally support collaboration among the expatriate and local workers in a field office. At best, those aid workers would not only exploit their joint knowledge but also explore novel ways of managing the challenges at hand. Yet differences between expatriate and local groups (e.g., in ethnicity, religion, education, and salary) often thwart intergroup collaboration in field offices and, by extension, any joint learning or creativity. In response to this issue, we study the role of field office leaders—specifically, how their boundary‐spanning behavior may inspire collaboration between the two groups and therefore facilitate joint learning and creativity. We propose that a leader's in‐group prototypicality additionally catalyzes this process—that is, a leader's behavior has more impact if s/he is seen as representing his/her group. We tested and found support for our hypothesized moderated mediation model in a field sample of 137 aid workers from 59 humanitarian organizations. Thus, our study generally highlights the pivotal role that field office leaders play for crucial outcomes in humanitarian aid operations. Furthermore, we offer concrete steps for field office leaders who want to inspire better collaboration between the expatriate and local aid workers they lead.</t>
@@ -25409,7 +26441,11 @@
       <c r="K512" t="n">
         <v>2018</v>
       </c>
-      <c r="P512" s="8" t="n"/>
+      <c r="P512" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures individual-level boundary spanning leadership and provides a standard zero-order correlation matrix.. Verbatim Evidence: "We measured boundary-spanning leadership using a three-item scale... TABLE 1 Means (M), standard deviations (SD), intercorrelations, and Cronbach's alpha"</t>
+        </is>
+      </c>
     </row>
     <row r="513" ht="18" customHeight="1" s="10">
       <c r="A513" t="inlineStr">
@@ -25422,6 +26458,16 @@
           <t>BSMA0510</t>
         </is>
       </c>
+      <c r="E513" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F513" t="inlineStr">
+        <is>
+          <t>No correlation matrix</t>
+        </is>
+      </c>
       <c r="G513" t="inlineStr">
         <is>
           <t>Organisations are increasingly investing in complex technological innovations, such as enterprise information systems, with the aim of improving the operation of the business, and in this way gaining competitive advantage. However, the implementation of technological innovations tends to have an excessive focus on either technological innovation effectiveness, or the resulting operational effectiveness. Focusing on either one of them is detrimental to long-term performance. Cross-functional teams have been used by many organisations as a way of involving expertise from different functional areas in the implementation of technologies. The role of boundary spanning actors is discussed as they bring a common language to the crossfunctional teams. Multiple regression analysis has been used to identify the structural relationships and provide an explanation for the influence of cross-functional teams, technological innovation effectiveness and operational effectiveness in the continuous improvement of operational performance. The findings indicate that cross functional teams have an indirect influence on continuous improvement of operational performance through the alignment between technological innovation effectiveness and operational effectiveness.</t>
@@ -25445,7 +26491,11 @@
       <c r="K513" t="n">
         <v>2011</v>
       </c>
-      <c r="P513" s="8" t="n"/>
+      <c r="P513" s="8" t="inlineStr">
+        <is>
+          <t>The paper does not provide a zero-order correlation matrix. Additionally, it focuses on cross-functional teams rather than measuring individual-level boundary spanning behaviors.. Verbatim Evidence: "Multiple regression analysis has been used to identify the structural relationships and provide an explanation for the influence of cross-functional teams, technological innovation effectiveness and operational effectiveness in the continuous improvement of operational performance."</t>
+        </is>
+      </c>
     </row>
     <row r="514" ht="18" customHeight="1" s="10">
       <c r="A514" t="inlineStr">
@@ -25458,6 +26508,16 @@
           <t>BSMA0511</t>
         </is>
       </c>
+      <c r="E514" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F514" t="inlineStr">
+        <is>
+          <t>Latent correlations</t>
+        </is>
+      </c>
       <c r="G514" t="inlineStr">
         <is>
           <t>Boundary spanners are pivotal in developing effective public–private collaboration in public infrastructure projects. As boundary spanners have to account for different interests, perspectives, and ways of working in public–private collaborations, engaging in boundary-spanning activities often comes with role stress, which can negatively impact their job performance. However, despite the significant levels of role stress associated with boundary spanning, there is a dearth of empirical studies on the role stress of boundary spanning public managers and how it can be reduced. In this study, we empirically investigate the reciprocal relationship between role stressors and boundary spanning and test if supporting organizational conditions can alleviate role stressors. The findings show that especially role conflict is detrimental for boundary-spanning activities. We further find that top-management support can diminish both role conflict and role ambiguity and that co-worker support can help in reducing the role ambiguity of boundary spanning public managers.</t>
@@ -25481,7 +26541,11 @@
       <c r="K514" t="n">
         <v>2024</v>
       </c>
-      <c r="P514" s="8" t="n"/>
+      <c r="P514" s="8" t="inlineStr">
+        <is>
+          <t>The paper only provides correlations between latent variables (used to establish discriminant validity), rather than raw, zero-order Pearson correlations, which violates Rule 7.. Verbatim Evidence: "TABLE 3 Descriptive statistics and correlation between latent variables and control variables. [...] To establish discriminant validity, the square root of average variance extracted (AVE) (shown in Table 2) must be higher than the shared variance with other constructs (shown in Table 3); and the lowest acceptable value of AVE is 0.5 (Fornell &amp; Larcker, 1981 ). These conditions are met, indicating that the constructs are distinct."</t>
+        </is>
+      </c>
     </row>
     <row r="515" ht="18" customHeight="1" s="10">
       <c r="A515" t="inlineStr">
@@ -25494,6 +26558,16 @@
           <t>BSMA0512</t>
         </is>
       </c>
+      <c r="E515" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F515" t="inlineStr">
+        <is>
+          <t>No Zero-Order Correlations (Latent Matrix)</t>
+        </is>
+      </c>
       <c r="G515" t="inlineStr">
         <is>
           <t>The public sector is increasingly collaborating with the private sector in the development of large-scale public infrastructure projects. However, the difficulties arising due to working across organizational boundaries are often detrimental to project performance. This article argues that boundary-spanning activities can enhance the quality of collaboration and subsequently the performance of projects. Boundary spanners utilize relational governance mechanisms and undertake conscious endeavors for building interorganizational relationships by engaging in activities, such as coordination and communication with the stakeholders. The data for this study are composed of 158 survey responses from lead public managers involved in Dutch national public infrastructure projects. The data are analyzed using structural equation modeling. The study demonstrates that the quality of collaboration has a significant impact on the performance of the project during the implementation phase. Further, we find that the different boundary-spanning activities are interconnected and that they have a significant positive relationship on project performance, with a mediating effect of collaboration. The study concludes that, and shows how boundary spanners are vital to the collaborative processes through which public infrastructure projects are implemented.</t>
@@ -25517,7 +26591,11 @@
       <c r="K515" t="n">
         <v>2023</v>
       </c>
-      <c r="P515" s="8" t="n"/>
+      <c r="P515" s="8" t="inlineStr">
+        <is>
+          <t>The paper provides a matrix explicitly labeled 'Correlation among Latent Variables' (Table 4) and a 'Discriminant Validity' matrix containing squared correlations (Table 3). It does not report raw, zero-order correlations as required.. Verbatim Evidence: "Table 4. Correlation among Latent Variables."</t>
+        </is>
+      </c>
     </row>
     <row r="516" ht="18" customHeight="1" s="10">
       <c r="A516" t="inlineStr">
@@ -25530,6 +26608,16 @@
           <t>BSMA0513</t>
         </is>
       </c>
+      <c r="E516" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F516" t="inlineStr">
+        <is>
+          <t>Code 99: Other - Team-level</t>
+        </is>
+      </c>
       <c r="G516" t="inlineStr">
         <is>
           <t>We report results from a longitudinal study of information systems development (ISD) teams. We use data drawn from 60 ISD teams at 22 sites of 15 Fortune 500 organizations to explore variations in performance relative to these teams’ social interactions. To do this, we characterize ISD as a form of new product development and focus on team-level social interactions with external stakeholders. Drawing on cluster analysis, we identify ﬁve patterns of team-level social interactions and the relationships of these patterns to a suite of objective and subjective measures of ISD performance. Analysis leads us to report three ﬁndings. First, data indicate that no one of the ﬁve identiﬁed patterns maximizes all performance measures. Second, data make clear that the most common approach to ISD is the least effective relative to our suite of performance measures. Third, data from this study show that early indications of ISD project success do not predict actual outcomes. These ﬁndings suggest two issues for research and practice. First, these ﬁndings indicate that varying patterns of social interactions lead to differences in ISD team performance. Second, the ﬁndings illustrate that singular measures of ISD performance are an oversimpliﬁcation and that multiple measures of ISD performance are unlikely to agree.</t>
@@ -25553,7 +26641,11 @@
       <c r="K516" t="n">
         <v>2010</v>
       </c>
-      <c r="P516" s="8" t="n"/>
+      <c r="P516" s="8" t="inlineStr">
+        <is>
+          <t>The study measures boundary spanning at the team level, rather than the individual level.. Verbatim Evidence: "Data collection instruments were specifically designed to be collected at the individual level and then aggregated (by averaging responses of the team’s members) to the team level for analysis"</t>
+        </is>
+      </c>
     </row>
     <row r="517" ht="18" customHeight="1" s="10">
       <c r="A517" t="inlineStr">
@@ -25566,6 +26658,16 @@
           <t>BSMA0514</t>
         </is>
       </c>
+      <c r="E517" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F517" t="inlineStr">
+        <is>
+          <t>Not Empirical / Introduction</t>
+        </is>
+      </c>
       <c r="G517" t="inlineStr">
         <is>
           <t>Great strides have been made in highlighting the strengths of the social work profession as a workforce vital to improving the health and well-being of individuals, families, and communities. Neverthe less, substantially more work is needed to advance education, practice, and research involving social workers’ potential and their contributions to improved care throughout the life course. This special issue offers exemplars of the power of social work in integrated settings with the capacity to address the scope of behavioral health, psychosocial, and physical health care needs. In today’s rapidly evolving heath care context, integrated care represents a promising direction for the future of health services, and may be leveraged to improve population health across the life course. Papers selected for this special issue focused on two themes: (a) defining the expanding roles and functions social workers fulfill in integrated health settings, and (b) identifying organizational and system factors that affect social workers’ delivery of interventions in integrated health models. This special issue further articulates the added-value of social workers on health care teams and the resulting improved outcomes for patients, families, and communities. Through increased evidence, such as the knowledge gained from this special issue, it is our hope that the profession continues to advance the boundary-spanning roles and capabilities of social workers in integrated health settings—both in the hospital and in community-based settings.</t>
@@ -25589,7 +26691,11 @@
       <c r="K517" t="n">
         <v>2019</v>
       </c>
-      <c r="P517" s="8" t="n"/>
+      <c r="P517" s="8" t="inlineStr">
+        <is>
+          <t>This paper is an introduction and overview to a special issue on social workers in integrated health care. It does not present empirical data, a correlation matrix, or quantitative measurements.. Verbatim Evidence: "Papers selected for this special issue focused on two themes: (a) defining the expanding roles and functions social workers fulfill in integrated health settings, and (b) identifying organizational and system factors that affect social workers’ delivery of interventions in integrated health models."</t>
+        </is>
+      </c>
     </row>
     <row r="518" ht="18" customHeight="1" s="10">
       <c r="A518" t="inlineStr">
@@ -25602,6 +26708,16 @@
           <t>BSMA0515</t>
         </is>
       </c>
+      <c r="E518" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F518" t="inlineStr">
+        <is>
+          <t>No Zero-Order Correlations</t>
+        </is>
+      </c>
       <c r="G518" t="inlineStr">
         <is>
           <t>The focus of this dissertation is the role of strategic flexibility and its effect on economic performance of firms in a cyclical industry. The performance consequences of the decision-making processes and CEO boundary-spanning activity are also examined.</t>
@@ -25625,7 +26741,11 @@
       <c r="K518" t="n">
         <v>1986</v>
       </c>
-      <c r="P518" s="8" t="n"/>
+      <c r="P518" s="8" t="inlineStr">
+        <is>
+          <t>The paper reports boundary spanning correlations only as partial correlations controlling for company size and age, omitting the required raw, zero-order correlations.. Verbatim Evidence: "Table 7-12 Partial Correlations Boundary Spanning and Performance Controlling for Company Size and Company Age"</t>
+        </is>
+      </c>
     </row>
     <row r="519" ht="18" customHeight="1" s="10">
       <c r="A519" t="inlineStr">

</xml_diff>

<commit_message>
chore: completed Batch 14 extraction
</commit_message>
<xml_diff>
--- a/BSMA_AI_Run_V2.xlsx
+++ b/BSMA_AI_Run_V2.xlsx
@@ -26758,6 +26758,16 @@
           <t>BSMA0516</t>
         </is>
       </c>
+      <c r="E519" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F519" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G519" t="inlineStr">
         <is>
           <t>This study investigates the role of entrepreneurial attitudes for small and medium‐sized enterprise managers' tendency to create knowledge acquisition ties with managers of other organizations in the context of an institutionalized high‐tech cluster. We examine how innovation orientation, perceived personal control, need for achievement, and self‐esteem influence boundary‐spanning tie creation as a crucial facet of entrepreneurial behavior in the cluster context. Applying exponential random graph models to survey data collected in a German biotech cluster, we find that innovation orientation and perceived personal control positively affect managers' tendency to rely on interpersonal ties to gather knowledge. In contrast, need for achievement and self‐esteem are negatively related to knowledge tie creation.</t>
@@ -26781,7 +26791,11 @@
       <c r="K519" t="n">
         <v>2018</v>
       </c>
-      <c r="P519" s="8" t="n"/>
+      <c r="P519" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures individual-level boundary-spanning knowledge ties across organizational boundaries and reports a valid zero-order correlation matrix including this variable and other individual characteristics.. Verbatim Evidence: "Our dependent variable is the occurrence of knowledge acquisition ties in an interpersonal knowledge network among managers... Since we are interested in knowledge acquisition across organizational boundaries, we did not include relationships between managers belonging to the same organization."</t>
+        </is>
+      </c>
     </row>
     <row r="520" ht="18" customHeight="1" s="10">
       <c r="A520" t="inlineStr">
@@ -26794,6 +26808,16 @@
           <t>BSMA0517</t>
         </is>
       </c>
+      <c r="E520" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F520" t="inlineStr">
+        <is>
+          <t>Level of Analysis</t>
+        </is>
+      </c>
       <c r="G520" t="inlineStr">
         <is>
           <t>Companies extend their boundaries through acquisitions to new industries, product lines, technologies, markets and geographic locations. Diversification research has focused predominantly on boundary extensions across industries. Using data on 167 intra-industry acquisitions in the pharmaceuticals industry between 1991 and 1996, we study boundary extension in an industry, integrating existing arguments to examine how proximity in intraindustry networks, geographic location, and technological domain influences the likelihood of acquisition. As expected, the proximity of two firms in these search contexts increases the likelihood that one will acquire the other, but the contexts are partial substitutes, proximity in one search context overcoming distance in other contexts.Thus, we find that while pharmaceutical companies are more likely to acquire technologically similar foreign companies, they are more likely to acquire technologically dissimilar alliance partners. Our results contribute to an improved understanding of who buys whom and in doing so, organizational boundary spanning through acquisitions.</t>
@@ -26817,7 +26841,11 @@
       <c r="K520" t="n">
         <v>2006</v>
       </c>
-      <c r="P520" s="8" t="n"/>
+      <c r="P520" s="8" t="inlineStr">
+        <is>
+          <t>The paper focuses on organizational boundary spanning (firms extending their boundaries through acquisitions) rather than individual-level boundary spanning behaviors.. Verbatim Evidence: "In this article we study how firms use acquisitions to extend their boundaries. Boundary extension involves the extension of a firm's scope to new geographical areas, technological domains, or networks."</t>
+        </is>
+      </c>
     </row>
     <row r="521" ht="18" customHeight="1" s="10">
       <c r="A521" t="inlineStr">
@@ -26830,6 +26858,16 @@
           <t>BSMA0518</t>
         </is>
       </c>
+      <c r="E521" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F521" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level</t>
+        </is>
+      </c>
       <c r="G521" t="inlineStr">
         <is>
           <t>Two competing theories suggest different ways in which networks resolve collective action problems: small, dense networks enhance credible commitments supportive of cooperative solutions, while large boundary-spanning networks enhance search and information exchange supportive of coordinated solutions. Our empirical study develops and tests the competing credibility and search hypotheses in 22 estuary policy arenas, where fragmentation of authority creates collective problems and opportunities for joint gains through collaboration. The results indicate that search rather than credibility appears to pose the greater obstacle to collaboration; well-connected centrally located organizations engage in more collaborative activities than those embedded in small, dense networks.</t>
@@ -26853,7 +26891,11 @@
       <c r="K521" t="n">
         <v>2008</v>
       </c>
-      <c r="P521" s="8" t="n"/>
+      <c r="P521" s="8" t="inlineStr">
+        <is>
+          <t>The study measures boundary-spanning network links between organizations rather than at the individual employee level.. Verbatim Evidence: "First, we define a network link between organization A..."</t>
+        </is>
+      </c>
     </row>
     <row r="522" ht="18" customHeight="1" s="10">
       <c r="A522" t="inlineStr">
@@ -26866,6 +26908,16 @@
           <t>BSMA0519</t>
         </is>
       </c>
+      <c r="E522" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F522" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G522" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this study is to analyze the effects of inpatriates’ abilities, motivation and opportunities on knowledge sharing and the moderating role of boundary spanning in this context. Design/methodology/approach – By integrating the ability–motivation–opportunity framework with the concept of boundary spanning four hypotheses are developed, which are tested against the data of 187 inpatriates working in Germany.</t>
@@ -26889,7 +26941,11 @@
       <c r="K522" t="n">
         <v>2019</v>
       </c>
-      <c r="P522" s="8" t="n"/>
+      <c r="P522" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures individual-level inpatriate boundary spanning and provides a valid zero-order correlation matrix.. Verbatim Evidence: "Inpatriate boundary spanning was measured by using a five-item scale (1 = strongly disagree – 7 = strongly agree) developed by Reiche (2011)."</t>
+        </is>
+      </c>
     </row>
     <row r="523" ht="18" customHeight="1" s="10">
       <c r="A523" t="inlineStr">
@@ -26900,6 +26956,16 @@
       <c r="B523" t="inlineStr">
         <is>
           <t>BSMA0520</t>
+        </is>
+      </c>
+      <c r="E523" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F523" t="inlineStr">
+        <is>
+          <t>NA</t>
         </is>
       </c>
       <c r="G523" t="inlineStr">
@@ -26936,7 +27002,11 @@
       <c r="K523" t="n">
         <v>2012</v>
       </c>
-      <c r="P523" s="8" t="n"/>
+      <c r="P523" s="8" t="inlineStr">
+        <is>
+          <t>The paper does not measure boundary spanning behaviors (it measures leadership dimensions) and does not provide a zero-order correlation matrix.. Verbatim Evidence: "The employees were asked to rate the importance of 45 leadership attributes to high-performing leadership in their particular business function. The attribute list was created from previous leadership studies... After examining the results the nine factors are labeled: ‘‘Charisma’’, ‘‘Supportive’’, ‘‘Responsible’’, ‘‘Vision’’, ‘‘Integrity’’, ‘‘Creative’’, ‘‘Intelligent’’, ‘‘Challenges the Process’’, and ‘‘Risk Taking’’."</t>
+        </is>
+      </c>
     </row>
     <row r="524" ht="18" customHeight="1" s="10">
       <c r="A524" t="inlineStr">
@@ -26949,6 +27019,16 @@
           <t>BSMA0521</t>
         </is>
       </c>
+      <c r="E524" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F524" t="inlineStr">
+        <is>
+          <t>Team-Level Analysis</t>
+        </is>
+      </c>
       <c r="G524" t="inlineStr">
         <is>
           <t>This study integrated theories of group effectiveness with social identity and social categorization theory to develop and test a model of team performance. The sample included 42 product and process development teams employed in three divisions of a Fortune 500 manufacturing firm. Performance data was collected at project midpoint and at project completion through both managers’ and team members’ assessments. The study found that team social identification was an important predictor of team performance, explaining variance beyond that explained by cohesiveness and external communication. Team social identification was influenced by top management support and recognition, project leader organizational influence, the extent to which members’ time was dedicated to the team, and team functional diversity. Implications for scholars and professional managers are discussed. 0 1997 Elsevier Science B.V.</t>
@@ -26972,7 +27052,11 @@
       <c r="K524" t="n">
         <v>1997</v>
       </c>
-      <c r="P524" s="8" t="n"/>
+      <c r="P524" s="8" t="inlineStr">
+        <is>
+          <t>The study measures boundary spanning (external communication) but aggregates all variables to the project group level (N=42 teams). It does not report individual-level correlations.. Verbatim Evidence: "Since the unit of analysis in this study was the group, items were specifically constructed to refer to the team or to the team’s work... The individual responses were aggregated to the project group level by computing the mean across project members."</t>
+        </is>
+      </c>
     </row>
     <row r="525" ht="18" customHeight="1" s="10">
       <c r="A525" t="inlineStr">
@@ -26985,6 +27069,16 @@
           <t>BSMA0522</t>
         </is>
       </c>
+      <c r="E525" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F525" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G525" t="inlineStr">
         <is>
           <t>This introduction bridges the often-separated bodies of research on institutional boundary work in the policy ﬁeld of “integration” and on migrant minorities’ responses to these boundaries. We engage with the contributions to this Special Issue and demonstrate the relevance of an intersectional analysis in studies on state “integration” policies and the boundaries they draw between communities and on migrant minorities’ strategies to navigate and respond to them. Through engaging with issues of “integration”, boundary-making, and intersectionality, we show how the Special Issue contributes to debates on “integration” and boundary work by presenting analyses of which subjectivities are accepted in “integration” policies’ reproduction of an (imagined) national community and how conditions of national membership do not apply equally to all individuals of migrant origins, nor to all social spaces. We advocate for research that is attentive to the relevant socio-political context, and where possible, responsive to self-identiﬁed needs of the aﬀected communities.</t>
@@ -27008,7 +27102,11 @@
       <c r="K525" t="n">
         <v>2023</v>
       </c>
-      <c r="P525" s="8" t="n"/>
+      <c r="P525" s="8" t="inlineStr">
+        <is>
+          <t>This document is an introduction to a special issue and does not contain empirical data or a correlation matrix measuring individual-level boundary spanning behaviors.. Verbatim Evidence: "Integration and intersectionality: boundaries and belonging "from above" and "from below". Introduction to the special issue"</t>
+        </is>
+      </c>
     </row>
     <row r="526" ht="18" customHeight="1" s="10">
       <c r="A526" t="inlineStr">
@@ -27021,6 +27119,16 @@
           <t>BSMA0523</t>
         </is>
       </c>
+      <c r="E526" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F526" t="inlineStr">
+        <is>
+          <t>Latent Construct Intercorrelations</t>
+        </is>
+      </c>
       <c r="G526" t="inlineStr">
         <is>
           <t>Despite extensive research on the negative outcomes of role ambiguity in boundary-spanning positions, insight into how to prevent frontline employees from experiencing role ambiguity is sparse. This study addresses questions as to how the problem-focused coping strategies used by frontline employees can eﬀectively reduce perceived role ambiguity. The gathered evidence indicates that only action coping is eﬀective, whereas instrumental support seeking in fact enhances perceived role ambiguity. An examination of intrinsic and extrinsic coping resources as drivers of coping has revealed that conscientiousness and supervisor support are helpful coping resources. Contrastively, neuroticism drives insuﬃcient coping and inhibits the eﬀective use of coping resources. We ﬁnd that managers of service ﬁrms should provide training to ensure eﬀective supervisor support; also, in recruitment procedures they should consider potential employees’ personality traits, to reduce and prevent role ambiguity experienced by frontline employees.</t>
@@ -27044,7 +27152,11 @@
       <c r="K526" t="n">
         <v>2021</v>
       </c>
-      <c r="P526" s="8" t="n"/>
+      <c r="P526" s="8" t="inlineStr">
+        <is>
+          <t>The paper does not provide raw zero-order correlations. The only correlation matrix provided (Table 2) is used for discriminant validity (Fornell-Larcker criterion) and contains latent construct intercorrelations with the square root of Average Variance Extracted (AVE) on the diagonal.. Verbatim Evidence: "All factors fulfill Fornell and Larcker’s (1981) discriminant validity criterion; the square root of the AVE of every factor is higher than its highest interrelation with any other factor (Table 2)."</t>
+        </is>
+      </c>
     </row>
     <row r="527" ht="18" customHeight="1" s="10">
       <c r="A527" t="inlineStr">
@@ -27057,6 +27169,16 @@
           <t>BSMA0524</t>
         </is>
       </c>
+      <c r="E527" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F527" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G527" t="inlineStr">
         <is>
           <t>This study explores patterns of individual boundary-spanning communication in a government-managed research and development setting. Individual position in the organization hierarchy and preference for risk, change, and new experiences are the most significant antecedents of general levels of boundary-spanning communication.</t>
@@ -27080,7 +27202,11 @@
       <c r="K527" t="n">
         <v>1989</v>
       </c>
-      <c r="P527" s="8" t="n"/>
+      <c r="P527" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures individual-level boundary spanning communication and provides a zero-order correlation matrix with Means and SDs.. Verbatim Evidence: "Individual boundary-spanning activity is defined as the weekly frequency or extent of communication, formal and informal, written and spoken, across organizational boundaries between tasks within project organizations and between research centers."</t>
+        </is>
+      </c>
     </row>
     <row r="528" ht="18" customHeight="1" s="10">
       <c r="A528" t="inlineStr">
@@ -27093,6 +27219,16 @@
           <t>BSMA0525</t>
         </is>
       </c>
+      <c r="E528" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F528" t="inlineStr">
+        <is>
+          <t>Non-Individual Anchors</t>
+        </is>
+      </c>
       <c r="G528" t="inlineStr">
         <is>
           <t>Multiple studies have found that the primary determinant of new product failure is an absence of innovativeness—the extent to which a new product provides meaningfully unique benefits. Given the persistence of this finding and the growing use of cross-functional teams in new product development projects, the authors examine how innovativeness is affected by various characteristics of cross-functional teams and contextual influences on the team. On the basis of a study of 141 cross-functional product development teams, the authors find that innovativeness is positively related to the strength of superordinate identity in the team, encouragement to take risk, customers' influence, and active monitoring of the project by senior management. Beyond a moderate level, social cohesion among team members has a negative effect on innovativeness. The effect of superordinate identity on innovativeness is strengthened by encouragement to take risk and weakened by social cohesion. Functional diversity has no effect on innovativeness. The authors discuss managerial and research implications of the findings.</t>
@@ -27116,7 +27252,11 @@
       <c r="K528" t="n">
         <v>2001</v>
       </c>
-      <c r="P528" s="8" t="n"/>
+      <c r="P528" s="8" t="inlineStr">
+        <is>
+          <t>The paper focuses on cross-functional product development teams and its constructs are measured at the team level, unit level, or product level. There are no individual-level boundary spanning behaviors measured.. Verbatim Evidence: "On the basis of a study of 141 cross-functional product development teams, the authors find that innovativeness is positively related to the strength of superordinate identity in the team"</t>
+        </is>
+      </c>
     </row>
     <row r="529" ht="18" customHeight="1" s="10">
       <c r="A529" t="inlineStr">
@@ -27129,6 +27269,16 @@
           <t>BSMA0526</t>
         </is>
       </c>
+      <c r="E529" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F529" t="inlineStr">
+        <is>
+          <t>NO_MATRIX</t>
+        </is>
+      </c>
       <c r="G529" t="inlineStr">
         <is>
           <t>Task performance is essential for organizations, so it continues to attract the attention of researchers, practitioners, and academics. Therefore, the purpose of this study is to explore the effect of boundary-spanning leadership and psychological empowerment on the task performance of employees in Indonesian companies through the mediation mechanism of proactive work behavior. Research data were obtained from 455 employees of companies in the financial, trade, service, and investment sectors in Indonesia. The paper employed accidental sampling using a Likert-scale questionnaire and structural equation modeling. The results show that boundary-spanning leadership, psychological empowerment, and proactive work behavior significantly affect task performance. Boundary-spanning leadership and psychological empowerment significantly affect proactive work behavior. Proactive work behavior mediated the causal relationship between boundary-spanning leadership and psychological empowerment with task performance. These findings encourage a new empirical model regarding the critical role of proactive work behavior in transmitting boundary-spanning leadership and psychological empowerment to task performance. This model can be used by scholars, researchers, and practitioners to investigate worker task performance more thoroughly and deeply from the perspectives of boundary-spanning leadership, psychological empowerment, and proactive work behavior. It can serve as a credo for corporate management professionals seeking to maximize proactive work behavior, psychological empowerment, and boundary-spanning leadership in order to enhance employee task performance. In the interim, scholars and researchers can utilize it as a guide for next task performance investigations.</t>
@@ -27152,7 +27302,11 @@
       <c r="K529" t="n">
         <v>2024</v>
       </c>
-      <c r="P529" s="8" t="n"/>
+      <c r="P529" s="8" t="inlineStr">
+        <is>
+          <t>The paper does not report a zero-order correlation matrix with Pearson r values; it only summarizes the range of correlation coefficients in the text.. Verbatim Evidence: "Additionally, the correlation coefficient values were in the range of .24 to .80. The significance of the results, comprising all constructs (variables), was established at p &lt; .01, depicting a mutual dependence among the constructs. Despite this mutual dependence, the correlation coefficient obtained was less than .8, showing the absence of features used to characterize multicollinearity."</t>
+        </is>
+      </c>
     </row>
     <row r="530" ht="18" customHeight="1" s="10">
       <c r="A530" t="inlineStr">
@@ -27165,6 +27319,16 @@
           <t>BSMA0527</t>
         </is>
       </c>
+      <c r="E530" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F530" t="inlineStr">
+        <is>
+          <t>No correlation matrix</t>
+        </is>
+      </c>
       <c r="G530" t="inlineStr">
         <is>
           <t>Over the last decade, there has been a tremendous growth and exploitation of open source geospatial software and technologies. A combination of factors is driving this momentum including the contributions made by hundreds of OSGeo developers and the leading role played by the Open Source Geospatial Foundation (OSGeo), aiming primarily to support and promote the collaborative development of open source geospatial technologies and data. This paper seeks to map out the social history of collaborative activities within the OSGeo ecosystem. We used the archival logs of developers’ contributions, specifically looking for boundary spanning activities where contributions crossed multiple projects. The analysis and visualization of these activities allow us to have a better understanding of the role of boundary spanning in the resourcing of each project, the incubation mechanism advocated by OSGeo, and the significance of the social interrelatedness among projects. The data consisted of the subversion (SVN) commit history made by individual developers in the programming code repository. We applied several network analytical and visualization techniques to explore the data. Our findings indicate that more than one in seven developers spanned multiple projects which potentially had the effects of shaping the projects’ directions, and increased knowledge flow and innovation. Also the OSGeo’s incubation mechanism provided an important encouragement for boundary spanning and increased knowledge sharing. By studying the social history of contributions, further tools can be developed in future to assist tracking of the social history, and make developers mindful of the significance of the interdependence among projects and hence continuously contribute to the healthiness of the OSGeo ecosystem.</t>
@@ -27188,7 +27352,11 @@
       <c r="K530" t="n">
         <v>2012</v>
       </c>
-      <c r="P530" s="8" t="n"/>
+      <c r="P530" s="8" t="inlineStr">
+        <is>
+          <t>The paper uses social network analysis and descriptive statistics to map developer contributions and boundary spanning, but does not provide any zero-order correlation matrices.. Verbatim Evidence: "The analysis and visualization of these activities allow us to have a better understanding of the role of boundary spanning... We applied several network analytical and visualization techniques to explore the data."</t>
+        </is>
+      </c>
     </row>
     <row r="531" ht="18" customHeight="1" s="10">
       <c r="A531" t="inlineStr">
@@ -27201,6 +27369,16 @@
           <t>BSMA0528</t>
         </is>
       </c>
+      <c r="E531" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F531" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="G531" t="inlineStr">
         <is>
           <t>Internet start-ups have the most dynamic organisational structure due to the rapid growth of network information technology. Based on social cognition theory and information processing theory, this study investigates the connection between boundary-spanning search and business model design, proposing two types of cognitive styles: adaptive and innovative. Based on the questionnaire survey data of 223 Internet start-ups, this study ﬁnds that: (1) boundary-spanning search of technical knowledge is positively related to the eﬃciency-centered business model. (2) boundary-spanning search of market knowledge is positively related to the novelty-centered business model; (3) hybrid boundary-spanning search is positively related to the combined business model. (4) cognitive style weakens or enhances the relationship between boundary-spanning search and business model design. The research provides practical guidance for Internet start-ups and contributes to a better understanding of the antecedent variables of the business model.</t>
@@ -27224,7 +27402,11 @@
       <c r="K531" t="n">
         <v>2024</v>
       </c>
-      <c r="P531" s="8" t="n"/>
+      <c r="P531" s="8" t="inlineStr">
+        <is>
+          <t>Firm-level boundary spanning instead of individual-level (measured at the firm level). Verbatim Evidence: "Boundary-spanning search was measured by the average communication frequency between the firm and external partners during new product or service development"</t>
+        </is>
+      </c>
     </row>
     <row r="532" ht="18" customHeight="1" s="10">
       <c r="A532" t="inlineStr">
@@ -27237,6 +27419,16 @@
           <t>BSMA0529</t>
         </is>
       </c>
+      <c r="E532" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F532" t="inlineStr">
+        <is>
+          <t>Latent Construct Intercorrelations</t>
+        </is>
+      </c>
       <c r="G532" t="inlineStr">
         <is>
           <t>Despite the enthusiasm for engaging in interorganizational collaboration to enable digital product innovation, firms often face challenges in integrating knowledge across organizational boundaries. Our research examines how collaborating firms use Interorganizational Systems (IOS) tools and project coordinators to overcome knowledge boundaries in different types of ideation tasks. Drawing on boundary-spanning theory, we conceptualize IOS tools as boundary objects, project coordinators as boundary spanners, and the interdependence of ideation tasks as moderators of the impacts of boundary objects and spanners on knowledge integration. Our findings suggest that IOS tools help overcome syntax and semantic knowledge boundaries by transferring and sharing information when the interdependence of idea implementation tasks is high, and project coordinators help overcome pragmatic knowledge boundaries by building reciprocity of innovation participants when the interdependence of idea generation tasks is high. Our research contributes to value co-creation literature by developing a boundary-spanning mechanism to explain the roles of boundary objects and boundary spanners in overcoming different knowledge boundaries to enable digital product innovation at the inter-firm level.</t>
@@ -27260,7 +27452,11 @@
       <c r="K532" t="n">
         <v>2023</v>
       </c>
-      <c r="P532" s="8" t="n"/>
+      <c r="P532" s="8" t="inlineStr">
+        <is>
+          <t>The unit of analysis is the project/firm level, not the individual level. Furthermore, the correlation matrix (Table 4) explicitly reports correlations among latent constructs.. Verbatim Evidence: "Square roots of AVE on the diagonal (in bold) and correlations among the latent constructs on the off-diagonal positions."</t>
+        </is>
+      </c>
     </row>
     <row r="533" ht="18" customHeight="1" s="10">
       <c r="A533" t="inlineStr">
@@ -27273,6 +27469,16 @@
           <t>BSMA0530</t>
         </is>
       </c>
+      <c r="E533" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F533" t="inlineStr">
+        <is>
+          <t>EXCLUDE: Firm Level</t>
+        </is>
+      </c>
       <c r="G533" t="inlineStr">
         <is>
           <t>Our paper proposes that corporate technological relatedness, or the degree to which business units within a corporation utilize similar technological knowledge, has both positive and negative effects on corporate R&amp;D activities. On the one hand, business units that employ similar technological knowledge have better absorptive capacity to source knowledge from each other. On the other hand, a higher level of technological relatedness means that each business unit possesses fewer opportunities to gain new knowledge not known to other units, thus promoting path dependence to each other. Using a patent data analysis of 201 firms in R&amp;D-intensive industries, we examine the effects of corporate technological relatedness on within-firm knowledge flow, boundary-spanning combinations of prior knowledge, and innovation impacts.</t>
@@ -27296,7 +27502,11 @@
       <c r="K533" t="n">
         <v>2010</v>
       </c>
-      <c r="P533" s="8" t="n"/>
+      <c r="P533" s="8" t="inlineStr">
+        <is>
+          <t>The study conducts analysis at the firm level rather than the individual level, using patent data from 201 public firms.. Verbatim Evidence: "The sample consists of 201 public firms in R&amp;D-intensive industries from the DISCLOSURE database."</t>
+        </is>
+      </c>
     </row>
     <row r="534" ht="18" customHeight="1" s="10">
       <c r="A534" t="inlineStr">
@@ -27309,6 +27519,16 @@
           <t>BSMA0531</t>
         </is>
       </c>
+      <c r="E534" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F534" t="inlineStr">
+        <is>
+          <t>Wrong Level of Analysis</t>
+        </is>
+      </c>
       <c r="G534" t="inlineStr">
         <is>
           <t>Research summary                 : Losing key employees to competitors allows an organization to engage in external boundary‐spanning activities. It may benefit the organization through access to external knowledge, but may also increase the risks of leaking knowledge to competitors. We propose that the destination of departed employees is a crucial contingency: benefits or risks only materialize when employees leave for competitors that differ from the focal organization along significant dimensions, such as country or status group. In the context of the global fashion industry, we find that key employees' moves to foreign competitors may increase (albeit at a diminishing rate) their former employers' creative performance. Furthermore, firms may suffer from losing key employees to higher‐ or same‐status competitors, but may benefit from losing them to lower‐status competitors.                                                                         Managerial summary                 : Losing key employees to competitors can provide organizations with access to external knowledge, but increase risks of leaking knowledge to competitors. We find that an organization's access to external knowledge and its risks of knowledge leakage through employee mobility may be affected by whether its employees leave for competitors in a foreign country or in a different status group. In the context of the global fashion industry, we show that key employees' moves to foreign competitors increase (up to a point) their former employers' creative performance. Furthermore, firms may suffer from losing key employees to higher‐ or same‐status competitors, but benefit from losing them to lower‐status competitors. Hence, executives in creative industries and possibly beyond could welcome losing employees to competitors in foreign countries or to lower‐status competitors                              . Copyright © 2016 John Wiley &amp; Sons, Ltd.</t>
@@ -27332,7 +27552,11 @@
       <c r="K534" t="n">
         <v>2017</v>
       </c>
-      <c r="P534" s="8" t="n"/>
+      <c r="P534" s="8" t="inlineStr">
+        <is>
+          <t>The unit of analysis is the organization (fashion houses), not the individual. The study measures firm-level creative performance.. Verbatim Evidence: "Our dependent variable incorporates the average number of points that a given fashion house's collection received from all of the buyers for a particular season."</t>
+        </is>
+      </c>
     </row>
     <row r="535" ht="18" customHeight="1" s="10">
       <c r="A535" t="inlineStr">
@@ -27345,6 +27569,16 @@
           <t>BSMA0532</t>
         </is>
       </c>
+      <c r="E535" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F535" t="inlineStr">
+        <is>
+          <t>Non-Individual Level</t>
+        </is>
+      </c>
       <c r="G535" t="inlineStr">
         <is>
           <t>Information processing theory suggests the need for different types of integration mechanisms in R &amp; D project management depending on levels of uncertainty and equivocality. This paper examines the use of these mechanisms and their links to project performance in a sample of 121 R &amp; D projects in a large research laboratory. Overall, it is found that formal leadership, planning and process specification, and to a lesser extent information technology use are related to project performance while the positive effects of horizontal structures are apparently balanced out by their costs. The integration mechanisms studied act on performance partly through their effect on horizontal communications. Modest support was found for the contingency hypotheses derived from information processing theory. It appears that managers adjusted their use of horizontal structures, planning and process specification, and informal leadership to project uncertainty but not to project equivocality. The positive effects of horizontal communications on performance were found to be greatest under high project equivocality as would be predicted by information processing arguments. Moreover, with the exception of formal leadership, the use of integration mechanisms did not enhance performance in contexts of low uncertainty and low equivocality. q 2000 Elsevier Science B.V. All rights reserved.</t>
@@ -27368,7 +27602,11 @@
       <c r="K535" t="n">
         <v>2000</v>
       </c>
-      <c r="P535" s="8" t="n"/>
+      <c r="P535" s="8" t="inlineStr">
+        <is>
+          <t>The study measures integration mechanisms and horizontal communication at the project level (N=121 R&amp;D projects), not at the individual employee level.. Verbatim Evidence: "This paperexamines the use of these mechanisms and their links to project performance in a sample of 121R&amp;D projects in a large research laboratory."</t>
+        </is>
+      </c>
     </row>
     <row r="536" ht="18" customHeight="1" s="10">
       <c r="A536" t="inlineStr">
@@ -27381,6 +27619,16 @@
           <t>BSMA0533</t>
         </is>
       </c>
+      <c r="E536" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F536" t="inlineStr">
+        <is>
+          <t>LoA_VIOLATION</t>
+        </is>
+      </c>
       <c r="G536" t="inlineStr">
         <is>
           <t>Many firms actively disclose research findings in scientific peer-reviewed journals. The literature highlights several potential benefits of such scientific boundary-spanning activities, including privileged access to academic information networks. However, scientific disclosure may lead to unintended knowledge spillovers. It remains unclear whether active engagement in science leads to higher returns. This paper investigates the impact of scientific activities on the firm’s market value, using accounting data for U.S. firms and matched patent and scientific publication data. We find evidence for the positive impact of scientific publications on a firm’s market value beyond the effects of research and development, patent stocks, and patent quality, and also document heterogeneity with respect to this impact between different industrial sectors.             This paper was accepted by David Hsu, entrepreneurship and innovation.</t>
@@ -27404,7 +27652,11 @@
       <c r="K536" t="n">
         <v>2016</v>
       </c>
-      <c r="P536" s="8" t="n"/>
+      <c r="P536" s="8" t="inlineStr">
+        <is>
+          <t>The paper conducts a firm-level analysis and does not measure individual-level boundary spanning behaviors. Additionally, it lacks a zero-order correlation matrix.. Verbatim Evidence: "Our empirical analysis uses firm-level information from the Compustat database and matched scientific publication and patent data for a representative sample of 1,739 stock market listed firms (9,920 firm-year observations)"</t>
+        </is>
+      </c>
     </row>
     <row r="537" ht="18" customHeight="1" s="10">
       <c r="A537" t="inlineStr">
@@ -27417,6 +27669,16 @@
           <t>BSMA0534</t>
         </is>
       </c>
+      <c r="E537" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F537" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G537" t="inlineStr">
         <is>
           <t>This paper proposes a radical empirical look on the concrete activities of project managers involved in creative projects, with a speciﬁc focus on ‘‘non-administrative’’ issues. Through four case studies in the video-game industry, multimedia, advertising and a circus, we propose an integrated synthesis of what creative project managers actually do. Beyond analytical, cognitive, psychological, symbolic and discursive activities, we identify four sets of activities carefully coined to acknowledge the everyday work of project manager involved in creative projects. We suggest that this project manager acts as a sense-maker, a web-weaver, a game-master and a ﬂowbalancer. This empirical ‘‘picture’’ raises questions on the technical and theoretical focus of research in project management where creativity is an utmost strategic issue.</t>
@@ -27440,7 +27702,11 @@
       <c r="K537" t="n">
         <v>2006</v>
       </c>
-      <c r="P537" s="8" t="n"/>
+      <c r="P537" s="8" t="inlineStr">
+        <is>
+          <t>The paper is an exploratory ethnographic field study based on qualitative empirical inductive studies and does not provide any quantitative data or correlation matrices.. Verbatim Evidence: "It is based on qualitative empirical inductive studies in creative industries, with a strong descriptive focus."</t>
+        </is>
+      </c>
     </row>
     <row r="538" ht="18" customHeight="1" s="10">
       <c r="A538" t="inlineStr">
@@ -27453,6 +27719,16 @@
           <t>BSMA0535</t>
         </is>
       </c>
+      <c r="E538" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F538" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G538" t="inlineStr">
         <is>
           <t>Manufacturers are often placing their intellectual property (IP) at risk by outsourcing to suppliers in countries with weak IP rights. Thus, understanding how to safeguard their IP from poaching, which is a supplier's unauthorized use of a buyer's proprietary information, is of critical practical importance for manufacturers that outsource to suppliers in countries with weak IP rights. To investigate this phenomenon, we use dyadic data from globally dispersed manufacturer–supplier relationships to examine how the IP rights of a supplier's location affects poaching and how IP rights influence the effectiveness of two transactional characteristics—supplier idiosyncratic investments and media‐rich communication—on poaching. We examine these two transaction characteristics because they are representative of two forms of safeguards which create self‐enforcing agreements that do not require legal enforcement—economic and relational. We find that the strength of IP rights not only has a direct effect on poaching, but it also influences the relationships for both transaction characteristics. Intriguingly, when IP rights are weak, we find that not only are supplier idiosyncratic investments less effective in reducing poaching, but increases in these investments are associated with an increase in poaching. This finding illustrates that the strength of IP rights is a determinant of the degree to which supplier idiosyncratic investments are transaction specific. For suppliers in countries with weak IP rights, media‐rich communication is found to be more effective in reducing poaching. This finding illustrates the importance of manufacturers’ boundary spanners in building relationships with suppliers in countries with weak IP rights.</t>
@@ -27476,7 +27752,11 @@
       <c r="K538" t="n">
         <v>2018</v>
       </c>
-      <c r="P538" s="8" t="n"/>
+      <c r="P538" s="8" t="inlineStr">
+        <is>
+          <t>The study examines boundary spanning communication at the firm-level rather than the individual-level.. Verbatim Evidence: "The unit of analysis for this study is a manufacturer (buyer)–supplier dyad."</t>
+        </is>
+      </c>
     </row>
     <row r="539" ht="18" customHeight="1" s="10">
       <c r="A539" t="inlineStr">
@@ -27489,6 +27769,16 @@
           <t>BSMA0536</t>
         </is>
       </c>
+      <c r="E539" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F539" t="inlineStr">
+        <is>
+          <t>Non-Individual Anchors</t>
+        </is>
+      </c>
       <c r="G539" t="inlineStr">
         <is>
           <t>To successfully satisfy large customers and meet financial objectives, dedicated sales teams need to manage two boundaries: a boundary within the selling firm and one with the customer organization. However, little is known about the process of managing these multiple boundaries. This study integrates job demands-resource theory with research on key account management and sales teams to examine (1) the main effect of customer boundary spanning on perceived customer satisfaction and team performance and (2) the moderating role of within-firm coordination activities at three levels: top management, cross-functional, and within-team. An empirical test of the model with data from 167 sales teams finds that the interaction between customer boundary spanning and within-firm coordination activities has opposite effects on perceived customer satisfaction and team performance outcomes. The results are robust to endogeneity and heteroskedasticity concerns.</t>
@@ -27512,7 +27802,11 @@
       <c r="K539" t="n">
         <v>2015</v>
       </c>
-      <c r="P539" s="8" t="n"/>
+      <c r="P539" s="8" t="inlineStr">
+        <is>
+          <t>The study measures boundary spanning at the team level rather than the individual employee level.. Verbatim Evidence: "We test these interactions in the dedicated sales team context using team-level variables... The final sample was 167 usable surveys after being aggregated to the team level."</t>
+        </is>
+      </c>
     </row>
     <row r="540" ht="18" customHeight="1" s="10">
       <c r="A540" t="inlineStr">
@@ -27525,6 +27819,16 @@
           <t>BSMA0537</t>
         </is>
       </c>
+      <c r="E540" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F540" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G540" t="inlineStr">
         <is>
           <t>This dissertation investigated the effects of intrinsic and extrinsic motivational orientations in a boundary spanning model of retail buyers. Contributions of the dissertation to the field of marketing include the following: First, a boundary spanning/role stress model was tested in the context of retail buyers. No previous work has empirically or conceptually investigated the ability of a boundary spanning/role stress model to explain retail buyers' work-related attitudes. Second, the boundary spanning/role stress model was extended with the inclusion of accumulated role benefits. Previous role stress studies consider only negative role perceptions; accumulated role benefits examines positive role perceptions. Third, the boundary spanning/role stress model considers only external influences of role set members on a role incumbent. In doing so, the model neglects the influence of the individual who is perceiving and interpreting these stimuli. To capture individual differences, effects of intrinsic and extrinsic motivational orientations of the buyers were tested in the model. Finally, scales were developed to measure intrinsic motivational orientations, extrinsic motivational orientations, boundary spanning beliefs, and accumulated role benefits.</t>
@@ -27548,7 +27852,11 @@
       <c r="K540" t="n">
         <v>1988</v>
       </c>
-      <c r="P540" s="8" t="n"/>
+      <c r="P540" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures individual-level boundary spanning behaviors (Boundary Spanning Beliefs) and provides a correlation matrix of zero-order correlations among summated scales.. Verbatim Evidence: "Observed zero order correlations among summated scales are reported in Table 4-17."</t>
+        </is>
+      </c>
     </row>
     <row r="541" ht="18" customHeight="1" s="10">
       <c r="A541" t="inlineStr">
@@ -27561,6 +27869,16 @@
           <t>BSMA0538</t>
         </is>
       </c>
+      <c r="E541" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F541" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G541" t="inlineStr">
         <is>
           <t>A widely-cited proposition in boundary theory states that it is difficult for individuals to transition between roles, especially when these roles are highly segmented. Surprisingly, this hypothesis has not been directly tested. We provide an empirical test of these propositions and draw from the self-regulation literature to expand boundary theory in exploring how episodes of cognitive role transitions impact job performance. We propose that cognitive role transitioning is cognitively demanding, which consumes the limited executive control resources that facilitate effective job performance. In a multilevel study of 619 employees providing 4371 episodes, we observed that work-to-family cognitive role transitioning was negatively related to job performance, and this effect was mediated by self-regulatory depletion. Although individuals with greater role integration were somewhat more likely to experience cognitive role transitions than those with segmented roles, these individuals were also buffered from the self-regulatory depletion that impairs effective job performance. Overall, these findings suggest that integration, rather than segmentation, may be a better long-term boundary management strategy for minimizing self-regulatory depletion and maintaining higher levels of job performance during inevitable work–family role transitions.</t>
@@ -27584,7 +27902,11 @@
       <c r="K541" t="n">
         <v>2016</v>
       </c>
-      <c r="P541" s="8" t="n"/>
+      <c r="P541" s="8" t="inlineStr">
+        <is>
+          <t>No raw zero-order correlation matrix available (Table 1 reports MLM fixed effects estimates). Verbatim Evidence: "Within-person correlations above diagonal (N = 3679–5908; pairwise) represent estimates from fixed effects MLM models."</t>
+        </is>
+      </c>
     </row>
     <row r="542" ht="18" customHeight="1" s="10">
       <c r="A542" t="inlineStr">
@@ -27597,6 +27919,16 @@
           <t>BSMA0539</t>
         </is>
       </c>
+      <c r="E542" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F542" t="inlineStr">
+        <is>
+          <t>Latent_Correlations</t>
+        </is>
+      </c>
       <c r="G542" t="inlineStr">
         <is>
           <t>Purpose – Boundary-spanning managers need to recognize, learn and implement external knowledge while balancing the conflicts emerging from new and existing knowledge. The authors’ study explores how a paradox mindset (PM) and a learning focus [learning goal orientation (LGO)] promote two managerial capabilities: absorptive capacity (ACAP) and ambidexterity. The authors’ study explores the inter-relationship between the mindsets and the capabilities required for innovative work behavior.</t>
@@ -27620,7 +27952,11 @@
       <c r="K542" t="n">
         <v>2022</v>
       </c>
-      <c r="P542" s="8" t="n"/>
+      <c r="P542" s="8" t="inlineStr">
+        <is>
+          <t>The paper only provides a matrix of latent inter-construct correlations used to demonstrate divergent validity (Fornell-Larcker criterion), not raw zero-order correlations.. Verbatim Evidence: "We established the discriminant validity by examining the cross-loadings and using the Fornell–Larcker criteria... Also for each construct, the square root of AVE was greater than the inter-construct correlations (See Table 2)."</t>
+        </is>
+      </c>
     </row>
     <row r="543" ht="18" customHeight="1" s="10">
       <c r="A543" t="inlineStr">
@@ -27633,6 +27969,16 @@
           <t>BSMA0540</t>
         </is>
       </c>
+      <c r="E543" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F543" t="inlineStr">
+        <is>
+          <t>EX03</t>
+        </is>
+      </c>
       <c r="G543" t="inlineStr">
         <is>
           <t>Supervisors may experience time differently from their subordinates, and little is known about the interplay between the time pressures experienced by supervisors and their teams. Focusing on team creativity as the outcome of interest, we explore how teams with varying time pressures function alongside the distinct time pressures experienced by their supervisors. In a polynomial regression and response surface analytical framework, team creativity was enhanced when there was a greater divergence between the time pressures of supervisors and team members. Conversely, creativity suffered when the time pressures of both parties were more aligned, whether at low or high levels.</t>
@@ -27656,7 +28002,11 @@
       <c r="K543" t="n">
         <v>2025</v>
       </c>
-      <c r="P543" s="8" t="n"/>
+      <c r="P543" s="8" t="inlineStr">
+        <is>
+          <t>Does not measure individual-level boundary spanning behaviors. The paper focuses on team-level and supervisor-level time pressure and team creativity.. Verbatim Evidence: "By conceptualizing supervisors’ time pressure as a distinct construct from the time pressure experienced by their subordinates, we advance the literature on time pressure by identifying different configurations of supervisor and team time pressure affecting team creativity."</t>
+        </is>
+      </c>
     </row>
     <row r="544" ht="18" customHeight="1" s="10">
       <c r="A544" t="inlineStr">
@@ -27669,6 +28019,16 @@
           <t>BSMA0541</t>
         </is>
       </c>
+      <c r="E544" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F544" t="inlineStr">
+        <is>
+          <t>No Boundary Spanning / No Correlation Matrix</t>
+        </is>
+      </c>
       <c r="G544" t="inlineStr">
         <is>
           <t>This empirical research compared job characteristics and organizational climate in the private and public sectors. Perceptions and satisfaction of 240 top managers from a variety of private and public organizations in Israel were compared. The hypotheses tested were that (a) performance-based rewards and (b) policies that promote efficiency would be significantly more prevalent in private sector organizations and (c) that higher levels of satisfaction would be expressed by managers in the private sector. Two-way analyses of variance, private versus public and production versus service organizations, were performed. Results yielded significant main effects for sector of ownership and provided strong support for the three hypotheses of the research. Interaction effects in specific scales were also in the hypothesized direction, revealing that the private/public sector differences are further amplified in service organizations. The relation of the findings of this research to those of comparable studies in the United States are discussed.</t>
@@ -27692,7 +28052,11 @@
       <c r="K544" t="n">
         <v>1986</v>
       </c>
-      <c r="P544" s="8" t="n"/>
+      <c r="P544" s="8" t="inlineStr">
+        <is>
+          <t>The paper does not measure boundary spanning behaviors and does not include a zero-order correlation matrix (the matrix is noted as 'available upon request').. Verbatim Evidence: "The correlations between the existence and satisfaction scores along the convergent diagonal of the multitrait-multimethod matrix ranged from .74 to .88, indicating a high level of convergent validity (table available upon request)."</t>
+        </is>
+      </c>
     </row>
     <row r="545" ht="18" customHeight="1" s="10">
       <c r="A545" t="inlineStr">
@@ -27705,6 +28069,16 @@
           <t>BSMA0542</t>
         </is>
       </c>
+      <c r="E545" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F545" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G545" t="inlineStr">
         <is>
           <t>The purpose of this study is to broaden our understanding of team boundary activities in promoting team innovation. The model examines the mediating role of boundary activities in the relationship between the structural variables of inter-team goal interdependence and team functional heterogeneity and team innovation. Sixty teams from high-technology companies were studied involving 196 team members and their 60 corresponding team leaders and unit managers to whom the leaders report. Results identified two dimensions of boundary activities: boundary-loosening activities and boundary-tightening activities. Overall, the results of the structural equation model confirmed the mediating role of team boundary activity. The results indicated a positive relationship between the two structural variables and boundary-loosening activities, a negative relationship between functional heterogeneity and boundary-tightening activities, and a positive relationship between the two dimensions of boundary activities and team innovation. Implications, limitations, and directions for further research on team boundary activities are discussed.</t>
@@ -27728,7 +28102,11 @@
       <c r="K545" t="n">
         <v>2014</v>
       </c>
-      <c r="P545" s="8" t="n"/>
+      <c r="P545" s="8" t="inlineStr">
+        <is>
+          <t>The study measures and analyzes boundary spanning at the team level rather than the individual level, aggregating member responses to team boundary activities.. Verbatim Evidence: "In the present study, the unit of analysis was the team. All the hypotheses referred to the team and such study variables as boundary activities and inter-team goal interdependence were framed at the team level, and aggregated to team level."</t>
+        </is>
+      </c>
     </row>
     <row r="546" ht="18" customHeight="1" s="10">
       <c r="A546" t="inlineStr">
@@ -27741,6 +28119,16 @@
           <t>BSMA0543</t>
         </is>
       </c>
+      <c r="E546" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F546" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G546" t="inlineStr">
         <is>
           <t>Boundary‐spanning individuals (BSIs) play a critical role in supply chain management, especially in small and medium‐sized enterprises (SMEs) where interactions with buyers and suppliers can depend heavily on just a few individuals. This study, utilizing data from Korean manufacturing‐sector SMEs, explores whether cooperative social value orientations of SMEs' BSIs influence the effects of collaborative buyer‐supplier initiatives. The results suggested that the performance implication of decision‐sharing initiative increases when BSIs have a high level of cooperative social value orientation. However, it also negatively moderates the relationship between risk/benefit sharing (involving financial losses or gains) and performance suggesting possible negative side effects. However, we found that such orientation also negatively moderates the relationship between risk/benefit sharing (involving direct financial losses or gains) and relationship performance suggesting possible negative side effects.</t>
@@ -27764,7 +28152,11 @@
       <c r="K546" t="n">
         <v>2019</v>
       </c>
-      <c r="P546" s="8" t="n"/>
+      <c r="P546" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures individual-level boundary spanning behaviors (Cooperative Social Value Orientation of BSIs) and provides a zero-order correlation matrix with means and standard deviations in Table 4.. Verbatim Evidence: "Table 4 Correlation Matrix and Descriptive Statistics"</t>
+        </is>
+      </c>
     </row>
     <row r="547" ht="18" customHeight="1" s="10">
       <c r="A547" t="inlineStr">
@@ -27777,6 +28169,16 @@
           <t>BSMA0544</t>
         </is>
       </c>
+      <c r="E547" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F547" t="inlineStr">
+        <is>
+          <t>Level of Analysis</t>
+        </is>
+      </c>
       <c r="G547" t="inlineStr">
         <is>
           <t>Purpose – This paper aims to explore the potential contribution of inter-unit network structure and intraunit task environment to the overall knowledge management (KM) effectiveness of an organization through different KM strategies.</t>
@@ -27800,7 +28202,11 @@
       <c r="K547" t="n">
         <v>2018</v>
       </c>
-      <c r="P547" s="8" t="n"/>
+      <c r="P547" s="8" t="inlineStr">
+        <is>
+          <t>The study measures boundary spanning behaviors (network structure) at the work unit level rather than the individual level. The individual-level variables do not include boundary spanning behaviors.. Verbatim Evidence: "For inter-unit analysis (H1 and H2), the unit of analysis is at the work unit level. Network structure, as described earlier, was measured at the work unit level by collecting responses from unit leaders."</t>
+        </is>
+      </c>
     </row>
     <row r="548" ht="18" customHeight="1" s="10">
       <c r="A548" t="inlineStr">
@@ -27813,6 +28219,16 @@
           <t>BSMA0545</t>
         </is>
       </c>
+      <c r="E548" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F548" t="inlineStr">
+        <is>
+          <t>NO_BS_MEASURE</t>
+        </is>
+      </c>
       <c r="G548" t="inlineStr">
         <is>
           <t>This paper examines the boundary role person (BRP) as an influence agent and investigates an aspect of his potential ability to influence the decision outcomes of other organizational members. It was found that as their information requirements increase under conditions of higher perceived environmental uncertainty, the constituent members attribute to the BRP greater power in the decision making process. The results further suggest that, in light of the BRP's position in the transference of information across the organization's boundary, the reliance on expert power appears to be the most effective basis of social power for dealing with other organizational members.</t>
@@ -27836,7 +28252,11 @@
       <c r="K548" t="n">
         <v>1979</v>
       </c>
-      <c r="P548" s="8" t="n"/>
+      <c r="P548" s="8" t="inlineStr">
+        <is>
+          <t>The study focuses on purchasing agents in boundary spanning roles but only measures environmental uncertainty, attributed power, and bases of social power. It does not measure boundary spanning behaviors.. Verbatim Evidence: "Specifically, this paper focuses on the purchasing agent and his interactions with members of the buying task group (BTG)... Measures [include] Environmental Uncertainty... Attributed Power... The Bases of Social Power"</t>
+        </is>
+      </c>
     </row>
     <row r="549" ht="18" customHeight="1" s="10">
       <c r="A549" t="inlineStr">
@@ -27849,6 +28269,16 @@
           <t>BSMA0546</t>
         </is>
       </c>
+      <c r="E549" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F549" t="inlineStr">
+        <is>
+          <t>No Zero-Order Correlation Matrix</t>
+        </is>
+      </c>
       <c r="G549" t="inlineStr">
         <is>
           <t>Wildfire is a cross-boundary, collective action issue. Previous research has demonstrated the importance of collaborative relationships in wildfire for purposes such as increasing capacity, trading information, and facilitating landscape-scale mitigation projects. However, a stakeholder’s location in social networks, as well as personal factors, may impact their collaboration. Furthermore, stakeholders must prioritize their own organizational goals and responsibilities, which may differ from those of their collaborators. I used interview and survey methods to investigate these questions in the context of wildfire management professionals in northwestern Wyoming. For the interviews, I selected 12 individuals with high betweenness centrality who were involved in wildfire management in different organizations and locations throughout the study area. I used semi-structured interviews and asked participants to describe how they use collaboration to accomplish both collective and organizational goals for wildfire management. I found that managers’ answers to this question could be divided into four themes:(1) Deciding when collaboration is and isn’t the right tool,(2) Utilizing jurisdictional and organizational differences,(3) Finding or designing multi-benefit projects, and (4) Choosing collaborators and building relationships. For the survey, I used chain referral sampling and asked about managers’ participation in 8 collaborative actions, as well as their scope and focus of work, their gender, their role in wildfire management, who they worked with most frequently. I then modeled managers’ participation in the collaborative actions using betweenness centrality, gender, focus, scale, and role as predictors. I found that higher betweenness centrality, a focus on wildfire, and working at the scale of multiple communities or jurisdictions all increased collaboration. Holding the self-identified roles of coordinating across jurisdictions or interests, engaging with landowners, providing leadership or authority, and responding to emergencies also increased collaboration. When all of the variables were combined in a single model, I found that working at the multiple community or jurisdiction scale and holding engaging, coordinating, or responding roles had the most significant impact on collaborative action in a combined model. I found that managers who identified as women had lower collaborative scores, possibly as a result of gender bias in the natural resource and wildfire fields. I also found that men were much more likely to nominate other men in the chain referral portion of the survey, suggesting that gender bias may influence research using this method.</t>
@@ -27872,7 +28302,11 @@
       <c r="K549" t="n">
         <v>2023</v>
       </c>
-      <c r="P549" s="8" t="n"/>
+      <c r="P549" s="8" t="inlineStr">
+        <is>
+          <t>The study measures individual-level boundary spanning behaviors (collaborative actions) but does not report a zero-order correlation matrix. It only provides descriptive statistics and the results of Generalized Linear Models (GLMs).. Verbatim Evidence: "I then created 5 generalized linear models (GLMs) to describe the relationship between collaborative behaviors and managers professional relationships, job characteristics, and personal factors."</t>
+        </is>
+      </c>
     </row>
     <row r="550" ht="18" customHeight="1" s="10">
       <c r="A550" t="inlineStr">
@@ -27885,6 +28319,16 @@
           <t>BSMA0547</t>
         </is>
       </c>
+      <c r="E550" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F550" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G550" t="inlineStr">
         <is>
           <t>Purpose – This study aims to develop and test a new formative theory of coping intelligence (CI). It asserts that problem- and emotion-focused coping strategies contribute differently to the overall CI latent construct, which, in turn, relates to three outcome variables – job satisfaction, life satisfaction and sales commission.</t>
@@ -27908,7 +28352,11 @@
       <c r="K550" t="n">
         <v>2018</v>
       </c>
-      <c r="P550" s="8" t="n"/>
+      <c r="P550" s="8" t="inlineStr">
+        <is>
+          <t>The study does not measure any boundary spanning behaviors. It measures coping strategies (problem-focused and emotion-focused), life satisfaction, job satisfaction, and sales commission among boundary spanners, but lacks an actual boundary spanning behavior construct.. Verbatim Evidence: "For the survey, we selected PFC and EFC from Ways of Coping Checklist (Folkman and Lazarus, 1988)."</t>
+        </is>
+      </c>
     </row>
     <row r="551" ht="18" customHeight="1" s="10">
       <c r="A551" t="inlineStr">
@@ -27921,6 +28369,16 @@
           <t>BSMA0548</t>
         </is>
       </c>
+      <c r="E551" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F551" t="inlineStr">
+        <is>
+          <t>No BS Measure</t>
+        </is>
+      </c>
       <c r="G551" t="inlineStr">
         <is>
           <t>In this study, we develop a new theoretical framework of Coping Intelligence (CI) which examines relationships between coping strategies and organizational commitment among boundary spanning employees. We collected data from 452 boundary spanning salespeople using multiple sources. Results demonstrate that a formative model of Coping Intelligence (CI) is superior to a reﬂective model and that problem-focused coping contributes to CI which, in turn, is related to affective and normative commitment. Further, our more parsimonious formative model illustrates that positive problem-focused coping and negative emotion-focused coping contribute to both affective and normative commitment. After controlling for gender and salespeople’s commission (from company’s personnel record) in separate analyses, results remain signiﬁcant. We provide additional insights: Females are likely to use emotion-focused coping than males, but gender is not related to organizational commitment. Salespeople’s commission is positively related to both affective and normative commitment but unrelated to coping strategies. We shed new lights on boundary spanning employees’ Coping Intelligence and organizational commitment and offer theoretical, empirical, and practical implications to coping strategies and business ethics.</t>
@@ -27944,7 +28402,11 @@
       <c r="K551" t="n">
         <v>2015</v>
       </c>
-      <c r="P551" s="8" t="n"/>
+      <c r="P551" s="8" t="inlineStr">
+        <is>
+          <t>The study uses boundary spanning employees (salespeople) as its sample but does not measure individual-level boundary spanning behaviors as a variable. It only measures coping strategies and organizational commitment.. Verbatim Evidence: "The components of Coping Intelligence, problem-focused coping (CI-P), action-focused coping (CI-A), and emotion-focused coping (CI-E), were measured using 33 items adapted from Folkman and Lazarus (1988) Ways of Coping Checklist."</t>
+        </is>
+      </c>
     </row>
     <row r="552" ht="18" customHeight="1" s="10">
       <c r="A552" t="inlineStr">
@@ -27957,6 +28419,16 @@
           <t>BSMA0549</t>
         </is>
       </c>
+      <c r="E552" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F552" t="inlineStr">
+        <is>
+          <t>Latent Correlations</t>
+        </is>
+      </c>
       <c r="G552" t="inlineStr">
         <is>
           <t>The current study draws upon socialization theory to investigate both antecedents and outcomes of support service utilization within a sales employee context. Research indicates high performing, in contrast to low performing, salespeople may be more adept at discerning the ways in which an organization’s support services can be useful to them. The empirical results obtained from sales personnel of a financial services firm suggest that effective socialization/communication is important in securing an employee’s reliance upon organizational support. Further, high-performing salespeople are more proactive and instrumental in relation to utilization of support services, while low-performing salespeople are more passive and conforming in interfacing with support. Implications to both practice and research are discussed.</t>
@@ -27980,7 +28452,11 @@
       <c r="K552" t="n">
         <v>2021</v>
       </c>
-      <c r="P552" s="8" t="n"/>
+      <c r="P552" s="8" t="inlineStr">
+        <is>
+          <t>The paper's correlation matrix reports latent construct intercorrelations instead of raw, zero-order correlations.. Verbatim Evidence: "Correlation coefficients in Table 2 represent the correlations among the latent variables."</t>
+        </is>
+      </c>
     </row>
     <row r="553" ht="18" customHeight="1" s="10">
       <c r="A553" t="inlineStr">
@@ -27993,6 +28469,16 @@
           <t>BSMA0550</t>
         </is>
       </c>
+      <c r="E553" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F553" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G553" t="inlineStr">
         <is>
           <t>Within business-to-business relationship marketing, boundary-spanning representatives play a crucial role in establishing and maintaining positive relations between their organizations. Spirituality, a workplace individual-level variable, is proposed to significantly influence buyer representatives’ relationship formation with their seller counterparts, which subsequently affects the relationship development between organizations. Here we identify aspects of spirituality within buyer representatives and present a conceptual framework that delineates the impact of spirituality upon individual perceptions of relational constructs such as trust and commitment. Structural equation modeling analyses support the inclusion of spirituality as a relevant construct in relationship marketing research. In addition, because cultural differences are known to exist regarding the role of spirituality, the impact of spirituality upon perception within relationship marketing is addressed with data collected from both American and Chinese buying representatives. The results indicate that spirituality is significantly related to perceptions about communication, commitment, and shared values for both sets of participants.</t>
@@ -28016,7 +28502,11 @@
       <c r="K553" t="n">
         <v>2010</v>
       </c>
-      <c r="P553" s="8" t="n"/>
+      <c r="P553" s="8" t="inlineStr">
+        <is>
+          <t>The study does not measure boundary spanning behaviors (subjects are merely boundary spanners) and fails to report a zero-order correlation matrix, providing only path coefficients and hierarchical regression coefficients.. Verbatim Evidence: "Table 1 presents thepath coefﬁcients and tvalues for all of the hypotheses."</t>
+        </is>
+      </c>
     </row>
     <row r="554" ht="18" customHeight="1" s="10">
       <c r="A554" t="inlineStr">
@@ -28029,6 +28519,16 @@
           <t>BSMA0551</t>
         </is>
       </c>
+      <c r="E554" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F554" t="inlineStr">
+        <is>
+          <t>No correlation matrix</t>
+        </is>
+      </c>
       <c r="G554" t="inlineStr">
         <is>
           <t>Abstract             This article examines the frequently cited argument that coordination issues in humanitarian relief can be addressed more effectively with greater centralized authority and argues for a new conceptualization of aid delivery. The former position suggests a hierarchical, top‐down view of the humanitarian relief theater, while this analysis contends that the relief implementation structure may be better conceived as consisting of a network of loosely coupled semiautonomous organizations (Weick, 1976). A network approach allows examination of aid coordination dynamics at multiple levels of analysis: individual (professional and personal), organizational and interorganizational (operational), and strategic (structural/contextual). So viewed, factors that influence relief delivery, including contextual or strategic conditions and organization‐scale concerns, may either encourage or dissuade coordination across institutional boundaries. We argue that trust is a key precondition to coordination and that its extension is in turn conditioned by a number of strategic and operating‐level factors. We concentrate on operational coordination, as strategic concerns are not often open to the control of lone organizational actors. Our analysis rests in part on in‐depth interviews (each consisted of open‐ended questions and lasted an average of ninety to one hundred minutes) with a small sample of experienced international nongovernmental organization relief professionals who were engaged in aid efforts in Kosovo following the 1999 intervention by the North Atlantic Treaty Organization in that region.</t>
@@ -28052,7 +28552,11 @@
       <c r="K554" t="n">
         <v>2006</v>
       </c>
-      <c r="P554" s="8" t="n"/>
+      <c r="P554" s="8" t="inlineStr">
+        <is>
+          <t>The paper is a qualitative study based on in-depth interviews with a small sample (N=5) and does not contain quantitative data or a correlation matrix.. Verbatim Evidence: "To begin to explore empirically the utility of this conceptualization of relief efforts, we conducted lengthy open-ended interviews with a small sample (N = 5) of experienced INGO professionals and leaders"</t>
+        </is>
+      </c>
     </row>
     <row r="555" ht="18" customHeight="1" s="10">
       <c r="A555" t="inlineStr">
@@ -28065,6 +28569,16 @@
           <t>BSMA0552</t>
         </is>
       </c>
+      <c r="E555" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F555" t="inlineStr">
+        <is>
+          <t>Qualitative Study / No Correlation Matrix</t>
+        </is>
+      </c>
       <c r="G555" t="inlineStr">
         <is>
           <t>This paper introduces the notion of “temporal boundary spanning” and highlights the key role of project management in resolving temporal tensions among partners participating in interorganizational projects (IOPs). The present study, which is based on data from 93 IOPs undertaken within a major change program, relies on in-depth, semi-structured interviews, observations, and detailed analyses of written documents and procedures from those IOPs. Based on the data, we inductively develop a practice-based theory that identiﬁes three main practices (framing, synchronizing, hyping) used to resolve the central temporal tensions observed in the studied IOPs. In that respect, the paper offers novel insights into the role and practice of project management in IOPs.</t>
@@ -28088,7 +28602,11 @@
       <c r="K555" t="n">
         <v>2019</v>
       </c>
-      <c r="P555" s="8" t="n"/>
+      <c r="P555" s="8" t="inlineStr">
+        <is>
+          <t>The study is a qualitative, practice-based theory building study relying on interviews, observations, and documents, lacking a quantitative correlation matrix.. Verbatim Evidence: "The present study, which is based on data from 93 IOPs undertaken within a major change program, relies on in-depth, semi-structured interviews, observations, and detailed analyses of written documents and procedures from those IOPs. Based on the data, we inductively develop a practice-based theory"</t>
+        </is>
+      </c>
     </row>
     <row r="556" ht="18" customHeight="1" s="10">
       <c r="A556" t="inlineStr">
@@ -28101,6 +28619,16 @@
           <t>BSMA0553</t>
         </is>
       </c>
+      <c r="E556" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F556" t="inlineStr">
+        <is>
+          <t>EXCLUDE_FIRM_LEVEL</t>
+        </is>
+      </c>
       <c r="G556" t="inlineStr">
         <is>
           <t>Currently, digital innovation is one of the biggest challenges facing small and medium-sized enterprises (SMEs). This study analyses how SMEs can achieve higher levels of digital innovation despite their lack of resources. Using a dataset consisting of 520 German SMEs, we propose and test a model in which corporate social responsibility enables knowledge-sharing and supports SMEs in acquiring the resources needed for digital innovation development. As hypothesised, we found empirical evidence for a positive mediation effect in which absorptive capacity links corporate social responsibility and an SME's digital innovation output. In sum, this study helps to explain the relationship between corporate social responsibility and an SME's digital innovation, thus presenting far-reaching implications for SME research and the emerging scholarly debate on digital innovation in resource-constrained organisations.</t>
@@ -28124,7 +28652,11 @@
       <c r="K556" t="n">
         <v>2022</v>
       </c>
-      <c r="P556" s="8" t="n"/>
+      <c r="P556" s="8" t="inlineStr">
+        <is>
+          <t>The study measures firm-level outcomes in SMEs, rather than individual-level boundary spanning behaviors.. Verbatim Evidence: "Using a dataset consisting of 520 German SMEs, we propose and test a model in which corporate social responsibility..."</t>
+        </is>
+      </c>
     </row>
     <row r="557" ht="18" customHeight="1" s="10">
       <c r="A557" t="inlineStr">
@@ -28137,6 +28669,16 @@
           <t>BSMA0554</t>
         </is>
       </c>
+      <c r="E557" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F557" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G557" t="inlineStr">
         <is>
           <t>Extant research has largely ignored the phenomenon of interorganizational teams, which consist of members from both supplier and customer companies. This study examines the degree to which team interorganizationality influences team performance in a business-to-business context. On the basis of resource-dependence theory and boundary theory, the author argues that team interorganizationality positively influences team effectiveness, particularly when uncertainty is high. The hypotheses testing is based on multiple informant data collected from members and leaders of 225 teams in various industries. The results show the positive influence of team interorganizationality on team effectiveness. In addition, uncertainty-related moderator variables (company-related, market-related, and technological uncertainty) strengthen the link between team interorganizationality and team effectiveness.</t>
@@ -28160,7 +28702,11 @@
       <c r="K557" t="n">
         <v>2006</v>
       </c>
-      <c r="P557" s="8" t="n"/>
+      <c r="P557" s="8" t="inlineStr">
+        <is>
+          <t>The study measures boundary spanning at the team level (interorganizational teams) rather than at the individual level.. Verbatim Evidence: "The unit of analysis for this study was a customer-related team in a B2B setting."</t>
+        </is>
+      </c>
     </row>
     <row r="558" ht="18" customHeight="1" s="10">
       <c r="A558" t="inlineStr">
@@ -28173,6 +28719,16 @@
           <t>BSMA0555</t>
         </is>
       </c>
+      <c r="E558" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F558" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G558" t="inlineStr">
         <is>
           <t>Purpose – Boundary-spanning exploration through establishing alliances is an effective strategy to explore technologies beyond local search in innovating firms. The purpose of this paper is to argue that it is useful to make a distinction in boundary-spanning exploration between what a firm learns from its alliance partners (explorative learning from partners (ELP)) and what it learns from other organisations (explorative learning from non-partners (ELN)).</t>
@@ -28196,7 +28752,11 @@
       <c r="K558" t="n">
         <v>2019</v>
       </c>
-      <c r="P558" s="8" t="n"/>
+      <c r="P558" s="8" t="inlineStr">
+        <is>
+          <t>The study analyzes firm-level interorganizational ties and technological exploration among ASIC producers, rather than individual-level boundary spanning behaviors.. Verbatim Evidence: "We constructed a panel data set covering the population of ASIC producers over the period 1987–2000."</t>
+        </is>
+      </c>
     </row>
     <row r="559" ht="18" customHeight="1" s="10">
       <c r="A559" t="inlineStr">

</xml_diff>

<commit_message>
chore: completed Batch 15 extraction
</commit_message>
<xml_diff>
--- a/BSMA_AI_Run_V2.xlsx
+++ b/BSMA_AI_Run_V2.xlsx
@@ -28769,6 +28769,16 @@
           <t>BSMA0556</t>
         </is>
       </c>
+      <c r="E559" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F559" t="inlineStr">
+        <is>
+          <t>No Correlation Matrix</t>
+        </is>
+      </c>
       <c r="G559" t="inlineStr">
         <is>
           <t>This chapter reviews literatures from organizational psychology and management to assess the impact of
@@ -28803,7 +28813,11 @@
       <c r="K559" t="n">
         <v>2015</v>
       </c>
-      <c r="P559" s="8" t="n"/>
+      <c r="P559" s="8" t="inlineStr">
+        <is>
+          <t>The paper is a book chapter reviewing literature and does not contain primary empirical data or a correlation matrix.. Verbatim Evidence: "This chapter reviews literatures from organizational psychology and management to assess the impact of member diversity on project team performance."</t>
+        </is>
+      </c>
     </row>
     <row r="560" ht="18" customHeight="1" s="10">
       <c r="A560" t="inlineStr">
@@ -28816,6 +28830,16 @@
           <t>BSMA0557</t>
         </is>
       </c>
+      <c r="E560" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F560" t="inlineStr">
+        <is>
+          <t>No Correlation Matrix</t>
+        </is>
+      </c>
       <c r="G560" t="inlineStr">
         <is>
           <t>Project value creation faces tensions between the project owner and the outsourced project manager, particularly in their crossorganizational and cross-temporal interactions. The interplay between cross-organizational and cross-temporal interactions brings signiﬁcant challenges to value creation. Therefore, this research aims to explore these cross-boundary tensions between the project owner and project manager in value creation. Q methodology was applied, involving 59 interviews for developing Q statements and 20 Q surveys for analyzing tension dimensions. This research identiﬁed four dimensions of cross-boundary tension: (1) structural tension between empowerment and control, (2) priority tension between short-term and long-term, (3) communication tension between convergence and divergence, and (4) involvement tension between assistance and intervention. This research could theoretically contribute to value creation from the owner–manager cross-boundary tension perspective and extend the scope of the temporal boundary. Additionally, it provides practical guidance for professionals to understand the implications of tensions and strike the right balance for optimal value creation.</t>
@@ -28839,7 +28863,11 @@
       <c r="K560" t="n">
         <v>2026</v>
       </c>
-      <c r="P560" s="8" t="n"/>
+      <c r="P560" s="8" t="inlineStr">
+        <is>
+          <t>The study uses Q methodology to explore cross-boundary tensions and does not provide a correlation matrix of quantitative variables or measure individual-level boundary spanning behaviors.. Verbatim Evidence: "Q methodology was applied, involving 59 interviews for developing Q statements and 20 Q surveys for analyzing tension dimensions."</t>
+        </is>
+      </c>
     </row>
     <row r="561" ht="18" customHeight="1" s="10">
       <c r="A561" t="inlineStr">
@@ -28852,6 +28880,16 @@
           <t>BSMA0558</t>
         </is>
       </c>
+      <c r="E561" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F561" t="inlineStr">
+        <is>
+          <t>No Correlation Matrix</t>
+        </is>
+      </c>
       <c r="G561" t="inlineStr">
         <is>
           <t>In multinational corporations (MNCs), cross-cultural interactions and collaboration are unavoidable. Cultural boundary spanning (CBS) is a behavior that has been shown to reduce conflict and ensure project success. It is a behavior that bridges internal and external organizational boundaries. This study examined if and how CBS functions (behaviors) change across national and cultural boundaries in MNCs. These boundaries were characterized by four demographic groups of people found within MNCs:(a) parent country nationals,(b) host country nationals,(c) third country nationals, and (d) parent country national expats. The findings of this research suggest that any of these demographic groups can perform CBS. Variances in the use of CBS functions between the groups were also identified. These variances seem to be influenced by the strength of the individual’s social networks and the interdependent leadership culture within the MNC.</t>
@@ -28875,7 +28913,11 @@
       <c r="K561" t="n">
         <v>2023</v>
       </c>
-      <c r="P561" s="8" t="n"/>
+      <c r="P561" s="8" t="inlineStr">
+        <is>
+          <t>The study provides only descriptive statistics (means and standard deviations) for boundary spanning functions based on a small sample survey (N=16) and qualitative interviews, lacking a quantitative correlation matrix with zero-order correlations.. Verbatim Evidence: "This study utilized an explanatory sequential mixed-methods research approach whereby an initial quantitative survey was utilized to set the stage for further exploration of the proposed theory through a set of qualitative semi-structured interviews (Creswell &amp; Creswell, 2018). To derive basic means and standard deviations of the variable of CBS functions across the groups of national and cultural staffing combinations in MNCs, a quantitative survey was employed."</t>
+        </is>
+      </c>
     </row>
     <row r="562" ht="18" customHeight="1" s="10">
       <c r="A562" t="inlineStr">
@@ -28888,6 +28930,16 @@
           <t>BSMA0559</t>
         </is>
       </c>
+      <c r="E562" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F562" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G562" t="inlineStr">
         <is>
           <t>In this study, the national cultures and the complex contexts of Japanese multinational organizations (MN0s) are studied in the US The present study assumes that there are influences of national cultures which maintain significant cultural stereotypes in MNO, and also there are complex contexts of MNOs which might create distinctive communication patterns among Americans and Japanese. The objectives of this study are to quantitatively analyze the cognitive and behavioral dimensions of communication between these two cultural groups and identify distinctive patterns of organizational communication in terms of MNO effectiveness. The frameworks for interactions (FINT) scale is used for measurement of individual communication frames (n= 152), and ego-networks are measured to analyze ingroup-outgroup communications (n= 66). Cultural difference is identified in communication frames and patterns of ingroup-outgroup communication. Results about communication frames and ingroup-outgroup communication contradict expectations of cross-cultural stereotypes. This result implies that convergence in communication frames and communicative interactions is a key to success in MNOs. Results also suggest that the importance of outgroup communication is in its boundary spanning function, while increasing outgroup communication is crucial for both Americans and Japanese to enhance their communicative convergence and increase the effectiveness of MNOs.</t>
@@ -28911,7 +28963,11 @@
       <c r="K562" t="n">
         <v>2000</v>
       </c>
-      <c r="P562" s="8" t="n"/>
+      <c r="P562" s="8" t="inlineStr">
+        <is>
+          <t>The study measures individual-level outgroup communication networks, recognized by the author as boundary spanning behavior, and provides a raw, zero-order correlation matrix.. Verbatim Evidence: "Japanese outgroup communication with Americans is recognized as the performance of boundary spanning roles in the MNOs."</t>
+        </is>
+      </c>
     </row>
     <row r="563" ht="18" customHeight="1" s="10">
       <c r="A563" t="inlineStr">
@@ -28924,6 +28980,16 @@
           <t>BSMA0560</t>
         </is>
       </c>
+      <c r="E563" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F563" t="inlineStr">
+        <is>
+          <t>No correlation matrix</t>
+        </is>
+      </c>
       <c r="G563" t="inlineStr">
         <is>
           <t>Even as knowledge-intensive firms adopt modes of work design that distribute authority across the workforce, the distribution of ownership and governance, termed “structural power”, continues to vary in these companies. Extant research suggests competing views that, in a knowledge-intensive industry, structural power is (a) irrelevant,(b) less consequential than work design, or (c) reinforces work design. Given these competing views, this project seeks to explore the consequences of variation in the distribution of structural power for knowledge-intensive work. Data comes from a multi-method comparison of knowledge-intensive work practices at two competing automated manufacturing equipment firms with contrasting distributions of structural power.</t>
@@ -28947,7 +29013,11 @@
       <c r="K563" t="n">
         <v>2016</v>
       </c>
-      <c r="P563" s="8" t="n"/>
+      <c r="P563" s="8" t="inlineStr">
+        <is>
+          <t>The study uses qualitative ethnographic data to examine boundary spanning, and does not report a quantitative zero-order correlation matrix for boundary spanning behaviors.. Verbatim Evidence: "In Chapter Four, I examine how structural power shapes the content of customer relationship management efforts, often called representative inter-organizational boundary spanning roles... In this chapter, I use longitudinal ethnographic data to examine how distributions of structural power shape the internal and external dimensions of representative inter-organizational boundary spanning."</t>
+        </is>
+      </c>
     </row>
     <row r="564" ht="18" customHeight="1" s="10">
       <c r="A564" t="inlineStr">
@@ -28960,6 +29030,16 @@
           <t>BSMA0561</t>
         </is>
       </c>
+      <c r="E564" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F564" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G564" t="inlineStr">
         <is>
           <t>This paper integrates insights from the literature on invention networks, gender, and the sociological literature to analyze differences in how firms participate in man-led and woman-led invention networks. We contribute to the current debate on whether clustering or boundary-spanning network properties are more important for invention by introducing gender as an important factor. We empirically test our hypotheses on a sample of more than 30,000 firms from around the world over time using OECD REGPAT global patent data. Our findings indicate that different network properties are important for firm invention in woman-led and man-led innovation networks. In man-led invention networks, firms strongly benefit from being in a boundary-spanning position and are negatively affected by clustering, whereas in woman-led invention networks, boundary spanning has a less pronounced positive effect, and clustering has a positive rather than negative effect. Our findings have substantial implications for firms and policymakers interested in invention and contribute to the studies of gender and invention networks.</t>
@@ -28983,7 +29063,11 @@
       <c r="K564" t="n">
         <v>2026</v>
       </c>
-      <c r="P564" s="8" t="n"/>
+      <c r="P564" s="8" t="inlineStr">
+        <is>
+          <t>The boundary spanning construct and outcomes are measured at the firm level, not the individual level.. Verbatim Evidence: "We empirically test our hypotheses on a sample of more than 30,000 firms from around the world over time using OECD REGPAT global patent data."</t>
+        </is>
+      </c>
     </row>
     <row r="565" ht="18" customHeight="1" s="10">
       <c r="A565" t="inlineStr">
@@ -28996,6 +29080,16 @@
           <t>BSMA0562</t>
         </is>
       </c>
+      <c r="E565" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F565" t="inlineStr">
+        <is>
+          <t>Wrong Level of Analysis</t>
+        </is>
+      </c>
       <c r="G565" t="inlineStr">
         <is>
           <t>This study forms a moderated mediating model by introducing the two variables of absorptive capacity and boundary-spanning search to explore the influence of strategic prospectivity on exaptation. The paper focuses on the mediating role of boundary-spanning search and the moderating role of absorptive capacity. The results show that (1) strategic prospectivity has a significant positive impact on exaptation and boundary-spanning search mediates the relationship between strategic prospectivity and exaptation. (2) Potential absorptive capacity and realized absorptive capacity strengthen the relationship between boundary-spanning search and exaptation. (3) Potential absorptive capacity regulates the mediating role of boundaryspanning search. The hypothesis that put forward that realized absorptive capacity positively regulates the mediating effect of boundary-spanning search has not been verified. The research findings enrich our understanding of the impact mechanisms of exaptation and offer valuable insights for Chinese enterprises seeking to promote exaptation practices.</t>
@@ -29019,7 +29113,11 @@
       <c r="K565" t="n">
         <v>2024</v>
       </c>
-      <c r="P565" s="8" t="n"/>
+      <c r="P565" s="8" t="inlineStr">
+        <is>
+          <t>The study measures boundary-spanning search and other variables at the firm/enterprise level rather than at the individual employee level.. Verbatim Evidence: "This paper selected the middle and senior management teams and core business personnel of Chinese manufacturing enterprises... a total of 276 valid questionnaires were obtained... The surveyed enterprises have been in operation for 5–15 years... The items include such statements as 'Enterprises are sensitive to the signals reflected by the market and take action.'"</t>
+        </is>
+      </c>
     </row>
     <row r="566" ht="18" customHeight="1" s="10">
       <c r="A566" t="inlineStr">
@@ -29032,6 +29130,16 @@
           <t>BSMA0563</t>
         </is>
       </c>
+      <c r="E566" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F566" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G566" t="inlineStr">
         <is>
           <t>In this paper, we investigate the processes of boundary spanning across subunits within organizational networks. We hypothesize that patterns of advice across organizational subunits are explained by diﬀerent triadic mechanisms depending on the organizational design of the intra-organizational network. In organizational networks characterized by limited hierarchical diﬀerentiation among members and horizontal coordination, we found triadic cyclic closure to be positively associated to boundary spanning across subunits; but when the network reﬂects an organizational structure with formal hierarchical diﬀerentiation among members, then we found triadic transitive closure to be associated to boundary spanning across subunits. We test these predictions in two empirical studies consisting of two organizational networks that diﬀer from each other in organizational design. We adopt a Bayesian approach for exponential random graph models speciﬁcally designed for the statistical analysis of interpersonal relationships within and across subgroups or subunits. We suggest that the eﬀects of informal, triadic network conﬁgurations on boundary spanning are contingent on formal organizational design.</t>
@@ -29055,7 +29163,11 @@
       <c r="K566" t="n">
         <v>2019</v>
       </c>
-      <c r="P566" s="8" t="n"/>
+      <c r="P566" s="8" t="inlineStr">
+        <is>
+          <t>No zero-order correlation matrix of individual-level variables. This is a social network analysis paper employing Exponential Random Graph Models (ERGMs) instead of providing raw correlations.. Verbatim Evidence: "For all the network models the estimates (posterior means, standard deviations, and MCMC errors) for the structural effects are presented in Table 3."</t>
+        </is>
+      </c>
     </row>
     <row r="567" ht="18" customHeight="1" s="10">
       <c r="A567" t="inlineStr">
@@ -29068,6 +29180,16 @@
           <t>BSMA0564</t>
         </is>
       </c>
+      <c r="E567" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F567" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G567" t="inlineStr">
         <is>
           <t>The mechanisms by which social networks and organizational vocabularies combine jointly to affect communication patterns across organizational boundaries remain largely unexplored. In this paper, we examine the mutually constitutive relation between the network ties through which organizational members communicate with each other and the vocabularies that they use to describe their organization. We suggest that the dynamic structure of social networks and organizational vocabularies is contingent on the formal design of organizational subunits. Within subunit boundaries, members who interact with each other are more likely to develop similar vocabularies over time. Interestingly, between subunits, the more two members share similar organizational vocabularies, the more likely they are to form a tie over time. We ﬁnd empirical evidence for these arguments in a longitudinal study conducted among the managers of a multiunit organization. Organizational vocabularies, we suggest, may sustain communication patterns across organizational boundaries, thus bridging cultural holes within organizations.</t>
@@ -29091,7 +29213,11 @@
       <c r="K567" t="n">
         <v>2020</v>
       </c>
-      <c r="P567" s="8" t="n"/>
+      <c r="P567" s="8" t="inlineStr">
+        <is>
+          <t>The unit of analysis is the dyad (4,680 dyads) rather than the individual, and the study focuses on dyadic interpersonal ties rather than individual boundary-spanning behavior.. Verbatim Evidence: "Overall, the data set consists of 4,680 dyads involving the 40 managers across the three periods."</t>
+        </is>
+      </c>
     </row>
     <row r="568" ht="18" customHeight="1" s="10">
       <c r="A568" t="inlineStr">
@@ -29104,6 +29230,16 @@
           <t>BSMA0565</t>
         </is>
       </c>
+      <c r="E568" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F568" t="inlineStr">
+        <is>
+          <t>Latent construct correlations</t>
+        </is>
+      </c>
       <c r="G568" t="inlineStr">
         <is>
           <t>Purpose – The aim of this paper is to investigate the link between store managers’ evaluation of how customers assess a shopping centre and their own evaluation of the centre and, based on that, the relevance of store managers in reflecting on and informing the management and marketing practices of the local shopping centre management.</t>
@@ -29127,7 +29263,11 @@
       <c r="K568" t="n">
         <v>2014</v>
       </c>
-      <c r="P568" s="8" t="n"/>
+      <c r="P568" s="8" t="inlineStr">
+        <is>
+          <t>The paper only provides a matrix of squared correlations for latent constructs, labeled 'Discriminant validity measures', which violates the rule requiring raw, zero-order correlations.. Verbatim Evidence: "Table II. Discriminant validity measures... Squared correlation matrix for latent constructs shown below the diagonal"</t>
+        </is>
+      </c>
     </row>
     <row r="569" ht="18" customHeight="1" s="10">
       <c r="A569" t="inlineStr">
@@ -29138,6 +29278,16 @@
       <c r="B569" t="inlineStr">
         <is>
           <t>BSMA0566</t>
+        </is>
+      </c>
+      <c r="E569" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F569" t="inlineStr">
+        <is>
+          <t>Non-Individual Anchors</t>
         </is>
       </c>
       <c r="G569" t="inlineStr">
@@ -29193,7 +29343,11 @@
       <c r="K569" t="n">
         <v>2004</v>
       </c>
-      <c r="P569" s="8" t="n"/>
+      <c r="P569" s="8" t="inlineStr">
+        <is>
+          <t>The boundary spanning behavior is measured at the project/team level rather than the individual level.. Verbatim Evidence: "This dissertation explores the development of core competence in emerging technology innovation projects, and the level of analysis is at the project level."</t>
+        </is>
+      </c>
     </row>
     <row r="570" ht="18" customHeight="1" s="10">
       <c r="A570" t="inlineStr">
@@ -29206,6 +29360,16 @@
           <t>BSMA0567</t>
         </is>
       </c>
+      <c r="E570" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F570" t="inlineStr">
+        <is>
+          <t>No Boundary Spanning Measure</t>
+        </is>
+      </c>
       <c r="G570" t="inlineStr">
         <is>
           <t>A major US workforce trend of the new Millennium has been the decline in membership in private-sector unions. From a 1954 peak of 35% of the workforce, membership now sets at 11% of the workforce. To increase union membership, industry labor leaders are reviving the notion of dual commitment-that a worker can be loyal to both employer and union (Rose, 1952). Earlier attempts at using a unitary dual measure encountered methodological problems, so we explored the commitment attitudes individually. In a Qualtrics-based field study of a Midwest Teamsters local, we look at the degree to which various workplace factors are indicators of organizational and union commitment attitudes. Using hierarchical regression analysis to test hypotheses, we found a positive relationship between union commitment and union participation, and a lesser level of organizational commitment among the boundary-spanning union shop stewards than among rank-and-file employees. Other post-hoc patterns also emerged. Implications for labor officials and managers are discussed, as are ideas for future research. The study offers both practical information for the union leadership, and theoretical testing of the dual commitment phenomenon.</t>
@@ -29229,7 +29393,11 @@
       <c r="K570" t="n">
         <v>2015</v>
       </c>
-      <c r="P570" s="8" t="n"/>
+      <c r="P570" s="8" t="inlineStr">
+        <is>
+          <t>The paper does not measure boundary spanning behavior as a continuous variable in its correlation matrix. While it discusses the categorical role of 'Shop Steward' as a boundary spanner, this variable is not included in the zero-order correlation matrix (Table 6).. Verbatim Evidence: "Research by Friedman and Podolny (1992) labels these people [shop stewards] as boundary spanners, and explains how they play a central role in intergroup relations."</t>
+        </is>
+      </c>
     </row>
     <row r="571" ht="18" customHeight="1" s="10">
       <c r="A571" t="inlineStr">
@@ -29242,6 +29410,16 @@
           <t>BSMA0568</t>
         </is>
       </c>
+      <c r="E571" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F571" t="inlineStr">
+        <is>
+          <t>No Boundary Spanning Measure</t>
+        </is>
+      </c>
       <c r="G571" t="inlineStr">
         <is>
           <t>Flexible work arrangements (FWAs) are widely implemented for organizational purposes including recruitment. Theoretically, these arrangements alter temporal and physical boundaries around work. However, the time and place dimensions are frequently confounded in research, making the separate and joint effect of each on various outcomes unclear. To determine the relative importance of                 FWA                 dimensions as anticipated resources, this study experimentally manipulates discretion over when (flextime) and where (flexplace) one is expected to work on anticipated organizational support (                 AOS                 ) and organization attraction. Prospective employees (                 N                  = 130) participated in a 3 × 3 within‐subject experiment in which they rated nine hypothetical organizations that varied in flextime and flexplace. Results indicated main effects for both flextime and flexplace on both                 AOS                 and organization attraction with flextime having the stronger impact. Although the combination of a high level of both flextime and flexplace yielded the highest ratings of                 AOS                 and organization attraction, the interaction between flextime and flexplace was not statistically significant, suggesting flextime and flexplace have independent effects on recruitment outcomes. Relationships between flextime and flexplace and organizational attraction were slightly stronger for individuals who prefer to integrate their work and non‐work roles. Managerial implications and directions for future research are discussed.                                                        Practitioner points                                                                        Potential applicants rate flextime without a required core time as significantly more supportive and attractive than flextime with core time.                                                           Potential applicants rate flextime with a required core time as significantly more supportive and attractive than no flextime.                                                           Potential applicants rate working from home 2 to 3 days a week as significantly more supportive and attractive than not being able to work from home at all.                                                           The supportiveness and attractiveness of flextime does not depend on the supportiveness or attractiveness of flexplace or vice versa.</t>
@@ -29265,7 +29443,11 @@
       <c r="K571" t="n">
         <v>2015</v>
       </c>
-      <c r="P571" s="8" t="n"/>
+      <c r="P571" s="8" t="inlineStr">
+        <is>
+          <t>The paper focuses on flexible work arrangements (flextime and flexplace) as boundary-spanning resources and experimentally manipulates them. It does not contain a measure of individual-level boundary spanning behaviors.. Verbatim Evidence: "To determine the relative importance of FWA dimensions as anticipated resources, this study experimentally manipulates discretion over when (flextime) and where (flexplace) one is expected to work on anticipated organizational support (AOS) and organization attraction."</t>
+        </is>
+      </c>
     </row>
     <row r="572" ht="18" customHeight="1" s="10">
       <c r="A572" t="inlineStr">
@@ -29278,6 +29460,16 @@
           <t>BSMA0569</t>
         </is>
       </c>
+      <c r="E572" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F572" t="inlineStr">
+        <is>
+          <t>Not an empirical quantitative study</t>
+        </is>
+      </c>
       <c r="G572" t="inlineStr">
         <is>
           <t>Twenty years ago, most companies developed their own products in a single location and brought them to market themselves. Today, original equipment manufacturers (OEMs) are enlisting partners on a global scale as subsystem designers and producers in order to create and deliver new products into the market more rapidly and more frequently. This is especially true for large, complex products from the aerospace, telecommunications, electronics, and software industries. To assure the delivery of information across organizational boundaries, new coordination mechanisms need to be adopted (boundary management). In this article, best practices are described on how OEMs and partners self-organize and use agile, cooperative techniques to maintain daily communication among numerous internal and partner engineers to better coordinate product design and system integration. This article focuses on examples from the aerospace industry; however; these tactics can be applied in any organization to innovate at faster rates, to make delivery times more predictable, and to realize shorter product development timelines.</t>
@@ -29301,7 +29493,11 @@
       <c r="K572" t="n">
         <v>2013</v>
       </c>
-      <c r="P572" s="8" t="n"/>
+      <c r="P572" s="8" t="inlineStr">
+        <is>
+          <t>The paper is a conceptual/practical article describing best practices for boundary management in product development and does not contain a correlation matrix or any empirical quantitative data.. Verbatim Evidence: "In this article, best practices are described on how OEMs and partners self-organize and use agile, cooperative techniques to maintain daily communication among numerous internal and partner engineers to better coordinate product design and system integration."</t>
+        </is>
+      </c>
     </row>
     <row r="573" ht="18" customHeight="1" s="10">
       <c r="A573" t="inlineStr">
@@ -29314,6 +29510,16 @@
           <t>BSMA0570</t>
         </is>
       </c>
+      <c r="E573" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F573" t="inlineStr">
+        <is>
+          <t>EX02</t>
+        </is>
+      </c>
       <c r="G573" t="inlineStr">
         <is>
           <t>The management of knowledge across country units is critical to multinational corporations (MNCs). Building on the argument that boundary spanning leads to the development of creative problem solving outcomes, this study advances the concept of MNC knowledge transformation and examines its relationship with solution creativity. Using questionnaire data on 67 problem solving projects, we ﬁnd that opportunity formation is an underlying mechanism linking MNC knowledge transformation to the development of creative solutions. These insights contribute to our understanding of boundary spanning in global organizations by substantiating MNC knowledge transformation and elaborating the relationship between boundary spanning and creative solution development. If successful at knowledge transformation, collaborators from across the MNC can construct previously unimagined opportunities for the generation of creative outcomes.</t>
@@ -29337,7 +29543,11 @@
       <c r="K573" t="n">
         <v>2017</v>
       </c>
-      <c r="P573" s="8" t="n"/>
+      <c r="P573" s="8" t="inlineStr">
+        <is>
+          <t>The study is excluded because it examines boundary spanning at the group/project level rather than the individual level, and the correlation matrix contains latent variable correlations from PLS-SEM instead of raw zero-order Pearson correlations.. Verbatim Evidence: "Our paper differs in its approach, examining boundary spanning at the group level... Note: Diagonal elements are square roots of AVEs, other elements are latent variable correlations."</t>
+        </is>
+      </c>
     </row>
     <row r="574" ht="18" customHeight="1" s="10">
       <c r="A574" t="inlineStr">
@@ -29350,6 +29560,16 @@
           <t>BSMA0571</t>
         </is>
       </c>
+      <c r="E574" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F574" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G574" t="inlineStr">
         <is>
           <t>There is a growing interest in the interrelated notions of the marketing concept, service quality, total quality management, and customer orientation. Salespeople are in a crucial position to make an impact in these particular areas because of their boundary spanning role between the customer and the organization. Customer-oriented selling has been promoted to salespeople as a way to impact the service and quality goals of an organization. However, little is known about the effectiveness of customer-oriented selling, as well as the factors influencing the extent to which salespeople engage in it. The purpose of this research is to explore some of the factors influencing customer-oriented selling so that researchers and practitioners may gain relevant insights on these issues.</t>
@@ -29373,7 +29593,11 @@
       <c r="K574" t="n">
         <v>1995</v>
       </c>
-      <c r="P574" s="8" t="n"/>
+      <c r="P574" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures individual-level boundary spanning behaviors (customer-oriented selling) and provides a raw zero-order correlation matrix containing means and standard deviations of the observed variables.. Verbatim Evidence: "Appendix M: Means, Standard Deviations, and Correlation Coefficients for the Major Variables in the Structural Equation Modeling"</t>
+        </is>
+      </c>
     </row>
     <row r="575" ht="18" customHeight="1" s="10">
       <c r="A575" t="inlineStr">
@@ -29386,6 +29610,16 @@
           <t>BSMA0572</t>
         </is>
       </c>
+      <c r="E575" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F575" t="inlineStr">
+        <is>
+          <t>Review Article</t>
+        </is>
+      </c>
       <c r="G575" t="inlineStr">
         <is>
           <t>Efforts to initiate new startups rely heavily on teams and networks. Research demonstrates that 95 percent of the individuals trying to start a business involved others in helping build the new business. This article provides an overview of the team performance literature that can be used when making managerial decisions about building and managing successful entrepreneurial teams. I integrate and review prior research in three areas that have been disconnected previously: 1) innovation networks and teams; 2) team boundary spanning and internal processes; and 3) shared ownership and team motivation. The integration and review in this article provide new insights towards an evidence-based approach on managing entrepreneurial teams.</t>
@@ -29409,7 +29643,11 @@
       <c r="K575" t="n">
         <v>2019</v>
       </c>
-      <c r="P575" s="8" t="n"/>
+      <c r="P575" s="8" t="inlineStr">
+        <is>
+          <t>This is a conceptual/review article providing an overview of team performance literature, lacking primary empirical data or a zero-order correlation matrix.. Verbatim Evidence: "This article provides an overview of the team performance literature that can be used when making managerial decisions about building and managing successful entrepreneurial teams."</t>
+        </is>
+      </c>
     </row>
     <row r="576" ht="18" customHeight="1" s="10">
       <c r="A576" t="inlineStr">
@@ -29422,6 +29660,16 @@
           <t>BSMA0573</t>
         </is>
       </c>
+      <c r="E576" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F576" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G576" t="inlineStr">
         <is>
           <t>In this article, we study the conditions under which having ties that span organizational boundaries (bridging ties) are conducive to the generation of innovations. Whereas previous research has shown that bridging ties have a positive impact on innovative performance, our analysis of 276 R&amp;D scientists and engineers reveals that there are no advantages associated with bridging per se. In contrast, our findings suggest that the advantages traditionally associated with bridging ties are contingent upon the nature of the ties forming the bridge—specifically, whether these bridging ties are Simmelian.</t>
@@ -29445,7 +29693,11 @@
       <c r="K576" t="n">
         <v>2010</v>
       </c>
-      <c r="P576" s="8" t="n"/>
+      <c r="P576" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures individual-level boundary spanning behavior (bridging ties across organizational labs via E-I index) and reports a valid zero-order bivariate correlation matrix.. Verbatim Evidence: "Given a relation among individuals in our sample, the E-I index for any actor i was constructed by considering the difference between the number of external ties and the number of internal ties. Taking Ei and Ii as the number of external and internal ties, respectively, then the E-I index for actor i is defined as..."</t>
+        </is>
+      </c>
     </row>
     <row r="577" ht="18" customHeight="1" s="10">
       <c r="A577" t="inlineStr">
@@ -29458,6 +29710,16 @@
           <t>BSMA0574</t>
         </is>
       </c>
+      <c r="E577" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F577" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
       <c r="G577" t="inlineStr">
         <is>
           <t>Prior research has emphasized the importance of boundary spanners in facilitating the transfer of knowledge between organizational units. The successful transfer of knowledge between organizational units is critical for a number of organizational processes and performance outcomes. The empirical evidence on the success of boundary spanners is mixed, however. Research findings indicate boundary spanners can either facilitate or inhibit the flow of knowledge between organizational units. We develop and test a theoretical argument emphasizing the importance of the broader network context in which boundary spanning occurs. In particular, we consider how tie strength, network cohesion, and network range affect the level of knowledge acquired in cross-unit knowledge transfer relationships. An analysis of knowledge transfer relationships among several hundred scientists indicates that each network feature had a positive effect on the level of knowledge acquired in cross-unit knowledge transfer relationships. Our findings illustrate how network features contribute to the flow of knowledge between organizational units and, therefore, how network context contributes to heterogeneity in boundary-spanning outcomes.</t>
@@ -29481,7 +29743,11 @@
       <c r="K577" t="n">
         <v>2012</v>
       </c>
-      <c r="P577" s="8" t="n"/>
+      <c r="P577" s="8" t="inlineStr">
+        <is>
+          <t>The study's correlation matrix is reported at the dyadic/relationship level (N=2,370 relationships) rather than the individual level, and boundary spanning is operationalized as a cross-unit transfer dyadic tie.. Verbatim Evidence: "The 249 individuals who completed the survey were involved in a total of 2,370 knowledge transfer relationships. Because there were multiple observations for each respondent and for each contact, the observed knowledge transfer relationships were not independent."</t>
+        </is>
+      </c>
     </row>
     <row r="578" ht="18" customHeight="1" s="10">
       <c r="A578" t="inlineStr">
@@ -29494,6 +29760,16 @@
           <t>BSMA0575</t>
         </is>
       </c>
+      <c r="E578" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F578" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G578" t="inlineStr">
         <is>
           <t>This study investigates the impact of environmental variability on communications within and outside a large R&amp;D laboratory. For high performing subunits, intra-project communication was found to be contingent on the nature of the unit’s task; extra-unit communication was inversely related to perceived environmental variability, suggesting that communication with external areas may be mediated by special boundary roles.</t>
@@ -29517,7 +29793,11 @@
       <c r="K578" t="n">
         <v>1979</v>
       </c>
-      <c r="P578" s="8" t="n"/>
+      <c r="P578" s="8" t="inlineStr">
+        <is>
+          <t>The boundary spanning communication is measured at the project level by pooling individual responses. Furthermore, the paper does not contain a correlation matrix.. Verbatim Evidence: "Because projects were the unit of analysis, individual responses were pooled."</t>
+        </is>
+      </c>
     </row>
     <row r="579" ht="18" customHeight="1" s="10">
       <c r="A579" t="inlineStr">
@@ -29530,6 +29810,16 @@
           <t>BSMA0576</t>
         </is>
       </c>
+      <c r="E579" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F579" t="inlineStr">
+        <is>
+          <t>Non-Individual Level</t>
+        </is>
+      </c>
       <c r="G579" t="inlineStr">
         <is>
           <t>Research indicates that certain boundary spanning individuals, labelled gatekeepers, can be an important linking mechanism between organizations and their external environments. This study investigates the role of gatekeepers in the transfer of information in a single R&amp;D setting by comparing directly the performance of project groups with and without gatekeepers. Results indicate that gatekeepers perform a linking role only for projects performing tasks that are locally oriented, while universally oriented tasks were most effectively linked to external areas by direct project member communication. Evidence also suggests that gatekeepers do more than mediate external information; they appear to facilitate the external communication of their more local project colleagues. Direct contact and contact mediated by gatekeepers, then, are two contrasting ways to link project groups with their external areas. The relative effectiveness of these linking mechanisms is contingent on the nature of the project's work.</t>
@@ -29553,7 +29843,11 @@
       <c r="K579" t="n">
         <v>1980</v>
       </c>
-      <c r="P579" s="8" t="n"/>
+      <c r="P579" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures boundary spanning at the project group level, not the individual level. It compares the performance of project groups with and without gatekeepers, and does not report a zero-order correlation matrix at the individual level.. Verbatim Evidence: "This study investigates the role of certain boundary spanning individuals, labelled gatekeepers, in the transfer of information in an R&amp;D setting by ccmparing the performance of project groups with and without gatekeepers."</t>
+        </is>
+      </c>
     </row>
     <row r="580" ht="18" customHeight="1" s="10">
       <c r="A580" t="inlineStr">
@@ -29566,6 +29860,16 @@
           <t>BSMA0577</t>
         </is>
       </c>
+      <c r="E580" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F580" t="inlineStr">
+        <is>
+          <t>No Correlation Matrix</t>
+        </is>
+      </c>
       <c r="G580" t="inlineStr">
         <is>
           <t>An investigation of alternative mechanisms by which information is imported into organizations indicates that informational boundary spanning is accomplished only by those individuals who are well connected internally and externally. These key individuals are nominated as technically competent in their unit and have personal characteristics to link effectively their unit to external areas.</t>
@@ -29589,7 +29893,11 @@
       <c r="K580" t="n">
         <v>1981</v>
       </c>
-      <c r="P580" s="8" t="n"/>
+      <c r="P580" s="8" t="inlineStr">
+        <is>
+          <t>The paper does not report a zero-order correlation matrix (Means, SD, and Correlations) for the measured variables, relying instead on contingency tables, ANOVAs, and discriminant analyses.. Verbatim Evidence: "Table 1 Individuals Nominated as 'Valuable Sources of External Information and New Ideas' and Communication Roles... Contingency Coefficient = .27"</t>
+        </is>
+      </c>
     </row>
     <row r="581" ht="18" customHeight="1" s="10">
       <c r="A581" t="inlineStr">
@@ -29602,6 +29910,16 @@
           <t>BSMA0578</t>
         </is>
       </c>
+      <c r="E581" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F581" t="inlineStr">
+        <is>
+          <t>EX_NO_MATRIX</t>
+        </is>
+      </c>
       <c r="G581" t="inlineStr">
         <is>
           <t>This field study investigates the characteristics of internal communication stars, the characteristics of boundary spanning individuals, and the extent to which boundary spanning individuals span multiple communication boundaries. The characteristics of boundary spanning individuals were found to be contingent on their subunit's work and on the information boundary they span. There is substantial boundary role overlap.</t>
@@ -29625,7 +29943,11 @@
       <c r="K581" t="n">
         <v>1981</v>
       </c>
-      <c r="P581" s="8" t="n"/>
+      <c r="P581" s="8" t="inlineStr">
+        <is>
+          <t>The paper does not provide a zero-order correlation matrix. It only reports discriminant analyses and comparisons of means (t-tests) between boundary spanners ('stars') and non-spanners.. Verbatim Evidence: "A stepwise discriminant analysis indicates that hierarchical level is the most powerful determinant of intra-departmental communication, and that professional orientation and laboratory tenure are other important determinants... (standardized discriminant coefficients are, respectively, .70, -.36 and -.34)."</t>
+        </is>
+      </c>
     </row>
     <row r="582" ht="18" customHeight="1" s="10">
       <c r="A582" t="inlineStr">
@@ -29638,6 +29960,16 @@
           <t>BSMA0579</t>
         </is>
       </c>
+      <c r="E582" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F582" t="inlineStr">
+        <is>
+          <t>Non-Individual Level / Discriminant Validity Matrix</t>
+        </is>
+      </c>
       <c r="G582" t="inlineStr">
         <is>
           <t>Prior literature has long examined innovation as a recombination process within or across the boundaries of technological domains. However, limited attention is paid to boundaries per se. Building upon recent development of categorical contrast, this study distinguishes domains with crisp boundaries from those with fuzzy boundaries and examines their effects on innovation outputs. Analyzing a large sample of US patents, we find that spanning crisp boundaries is more likely to generate impactful inventions but at the same time leads to significantly higher recombinant uncertainty. We continue to explore what types of inventors are better able to span such types of domain boundaries. Focusing specifically on the role of inventors’ knowledge expertise, we find that while both knowledge depth and breadth enhance the impact of technologies that span crisp boundaries, knowledge breadth is also found to escalate the associated uncertainty. Our emphasis on the contrast of technological domains contributes to the literature on recombinative innovation and boundary spanning.</t>
@@ -29661,7 +29993,11 @@
       <c r="K582" t="n">
         <v>2023</v>
       </c>
-      <c r="P582" s="8" t="n"/>
+      <c r="P582" s="8" t="inlineStr">
+        <is>
+          <t>The boundary spanning construct is measured at the firm level (Internet start-ups) rather than the individual level. Additionally, the correlation matrix reports latent construct intercorrelations and the square root of the AVE for discriminant validity, rather than raw zero-order Pearson correlations.. Verbatim Evidence: "Table 3. Correlation matrix and descriptive statistics. ... Note: N = 223; *p &lt; 0.05; **p &lt; 0.01. Bold values are the square root of AVE."</t>
+        </is>
+      </c>
     </row>
     <row r="583" ht="18" customHeight="1" s="10">
       <c r="A583" t="inlineStr">
@@ -29674,6 +30010,16 @@
           <t>BSMA0580</t>
         </is>
       </c>
+      <c r="E583" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F583" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G583" t="inlineStr">
         <is>
           <t>Abstract             Although recent years have seen a proliferation of research on organizational ambidexterity, important questions remain about the role that leaders play in leveraging learning ambidexterity for organizational benefits. Drawing on the conservation of resources theory, we investigate the indirect links between servant leadership and middle managers’ learning ambidexterity, with structural empowerment and role breadth self‐efficacy (RBSE) as serial mediators. We also examine the importance of leader boundary‐spanning behaviour as a moderating factor for these relationships. Using time‐lagged and multi‐source data from 344 middle managers and their supervisors, we show that servant leadership has a positive indirect influence on two forms of learning ambidexterity: exploitative and explorative learning. In particular, servant leadership promotes structural empowerment (as a contextual resource), which in turn influences RBSE (as a personal resource) and encourages learning ambidexterity. In addition, we show that when leaders engage in boundary‐spanning behaviour, these indirect relationships become more prominent. This research offers new theoretical and practical insights to assist organizations in improving learning ambidexterity and achieving higher levels of performance.</t>
@@ -29697,7 +30043,11 @@
       <c r="K583" t="n">
         <v>2024</v>
       </c>
-      <c r="P583" s="8" t="n"/>
+      <c r="P583" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures individual-level boundary spanning behaviour (leader's boundary-spanning behaviour) and provides a raw zero-order correlation matrix (Table 2: Means and correlations).. Verbatim Evidence: "Leader boundary-spanning behaviour was also assessed at Time 1 using a six-item scale (α=0.94) developed by Marrone, Tesluk and Carson (2007). Sample item: 'My supervisor reaches out to individuals outside of our organization that can offer expertise or ideas about the task at hand'."</t>
+        </is>
+      </c>
     </row>
     <row r="584" ht="18" customHeight="1" s="10">
       <c r="A584" t="inlineStr">
@@ -29710,6 +30060,16 @@
           <t>BSMA0581</t>
         </is>
       </c>
+      <c r="E584" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F584" t="inlineStr">
+        <is>
+          <t>Non-Individual Anchor</t>
+        </is>
+      </c>
       <c r="G584" t="inlineStr">
         <is>
           <t>We explore whether and how the beneﬁts of openness in innovation are different for small plants (less than 50 employees) compared to medium and large plants. Using panel data from Irish manufacturing we ﬁnd that the contribution of the “breadth” of openness (i.e., the variety of plants’ innovation linkages) on innovation performance is stronger for small plants than for larger plants. Both small and larger plants face diminishing returns as the breadth of openness increases, but small plants experience negative returns at lower level of the breadth of openness than larger plants. Our results suggest that small plants can gain signiﬁcantly from using wider set of innovation linkages, but for such plants appropriate partner choice is a particularly important issue. Small plants also gain signiﬁcantly more than larger ones from investing in the linkages within the supply chain.</t>
@@ -29733,7 +30093,11 @@
       <c r="K584" t="n">
         <v>2014</v>
       </c>
-      <c r="P584" s="8" t="n"/>
+      <c r="P584" s="8" t="inlineStr">
+        <is>
+          <t>The study measures boundary spanning (external knowledge linkages) at the plant/firm level, not the individual level, and does not provide a correlation matrix.. Verbatim Evidence: "We explore whether and how the benefits of openness in innovation are different for small plants (less than 50 employees) compared to medium and large plants."</t>
+        </is>
+      </c>
     </row>
     <row r="585" ht="18" customHeight="1" s="10">
       <c r="A585" t="inlineStr">
@@ -29746,6 +30110,16 @@
           <t>BSMA0582</t>
         </is>
       </c>
+      <c r="E585" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F585" t="inlineStr">
+        <is>
+          <t>No Boundary Spanning Measure</t>
+        </is>
+      </c>
       <c r="G585" t="inlineStr">
         <is>
           <t>The literature recognizes that the sales profession is an inherently competitive and self-interested occupation that can be negatively impacted by deviant behavior and rationalizations of unethical conduct. The unique boundary-spanning nature and autonomy of such work means that there is often little management oversight of sales professionals' behavior, which may lead to misbehavior and poor work attitudes. Yet, evidence suggests that the development of corporate ethical values (CEVs) can mitigate concerns about unethical conduct, suggesting that these principles might be used to reduce workplace bullying and enhance job satisfaction. Using a self-report questionnaire, information was collected from national and regional samples of selling professionals employed in different organizations located in the USA (N = 356). While controlling for the effects of sampling and social desirability, results indicated that increased communication of an ethics code was associated with stronger perceptions of CEVs, while ethical values were negatively related to perceptions of workplace bullying and positively related to job satisfaction. Workplace bullying was also negatively related to job satisfaction. The findings suggest that an ethical work environment should be instituted in sales organizations to reduce misconduct and enhance work attitudes.</t>
@@ -29769,7 +30143,11 @@
       <c r="K585" t="n">
         <v>2015</v>
       </c>
-      <c r="P585" s="8" t="n"/>
+      <c r="P585" s="8" t="inlineStr">
+        <is>
+          <t>The paper examines workplace bullying, job satisfaction, and corporate ethics among selling professionals. It does not measure any individual-level boundary spanning behaviors (e.g., adaptive selling, customer orientation) but rather focuses on intra-organizational interpersonal deviance.. Verbatim Evidence: "The findings suggest that an ethical work environment should be instituted in sales organizations to reduce misconduct and enhance work attitudes. Keywords: corporate ethical values; workplace bullying; job satisfaction"</t>
+        </is>
+      </c>
     </row>
     <row r="586" ht="18" customHeight="1" s="10">
       <c r="A586" t="inlineStr">
@@ -29782,6 +30160,16 @@
           <t>BSMA0583</t>
         </is>
       </c>
+      <c r="E586" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F586" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G586" t="inlineStr">
         <is>
           <t>Programme management is increasingly used in The Netherlands to realize more integrated regional development, where diﬀerent sectoral policy objectives are combined. To understand how integration of diﬀerent objectives is realized in programme management approaches, it is important to have in depth knowledge on how actors manage social, cognitive and physical boundaries. Therefore, this article analyses how actors manage boundaries in a regional integrative programme. Within this case we focus on two integration attempts: one which has succeeded relatively well and one which was less successful. The analysis shows the importance of boundary spanning actions, such as jointly working on strategy documents, organizing events where actors can formally and informally interact, and the activities of a political change agent. Adding to previous insights, we ﬁnd four additional explanations for successful integration which shed new light on how boundaries can be best managed in future programmatic approaches: the inﬂuence of contextual factors on boundary management and its success, the need to address both the social and cognitive dimension of boundaries, the need to make the programme attractive for the actors governing the issues it wants to integrate with, and the role of boundary drawing to create an understanding and respect for boundaries.</t>
@@ -29805,7 +30193,11 @@
       <c r="K586" t="n">
         <v>2020</v>
       </c>
-      <c r="P586" s="8" t="n"/>
+      <c r="P586" s="8" t="inlineStr">
+        <is>
+          <t>Qualitative longitudinal case study based on interviews and observations. No quantitative effect sizes or zero-order correlations are reported.. Verbatim Evidence: "To study in-depth the micro-interactions of boundary management and explore boundary actions and configurations of actions over time we use a single longitudinal case study design... Data is gathered by: (a) semi-structured interviews; (b) document analysis; and (c) observations of actors’ interactions"</t>
+        </is>
+      </c>
     </row>
     <row r="587" ht="18" customHeight="1" s="10">
       <c r="A587" t="inlineStr">
@@ -29818,6 +30210,16 @@
           <t>BSMA0584</t>
         </is>
       </c>
+      <c r="E587" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F587" t="inlineStr">
+        <is>
+          <t>No Boundary Spanning Measure</t>
+        </is>
+      </c>
       <c r="G587" t="inlineStr">
         <is>
           <t>As work increasingly transcends organizational boundaries, employee psychological empowerment benefits from resources provided by others outside of the employee's own team, department, or organization. These intergroup collaborations, however, may be inhibited by social identity and social categorization processes, so that the empowerment potential of these relations remains largely untapped. In this study (N = 213), we demonstrate that intergroup leadership is linked to employee psychological empowerment via intergroup relational identification and access to resources. In this way, this study demonstrates the empowering potential of intergroup leadership and intergroup relational identification for employees who collaborate across group barriers. We finish this paper by discussing the main implications for both empowerment and intergroup leadership theory, suggesting fruitful avenues for future research and highlighting the practical value for those who are motivated to increase psychological empowerment among boundary-spanning employees.</t>
@@ -29841,7 +30243,11 @@
       <c r="K587" t="n">
         <v>2020</v>
       </c>
-      <c r="P587" s="8" t="n"/>
+      <c r="P587" s="8" t="inlineStr">
+        <is>
+          <t>The study does not measure individual-level boundary spanning behaviors. It measures intergroup leadership, intergroup relational identification, access to resources, and psychological empowerment.. Verbatim Evidence: "We measured the extent to which employees had access to resources needed for optimal performance at work from all other individuals (i.e., others within and outside their organization, friends, acquaintances, etc.) with four items."</t>
+        </is>
+      </c>
     </row>
     <row r="588" ht="18" customHeight="1" s="10">
       <c r="A588" t="inlineStr">
@@ -29854,6 +30260,16 @@
           <t>BSMA0585</t>
         </is>
       </c>
+      <c r="E588" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F588" t="inlineStr">
+        <is>
+          <t>Non-Individual Anchor</t>
+        </is>
+      </c>
       <c r="G588" t="inlineStr">
         <is>
           <t>Post-bureaucratic, collaborative organizational arrangements possess great potential for innovation, but alignment of the dissimilar goals, values and interests of participants is required. We propose and empirically test how visionary leadership can increase innovation in multidisciplinary teams, by fostering internal team cohesion and external team boundary management. We rely on longitudinal, multi-source data concerning social welfare professionals and their team leaders across 95 teams. Our results show that visionary leadership is positively related to improved team cohesion and team boundary management over time. The positive relationship between visionary leadership and team innovation is mediated by team cohesion, but not team boundary management.</t>
@@ -29877,7 +30293,11 @@
       <c r="K588" t="n">
         <v>2021</v>
       </c>
-      <c r="P588" s="8" t="n"/>
+      <c r="P588" s="8" t="inlineStr">
+        <is>
+          <t>The study measures boundary spanning (boundary management) at the team level, explicitly aggregating individual responses to the team level for its analysis. This violates the rule that boundary spanning must be measured at the individual level.. Verbatim Evidence: "The individual responses are aggregated to the team level, for which intraclass correlation coefficients are calculated in the analysis section."</t>
+        </is>
+      </c>
     </row>
     <row r="589" ht="18" customHeight="1" s="10">
       <c r="A589" t="inlineStr">
@@ -29890,6 +30310,16 @@
           <t>BSMA0586</t>
         </is>
       </c>
+      <c r="E589" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F589" t="inlineStr">
+        <is>
+          <t>Team-level measurement of boundary spanning</t>
+        </is>
+      </c>
       <c r="G589" t="inlineStr">
         <is>
           <t>The knowledge integration perspective on team innovation holds that information elaboration – the exchange, discussion, and integration of task-relevant information and perspectives – is the core team process driving team innovation. Factors reflecting the informational resources the team can draw on through information elaboration therefore are important influences on team innovation. In this respect, team innovation research points to team functional diversity and to team boundary spanning scouting to acquire information from outside the team. Team innovation research also makes clear that informational resources (as reflected in functional diversity and boundary spanning scouting) do not guarantee team information elaboration, and that identifying moderation in this relationship is particularly valuable. Building on this state of the science, we focus on the moderating role of the team diversity mindset – members' shared understanding of the importance of information elaboration for team performance – in the relationships of team functional diversity and boundary spanning scouting with information elaboration and team innovation. A multi-wave and multisource survey of N = 215 teams involved in knowledge work in various Chinese organizations supported our research model for team boundary spanning scouting but not for team functional diversity.</t>
@@ -29913,7 +30343,11 @@
       <c r="K589" t="n">
         <v>2024</v>
       </c>
-      <c r="P589" s="8" t="n"/>
+      <c r="P589" s="8" t="inlineStr">
+        <is>
+          <t>The study measures boundary spanning at the team level rather than the required individual level.. Verbatim Evidence: "Boundary spanning scouting was measured with Ancona and Caldwell's (1992) three-item scale at T1. We asked the team members to what extent they agreed (1 = strongly disagree; 7 = strongly agree) with the following items 'our team finds out what competing companies or teams are doing on similar projects', 'our team scans the environment inside and outside the company for ideas or expertise', and 'our team collects information or ideas from individuals outside the team'."</t>
+        </is>
+      </c>
     </row>
     <row r="590" ht="18" customHeight="1" s="10">
       <c r="A590" t="inlineStr">
@@ -29926,6 +30360,16 @@
           <t>BSMA0587</t>
         </is>
       </c>
+      <c r="E590" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F590" t="inlineStr">
+        <is>
+          <t>Wrong Level of Analysis</t>
+        </is>
+      </c>
       <c r="G590" t="inlineStr">
         <is>
           <t>Previous research has extensively analyzed the role, and indicated the importance, of network management for the functioning and performance of public or governance networks. In this article, we focus on the inﬂuence of boundary spanning actors in such networks—an aspect less examined in the governance network literature. Boundary spanners are considered to be important for governance network performance. Building on the literature, we expect a mediating role of trust in this relationship. To empirically test these relationships, we conducted survey research (N = 141) among project managers involved in urban governance networks: networks around complex urban projects that include the organizations involved in the governance process (the formulation of policies, decision making, and implementation) in these complex projects. We found a strong positive relationship between the presence of boundary spanners and trust and governance network performance. The results indicate a partially mediating role of trust in this relationship. Furthermore, we found that these boundary spanners originated mainly from private and societal organizations, and less from governmental organizations.</t>
@@ -29949,7 +30393,11 @@
       <c r="K590" t="n">
         <v>2014</v>
       </c>
-      <c r="P590" s="8" t="n"/>
+      <c r="P590" s="8" t="inlineStr">
+        <is>
+          <t>The study measures the perceived presence of boundary spanners at the macro network/project level rather than assessing individual-level boundary spanning behaviors.. Verbatim Evidence: "Our unit of analysis is on the level of the governance network. We study the presence of boundary spanners in the network... We therefore asked the leading project manager of each network to what extent they witnessed boundary spanners in the network."</t>
+        </is>
+      </c>
     </row>
     <row r="591" ht="18" customHeight="1" s="10">
       <c r="A591" t="inlineStr">
@@ -29962,6 +30410,16 @@
           <t>BSMA0588</t>
         </is>
       </c>
+      <c r="E591" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F591" t="inlineStr">
+        <is>
+          <t>No Correlation Matrix</t>
+        </is>
+      </c>
       <c r="G591" t="inlineStr">
         <is>
           <t>Recent team boundary spanning literature has recommended a shift toward assessing the role of virtual tools – such as social media. Simultaneously the proliferation of Enterprise Social Media (ESM) points to the need to theorize and investigate the supra-individual usage of these tools, such as their usefulness for organizational groups. This paper responds to both mandates through a theoretical integration of the team boundary spanning and existing ESM literature. Using data from two studies – one qualitative and one quantitative – this papers addresses two important research questions regarding the empirical relationship between team boundary spanning and ESM for understanding (i) the types of team boundary-spanning activities that group members enact through ESM and (ii) the effects of ESM on extra-team stakeholders’ perceptions and reciprocating actions vis-à-vis the team boundary-spanning activities of these group members. The results of this study show that ESM, largely as a function of their visibility affordance, supports a narrow set of representational activities, but offers only limited support for information search and coordination. Furthermore, the ﬁndings reveal that ESM activity has a positive effect on extra-team stakeholders’ recognition and ﬁnancial support of the representational ESM posts emanating from the boundary-spanning group. Important implications for theory, strategy, and design are discussed.</t>
@@ -29985,7 +30443,11 @@
       <c r="K591" t="n">
         <v>2016</v>
       </c>
-      <c r="P591" s="8" t="n"/>
+      <c r="P591" s="8" t="inlineStr">
+        <is>
+          <t>The paper does not report a zero-order correlation matrix. Additionally, the study focuses on team boundary spanning and the perceptions of extra-team stakeholders rather than individual-level boundary spanning behaviors.. Verbatim Evidence: "Recent team boundary spanning literature has recommended a shift toward assessing the role of virtual tools... this papers addresses two important research questions regarding the empirical relationship between team boundary spanning and ESM"</t>
+        </is>
+      </c>
     </row>
     <row r="592" ht="18" customHeight="1" s="10">
       <c r="A592" t="inlineStr">
@@ -29998,6 +30460,16 @@
           <t>BSMA0589</t>
         </is>
       </c>
+      <c r="E592" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F592" t="inlineStr">
+        <is>
+          <t>No BSB</t>
+        </is>
+      </c>
       <c r="G592" t="inlineStr">
         <is>
           <t>Abstract                            Work increasingly takes place across organizational boundaries. This has implications for workers’ commitments to a plethora of targets, including the organization and the client, as well as for the conflicting nature of the interrelation between these commitments. In this paper, we draw on commitment system theory (CST), which views commitment as a malleable and interconnected system. Using a pragmatic abductive and quantitative discovery approach, we distinguish and develop commitment systems to consist of               strength               , including the multiple targets and types of commitment, as well as               interaction               between commitments, including               coupling               and               nature               . In particular, we develop a theoretical understanding of the               nature               dimension by identifying two target‐neutral types of conflict and one context‐ and target‐specific type of conflict. Three commitment systems are identified: ‘               balanced system               ’, ‘               conflicting system               ’, and ‘               detached system               ’. Furthermore, we provide insights into how job demands resources and contextual job aspects influence membership of these commitment systems. This paper is the first to empirically explore commitment as a system, and it advances the theoretical understanding of commitment systems in a cross‐boundary space. Our study discusses the theoretical, methodological and practical implications for cross‐boundary organizations that compete with their clients for the commitment of their employees.</t>
@@ -30021,7 +30493,11 @@
       <c r="K592" t="n">
         <v>2023</v>
       </c>
-      <c r="P592" s="8" t="n"/>
+      <c r="P592" s="8" t="inlineStr">
+        <is>
+          <t>The paper does not measure any individual-level boundary spanning behaviors. It measures variables such as commitment to the organization and client, perceived support, role ambiguity, role overload, and intention to quit.. Verbatim Evidence: "Table 2. Descriptive statistics, correlations, and reliabilities... Variables: 1 AC organization, 2 NC organization, 3 CC organization, 4 AC client, 5 NC client, 6 CC client, 7 Value-based conflict, 8 Behaviour-based conflict, 9 Cross-boundary conflict, 10 PS organization, 11 PS client, 12 PS supervisor, 13 RA organization, 14 RA client, 15 Job role overload, 16 ITQ organization, 17 ITQ client."</t>
+        </is>
+      </c>
     </row>
     <row r="593" ht="18" customHeight="1" s="10">
       <c r="A593" t="inlineStr">
@@ -30034,6 +30510,16 @@
           <t>BSMA0590</t>
         </is>
       </c>
+      <c r="E593" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F593" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G593" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this paper is to investigate how different team learning activities relate to different types of team performance as rated by team members and managers. Design/methodology/approach – The 624 respondents, working in 88 teams in seven different organizations indicate their perceptions of team learning and their performance ratings of the team. Moreover, managers in the organization are asked to evaluate the team performance.</t>
@@ -30057,7 +30543,11 @@
       <c r="K593" t="n">
         <v>2009</v>
       </c>
-      <c r="P593" s="8" t="n"/>
+      <c r="P593" s="8" t="inlineStr">
+        <is>
+          <t>The study analyzes team learning activities and their impact on team performance, with variables aggregated to the team level and correlations reported in a between-teams correlation matrix.. Verbatim Evidence: "Table I reports the descriptive statistics and the between teams correlations between our scales."</t>
+        </is>
+      </c>
     </row>
     <row r="594" ht="18" customHeight="1" s="10">
       <c r="A594" t="inlineStr">
@@ -30070,6 +30560,16 @@
           <t>BSMA0591</t>
         </is>
       </c>
+      <c r="E594" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F594" t="inlineStr">
+        <is>
+          <t>Latent construct correlations / No BSB</t>
+        </is>
+      </c>
       <c r="G594" t="inlineStr">
         <is>
           <t>Widespread use of social media across work and non-work boundaries has heightened concerns about employee engagement in the contemporary workforce. This study examines how employees’ boundary management preferences inﬂuence their work communication on social media, and how these factors impact their engagement. Results from three waves of survey data (N = 361) demonstrate that work communication mediates the relationship between employee boundary preferences and engagement, supporting the hypothesized causal structure over alternative models. Overall, the ﬁndings contribute a novel perspective on employee engagement by showing that mediated work communication plays a central role in constructing engagement, rather than merely demonstrating it. We discuss how organizations can leverage this knowledge to address critical concerns about workplace (dis)engagement in the digital age.</t>
@@ -30093,7 +30593,11 @@
       <c r="K594" t="n">
         <v>2018</v>
       </c>
-      <c r="P594" s="8" t="n"/>
+      <c r="P594" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures work-life boundary management preferences (not organizational boundary spanning behaviors) and Table 1 reports latent construct correlations (factor correlations) rather than raw, zero-order Pearson correlations.. Verbatim Evidence: "Factor correlations within waves ranged from .08 to .36 demonstrating that the latent constructs as sufficiently distinct (i.e., discriminant validity). Correlations across waves between the same factors ranged from .55 to .80. This suggests that the constructs are relatively stable across measurement points (see Table 1)."</t>
+        </is>
+      </c>
     </row>
     <row r="595" ht="18" customHeight="1" s="10">
       <c r="A595" t="inlineStr">
@@ -30106,6 +30610,16 @@
           <t>BSMA0592</t>
         </is>
       </c>
+      <c r="E595" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F595" t="inlineStr">
+        <is>
+          <t>Not an empirical quantitative study</t>
+        </is>
+      </c>
       <c r="G595" t="inlineStr">
         <is>
           <t>This study focuses on the boundary-spanning nature of sustainable business model innovation, studying multi-stakeholder engagement and alignment. Drawing on the concept of boundary work, we explore the different types of organizational boundary changes between focal companies and their external stakeholders, investigating specifically the process of exploring, negotiating, disrupting and realigning organizational boundaries. Based on an exploratory study of nine different sustainable business model initiatives from for-profit and non-profit organizations, our analysis shows how actors involved need to find alignment at normative, instrumental and strategic dimensions in order to achieve sustainable value creation. However, complexity for alignment emerges through different understandings of value, diverging interests, division of risks and responsibilities, and existing processes and activities that limits actors’ openness to align. Mutual boundary changes are thus necessary in the process of multi-stakeholder engagement in order to enhance organizations’ understanding of value and to capture the envisioned value. This paper functions as an agenda-setting paper, presenting first insights on how the boundary work lens can advance our understanding of alignment processes between focal organizations and their external stakeholders, required for sustainable business model innovation.</t>
@@ -30129,7 +30643,11 @@
       <c r="K595" t="n">
         <v>2020</v>
       </c>
-      <c r="P595" s="8" t="n"/>
+      <c r="P595" s="8" t="inlineStr">
+        <is>
+          <t>The study is a qualitative exploratory comparative case study based on semi-structured interviews. It does not measure individual-level variables or provide a quantitative correlation matrix.. Verbatim Evidence: "To analyze the role of boundary work in SBMI, we used an exploratory comparative case study approach whereby the unit of analysis is the company"</t>
+        </is>
+      </c>
     </row>
     <row r="596" ht="18" customHeight="1" s="10">
       <c r="A596" t="inlineStr">
@@ -30142,6 +30660,16 @@
           <t>BSMA0593</t>
         </is>
       </c>
+      <c r="E596" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F596" t="inlineStr">
+        <is>
+          <t>No Correlation Matrix</t>
+        </is>
+      </c>
       <c r="G596" t="inlineStr">
         <is>
           <t>The goal of this article is to explore the role that shame and embarrassment play within an organization boundary-spanning context. For a sample of 458 salespeople selling ﬁnancial services, measures are developed and hypotheses are tested concerning the effects of shame and embarrassment. The results suggest that the tendency to experience shame and embarrassment in personal selling leads to protective reactions (e.g., avoidance behaviors), and these, in turn, negatively impact performance (e.g., sales volume and quality of sales interaction). Hypotheses are tested on ﬁtting and validation samples, both for salespeople focusing on prospecting tasks and salespeople focusing on relationship building. 2002 Wiley Periodicals, Inc.</t>
@@ -30165,7 +30693,11 @@
       <c r="K596" t="n">
         <v>2002</v>
       </c>
-      <c r="P596" s="8" t="n"/>
+      <c r="P596" s="8" t="inlineStr">
+        <is>
+          <t>The paper does not report a correlation matrix containing zero-order correlations (Pearson r values) between the studied variables.. Verbatim Evidence: "All analyses were performed on the covariance matrices as input (e.g., Cudeck, 1989)."</t>
+        </is>
+      </c>
     </row>
     <row r="597" ht="18" customHeight="1" s="10">
       <c r="A597" t="inlineStr">
@@ -30178,6 +30710,16 @@
           <t>BSMA0594</t>
         </is>
       </c>
+      <c r="E597" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F597" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G597" t="inlineStr">
         <is>
           <t>This dissertation examines the consequences of Electronic Data Interchange (EDI) use on interorganizational relations (IR) in the retail industry. EDI is a type of interorganizational information system that facilitates the exchange of business documents in structured, machine processable form. The research model links EDI use and three IR dimensions--structural, behavioral, and outcome. Based on relevant literature from organizational theory and marketing channels, fourteen hypotheses were proposed for the relationships among EDI use and the three IR dimensions.</t>
@@ -30201,7 +30743,11 @@
       <c r="K597" t="n">
         <v>1994</v>
       </c>
-      <c r="P597" s="8" t="n"/>
+      <c r="P597" s="8" t="inlineStr">
+        <is>
+          <t>Data was collected at the organizational level.. Verbatim Evidence: "Since the study seeks to measure organizational level constructs, data were collected from key informants (Anderson, 1987) in the sample organizations."</t>
+        </is>
+      </c>
     </row>
     <row r="598" ht="18" customHeight="1" s="10">
       <c r="A598" t="inlineStr">
@@ -30214,6 +30760,16 @@
           <t>BSMA0595</t>
         </is>
       </c>
+      <c r="E598" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F598" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G598" t="inlineStr">
         <is>
           <t>Purpose – This paper aims to draw upon motivated information processing theory to examine the sequential mediating roles of perspective taking and boundary spanning between transformational leadership and the creative performance of knowledge workers.</t>
@@ -30237,7 +30793,11 @@
       <c r="K598" t="n">
         <v>2021</v>
       </c>
-      <c r="P598" s="8" t="n"/>
+      <c r="P598" s="8" t="inlineStr">
+        <is>
+          <t>The study measures individual-level boundary spanning behaviors and provides a valid zero-order correlation matrix.. Verbatim Evidence: "Boundary spanning was accessed using the four-item subscale taken from Marrone et al. (2007). A sample item was, 'I proactively seek the advice and support of my faculty advisor'."</t>
+        </is>
+      </c>
     </row>
     <row r="599" ht="18" customHeight="1" s="10">
       <c r="A599" t="inlineStr">

</xml_diff>

<commit_message>
chore: completed Batch 16 extraction
</commit_message>
<xml_diff>
--- a/BSMA_AI_Run_V2.xlsx
+++ b/BSMA_AI_Run_V2.xlsx
@@ -30810,6 +30810,16 @@
           <t>BSMA0596</t>
         </is>
       </c>
+      <c r="E599" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F599" t="inlineStr">
+        <is>
+          <t>EXCL-01</t>
+        </is>
+      </c>
       <c r="G599" t="inlineStr">
         <is>
           <t>For teams developing products or services to meet customer needs, customer adoption of team deliverables is core to their success. When such teams focus on complex, tailored deliverables, customer adoption can be expected to benefit from team information elaboration—the exchange, discussion, and integration of team members' knowledge and perspectives—to develop solutions for customer needs. We aim to shed light on how teams can focus on the customer's perspective within the elaboration process to drive customer adoption. We propose that whereas engaging with the customer's perspective is key to customer adoption, teams may only do this to a modest degree unless they are stimulated to put the customer perspective center-stage. Extending information elaboration theory by drawing on the attention-based view, we propose that customer-oriented boundary spanning—engaging with the customer to champion the customer's perspective within the team—strengthens the shared objective of serving the customer to guide information elaboration and increase the quality of knowledge work. We argue that this effect is moderated by team functional background diversity: increased attention to the customer's perspective guides teams to better use their informational resources and this benefit is stronger with greater functional background diversity. These predictions were supported in a field experiment with a customer-oriented boundary spanning intervention (N = 144 teams). Shared objectives and information elaboration sequentially mediated the effect of customer-oriented boundary spanning and the indirect effect from customer-oriented boundary spanning to customer adoption was stronger with greater functional diversity.</t>
@@ -30833,7 +30843,11 @@
       <c r="K599" t="n">
         <v>2025</v>
       </c>
-      <c r="P599" s="8" t="n"/>
+      <c r="P599" s="8" t="inlineStr">
+        <is>
+          <t>The study's unit of analysis is the team, not the individual, and boundary spanning is manipulated/measured at the team level.. Verbatim Evidence: "The unit of analysis is the customer engagement team with team sizes ranging from 3 to 27... Individual team member responses were aggregated to the team level by computing the means resulting in 162 team cases. ... The remaining N=144 teams are the basis for the analysis"</t>
+        </is>
+      </c>
     </row>
     <row r="600" ht="18" customHeight="1" s="10">
       <c r="A600" t="inlineStr">
@@ -30846,6 +30860,16 @@
           <t>BSMA0597</t>
         </is>
       </c>
+      <c r="E600" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F600" t="inlineStr">
+        <is>
+          <t>NON_INDIVIDUAL</t>
+        </is>
+      </c>
       <c r="G600" t="inlineStr">
         <is>
           <t>In this study, I assess the causal impact of boundary spanning on team innovation. I explore conditions and processes in 144 engagement teams in an enterprise software company driving innovation with customers in North America across industries. In this context, innovation is defined as the development and implementation of technology-based ideas in organizations. Using an integrated conditional process analysis, I find that boundary-spanning team practices combined with a shared vision and functional background diversity lead to a significant team innovation increase. I further assess the team process of information elaboration through which functional diversity and boundary spanning foster solution use. In particular, I argue that boundary spanning amplifies the effects of shared vision and information elaboration, leading to significantly increased team innovation. Consistent with this argument, I find that functional diversity's positive impact on team innovation through information elaboration is conditional on a shared vision, whereas the impact is more significant when team members share a commitment to common goals for their work. Therefore, my findings contribute actionable insight into how to enable cross-functional engagement teams to successfully drive customer innovation with enterprise software in the technology industry.</t>
@@ -30869,7 +30893,11 @@
       <c r="K600" t="n">
         <v>2021</v>
       </c>
-      <c r="P600" s="8" t="n"/>
+      <c r="P600" s="8" t="inlineStr">
+        <is>
+          <t>The unit of analysis is the team, and boundary spanning is measured as a team-level binary treatment variable.. Verbatim Evidence: "The unit of analysis is the customer engagement team with team sizes ranging from 3 to 27 and a median of 9 members... The boundary-spanning treatment was measured with a binary variable separating treatment and control group wherein zero identified the control group and one the treatment group."</t>
+        </is>
+      </c>
     </row>
     <row r="601" ht="18" customHeight="1" s="10">
       <c r="A601" t="inlineStr">
@@ -30882,6 +30910,16 @@
           <t>BSMA0598</t>
         </is>
       </c>
+      <c r="E601" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F601" t="inlineStr">
+        <is>
+          <t>EXCLUDE - Qualitative</t>
+        </is>
+      </c>
       <c r="G601" t="inlineStr">
         <is>
           <t>Being connected to the Internet through various mobile devices is pervasive in our daily professional and private lives. Yet, the way people connect, including when, with whom and through which communication channels differs, manifesting individuals’ idiosyncratic connectivity patterns. In team collaboration, where individuals are dependent on each other’s availability and responsiveness, differences in team members’ connectivity patterns can lead to clashing expectations concerning connectivity. This, in turn, can compromise individuals’ well-being and productivity and threaten team collaboration outcomes. In this paper, we address the question of how to manage connectivity in interdependent teams and align connectivity patterns to facilitate successful collaboration while at the same time safeguarding individuals’ connectivity boundaries. To address this question, we conducted a qualitative case study that involved 39 semi-structured interviews with employees and members of the management board of an international consultancy headquartered in Germany. Building on concepts established in boundary theory, we coined the term “connectivity boundaries” and identiﬁed the six boundary work tactics, externalizing, accommodating, adapting, pushing, sacriﬁcing, and enforcing that allow team members to create, maintain, temporarily change, and reclaim their connectivity boundaries and achieve team collaboration success. We developed propositions that highlight which contextual factors and goals are associated with which boundary work tactic.</t>
@@ -30905,7 +30943,11 @@
       <c r="K601" t="n">
         <v>2024</v>
       </c>
-      <c r="P601" s="8" t="n"/>
+      <c r="P601" s="8" t="inlineStr">
+        <is>
+          <t>The study is a qualitative case study and does not provide quantitative correlation data.. Verbatim Evidence: "we conducted a qualitative case study that involved 39 semi-structured interviews with employees"</t>
+        </is>
+      </c>
     </row>
     <row r="602" ht="18" customHeight="1" s="10">
       <c r="A602" t="inlineStr">
@@ -30918,6 +30960,16 @@
           <t>BSMA0599</t>
         </is>
       </c>
+      <c r="E602" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F602" t="inlineStr">
+        <is>
+          <t>Wrong Level of Analysis</t>
+        </is>
+      </c>
       <c r="G602" t="inlineStr">
         <is>
           <t>In the era of digital economy, business model innovation (BMI) has become an important way for companies to achieve digital transformation and gain new competitive advantages, but there is still a lack of research on the impact mechanism of BMI. Based on the social network theory perspective, this paper explores the influence of external social network (ESN) on BMI and the mediating role of business model boundary-spanning search (BMBS) and the moderating role of slack resources (SR). Through the survey and data analysis of 201 Chinese companies, this paper found that ESN has a significant positive impact on BMI. In addition, BMBS played a partial mediating role between ESN and BMI. At the same time, SR positively moderates the relationship between BMBS and BMI and the mediating effect of BMBS. The findings enrich the study about the influencing mechanism of BMI and provide insights into the BMI practice of companies in the context of digital transformation.</t>
@@ -30941,7 +30993,11 @@
       <c r="K602" t="n">
         <v>2024</v>
       </c>
-      <c r="P602" s="8" t="n"/>
+      <c r="P602" s="8" t="inlineStr">
+        <is>
+          <t>The study measures boundary spanning at the firm/company level rather than the individual level.. Verbatim Evidence: "Since the research variables of this paper focus on the company level, higher requirements are put forward for the questionnaire filling."</t>
+        </is>
+      </c>
     </row>
     <row r="603" ht="18" customHeight="1" s="10">
       <c r="A603" t="inlineStr">
@@ -30954,6 +31010,16 @@
           <t>BSMA0600</t>
         </is>
       </c>
+      <c r="E603" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F603" t="inlineStr">
+        <is>
+          <t>No Empirical Data</t>
+        </is>
+      </c>
       <c r="G603" t="inlineStr">
         <is>
           <t>Social movement scholarship has increasingly sought to understand the relational dynamics of internal movement activity, from investigating the factors that enable movement coalitions to analyzing the trade-offs of organizational hybridity. We bring these and other related phenomena together under the label of boundary-spanning processes. Speciﬁcally, we organize research on boundary-spanning in social movements by identifying three types of boundaries that have symbolic signiﬁcance as categorical demarcations: (a) issue and identity boundaries, (b) organizational boundaries, and (c) tactical boundaries. We then elucidate the tension in work that has examined how each form of boundary-spanning either promotes or hinders the realization of three important movement outcomes: (a) mobilization, (b) internal movement solidarity and scope, and (c) external social and political change. We relate our three types of boundary-spanning to these three types of outcomes in an organizing framework to locate future opportunities for research on boundary-spanning in social movements.</t>
@@ -30977,7 +31043,11 @@
       <c r="K603" t="n">
         <v>2018</v>
       </c>
-      <c r="P603" s="8" t="n"/>
+      <c r="P603" s="8" t="inlineStr">
+        <is>
+          <t>The paper is a theoretical review rather than an empirical study and does not contain a quantitative correlation matrix.. Verbatim Evidence: "Specifically, we organize research on boundary-spanning in social movements by identifying three types of boundaries that have symbolic significance as categorical demarcations: (a) issue and identity boundaries, (b) organizational boundaries, and (c) tactical boundaries."</t>
+        </is>
+      </c>
     </row>
     <row r="604" ht="18" customHeight="1" s="10">
       <c r="A604" t="inlineStr">
@@ -30990,6 +31060,16 @@
           <t>BSMA0601</t>
         </is>
       </c>
+      <c r="E604" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F604" t="inlineStr">
+        <is>
+          <t>Firm-Level Analysis / Latent Construct Correlations</t>
+        </is>
+      </c>
       <c r="G604" t="inlineStr">
         <is>
           <t>This study develops a model to examine whether intraﬁrm, hard and soft IT skills have cross-boundary effects on interﬁrm collaboration and integration, thus leading to better supply-chain performance. A model with eight hypotheses was developed and tested using data collected from 250 Taiwanese manufacturing ﬁrms. Seven hypotheses ﬁnd empirical support. The results show that intraﬁrm IT skills indeed can beneﬁt interﬁrm collaboration and integration and thus, supply-chain performance. Our ﬁndings suggest that the value of skilled IT professionals for interﬁrm integration, supply-chain performance and collaborative relationships between ﬁrms is critical for realizing that value.</t>
@@ -31013,7 +31093,11 @@
       <c r="K604" t="n">
         <v>2014</v>
       </c>
-      <c r="P604" s="8" t="n"/>
+      <c r="P604" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures constructs at the firm/department level rather than individual-level boundary spanning behaviors (e.g., 'Our firm and its major supplier...'). Additionally, the correlation matrix (Table 4) contains latent construct correlations used for discriminant validity, rather than raw, zero-order correlations.. Verbatim Evidence: "Our firm and its major supplier coordinate their efforts harmoniously. [...] Second, the square root of the AVE of a construct should be greater than the correlations between the construct and all other constructs in the model [29]. As shown in Table 4 and Appendix B, both criteria are clearly met, demonstrating sufficient construct validity of the scales."</t>
+        </is>
+      </c>
     </row>
     <row r="605" ht="18" customHeight="1" s="10">
       <c r="A605" t="inlineStr">
@@ -31026,6 +31110,16 @@
           <t>BSMA0602</t>
         </is>
       </c>
+      <c r="E605" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F605" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G605" t="inlineStr">
         <is>
           <t>Building upon the ambidexterity perspective, this study conceptualizes boundary-spanning activities as both transactional and learning to illuminate their different effects on IT employees’ job satisfaction. Specifically, we offer an overarching theoretical framework rooted in ambidexterity by connecting the role theory and knowledge acquisition perspective to reconcile the inconsistency of extant findings. Role overload has a mediating effect on the relationship between boundary-spanning activities (both transactional and learning) and job satisfaction, whereas knowledge acquisition mediates the relationship between learning boundary-spanning activities and job satisfaction. Furthermore, high achievement motivation and learning goal orientation moderate the positive effect of learning boundary-spanning activities on job satisfaction. The quantitative analysis of IT employees in Chinese state-owned enterprises largely supports our hypotheses. We conclude this paper by discussing theoretical and managerial implications for ambidexterity, boundary spanning, and job satisfaction.</t>
@@ -31049,7 +31143,11 @@
       <c r="K605" t="n">
         <v>2019</v>
       </c>
-      <c r="P605" s="8" t="n"/>
+      <c r="P605" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures individual-level boundary spanning activities (transactional and learning) of IT employees and contains a valid zero-order correlation matrix with Means and SDs.. Verbatim Evidence: "Table 1 Descriptive statistics and correlation coefficient of the variables"</t>
+        </is>
+      </c>
     </row>
     <row r="606" ht="18" customHeight="1" s="10">
       <c r="A606" t="inlineStr">
@@ -31062,6 +31160,16 @@
           <t>BSMA0603</t>
         </is>
       </c>
+      <c r="E606" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F606" t="inlineStr">
+        <is>
+          <t>Not Individual-Level BSB</t>
+        </is>
+      </c>
       <c r="G606" t="inlineStr">
         <is>
           <t>Drawing on the knowledge-based view, this study examines the effect of business process digitisation on firm innovation performance. Furthermore, we investigate the mediating role of knowledge search (i.e., local search and boundary-spanning search) and the moderating effect of digital culture by focusing on the relationship between business process digitisation and firm innovation performance. The results, based on 330 questionnaire survey responses, show that business process digitisation has a positive effect on firm innovation performance, knowledge search plays a mediating role between business process digitisation and firm innovation performance, and digital culture has a positive moderating effect, which is mainly reflected in business process digitisation and boundary-spanning search. This study provides inspiration for firms to improve innovation performance through business process digitisation and expands the literature on knowledge search and firm innovation in the digital context.</t>
@@ -31085,7 +31193,11 @@
       <c r="K606" t="n">
         <v>2024</v>
       </c>
-      <c r="P606" s="8" t="n"/>
+      <c r="P606" s="8" t="inlineStr">
+        <is>
+          <t>The paper does not measure an individual-level boundary spanning behavior. Horizontal knowledge transfer is measured as a dyad-level construct (the sum of the Chinese and foreign managers' scores), and vertical knowledge transfer is measured as an organizational-level outcome (the extent to which the parent firm acquired knowledge).. Verbatim Evidence: "We calculated the sum of the scores of the dyadic Chinese and foreign managers to measure the total knowledge learned and generated in the IJVs for subsequent analyses."</t>
+        </is>
+      </c>
     </row>
     <row r="607" ht="18" customHeight="1" s="10">
       <c r="A607" t="inlineStr">
@@ -31098,6 +31210,16 @@
           <t>BSMA0604</t>
         </is>
       </c>
+      <c r="E607" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F607" t="inlineStr">
+        <is>
+          <t>DISCRIMINANT_VALIDITY_MATRIX</t>
+        </is>
+      </c>
       <c r="G607" t="inlineStr">
         <is>
           <t>Purpose – This study aims to examine the inﬂuence of perceived organizational support (POS) on boundary-spanning behaviors (BSBs) among frontline employees in the hospitality industry. It also considered perceived supervisory support (PSS) as a moderating factor within a conceptual model.</t>
@@ -31121,7 +31243,11 @@
       <c r="K607" t="n">
         <v>2024</v>
       </c>
-      <c r="P607" s="8" t="n"/>
+      <c r="P607" s="8" t="inlineStr">
+        <is>
+          <t>The paper does not report a standard zero-order correlation matrix with Means and SDs. It only provides a Discriminant Validity assessment matrix (Table 3), which is explicitly forbidden by the zero-order correlation lock rule.. Verbatim Evidence: "Table 3. Discriminant validity assessment"</t>
+        </is>
+      </c>
     </row>
     <row r="608" ht="18" customHeight="1" s="10">
       <c r="A608" t="inlineStr">
@@ -31134,6 +31260,16 @@
           <t>BSMA0605</t>
         </is>
       </c>
+      <c r="E608" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F608" t="inlineStr">
+        <is>
+          <t>No Zero-Order Correlation Matrix</t>
+        </is>
+      </c>
       <c r="G608" t="inlineStr">
         <is>
           <t>Purpose – This study aims to investigate the antecedents of frontline employees’ boundary-spanning behaviors in the hospitality industry. Anchored in transactional stress theory, affective events theory and motivation theories, a conceptual model was built to explore the impacts of hindrance stressors on boundary-spanning behavior.</t>
@@ -31157,7 +31293,11 @@
       <c r="K608" t="n">
         <v>2021</v>
       </c>
-      <c r="P608" s="8" t="n"/>
+      <c r="P608" s="8" t="inlineStr">
+        <is>
+          <t>The paper does not provide a raw, zero-order correlation matrix. The matrix provided in Table 3 is explicitly labeled 'Discriminant validity assessment', where the diagonal represents AVEs and the off-diagonal represents squared correlation coefficients.. Verbatim Evidence: "As shown in Table 3, AVE scores for all dimensions, presented in the diagonal of the matrix, exceeded the squares of paired correlation coefficients, shown in the off-diagonal of the matrix, satisfying discriminant validity (Chin, 1998)."</t>
+        </is>
+      </c>
     </row>
     <row r="609" ht="18" customHeight="1" s="10">
       <c r="A609" t="inlineStr">
@@ -31170,6 +31310,16 @@
           <t>BSMA0606</t>
         </is>
       </c>
+      <c r="E609" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F609" t="inlineStr">
+        <is>
+          <t>No Valid Correlation Matrix</t>
+        </is>
+      </c>
       <c r="G609" t="inlineStr">
         <is>
           <t>The present study explores the antecedents of frontline employees’ boundary-spanning behaviors in the hospitality industry. Based on social exchange theory and role theory, a conceptual model was built to explore how three dimensions of perceived organizational support (perceived supervisory support, internal communication, and training) cultivate frontline employees’ boundary-spanning behaviors through job satisfaction and organizational commitment. Based on the analysis of 597 hospitality frontline employees in the United States, which were recruited through Amazon Mechanical Turk, this study shows the differential impacts of organizational support types on driving boundary spanning staff to effectively operate on the boundary. Theoretical and practical implications of the findings are articulated.</t>
@@ -31193,7 +31343,11 @@
       <c r="K609" t="n">
         <v>2022</v>
       </c>
-      <c r="P609" s="8" t="n"/>
+      <c r="P609" s="8" t="inlineStr">
+        <is>
+          <t>The paper does not provide a raw, zero-order correlation matrix (with Means and SDs). Instead, it only provides Table 2 labeled 'Assessment of discriminant validity', which contains AVEs on the diagonal and squared or latent correlations off the diagonal.. Verbatim Evidence: "Table 2. Assessment of discriminant validity."</t>
+        </is>
+      </c>
     </row>
     <row r="610" ht="18" customHeight="1" s="10">
       <c r="A610" t="inlineStr">
@@ -31206,6 +31360,16 @@
           <t>BSMA0607</t>
         </is>
       </c>
+      <c r="E610" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F610" t="inlineStr">
+        <is>
+          <t>Level of Analysis (Firm)</t>
+        </is>
+      </c>
       <c r="G610" t="inlineStr">
         <is>
           <t>Building on resource‐based theory and resource orchestration theory, we investigate the impact of two characteristics of boundary‐spanning search, search breadth and search depth, on firms' exploitative and exploratory green innovations. We also examine the moderating role of resource orchestration capability. The results of data analysis from 186 manufacturing firms in China show that both search breadth and search depth have inverted U‐shaped relationships with exploitative and exploratory green innovations. Furthermore, resource orchestration capability is found to moderate the inverted U‐shaped relationship between boundary‐spanning search and green innovation. Specifically, with high resource orchestration capability, the inverted U‐shaped relationships of search breadth with exploitative and exploratory green innovations are flattened, whereas the relationships of search depth with exploitative and exploratory green innovations are almost linear. Our research contributes to the literature on green innovation by uncovering the complex effects of boundary‐spanning search on exploitative and exploratory green innovations.</t>
@@ -31229,7 +31393,11 @@
       <c r="K610" t="n">
         <v>2020</v>
       </c>
-      <c r="P610" s="8" t="n"/>
+      <c r="P610" s="8" t="inlineStr">
+        <is>
+          <t>The study measures boundary spanning search at the firm level (manufacturing firms) rather than the individual level.. Verbatim Evidence: "The results of data analysis from 186 manufacturing firms in China show that both search breadth and search depth have inverted U-shaped relationships with exploitative and exploratory green innovations."</t>
+        </is>
+      </c>
     </row>
     <row r="611" ht="18" customHeight="1" s="10">
       <c r="A611" t="inlineStr">
@@ -31242,6 +31410,16 @@
           <t>BSMA0608</t>
         </is>
       </c>
+      <c r="E611" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F611" t="inlineStr">
+        <is>
+          <t>Wrong Level of Analysis</t>
+        </is>
+      </c>
       <c r="G611" t="inlineStr">
         <is>
           <t>Green innovation is critical for firms' sustainable development, and its antecedents have attracted extensive attention. However, how proactive boundary-spanning search enhances firms' green innovation remains unclear. Building on the resourcebased view and dynamic capabilities theory, we explore the impact of proactive boundary-spanning search on firms' green innovation and investigate the mediating role of two types of organizational resilience. Survey data are collected from 218 manufacturing firms in China, and hierarchical regression and bootstrap analysis are used to test hypotheses. The results demonstrate that proactive boundaryspanning search not only has an inverted U-shaped relationship with radical green innovation and incremental green innovation, but also has an inverted U-shaped relationship with precursor resilience and improvisation resilience. Moreover, the results show that precursor resilience and improvisation resilience partially mediate the inverted U-shaped relationship between proactive boundary-spanning search and the two types of green innovation. This research reveals the nonlinear relationship between proactive boundary-spanning search and green innovation, which enriches the research of green innovation by considering organizational resilience.</t>
@@ -31265,7 +31443,11 @@
       <c r="K611" t="n">
         <v>2023</v>
       </c>
-      <c r="P611" s="8" t="n"/>
+      <c r="P611" s="8" t="inlineStr">
+        <is>
+          <t>The study focuses on boundary-spanning search at the firm level, not the individual level.. Verbatim Evidence: "Proactive boundary-spanning search was adapted from Katila and Ahuja (2002) and Wang et al. (2020), including four items: "Our firm has many channels to search new domain knowledge ahead of competitors...""</t>
+        </is>
+      </c>
     </row>
     <row r="612" ht="18" customHeight="1" s="10">
       <c r="A612" t="inlineStr">
@@ -31278,6 +31460,16 @@
           <t>BSMA0609</t>
         </is>
       </c>
+      <c r="E612" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F612" t="inlineStr">
+        <is>
+          <t>Non-Individual Level</t>
+        </is>
+      </c>
       <c r="G612" t="inlineStr">
         <is>
           <t>Purpose – This paper aims to analyze the mechanism underlying the impact of boundary-spanning search (BS) on the sustainable development ability (SDA) of service-oriented manufacturing enterprises and to emphasize the intermediary role of knowledge integration (KI). The moderating role of knowledge inertia on the link between BS and KI is also investigated.</t>
@@ -31301,7 +31493,11 @@
       <c r="K612" t="n">
         <v>2023</v>
       </c>
-      <c r="P612" s="8" t="n"/>
+      <c r="P612" s="8" t="inlineStr">
+        <is>
+          <t>The study measures boundary-spanning search at the enterprise (firm) level, not at the individual level. The sample consists of 110 service-oriented manufacturing enterprises.. Verbatim Evidence: "BS refers to the behavior of enterprises to search for external knowledge resources across organizational boundaries (Grimpe and Sofka, 2009)."</t>
+        </is>
+      </c>
     </row>
     <row r="613" ht="18" customHeight="1" s="10">
       <c r="A613" t="inlineStr">
@@ -31314,6 +31510,16 @@
           <t>BSMA0610</t>
         </is>
       </c>
+      <c r="E613" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F613" t="inlineStr">
+        <is>
+          <t>Non-Individual Level</t>
+        </is>
+      </c>
       <c r="G613" t="inlineStr">
         <is>
           <t>Previous studies on IT alignment have attempted to address if, and how, the presence of IT outsourcing can help attain IT alignment. In this study, we advance the literature by investigating how organizations appropriate IT outsourcing for achieving IT alignment. Specifically, drawing on the adaptive structuration theory (AST), we construct a model examining factors associated with outsourcing appropriation, including consensus of appropriation (COA) and faithfulness of appropriation (FOA), and how the latter are associated with IT alignment. To test our proposed model, we use a questionnaire survey of 170 IT executives working in Chinese firms. Our results indicate that both shared IT affordance for knowledge acquisition and boundary spanning positively affect COA and FOA. Boundary buffering positively affects the FOA, but not the COA. Further, our results also show the positive effects on IT alignment from COA and FOA, and the significant moderating effects of adoption of cloud computing and the non-significant moderating effects of degree of outsourcing in the relationships. Interestingly, the moderating effects of three cloud computing adoption modes (SaaS, PaaS, and IaaS) on the impact of outsourcing appropriation on IT alignment vary significantly. These findings enrich our understanding towards how to appropriate IT outsourcing for IT alignment and contribute to the literature on IT alignment in IT outsourcing.</t>
@@ -31337,7 +31543,11 @@
       <c r="K613" t="n">
         <v>2023</v>
       </c>
-      <c r="P613" s="8" t="n"/>
+      <c r="P613" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures boundary spanning and boundary buffering behaviors at the organizational/departmental level (i.e., the IT department), rather than at the individual level.. Verbatim Evidence: "The boundary spanning and boundary buffering scales were measured using four items adopted by Faraj and Yan (2009), and were mainly concerned with the boundary spanning and boundary buffering behavior of IT departments with the IT department as the boundary. An example for boundary spanning was “To what extent does the IT department encourage its staff to solicit information and resources from elsewhere in and/or beyond the department”"</t>
+        </is>
+      </c>
     </row>
     <row r="614" ht="18" customHeight="1" s="10">
       <c r="A614" t="inlineStr">
@@ -31350,6 +31560,16 @@
           <t>BSMA0611</t>
         </is>
       </c>
+      <c r="E614" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F614" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G614" t="inlineStr">
         <is>
           <t>Based on social information processing theory, we provide a novel theoretical account of how and when leader humor influences subordinate boundary-spanning behavior. We develop a moderated mediation model explicating the mechanism of psychological safety and the boundary condition of subordinate interpersonal influence. Using multiwave data, we tested our research hypotheses with a sample of 452 members from 140 teams in a Chinese information technology (IT) company. Results showed that leader humor positively affects subordinate boundary-spanning behavior               via               increased psychological safety. Moreover, this mediated effect is stronger when subordinates have high interpersonal influence. These findings offer theoretical and practical insights into boundary-spanning activities and leader humor, which we discuss.</t>
@@ -31373,7 +31593,11 @@
       <c r="K614" t="n">
         <v>2022</v>
       </c>
-      <c r="P614" s="8" t="n"/>
+      <c r="P614" s="8" t="inlineStr">
+        <is>
+          <t>The study measures individual-level boundary-spanning behavior and provides a valid zero-order correlation matrix.. Verbatim Evidence: "We measured boundary-spanning behavior with a six-item scale developed by Marrone et al. (2007). Subordinates were asked to evaluate the extent to which they engage in boundary-spanning behavior."</t>
+        </is>
+      </c>
     </row>
     <row r="615" ht="18" customHeight="1" s="10">
       <c r="A615" t="inlineStr">
@@ -31386,6 +31610,16 @@
           <t>BSMA0612</t>
         </is>
       </c>
+      <c r="E615" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F615" t="inlineStr">
+        <is>
+          <t>EXC_LATENT_CORRELATIONS</t>
+        </is>
+      </c>
       <c r="G615" t="inlineStr">
         <is>
           <t>The turnover of IT professionals is a perpetual challenge for non-IT organizations. Based on selfcategorization theory, this study proposes that IT employees’ turnover may be mitigated by fostering their identification with non-IT organizations, which can be done by meeting various facilitative conditions. Guided by intergroup contact theory, we identify IT employees’ perceived alignment between IT and the core business of an organization (business-IT alignment), the extent of boundaryspanning activities that IT employees engage in, and the closeness of the relationships between IT and non-IT employees as the drivers of their organizational identification. Using survey data collected from organizations in different industries, we obtained empirical evidence supporting the positive effects of the perceived business-IT alignment, the extent of boundary-spanning activities, and the relationship closeness between IT and non-IT employees on IT employees’ organizational identification. Additionally, there was a three-way interaction effect among the three drivers such that the relationship closeness between IT and non-IT employees reduced the positive effect of the extent of boundary-spanning activities on IT employees’ organizational identification when business-IT alignment was low. However, this negative moderating effect diminished when business-IT alignment increased. The findings of this research advance the literature and offer practical guidelines for non-IT organizations on how to enhance their IT employees’ organizational identification and how to mitigate their turnover intentions.</t>
@@ -31409,7 +31643,11 @@
       <c r="K615" t="n">
         <v>2022</v>
       </c>
-      <c r="P615" s="8" t="n"/>
+      <c r="P615" s="8" t="inlineStr">
+        <is>
+          <t>The paper only provides a correlation matrix used for assessing discriminant validity, containing latent interconstruct correlations rather than raw, zero-order Pearson correlations.. Verbatim Evidence: "Discriminant validity was assessed by comparing the square root of the average variance extracted (AVE) of a construct with interconstruct correlations. Correlation results in Table 7 show that all constructs demonstrated satisfactory discriminant validity."</t>
+        </is>
+      </c>
     </row>
     <row r="616" ht="18" customHeight="1" s="10">
       <c r="A616" t="inlineStr">
@@ -31422,6 +31660,16 @@
           <t>BSMA0613</t>
         </is>
       </c>
+      <c r="E616" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F616" t="inlineStr">
+        <is>
+          <t>Non-Individual Level</t>
+        </is>
+      </c>
       <c r="G616" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this paper is to investigate the individual effects of boundary-spanning search from suppliers (supplier-side search (SS)). It is proposed that SS contributes to innovation ambidexterity (IA) and then business performance (BP). Further, this paper includes buyer–supplier relationships (BSRs) and competitive intensity (CI) as moderators to clarify boundary conditions.</t>
@@ -31445,7 +31693,11 @@
       <c r="K616" t="n">
         <v>2019</v>
       </c>
-      <c r="P616" s="8" t="n"/>
+      <c r="P616" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures supplier-side boundary-spanning search at the firm level, rather than the individual level, violating the unit of analysis requirement.. Verbatim Evidence: "Supplier-side search. According to the work of Laursen and Salter (2006), SS refers to the extent to which a firm draws intensively from its suppliers."</t>
+        </is>
+      </c>
     </row>
     <row r="617" ht="18" customHeight="1" s="10">
       <c r="A617" t="inlineStr">
@@ -31458,6 +31710,16 @@
           <t>BSMA0614</t>
         </is>
       </c>
+      <c r="E617" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F617" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G617" t="inlineStr">
         <is>
           <t>Frontline service employees (FSEs)’ customer-oriented boundary spanning behaviors (COBSBs) are prosocial behaviors adapted to the job requirements and work environment of customer service personnel. It is a significant strategic imperative for achieving excellent performance in the tourism organizations. Building on social exchange theory, this study uncovered that inclusive leadership motivates FSEs’ COBSBs. Using hierarchical multiple regression analysis with time-lagged data, we find that inclusive leadership promotes FSEs’ COBSBs by enhancing their felt obligations. Moreover, the need for affiliation enhances the direct effect that inclusive leadership has on felt obligations and its indirect effect on FSEs’ COBSBs via felt obligations.</t>
@@ -31481,7 +31743,11 @@
       <c r="K617" t="n">
         <v>2024</v>
       </c>
-      <c r="P617" s="8" t="n"/>
+      <c r="P617" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures individual-level customer-oriented boundary spanning behaviors (COBSBs) and provides a raw zero-order correlation matrix (Table 2) that includes these measures alongside demographic control variables.. Verbatim Evidence: "Table 2. Means, Standard Deviations and Correlations of All Variables in the Study."</t>
+        </is>
+      </c>
     </row>
     <row r="618" ht="18" customHeight="1" s="10">
       <c r="A618" t="inlineStr">
@@ -31494,6 +31760,16 @@
           <t>BSMA0615</t>
         </is>
       </c>
+      <c r="E618" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F618" t="inlineStr">
+        <is>
+          <t>Non-Individual Level</t>
+        </is>
+      </c>
       <c r="G618" t="inlineStr">
         <is>
           <t>This study utilizes network exploitation and exploration theory to distinguish the exploitative and exploratory mechanisms (government support and boundary-spanning learning, respectively) that convert political ties into firm innovativeness. It also examines the moderating roles market uncertainty plays in how political ties influence firm innovativeness. An empirical analysis of 262 manufacturers in China indicates that both government support and boundary-spanning learning mediate the link between political ties and firm innovativeness. Market uncertainty negatively moderates the impact of political ties on boundary-spanning learning but does not significantly moderate their impact on government support. Moreover, market uncertainty moderates the impact of government support on firm innovativeness negatively but moderates the impacts of boundary-spanning learning on firm innovativeness positively. This study theorizes two mediating factors for how firms exploit and explore their political ties to increase their innovativeness and enriches the knowledge of how market uncertainty affects the relationship between political ties and innovation.</t>
@@ -31517,7 +31793,11 @@
       <c r="K618" t="n">
         <v>2022</v>
       </c>
-      <c r="P618" s="8" t="n"/>
+      <c r="P618" s="8" t="inlineStr">
+        <is>
+          <t>The study measures boundary spanning learning at the firm level (manufacturing companies) rather than the individual level.. Verbatim Evidence: "An empirical analysis of 262 manufacturers in China indicates that both government support and boundary-spanning learning mediate the link between political ties and firm innovativeness."</t>
+        </is>
+      </c>
     </row>
     <row r="619" ht="18" customHeight="1" s="10">
       <c r="A619" t="inlineStr">
@@ -31530,6 +31810,16 @@
           <t>BSMA0616</t>
         </is>
       </c>
+      <c r="E619" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F619" t="inlineStr">
+        <is>
+          <t>EX-NoMatrix</t>
+        </is>
+      </c>
       <c r="G619" t="inlineStr">
         <is>
           <t>Organizational values and beliefs significantly influence employee decision making and behavior and manifest themselves as multiple climates existing within a single organization. A subset of organizational climate is an ethical climate, embodying normative values and beliefs involving moral issues shared by the employees of the organization. Reseachers have found multiple ethical climates present in an organization.</t>
@@ -31553,7 +31843,11 @@
       <c r="K619" t="n">
         <v>1995</v>
       </c>
-      <c r="P619" s="8" t="n"/>
+      <c r="P619" s="8" t="inlineStr">
+        <is>
+          <t>The paper does not contain a correlation matrix. It only contains means for different department types in tables 1, 2, and 3.. Verbatim Evidence: "Table 1 Locus of Analysis Decision Making by Department Types"</t>
+        </is>
+      </c>
     </row>
     <row r="620" ht="18" customHeight="1" s="10">
       <c r="A620" t="inlineStr">
@@ -31566,6 +31860,16 @@
           <t>BSMA0617</t>
         </is>
       </c>
+      <c r="E620" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F620" t="inlineStr">
+        <is>
+          <t>No Correlation Matrix</t>
+        </is>
+      </c>
       <c r="G620" t="inlineStr">
         <is>
           <t>Boundary‐spanning communication has been found to be important to various types of organizations and groups as a source of new information and awareness of environmental changes. Although the importance of formal, public channels in building the knowledge base of a field has long been recognized, most studies of boundary‐spanning activity have been limited to direct, personal (informal) communication. This study examines both informal and formal communication patterns of three groups in order to determine whether, in fact, a variety of media are used in boundary‐spanning communication. The groups selected were the members of three professions which fill intermediary positions between the creators and consumers of cultural products; one located in academia and two in the private sector. Major findings were that: (1) A boundary‐spanning structure linking 82.2% of the survey respondents was composed of both informal and formal media. (2) The professions differed in which type of channel was most heavily used, but were similar in their perceptions of the importance of the channels. (3) Individuals central to the informal part of the structure were also more likely to use the formal parts of the structure. (4) Boundary‐spanning media were among the five most frequently cited media for all three of the professions.</t>
@@ -31589,7 +31893,11 @@
       <c r="K620" t="n">
         <v>1992</v>
       </c>
-      <c r="P620" s="8" t="n"/>
+      <c r="P620" s="8" t="inlineStr">
+        <is>
+          <t>The paper does not provide a correlation matrix with zero-order correlations. It only reports percentages, means, and Chi-square statistics for communication channel usage.. Verbatim Evidence: "Table 1. Perceived importance of the three boundary-spanning channels... Table 3. Mean ratings of informal and formal channels, by professional group."</t>
+        </is>
+      </c>
     </row>
     <row r="621" ht="18" customHeight="1" s="10">
       <c r="A621" t="inlineStr">
@@ -31602,6 +31910,16 @@
           <t>BSMA0618</t>
         </is>
       </c>
+      <c r="E621" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F621" t="inlineStr">
+        <is>
+          <t>Qualitative Study</t>
+        </is>
+      </c>
       <c r="G621" t="inlineStr">
         <is>
           <t>Research-practice partnerships (RPPs) offer promising approaches to improve educational outcomes. Navigating boundaries between contexts is essential for RPP effectiveness, yet much work remains to establish a conceptual framework of boundary spanning in partnerships. Our longitudinal comparative case study draws from our experiences as graduate student boundary spanners in three long-term partnerships to examine boundary spanning roles in RPPs, with particular attention to the ways in which power permeates partnership work. Using qualitative, critically reflexive analysis of meeting artifacts and field notes, we found that our boundary spanning roles varied along five spectrums: institutional focus, task orientation, expertise, partnership disposition, and agency. Our roles were shaped by the organizational, cultural, relational, and historical features of the partnerships and contexts of interaction. We aim to promote the development of effective RPP strategies by leveraging the perspectives and positionality of graduate students in order to advance understanding of boundary spanning roles.</t>
@@ -31625,7 +31943,11 @@
       <c r="K621" t="n">
         <v>2021</v>
       </c>
-      <c r="P621" s="8" t="n"/>
+      <c r="P621" s="8" t="inlineStr">
+        <is>
+          <t>The paper is a qualitative case study that does not report quantitative metrics (Means, SD, Correlations) or measure individual-level boundary spanning behaviors quantitatively.. Verbatim Evidence: "Using qualitative, critically reflexive analysis of meeting artifacts and field notes, we found that our boundary spanning roles varied along five spectrums..."</t>
+        </is>
+      </c>
     </row>
     <row r="622" ht="18" customHeight="1" s="10">
       <c r="A622" t="inlineStr">
@@ -31638,6 +31960,16 @@
           <t>BSMA0619</t>
         </is>
       </c>
+      <c r="E622" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F622" t="inlineStr">
+        <is>
+          <t>NON-INDIVIDUAL LEVEL</t>
+        </is>
+      </c>
       <c r="G622" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this paper is to get deeper insight into the complex nature of the relationship between team learning conditions, team learning behaviours (TLBs) and innovative work behaviour (IWB) by considering and combining different neglected aspects in research.</t>
@@ -31661,7 +31993,11 @@
       <c r="K622" t="n">
         <v>2018</v>
       </c>
-      <c r="P622" s="8" t="n"/>
+      <c r="P622" s="8" t="inlineStr">
+        <is>
+          <t>The boundary spanning construct (a Team Learning Behaviour) is conceptualized and measured at the team level, with the items referring to the team, and aggregated to the team level for analysis.. Verbatim Evidence: "Due to the nested nature of the data of individuals in work teams and the conceptual meaning of the constructs at the team level, we aggregated the TLBs and team learning conditions at team level."</t>
+        </is>
+      </c>
     </row>
     <row r="623" ht="18" customHeight="1" s="10">
       <c r="A623" t="inlineStr">
@@ -31674,6 +32010,16 @@
           <t>BSMA0620</t>
         </is>
       </c>
+      <c r="E623" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F623" t="inlineStr">
+        <is>
+          <t>No individual boundary spanning</t>
+        </is>
+      </c>
       <c r="G623" t="inlineStr">
         <is>
           <t>Teams have a high potential for innovation development by carrying out innovative work behaviour (IWB), but research remains limited on how engagement in team learning behaviours (TLBs) can foster IWB among team members. Especially longitudinal studies investigating the dynamic character of both constructs are missing. To clarify the relationship between TLBs and IWB over time, we conducted a threewave longitudinal survey among interdisciplinary work teams in German vocational education. Based on a sample of 66 work teams with 275 team members consisting of vocational educators, such as teachers, school principals and social workers, a manifest cross-lagged panel model was estimated to capture the dynamic relationship between TLBs and IWB. The hierarchical structure was taken into account and missing data were imputed. The results indicate that knowledge sharing and team reﬂexivity at the beginning of the teamwork predict future engagement in dimensions of IWB. In the further course of the teamwork boundary spanning becomes an important TLB for IWB. The TLBs that are relevant for IWB are inﬂuenced by task interdependence and team structure. The results provide insight into how IWB can be fostered through TLBs over time. At the beginning of a work task, knowledge sharing and team reﬂexivity should be fostered by encouraging discussion and enriching diﬀerent perspectives to reach high engagement in IWB. In the further course of teamwork information should be gathered from outside the team, for instance by inviting experts.</t>
@@ -31697,7 +32043,11 @@
       <c r="K623" t="n">
         <v>2019</v>
       </c>
-      <c r="P623" s="8" t="n"/>
+      <c r="P623" s="8" t="inlineStr">
+        <is>
+          <t>The study conceptualizes and measures boundary spanning as a team-level learning behavior using team-referent items, rather than capturing boundary spanning at the individual level.. Verbatim Evidence: "Boundary spanning was assessed using Hirst and Mann’s (2004) four-item scale, including such items as (a) ‘When necessary, team members consult with individuals who possess knowledge relevant to the project’"</t>
+        </is>
+      </c>
     </row>
     <row r="624" ht="18" customHeight="1" s="10">
       <c r="A624" t="inlineStr">
@@ -31710,6 +32060,16 @@
           <t>BSMA0621</t>
         </is>
       </c>
+      <c r="E624" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F624" t="inlineStr">
+        <is>
+          <t>No BSB</t>
+        </is>
+      </c>
       <c r="G624" t="inlineStr">
         <is>
           <t>Summary             We examine how demographic context influences the trust that boundary spanners experience in their dyadic relationships with clients. Because of the salience of age as a demographic characteristic as well as the increasing prevalence of age diversity and intergenerational conflict in the workplace, we focus on team age diversity as a demographic social context that affects trust between boundary spanners and their clients. Using social categorization theory and theories of social capital, we develop and test our contextual argument that a boundary spanner's experience of being trusted is influenced by the social categorization processes that occur in dyadic interactions with a specific client and, simultaneously, by similar social categorization processes that influence the degree to which the client team as a whole serves as a cooperative resource for demographically similar versus dissimilar boundary spanner–client dyads. Using a sample of 168 senior boundary spanners from the consulting industry, we find that generational diversity among client team members from a client organization undermines the perception of being trusted within homogeneous boundary spanner–client dyads while it enhances the perception of being trusted within heterogeneous dyads. The perception of being trusted is an important aspect of cross‐boundary relationships because it influences coordination and the costs associated with coordination. © 2015 The Author Journal of Organizational Behavior Published by John Wiley &amp; Sons Ltd</t>
@@ -31733,7 +32093,11 @@
       <c r="K624" t="n">
         <v>2016</v>
       </c>
-      <c r="P624" s="8" t="n"/>
+      <c r="P624" s="8" t="inlineStr">
+        <is>
+          <t>The study focuses on how demographic context and age diversity influence the perception of being trusted among boundary spanners. It measures the boundary spanner's perception of being trusted by clients, but it does not actually measure any boundary spanning behaviors.. Verbatim Evidence: "Consistent with Lau et al. (2014), we used two different dimensions of being trusted, behavioral reliance and disclosure (i.e., information sharing)."</t>
+        </is>
+      </c>
     </row>
     <row r="625" ht="18" customHeight="1" s="10">
       <c r="A625" t="inlineStr">
@@ -31746,6 +32110,16 @@
           <t>BSMA0622</t>
         </is>
       </c>
+      <c r="E625" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F625" t="inlineStr">
+        <is>
+          <t>NO_CORR</t>
+        </is>
+      </c>
       <c r="G625" t="inlineStr">
         <is>
           <t>Inter‐organizational frameworks of intervention dominate the resolution of complex societal problems facing the UK and many other countries. Strategic alliances, joint working arrangements, networks, partnerships and many other forms of collaboration across sectoral and organizational boundaries currently proliferate across the policy landscape. However, the discourse is positioned at an institutional and organizational level, and comparatively little attention is accorded to the pivotal role of individual actors in the management of inter‐organizational relationships. This paper attempts to redress this balance by focusing on the skills, competencies and behaviour of boundary spanners. A critical review of the relevant literature, both from an institutional and relational perspective, is undertaken. This is complemented by some new empirical research that involves an engagement with groups of particular types of boundary spanner using a combination of surveys and in‐depth interviews. Finally, a discussion makes connections between the existing literature and the research findings and offers suggestions for future areas of enquiry.</t>
@@ -31769,7 +32143,11 @@
       <c r="K625" t="n">
         <v>2002</v>
       </c>
-      <c r="P625" s="8" t="n"/>
+      <c r="P625" s="8" t="inlineStr">
+        <is>
+          <t>The paper is an exploratory study using postal surveys and interviews to identify boundary spanning competencies. It does not report any quantitative zero-order correlation matrix.. Verbatim Evidence: "The fieldwork and data collection consists of two interconnected phases (table 3). Phase 1 is directed to an initial identification and categorization of boundary spanning competencies together with a short attitudinal investigation."</t>
+        </is>
+      </c>
     </row>
     <row r="626" ht="18" customHeight="1" s="10">
       <c r="A626" t="inlineStr">
@@ -31782,6 +32160,16 @@
           <t>BSMA0623</t>
         </is>
       </c>
+      <c r="E626" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F626" t="inlineStr">
+        <is>
+          <t>Not individual level</t>
+        </is>
+      </c>
       <c r="G626" t="inlineStr">
         <is>
           <t>This study examines the concept of intra-organizational links as a way for boundary spanners to bring into the project group the information needed to deal with task uncertainty. Several studies have shown that heterogeneous groups are superior to homogeneous groups when novel or creative solutions need to be developed to deal with tasks characterized by high task uncertainty. For boundary spanners in engineering project groups, it is proposed that cross-departmental technical advice links are another source of the information needed to deal with task uncertainty. An empirical test supports the proposition that for high-performing project groups, boundary-spanning technical advice links may compensate for a lack of internal group heterogeneity and vice versa. This is not the case for low-performing project groups. Implications of these finding are presented, including the direction that the open innovation research stream might take to address the findings of this study.</t>
@@ -31805,7 +32193,11 @@
       <c r="K626" t="n">
         <v>2018</v>
       </c>
-      <c r="P626" s="8" t="n"/>
+      <c r="P626" s="8" t="inlineStr">
+        <is>
+          <t>The unit of analysis is the project group, and all variables were aggregated to group means.. Verbatim Evidence: "Since the project group is the unit of analysis in the present study, all variables were aggregated to group means."</t>
+        </is>
+      </c>
     </row>
     <row r="627" ht="18" customHeight="1" s="10">
       <c r="A627" t="inlineStr">
@@ -31818,6 +32210,16 @@
           <t>BSMA0624</t>
         </is>
       </c>
+      <c r="E627" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F627" t="inlineStr">
+        <is>
+          <t>Latent Correlations</t>
+        </is>
+      </c>
       <c r="G627" t="inlineStr">
         <is>
           <t>The importance of frontline employees for the success of organizations is recognized by researches and practitioners alike. However, their importance for the innovativeness of companies resulting from their boundary spanning role is often underestimated and has received little attention in prior research. The present paper contributes to the literature by empirically investigating idea fishing behaviors, and, in particular, the relationship between idea gathering and idea dissemination behaviors, of frontline employees from different industrial and business services firms. Furthermore, the impact of motivators such as job satisfaction and desire for upward mobility and the effects of other important conditions such as role stress and internal network on idea gathering and dissemination are assessed. Results of our study show that the proposed chain of idea gathering leading to idea dissemination and resulting in innovation holds. Furthermore, the various effects of role stress underline the importance of differentiating between different forms of role conflict and ambiguity. Based on these findings, implications for management and research are derived.</t>
@@ -31841,7 +32243,11 @@
       <c r="K627" t="n">
         <v>2016</v>
       </c>
-      <c r="P627" s="8" t="n"/>
+      <c r="P627" s="8" t="inlineStr">
+        <is>
+          <t>The correlation matrix is explicitly labeled as 'Correlations of latent constructs' and includes 'Average variance extracted', indicating these are not raw zero-order correlations.. Verbatim Evidence: "TABLE 3 Correlations of latent constructs"</t>
+        </is>
+      </c>
     </row>
     <row r="628" ht="18" customHeight="1" s="10">
       <c r="A628" t="inlineStr">
@@ -31854,6 +32260,16 @@
           <t>BSMA0625</t>
         </is>
       </c>
+      <c r="E628" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F628" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G628" t="inlineStr">
         <is>
           <t>There is increasing recognition that group members learn not only within the group (i.e., local learning), but also externally (i.e., distal learning), and these two group learning processes may facilitate group performance in different ways. Yet, despite this recognition, there is much that is not understood about whether they complement or inhibit each other in affecting group performance, and whether group social and task conditions that foster one type of learning do so at the expense of the other. The findings from this field study of teams from four firms show that (1) local learning and distal learning are positively related to group efficiency and group innovativeness, respectively; (2) distal learning negatively interacts with local learning to impede group efficiency; and (3) high levels of group cohesion promote distal learning but diminish local learning. Overall, these findings suggest that there are not only performance trade-offs to engaging in either only local or distal learning, but also performance disadvantages to engaging in both types of group learning because distal learning impedes local learning from achieving a high level of group efficiency. In addition, there is preliminary evidence to suggest that tensions can arise from simultaneously managing both types of group learning because a high level of group cohesion increases distal learning but decreases local learning.</t>
@@ -31877,7 +32293,11 @@
       <c r="K628" t="n">
         <v>2004</v>
       </c>
-      <c r="P628" s="8" t="n"/>
+      <c r="P628" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures distal learning (boundary spanning) and its correlations at the group level (N=73 teams), violating the requirement for individual-level analysis.. Verbatim Evidence: "The final sample size comprised 73 teams... The team size ranged from 3 to 25 members"</t>
+        </is>
+      </c>
     </row>
     <row r="629" ht="18" customHeight="1" s="10">
       <c r="A629" t="inlineStr">
@@ -31890,6 +32310,16 @@
           <t>BSMA0626</t>
         </is>
       </c>
+      <c r="E629" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F629" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G629" t="inlineStr">
         <is>
           <t>Drawing from the structural perspective of social capital theory, this research investigates how internal and external advice network structures inﬂuence knowledge overlap and variety and, how these knowledge dimensions in turn inﬂuence group effectiveness. Findings from two studies on knowledge-intensive groups indicate that different advice network structures are associated with knowledge overlap and knowledge variety, and only knowledge variety was signiﬁcantly associated with group effectiveness. In addition, despite implicit understanding that advice networks aid performance through enhancing knowledge outcomes, only knowledge variety was found to mediate the relationship between external network and group effectiveness. Implications for theory and practice are discussed. Copyright # 2007 John Wiley &amp; Sons, Ltd.</t>
@@ -31913,7 +32343,11 @@
       <c r="K629" t="n">
         <v>2008</v>
       </c>
-      <c r="P629" s="8" t="n"/>
+      <c r="P629" s="8" t="inlineStr">
+        <is>
+          <t>The study measures external network and knowledge at the group level, not the individual level. The unit of analysis is organizational work groups.. Verbatim Evidence: "Group network data were collected from 50 work groups from three firms"</t>
+        </is>
+      </c>
     </row>
     <row r="630" ht="18" customHeight="1" s="10">
       <c r="A630" t="inlineStr">
@@ -31926,6 +32360,16 @@
           <t>BSMA0627</t>
         </is>
       </c>
+      <c r="E630" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F630" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G630" t="inlineStr">
         <is>
           <t>Prior research has highlighted that network sparseness and network centrality enhance innovativeness through access to information and inﬂuence, respectively. We advance this perspective by exploring the extent to which individual actions are needed to mobilize information and inﬂuence accessed through social networks, and whether such information and inﬂuence would mutually reinforce to enhance managerial innovativeness. Our ﬁndings found partial support for the idea that actions are needed to actualize potential resources embedded in social networks, as centrally positioned managers enjoy higher innovativeness when they engage in ambassador activities. We also found that advice network sparseness and advice network centrality had independent, not interactive relationships with managerial innovativeness, suggesting that they offer distinct routes to achieving managerial innovativeness. Overall, our research clariﬁes the relationships of two important social network attributes on managerial innovativeness, and also sheds new light on how managerial action matters in realizing social network advantages for innovative ends.</t>
@@ -31949,7 +32393,11 @@
       <c r="K630" t="n">
         <v>2014</v>
       </c>
-      <c r="P630" s="8" t="n"/>
+      <c r="P630" s="8" t="inlineStr">
+        <is>
+          <t>The paper provides a zero-order correlation matrix including individual-level measures of boundary spanning behaviors (scout and ambassador activities) and managerial innovativeness.. Verbatim Evidence: "Table I reports means, standard deviations, and intercorrelations among the variables."</t>
+        </is>
+      </c>
     </row>
     <row r="631" ht="18" customHeight="1" s="10">
       <c r="A631" t="inlineStr">
@@ -31962,6 +32410,16 @@
           <t>BSMA0628</t>
         </is>
       </c>
+      <c r="E631" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F631" t="inlineStr">
+        <is>
+          <t>No Zero-Order Correlation Matrix</t>
+        </is>
+      </c>
       <c r="G631" t="inlineStr">
         <is>
           <t>Productive relationships between a company and its customers are often the result of positive relationships between the company and its boundary spanning employees. The career entry transition marks the beginning of these interpersonal relationships, which have a significant impact on marketing performance. Using a sample of newly hired boundary spanning employees, we examine the influence of individual difference factors on boundary spanners’ appraisals of the career entry transition. Significant relationships are found between boundary spanners’ positive and negative appraisals of the transition and personal and non-organizational factors: perceived centrality of the work role, availability of resources (finances, social support, personal hope), and sense of coherence.</t>
@@ -31985,7 +32443,11 @@
       <c r="K631" t="n">
         <v>2004</v>
       </c>
-      <c r="P631" s="8" t="n"/>
+      <c r="P631" s="8" t="inlineStr">
+        <is>
+          <t>The paper does not provide a zero-order correlation matrix. It only reports the results of multiple regression analyses (Tables 1 and 2).. Verbatim Evidence: "Multiple regression analysis was conducted to test this prediction."</t>
+        </is>
+      </c>
     </row>
     <row r="632" ht="18" customHeight="1" s="10">
       <c r="A632" t="inlineStr">
@@ -31998,6 +32460,16 @@
           <t>BSMA0629</t>
         </is>
       </c>
+      <c r="E632" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F632" t="inlineStr">
+        <is>
+          <t>No Empirical Data</t>
+        </is>
+      </c>
       <c r="G632" t="inlineStr">
         <is>
           <t>Over the last five years, the once vaulted system known as product management has been under attack. Challenged by a variety of mega‐trends, including rising consumer expectations and expertise, revolutionary changes in technology, and shifting power in channels of distribution, product managers now face an environment much more demanding than that of the past. Examines the role of product managers of consumer goods in this new environment, within the context of a conceptual model developed to understand better the dynamics underlying their job performance and satisfaction. The model highlights the interactions among boundary spanning, information power and interfunctional coordination, and incorporates the concepts of strategic orientation, role conflict and role ambiguity. In all, 17 propositions are advanced for future empirical testing.</t>
@@ -32021,7 +32493,11 @@
       <c r="K632" t="n">
         <v>1994</v>
       </c>
-      <c r="P632" s="8" t="n"/>
+      <c r="P632" s="8" t="inlineStr">
+        <is>
+          <t>The paper presents a theoretical model and does not contain empirical data or a correlation matrix.. Verbatim Evidence: "While theoretically compelling, empirical verification of the proposed linkages in the model is required. Future research should focus on a number of key questions..."</t>
+        </is>
+      </c>
     </row>
     <row r="633" ht="18" customHeight="1" s="10">
       <c r="A633" t="inlineStr">
@@ -32034,6 +32510,16 @@
           <t>BSMA0630</t>
         </is>
       </c>
+      <c r="E633" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F633" t="inlineStr">
+        <is>
+          <t>Non-Individual Level</t>
+        </is>
+      </c>
       <c r="G633" t="inlineStr">
         <is>
           <t>Motivated by the inconsistent findings of the linkage between early supplier involvement practice and new product development success, this study adopts both the resource-based perspective and agency theory to investigate dynamic relationships between the manufacturer and supplier during the collaboration process. Survey data were used to empirically examine the impact of the resource factor (i.e. collaboration effect) and agency factors (i.e. interaction effect) on project team effectiveness. The results showed that selecting suppliers with appropriate knowledge and resources is necessary yet insufficient to improve project team effectiveness. The agency problem plays a dominant role in determining the quality of collaboration. In particular, the study identified information sharing and task programmability as two key governance mechanisms to curb suppliers’ opportunistic behaviour. The study provides insightful managerial and policy implications for firms considering early supplier involvement practice in their innovation process.</t>
@@ -32057,7 +32543,11 @@
       <c r="K633" t="n">
         <v>2010</v>
       </c>
-      <c r="P633" s="8" t="n"/>
+      <c r="P633" s="8" t="inlineStr">
+        <is>
+          <t>The paper examines early supplier involvement (ESI) in new product development (NPD) projects at the firm or project-team level. It does not measure individual-level boundary spanning behaviors.. Verbatim Evidence: "The unit of analysis in this study is a specific case of supplier involvement in the NPD process."</t>
+        </is>
+      </c>
     </row>
     <row r="634" ht="18" customHeight="1" s="10">
       <c r="A634" t="inlineStr">
@@ -32070,6 +32560,16 @@
           <t>BSMA0631</t>
         </is>
       </c>
+      <c r="E634" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F634" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G634" t="inlineStr">
         <is>
           <t>This study is the first to examine the mediating role of boundary-spanning search and the moderating role of partner similarity in horizontal coopetition for sustainable product innovation. Analyzing empirical data from 236 Chinese firms, we found that horizontal coopetition positively impacts both proactive search (aimed at surpassing competitors) and responsive search (aimed at following competitors), with a stronger influence on proactive search. Both search types mediate the relationship between horizontal coopetition and sustainable product innovation. Furthermore, greater competing similarity (e.g., market coverage) between firms and their partners increases firms' inclination toward proactive search under the influence of horizontal coopetition but weakens their tendency for responsive search. Conversely, greater cooperating similarity (e.g., corporate culture) increases firms' inclination toward responsive search under the influence of horizontal coopetition but weakens their tendency for proactive search.</t>
@@ -32093,7 +32593,11 @@
       <c r="K634" t="n">
         <v>2025</v>
       </c>
-      <c r="P634" s="8" t="n"/>
+      <c r="P634" s="8" t="inlineStr">
+        <is>
+          <t>Boundary spanning behavior is measured at the firm level rather than the individual level.. Verbatim Evidence: "Our company prefers to collect information with no identifiable strategic market needs to ensure experimentation in the project, aiming to surpass competitors"</t>
+        </is>
+      </c>
     </row>
     <row r="635" ht="18" customHeight="1" s="10">
       <c r="A635" t="inlineStr">
@@ -32106,6 +32610,16 @@
           <t>BSMA0632</t>
         </is>
       </c>
+      <c r="E635" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F635" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G635" t="inlineStr">
         <is>
           <t>Purpose – Two challenges faced by automotive component design projects within contracted design agencies are (1) specification changes requested by the manufacturers and (2) product information or core technology knowledge leakage to external actors. We examine the effects of targeted boundary activities that address these challenges under the contingencies of environmental uncertainty and project complexity.</t>
@@ -32129,7 +32643,11 @@
       <c r="K635" t="n">
         <v>2020</v>
       </c>
-      <c r="P635" s="8" t="n"/>
+      <c r="P635" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures individual-level boundary buffering behaviors of the project manager and provides a valid zero-order correlation matrix containing Means, SDs, and correlations.. Verbatim Evidence: "The project manager conducts the following activities (1—strongly disagree; 5—strongly agree): (1) Deflect outside pressures on the team... Finally, descriptive statistics and correlations for the variables are shown in Table IV."</t>
+        </is>
+      </c>
     </row>
     <row r="636" ht="18" customHeight="1" s="10">
       <c r="A636" t="inlineStr">
@@ -32142,6 +32660,16 @@
           <t>BSMA0633</t>
         </is>
       </c>
+      <c r="E636" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F636" t="inlineStr">
+        <is>
+          <t>Wrong Level of Analysis</t>
+        </is>
+      </c>
       <c r="G636" t="inlineStr">
         <is>
           <t>Transnational knowledge networks provide organizations with information useful in addressing shared problems. Social media may enable the formation of those networks, yet their role in the process has received little attention. This article examines the structure and antecedents of two networks facilitated by the microblogging platform Twitter operating in the policy domain of emergency management. One network includes national-level government agencies responsible for disaster response and recovery operations; the other includes nongovernmental organizations in the form of Red Cross and Red Crescent national societies. We use a logistic regression quadratic assignment procedure to test hypotheses derived from related literature. While findings indicate that shared language and geographic proximity shaped network formation, both networks exhibit boundary spanning behavior in which organizations sought out information from high-profile, resource-rich organizations. Those organizations helped to connect otherwise regionally bound clusters and demonstrate the nascent potential of social media to create global transnational knowledge networks.</t>
@@ -32165,7 +32693,11 @@
       <c r="K636" t="n">
         <v>2017</v>
       </c>
-      <c r="P636" s="8" t="n"/>
+      <c r="P636" s="8" t="inlineStr">
+        <is>
+          <t>The study analyzes network formation among national-level organizations (government agencies and NGOs) rather than individual-level boundary spanning behaviors. Furthermore, the paper does not report a zero-order correlation matrix.. Verbatim Evidence: "This article examines the structure and antecedents of two networks facilitated by the microblogging platform Twitter operating in the policy domain of emergency management. One network includes national-level government agencies responsible for disaster response and recovery operations; the other includes nongovernmental organizations in the form of Red Cross and Red Crescent national societies. [...] Thus, our unit of analysis is the directional dyad."</t>
+        </is>
+      </c>
     </row>
     <row r="637" ht="18" customHeight="1" s="10">
       <c r="A637" t="inlineStr">
@@ -32178,6 +32710,16 @@
           <t>BSMA0634</t>
         </is>
       </c>
+      <c r="E637" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F637" t="inlineStr">
+        <is>
+          <t>Wrong Level of Analysis</t>
+        </is>
+      </c>
       <c r="G637" t="inlineStr">
         <is>
           <t>Drawing on social network theory, our study develops a theoretical model delineating the impact of informational faultlines, paradoxical leadership, and team boundary work on idea implementation. Drawing from empirical research using a dataset of 82 teams from multi-source and multi-timepoints, our findings reveal that informational faultlines positively influence team boundary work (boundary spanning, buffering, and reinforcement) and idea implementation. Team boundary work (boundary spanning, buffering, and reinforcement) mediates the relationship between informational faultlines and idea implementation. Paradoxical leadership moderates the mediating effect of boundary buffering and spanning between informational faultlines and idea implementation. The findings of our study provide theoretical insights and practical implications for the management of innovative teams in businesses, team establishment, and the recruitment and selection of leaders.</t>
@@ -32201,7 +32743,11 @@
       <c r="K637" t="n">
         <v>2025</v>
       </c>
-      <c r="P637" s="8" t="n"/>
+      <c r="P637" s="8" t="inlineStr">
+        <is>
+          <t>The study aggregates boundary work measures to the team level (N=82) and only provides a team-level correlation matrix. It does not report individual-level correlations.. Verbatim Evidence: "This confirms that the study’s sample can be successfully aggregated from the individual level to the team level, thereby providing a solid foundation for subsequent analyses... Table 4 Descriptive statistics and correlations... Notes: N = 82."</t>
+        </is>
+      </c>
     </row>
     <row r="638" ht="18" customHeight="1" s="10">
       <c r="A638" t="inlineStr">
@@ -32214,6 +32760,16 @@
           <t>BSMA0635</t>
         </is>
       </c>
+      <c r="E638" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F638" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G638" t="inlineStr">
         <is>
           <t>Although research suggests that subordinates’ boundary spanning may result in unintended negative responses from their supervisors, little is known about which supervisors are likely to react adversely and which are not. We draw on self-protection theory to answer this question. Specifically, we argue that when supervisors experience low levels of managerial self-efficacy, boundary spanning behavior threatens their perceived work status within the team, resulting in abusive supervisory behavior. The results of two field survey studies and an experimental study support our hypotheses. Our research identifies managerial barriers that may hinder boundary spanning behavior at work and provides invaluable insights into how upper-level organizations may create constructive work contexts that encourage employees to engage in such behavior.</t>
@@ -32237,7 +32793,11 @@
       <c r="K638" t="n">
         <v>2023</v>
       </c>
-      <c r="P638" s="8" t="n"/>
+      <c r="P638" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures individual-level boundary spanning behaviors (subordinates) and contains valid zero-order correlation matrices (Tables 1, 4, 7) that are not latent construct intercorrelations.. Verbatim Evidence: "Subordinate boundary spanning behavior. We measured subordinate boundary spanning behavior using the 15-item scale from Ancona and Caldwell (1992)."</t>
+        </is>
+      </c>
     </row>
     <row r="639" ht="18" customHeight="1" s="10">
       <c r="A639" t="inlineStr">

</xml_diff>

<commit_message>
chore: completed Batch 17 extraction
</commit_message>
<xml_diff>
--- a/BSMA_AI_Run_V2.xlsx
+++ b/BSMA_AI_Run_V2.xlsx
@@ -32810,6 +32810,16 @@
           <t>BSMA0636</t>
         </is>
       </c>
+      <c r="E639" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F639" t="inlineStr">
+        <is>
+          <t>No Empirical Data</t>
+        </is>
+      </c>
       <c r="G639" t="inlineStr">
         <is>
           <t>Estimating customer lifetime value is becoming increasingly important in order to identify and invest on prospective profitable customers. This paper reviews three research streams in this field: models for calculation of CLV; models of customer base analysis; normative models of CLV in order to evaluate the usefulness of customer lifetime value as a metric for customer selection and marketing resource allocation. Lifetime value can be used to inform the nature and quality of relationship that an organization might have with customers. Customers who are selected on the basis of their lifetime value provide higher profits in future periods than do customers selected on the basis of several other customer-based metrics. Managers can improve profits by designing marketing communications that maximize CLV.</t>
@@ -32833,7 +32843,11 @@
       <c r="K639" t="n">
         <v>2009</v>
       </c>
-      <c r="P639" s="8" t="n"/>
+      <c r="P639" s="8" t="inlineStr">
+        <is>
+          <t>The paper is a theoretical review of customer lifetime value (CLV) models. It does not contain any empirical data, zero-order correlation matrix, or measures of individual-level boundary spanning behaviors.. Verbatim Evidence: "This paper reviews three research streams in this field: models for calculation of CLV; models of customer base analysis; normative models of CLV"</t>
+        </is>
+      </c>
     </row>
     <row r="640" ht="18" customHeight="1" s="10">
       <c r="A640" t="inlineStr">
@@ -32846,6 +32860,16 @@
           <t>BSMA0637</t>
         </is>
       </c>
+      <c r="E640" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F640" t="inlineStr">
+        <is>
+          <t>Firm-Level</t>
+        </is>
+      </c>
       <c r="G640" t="inlineStr">
         <is>
           <t>Radical green innovation has emerged as an effective strategy for firms to achieve sustainable development in the volatility, uncertainty, complexity, and ambiguity (VUCA) environment. Although the importance of external knowledge acquisition has been recognized, the mechanism of how proactive boundary-spanning search affects radical green innovation is still blurred. Drawing on the resource-based view and dynamic capabilities theory, this research discusses the impact of two types of proactive boundary-spanning search on radical green innovation and considers the mediating role of organizational resilience and the moderating role of big data analytics capability. Based on data collected from 294 manufacturing firms in China, the results show that both value-chain-based proactive search and industry–university-based proactive search positively influence radical green innovation. Furthermore, organizational resilience fully mediates the relationship between value-chain-based proactive search and radical green innovation, and partially mediates the relationship between industry–university-based proactive search and radical green innovation. Moreover, we demonstrate that big data analytics capability moderates the relationship between industry–university-based proactive search and radical green innovation. This research clarifies not only the mechanism of proactive boundary-spanning search driving radical green innovation by highlighting the mediating role of organizational resilience and the moderating role of big data analytics capability, but also provides theoretical and managerial implications for manufacturing firms and other stakeholders to carry out radical green innovation.</t>
@@ -32869,7 +32893,11 @@
       <c r="K640" t="n">
         <v>2024</v>
       </c>
-      <c r="P640" s="8" t="n"/>
+      <c r="P640" s="8" t="inlineStr">
+        <is>
+          <t>The study measures proactive boundary-spanning search at the firm level rather than the individual level.. Verbatim Evidence: "four items were designed, including “Our firm can search knowledge and data about green innovation from suppliers ahead of competitors”"</t>
+        </is>
+      </c>
     </row>
     <row r="641" ht="18" customHeight="1" s="10">
       <c r="A641" t="inlineStr">
@@ -32882,6 +32910,16 @@
           <t>BSMA0638</t>
         </is>
       </c>
+      <c r="E641" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F641" t="inlineStr">
+        <is>
+          <t>Latent Correlations / Team-level</t>
+        </is>
+      </c>
       <c r="G641" t="inlineStr">
         <is>
           <t>Purpose – The consulting team intervenes in the integrated construction consulting (ICC) network structure centered on “client-contractor-consultant.” Team boundary-spanning behavior (TBB) driven by the network structure is crucial to project performance. This article investigated how to stimulate the consulting project performance (CPP) improvement by considering the interactive effect of network structure and TBB. To be specific, this paper explored the configuration between structural characteristics of project networks, the dimension of TBB, and project performance in ICC projects.</t>
@@ -32905,7 +32943,11 @@
       <c r="K641" t="n">
         <v>2024</v>
       </c>
-      <c r="P641" s="8" t="n"/>
+      <c r="P641" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures boundary-spanning behavior at the team level (Team Boundary-Spanning Behavior). Additionally, the correlation matrix (Table 2) reports latent construct correlations generated using Smart PLS 3.0 for testing discriminant validity, rather than raw, zero-order correlations.. Verbatim Evidence: "After testing the convergent validity, the AVE method was used to further analyze the discriminant validity of the scale... The large sample data were imported into Smart PLS 3.0, and the statistical results of the correlations among the variables were calculated, as shown in Table 2."</t>
+        </is>
+      </c>
     </row>
     <row r="642" ht="18" customHeight="1" s="10">
       <c r="A642" t="inlineStr">
@@ -32918,6 +32960,16 @@
           <t>BSMA0639</t>
         </is>
       </c>
+      <c r="E642" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F642" t="inlineStr">
+        <is>
+          <t>Not Individual-Level</t>
+        </is>
+      </c>
       <c r="G642" t="inlineStr">
         <is>
           <t>Resources are basic element of business model innovation, but most enterprises face serious resource constraints due to their capability limitations. This study focuses on boundary-spanning behaviour of top management team and bricolage, to explore their inﬂuence mechanism on business model innovation. A hierarchical regression analysis is carried out on data from China. Responses from 163 enterprises indicate that top management team boundary-spanning behaviour has a signiﬁcantly positive inﬂuence on business model innovation, that bricolage has a signiﬁcantly positive eﬀect on business model innovation, and that bricolage plays a signiﬁcant intermediary role between top management team boundary-spanning behaviour and business model innovation. This study enriches theoretical and empirical researches on business model innovation while serving as a valuable reference for business practice.</t>
@@ -32941,7 +32993,11 @@
       <c r="K642" t="n">
         <v>2020</v>
       </c>
-      <c r="P642" s="8" t="n"/>
+      <c r="P642" s="8" t="inlineStr">
+        <is>
+          <t>The boundary spanning construct is measured at the Top Management Team (TMT) level rather than the individual level.. Verbatim Evidence: "The original measurement scale of team boundary-spanning behaviour was designed by Ancona and Caldwell (1992)... so we draw nine items from it to measure TMT boundary-spanning behaviour."</t>
+        </is>
+      </c>
     </row>
     <row r="643" ht="18" customHeight="1" s="10">
       <c r="A643" t="inlineStr">
@@ -32954,6 +33010,16 @@
           <t>BSMA0640</t>
         </is>
       </c>
+      <c r="E643" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F643" t="inlineStr">
+        <is>
+          <t>Not Individual-Level</t>
+        </is>
+      </c>
       <c r="G643" t="inlineStr">
         <is>
           <t>Purpose – This study aims to investigate how market orientation (MO) motivates ﬁrms to develop business model innovation and how such effects are moderated by strategic ﬂexibility. Design/methodology/approach – In this study, a questionnaire-based survey was undertaken to test the proposed hypotheses. The empirical study was conducted on a sample of 204 ﬁrms using two key informants (408 respondents) in China. The regression model is used to test the proposed model.</t>
@@ -32977,7 +33043,11 @@
       <c r="K643" t="n">
         <v>2020</v>
       </c>
-      <c r="P643" s="8" t="n"/>
+      <c r="P643" s="8" t="inlineStr">
+        <is>
+          <t>The study focuses on firm-level capabilities (market orientation, strategic flexibility, and business model innovation) rather than individual-level boundary spanning behaviors.. Verbatim Evidence: "The empirical study was conducted on a sample of 204 firms using two key informants (408 respondents) in China."</t>
+        </is>
+      </c>
     </row>
     <row r="644" ht="18" customHeight="1" s="10">
       <c r="A644" t="inlineStr">
@@ -32990,6 +33060,16 @@
           <t>BSMA0641</t>
         </is>
       </c>
+      <c r="E644" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F644" t="inlineStr">
+        <is>
+          <t>Code 99: Other - No Boundary Spanning Construct</t>
+        </is>
+      </c>
       <c r="G644" t="inlineStr">
         <is>
           <t>The meteoric rise in the popularity of social networking sites (SNSs) has connected many employees with their contacts from work. However, clashes are catalyzed when individuals’ professional identities collide with their social ones. This paper aims to explore hotel employees’ identity conflicts stemming from cross-boundary friendships. Building on cognitive dissonance theory and conservation of resources theory, a multilevel model is proposed to examine how befriending colleagues on SNSs induces unfavorable workplace consequences through the mediation effect of identity conflict. The model further scrutinizes whether task interdependence intensifies this negative spillover. This study probes a novel identity issue aroused by SNS interactions in a professional context and advances research on interpersonal dynamics in organizations. It also provides new insights on the role of team-level situational factors. The results generate managerial implications for hotels and employees, suggesting that both groups should be better prepared for possible dilemmas embedded in crossboundary relationships.</t>
@@ -33013,7 +33093,11 @@
       <c r="K644" t="n">
         <v>2021</v>
       </c>
-      <c r="P644" s="8" t="n"/>
+      <c r="P644" s="8" t="inlineStr">
+        <is>
+          <t>The study focuses on work-life boundary management (cross-boundary friendships via SNS with intra-team members) rather than individual-level boundary spanning behavior across organizational or unit boundaries.. Verbatim Evidence: "The rise of SNSs has profoundly changed the ways in which employees interact with each other, blurring the work–life boundaries and bridging domains which were once well defined"</t>
+        </is>
+      </c>
     </row>
     <row r="645" ht="18" customHeight="1" s="10">
       <c r="A645" t="inlineStr">
@@ -33026,6 +33110,16 @@
           <t>BSMA0642</t>
         </is>
       </c>
+      <c r="E645" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F645" t="inlineStr">
+        <is>
+          <t>Wrong Level of Analysis</t>
+        </is>
+      </c>
       <c r="G645" t="inlineStr">
         <is>
           <t>Purpose – In today’s complex and rapidly changing business environment, cross-boundary growth is increasingly critical to the survival or even success of organizations. The purpose of this study is to examine the forming mechanism of ﬁrm’s cross-boundary growth by integrating the two important antecedent factors of performance pressure and managerial discretion into a united framework and theoretically analyze the direct role of performance pressure on ﬁrm’s cross-boundary growth as well as reveal the moderating role of managerial discretion. Also, the authors select listed manufacturing companies in China as samples to empirically test the research hypotheses.</t>
@@ -33049,7 +33143,11 @@
       <c r="K645" t="n">
         <v>2024</v>
       </c>
-      <c r="P645" s="8" t="n"/>
+      <c r="P645" s="8" t="inlineStr">
+        <is>
+          <t>The study focuses on firm-level cross-boundary growth (cross-industry and cross-regional) using data from listed manufacturing companies, rather than individual-level boundary spanning behaviors.. Verbatim Evidence: "This study adopts the A-stock manufacturing listed companies on the main boards of Shenzhen and Shanghai in China from 2013 to 2016 as the sample."</t>
+        </is>
+      </c>
     </row>
     <row r="646" ht="18" customHeight="1" s="10">
       <c r="A646" t="inlineStr">
@@ -33062,6 +33160,16 @@
           <t>BSMA0643</t>
         </is>
       </c>
+      <c r="E646" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F646" t="inlineStr">
+        <is>
+          <t>Non-Individual Level</t>
+        </is>
+      </c>
       <c r="G646" t="inlineStr">
         <is>
           <t>Purpose – The rapid advancement of digital transformation requires a shift in firms’ focus from past met needs to both latent future and unmet past needs. However, how boundary-spanning search with future orientation and past orientation affects breakthrough innovation remains unclear. This study thus aims to investigate the relationship between boundary-spanning search and breakthrough innovation from the perspective of search orientation.</t>
@@ -33085,7 +33193,11 @@
       <c r="K646" t="n">
         <v>2024</v>
       </c>
-      <c r="P646" s="8" t="n"/>
+      <c r="P646" s="8" t="inlineStr">
+        <is>
+          <t>Boundary spanning behavior is measured at the firm level, not the individual level.. Verbatim Evidence: "Boundary-spanning search refers to firms’ knowledge search activities that cross organizational or technical boundaries"</t>
+        </is>
+      </c>
     </row>
     <row r="647" ht="18" customHeight="1" s="10">
       <c r="A647" t="inlineStr">
@@ -33098,6 +33210,16 @@
           <t>BSMA0644</t>
         </is>
       </c>
+      <c r="E647" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F647" t="inlineStr">
+        <is>
+          <t>Firm-Level Analysis</t>
+        </is>
+      </c>
       <c r="G647" t="inlineStr">
         <is>
           <t>Although the critical role of boundary-spanning search in facilitating sustainable competitive advantage (SCA) has been recognized, how boundary-spanning search affects SCA under the conditions that competitors also search remains unclear. By considering competition, this study divides boundary-spanning search into proactive and responsive searches, and develops a theoretical model, in which proactive and responsive searches respectively influence exploratory and exploitative innovations, and subsequently enhance SCA. Empirical results from Chinese advanced manufacturing firms show that proactive and responsive searches have inverted Ushaped effects on SCA. Additionally, when the levels of proactive and responsive searches are low and moderate, exploratory innovation plays a complementary mediating role between proactive search and SCA, whereas exploitative innovation plays a complementary mediating role between responsive search and SCA. When considering competition, this study offers a crucial condition under which exploratory and exploitative innovations can transform the efforts of boundary-spanning search to SCA.</t>
@@ -33121,7 +33243,11 @@
       <c r="K647" t="n">
         <v>2021</v>
       </c>
-      <c r="P647" s="8" t="n"/>
+      <c r="P647" s="8" t="inlineStr">
+        <is>
+          <t>The study measures boundary spanning (proactive and responsive search) at the firm level, not the individual level. All scale items refer to 'My firm'.. Verbatim Evidence: "Table 2 Reliability and convergent validity. Items: Proactive search... 1. My firm discovers opportunities in new market or targets new customers ahead of competitors... 2. My firm invents new products with unique features ahead of competitors..."</t>
+        </is>
+      </c>
     </row>
     <row r="648" ht="18" customHeight="1" s="10">
       <c r="A648" t="inlineStr">
@@ -33134,6 +33260,16 @@
           <t>BSMA0645</t>
         </is>
       </c>
+      <c r="E648" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F648" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G648" t="inlineStr">
         <is>
           <t>Summary                            Team creativity, as one of the most important sources of organizational competitiveness and continuous innovation, requires rich and non‐redundant information from both internal and external sources. Although an emerging line of research has shed light on the role of team boundary‐spanning activity in promoting creativity, it has solely focused on the mean level of team boundary‐spanning activity and rarely addressed the fact that not all team members engage in boundary‐spanning behaviors to the same extent. In this study, we broaden the existing knowledge by examining               when               and               how               the pattern of team boundary spanning, particularly the differentiation in team member boundary‐spanning activities, promotes team creativity. Based on the categorization‐elaboration model, we propose a curvilinear relationship between team member boundary‐spanning differentiation and creativity that is mediated through information sharing. Further, we add an important layer of understanding to the nature of this curvilinear relationship by identifying team goal interdependence as an important moderator. Using multisource data collected from two time points in 70 teams, we have received general support for our hypotheses. As such, we enrich the conversation about the importance of team boundary spanning by answering “               Whether               team boundary‐spanning differentiation fosters creativity, and               when               and               how               ?”</t>
@@ -33157,7 +33293,11 @@
       <c r="K648" t="n">
         <v>2022</v>
       </c>
-      <c r="P648" s="8" t="n"/>
+      <c r="P648" s="8" t="inlineStr">
+        <is>
+          <t>The study aggregates boundary spanning to the team level (TMBSD and mean boundary-spanning) and only reports correlations at the team level (N=70 teams). No individual-level correlations are provided.. Verbatim Evidence: "we calculated TMBSD using the within-group standard deviation of individual boundary spanning... TABLE 1 Means, standard deviations, and intercorrelations of variables... Note :n=70;"</t>
+        </is>
+      </c>
     </row>
     <row r="649" ht="18" customHeight="1" s="10">
       <c r="A649" t="inlineStr">
@@ -33170,6 +33310,16 @@
           <t>BSMA0646</t>
         </is>
       </c>
+      <c r="E649" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F649" t="inlineStr">
+        <is>
+          <t>Non-Individual Level</t>
+        </is>
+      </c>
       <c r="G649" t="inlineStr">
         <is>
           <t>As an important strategic decision for enterprise sustainability, the green entrepreneurial orientation can facilitate boundary-spanning search for external knowledge and resources to achieve triadic sustainable economic, environmental, and social performance. Based on organizational search theory and dynamic capability theory, this study introduces environmental dynamism into the model of the relationship between green entrepreneurial orientation, boundary-spanning search and enterprise triadic sustainable performance. By analyzing the questionnaire data from 202 managers of manufacturing SMEs, the study explores the internal and external influences of green entrepreneurial orientation on the enterprise sustainable performance. The results show that: green entrepreneurial orientation has a positive impact on enterprise economic, environmental and social performance; boundary-spanning search plays a fully mediating role between green entrepreneurial orientation and enterprise economic, environmental and social performance; environmental dynamism, as a key external environmental factor, positively regulates the relationship between boundary-spanning search and enterprise economic performance and environmental performance, and negatively regulates the relationship between boundary-spanning search and social performance. This study clearly demonstrates how green entrepreneurial orientation in the environmental era can drive triadic sustainable performance improvement of enterprises. In addition, this study argues that boundary-spanning search is an important tool that enables manufacturing SMEs to achieve a triad of coordinated sustainable development of economic, environmental and social benefits in a dynamic environment.</t>
@@ -33193,7 +33343,11 @@
       <c r="K649" t="n">
         <v>2022</v>
       </c>
-      <c r="P649" s="8" t="n"/>
+      <c r="P649" s="8" t="inlineStr">
+        <is>
+          <t>The study conceptualizes and measures boundary-spanning search at the enterprise/organizational level (SMEs) rather than the individual employee level.. Verbatim Evidence: "Boundary-spanning search is an essential way to acquire external knowledge, which is a way for enterprises to search for novel and heterogeneous knowledge and resources across organizational or technological boundaries"</t>
+        </is>
+      </c>
     </row>
     <row r="650" ht="18" customHeight="1" s="10">
       <c r="A650" t="inlineStr">
@@ -33206,6 +33360,16 @@
           <t>BSMA0647</t>
         </is>
       </c>
+      <c r="E650" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F650" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G650" t="inlineStr">
         <is>
           <t>Innovation often involves high uncertainty, making it difficult for a single entrepreneurial decision-making logic to navigate effectively. Grounded in resource orchestration theory, we advance the discussion on entrepreneurial decision-making logics by examining the interplay between causation and effectuation, and their interactive impacts on innovation within new ventures. Using a multi-wave survey of 404 founding team members from 91 new ventures, we find that new venture innovation is enhanced by the synergy of causation and effectuation. Furthermore, the boundary-spanning behavior of founding teams mediates the relationship between the synergy and new venture innovation, and founding team trust positively moderates this mediated relationship. These insights contribute to understanding the entrepreneurial decision-making logics and strategic behaviors of founding teams as they pursue innovation.</t>
@@ -33229,7 +33393,11 @@
       <c r="K650" t="n">
         <v>2026</v>
       </c>
-      <c r="P650" s="8" t="n"/>
+      <c r="P650" s="8" t="inlineStr">
+        <is>
+          <t>Boundary spanning behavior is measured and analyzed at the founding team level rather than at the individual level.. Verbatim Evidence: "Before aggregating individual-level data into founding team-level variables, we computed well-accepted statistical indexes such as the Index of Within-Group Interrater Agreement (Rwg) (James et al., 1993) and Interclass Correlation Coefficient (ICC (1) and ICC (2))."</t>
+        </is>
+      </c>
     </row>
     <row r="651" ht="18" customHeight="1" s="10">
       <c r="A651" t="inlineStr">
@@ -33242,6 +33410,16 @@
           <t>BSMA0648</t>
         </is>
       </c>
+      <c r="E651" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F651" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G651" t="inlineStr">
         <is>
           <t>This study examines the impact of emotional intelligence (EI) on boundaryspanning behavior, relationship quality, and performance among door‐todoor salespeople. Data is collected from salespeople and customers of South Korean door‐to‐door cosmetics businesses and analyzed using structural equation modeling. The findings show that EI positively affects boundaryspanning behavior. Similarly, boundary‐spanning behavior improves relationship quality, which improves both sales performance and customer satisfaction. This suggests that EI plays an important role in salespeople's boundaryspanning behavior, thereby enhancing relationship quality, sales performance, and customer satisfaction. Unlike previous studies, this study makes use of actual sales volumes, salespeople's self‐reporting responses, and salespeople's customer‐reporting, which adds to the findings' uniqueness. The present study highlights that EI improves boundary‐spanning behavior, which is vital in developing relationship quality, improving sales performance, and increasing customer satisfaction. The study uses triadic data from door‐to‐door salespeople, customers, and sales organizations extensively, which is unusual in this field.</t>
@@ -33265,7 +33443,11 @@
       <c r="K651" t="n">
         <v>2024</v>
       </c>
-      <c r="P651" s="8" t="n"/>
+      <c r="P651" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures individual-level boundary-spanning behaviors (external representation, internal influence, and service delivery behaviors) of salespeople and provides a valid zero-order correlation matrix with means and standard deviations.. Verbatim Evidence: "we investigate three types of boundary-spanning behaviors that salespeople may engage in... (1) External representation behavior... (2) internal influence behavior... and (3) service delivery behavior"</t>
+        </is>
+      </c>
     </row>
     <row r="652" ht="18" customHeight="1" s="10">
       <c r="A652" t="inlineStr">
@@ -33278,6 +33460,16 @@
           <t>BSMA0649</t>
         </is>
       </c>
+      <c r="E652" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F652" t="inlineStr">
+        <is>
+          <t>EXCLUDE: Firm-Level</t>
+        </is>
+      </c>
       <c r="G652" t="inlineStr">
         <is>
           <t>Despite the general agreement of the importance of resources and capabilities to strategic change, the broader question of how resources and capabilities affect strategic change itself remains unresolved. This research focuses on one characteristic of the process of strategic change, i.e., its speed. This study investigates the relationship between dynamic capabilities, the speed of strategic change, and performance. We propose that technological capabilities, marketing capabilities, and market-linking capabilities, due to their absorptive capacity and boundary spanning attributes, will facilitate the speed of strategic change. Furthermore, the risk orientation of managers will moderate this effect such that it would be strengthened for relatively risk-taking managers. Finally, we argue that the speed of strategic change will have an inverted-U relationship with organizational performance. We test these hypotheses on a sample of 213 Chinese ﬁrms and ﬁnd that while dynamic capabilities facilitate rapid strategic change, the risk orientation of decision makers moderates this relationship, but not all as hypothesized. While faster implementation of strategic change has a positive effect on performance, strategic change carried out too quickly has negative performance repercussions. Our ﬁndings suggest that ﬁrms not only need to adjust strategies to complement the changing environment, but also have corresponding capabilities to enable rapid strategic change.</t>
@@ -33301,7 +33493,11 @@
       <c r="K652" t="n">
         <v>2015</v>
       </c>
-      <c r="P652" s="8" t="n"/>
+      <c r="P652" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures dynamic capabilities, including market-linking capabilities (boundary spanning), at the firm level rather than the individual level.. Verbatim Evidence: "Market-linking capabilities were composed of five items [31], [55], including, relative to our major competitors: 1) stronger customer-linking capabilities (i.e., creating and managing durable customer relationships)"</t>
+        </is>
+      </c>
     </row>
     <row r="653" ht="18" customHeight="1" s="10">
       <c r="A653" t="inlineStr">
@@ -33314,6 +33510,16 @@
           <t>BSMA0650</t>
         </is>
       </c>
+      <c r="E653" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F653" t="inlineStr">
+        <is>
+          <t>No Boundary Spanning Measure</t>
+        </is>
+      </c>
       <c r="G653" t="inlineStr">
         <is>
           <t>With the development of economy, the innovation of enterprises can not meet the needs of enterprises. Knowledge transfer in industry-university-research alliance is the process of knowledge creation from universities and scientific research institutes, transfer to the enterprise and use the knowledge to create value. The establishment of industry-university-research alliance is conducive to the realization of knowledge transfer in universities and scientific research institutions to enterprises, expanding the knowledge stock of enterprises, and improving the ability of independent innovation. This paper summarizes the research results of domestic and foreign scholars, defines the connotation of industry-university-research alliance and alliance knowledge transfer, discussed the influence factors of alliance knowledge transfer, and makes research on knowledge transfer promotion measures. It can be used for reference to improve the knowledge transfer effect.</t>
@@ -33337,7 +33543,11 @@
       <c r="K653" t="n">
         <v>2017</v>
       </c>
-      <c r="P653" s="8" t="n"/>
+      <c r="P653" s="8" t="inlineStr">
+        <is>
+          <t>The paper does not measure individual-level boundary spanning behaviors and does not contain a correlation matrix.. Verbatim Evidence: "The terms 'boundary spanning', 'correlation', and 'matrix' do not appear anywhere in the text."</t>
+        </is>
+      </c>
     </row>
     <row r="654" ht="18" customHeight="1" s="10">
       <c r="A654" t="inlineStr">
@@ -33350,6 +33560,16 @@
           <t>BSMA0651</t>
         </is>
       </c>
+      <c r="E654" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F654" t="inlineStr">
+        <is>
+          <t>EXC_NO_CORR</t>
+        </is>
+      </c>
       <c r="G654" t="inlineStr">
         <is>
           <t>In a recent study by CCL, 86 percent of senior executives said it is "extremely important" to work across boundaries in their current leadership roles. Yet, only 7 percent of these executives believe they are currently "very effective" at doing so. Closing this gap is both a critical challenge and a transformative opportunity for leaders and organizations in today's business environment. This white paper explores why boundary spanning leadership matters and how to make it happen.</t>
@@ -33373,7 +33593,11 @@
       <c r="K654" t="n">
         <v>2016</v>
       </c>
-      <c r="P654" s="8" t="n"/>
+      <c r="P654" s="8" t="inlineStr">
+        <is>
+          <t>This document is an industry white paper by the Center for Creative Leadership. It presents descriptive survey percentages rather than quantitative empirical findings, and it does not contain a correlation matrix.. Verbatim Evidence: "Data were collected from 128 CCL participants who attended the Leadership at the Peak program between September 2008 and April 2009... Figure 9 presents the top 10 trends, ranked by the number of times they were cited as having an impact on the organization’s strategy."</t>
+        </is>
+      </c>
     </row>
     <row r="655" ht="18" customHeight="1" s="10">
       <c r="A655" t="inlineStr">
@@ -33386,6 +33610,16 @@
           <t>BSMA0652</t>
         </is>
       </c>
+      <c r="E655" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F655" t="inlineStr">
+        <is>
+          <t>Code 99: Other - Firm-level</t>
+        </is>
+      </c>
       <c r="G655" t="inlineStr">
         <is>
           <t>Purpose – The role of management control is frequently emphasized in connection with inter-organizational relationships and value networks. For example, boundary-spanning cost and accounting control techniques have been studied in multifaceted empirical settings. The prevalence of such techniques is, however, currently unknown in conjunction with companies’ interests to increase inter-organizational integration in general. Additionally, also the nexus between the internal state of cost management and the company’s willingness to develop inter-organizational relationships requires further investigation. The paper aims to discuss these issues. Design/methodology/approach – The study is based on an extensive survey that was responded to by more than 1,500 CEOs and CFOs from large, medium-sized and small Finnish enterprises in a variety of industries. As the authors chose the mixed-methods approach, both quantitative and qualitative data were collected for the study.</t>
@@ -33409,7 +33643,11 @@
       <c r="K655" t="n">
         <v>2018</v>
       </c>
-      <c r="P655" s="8" t="n"/>
+      <c r="P655" s="8" t="inlineStr">
+        <is>
+          <t>The paper conducts a firm-level analysis of organizational cost management and inter-organizational integration, rather than measuring individual-level boundary spanning behaviors.. Verbatim Evidence: "The study is based on an extensive survey that was responded to by more than 1,500 CEOs and CFOs from large, medium-sized and small Finnish enterprises in a variety of industries."</t>
+        </is>
+      </c>
     </row>
     <row r="656" ht="18" customHeight="1" s="10">
       <c r="A656" t="inlineStr">
@@ -33422,6 +33660,16 @@
           <t>BSMA0653</t>
         </is>
       </c>
+      <c r="E656" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F656" t="inlineStr">
+        <is>
+          <t>Firm-level</t>
+        </is>
+      </c>
       <c r="G656" t="inlineStr">
         <is>
           <t>This work examines how the strategic choice and performance of late movers are inﬂuenced by the top management team’s external ties, inside and outside the ﬁrm’s industry. Using a multiyear sample of ﬁrms from the computer industry, we found that intra-industry trade-association ties of top managers led to the adoption of a resource-imitation strategy by late movers while extra-industry importation and professional-association ties led to the adoption of a resource-substitution strategy. We also found that trade association ties had a negative effect on the performance of late movers using resource-substitution, while top managers’ service on other ﬁrms’ boards had a positive inﬂuence on the performance of those ﬁrms. Our ﬁndings not only conﬁrm the importance of the role of ﬁt in strategy and performance, but they also highlight the importance of the management and control of boundary-spanning activities.</t>
@@ -33445,7 +33693,11 @@
       <c r="K656" t="n">
         <v>2009</v>
       </c>
-      <c r="P656" s="8" t="n"/>
+      <c r="P656" s="8" t="inlineStr">
+        <is>
+          <t>The study measures boundary spanning (external ties) at the top management team (TMT) and firm level, rather than at the individual level.. Verbatim Evidence: "This work examines how the strategic choice and performance of late movers are inﬂuenced by the top management team’s external ties, inside and outside the ﬁrm’s industry."</t>
+        </is>
+      </c>
     </row>
     <row r="657" ht="18" customHeight="1" s="10">
       <c r="A657" t="inlineStr">
@@ -33458,6 +33710,16 @@
           <t>BSMA0654</t>
         </is>
       </c>
+      <c r="E657" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F657" t="inlineStr">
+        <is>
+          <t>1 = No effect size of interest</t>
+        </is>
+      </c>
       <c r="G657" t="inlineStr">
         <is>
           <t>Purpose – This study aims to investigate the effect of social undermining on the service employees’ boundary-spanning behavior though perceived ﬁt with job (P-J ﬁt). This study also aims to examine the moderating role of ethical climate in the relationship between service employees’ perceived ﬁt with job (P-J ﬁt) and boundary-spanning behavior.</t>
@@ -33481,7 +33743,11 @@
       <c r="K657" t="n">
         <v>2013</v>
       </c>
-      <c r="P657" s="8" t="n"/>
+      <c r="P657" s="8" t="inlineStr">
+        <is>
+          <t>The paper only provides 'Measure correlations' which appear to be latent construct intercorrelations from a CFA (discriminant validity testing), and completely omits raw means and standard deviations.. Verbatim Evidence: "Evidence of discriminant validity is provided by the fact that all of the construct intercorrelations were significantly (p &lt; 0.05) less than 1.00"</t>
+        </is>
+      </c>
     </row>
     <row r="658" ht="18" customHeight="1" s="10">
       <c r="A658" t="inlineStr">
@@ -33494,6 +33760,16 @@
           <t>BSMA0655</t>
         </is>
       </c>
+      <c r="E658" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F658" t="inlineStr">
+        <is>
+          <t>Latent Correlations Only</t>
+        </is>
+      </c>
       <c r="G658" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this model is to explain how person – organization fit (P – O fit) and competitive intensity, conceptualized as a job resource and a job demand, respectively, ultimately affect the development of frontline employee boundary-spanning behavior (BSB).</t>
@@ -33517,7 +33793,11 @@
       <c r="K658" t="n">
         <v>2014</v>
       </c>
-      <c r="P658" s="8" t="n"/>
+      <c r="P658" s="8" t="inlineStr">
+        <is>
+          <t>The paper does not report a raw, zero-order correlation matrix, nor does it report Means and Standard Deviations. The presented correlation matrix (Table I) contains latent construct intercorrelations derived from a confirmatory factor analysis (CFA) measurement model, which is used for assessing discriminant validity and common method variance.. Verbatim Evidence: "Evidence of discriminant validity is provided by the fact that all of the construct intercorrelations were significantly (p &lt; 0.05) less than 1.00; and the variance shared by any two constructs (i.e. the square of their intercorrelation) was always less than the [average variance extracted]."</t>
+        </is>
+      </c>
     </row>
     <row r="659" ht="18" customHeight="1" s="10">
       <c r="A659" t="inlineStr">
@@ -33530,6 +33810,16 @@
           <t>BSMA0656</t>
         </is>
       </c>
+      <c r="E659" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F659" t="inlineStr">
+        <is>
+          <t>EXCL_NON_INDIVIDUAL</t>
+        </is>
+      </c>
       <c r="G659" t="inlineStr">
         <is>
           <t>Individuals in work teams frequently cross boundaries across teams, often by using information and communication technologies (ICTs). The current study investigates the effects of members’ boundary work and the visibility affordance of teams’ ICTs on Transactive Memory Systems (TMS) in teams. Survey data from 212 fulltime employees whose work hours were divided between multiple teams reveals that boundary spanning enhances the focal team’s TMS specialization and credibility and negatively inﬂuences TMS coordination. Additionally, boundary reinforcement positively affects TMS credibility and coordination. The visibility affordance has a direct positive effect on all three dimensions of TMS and a moderating effect for boundary reinforcement such that higher visibility overrides the positive direct effect of boundary reinforcement on TMS. These ﬁndings suggest that different types of boundary work contribute to different dimensions of TMS and that teams might consider prioritizing the use of ICTs with high visibility to enhance their TMS.</t>
@@ -33553,7 +33843,11 @@
       <c r="K659" t="n">
         <v>2024</v>
       </c>
-      <c r="P659" s="8" t="n"/>
+      <c r="P659" s="8" t="inlineStr">
+        <is>
+          <t>The study measures boundary spanning at the team level (team norms/culture) rather than at the individual level.. Verbatim Evidence: "Boundary spanning was measured using items including “Does the team value team members for making use of their relationships with others on behalf of the team?,” and “Does your primary team encourage its members to solicit information and resources from elsewhere in and/or beyond the team?”"</t>
+        </is>
+      </c>
     </row>
     <row r="660" ht="18" customHeight="1" s="10">
       <c r="A660" t="inlineStr">
@@ -33566,6 +33860,16 @@
           <t>BSMA0657</t>
         </is>
       </c>
+      <c r="E660" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F660" t="inlineStr">
+        <is>
+          <t>No BSMA Measure</t>
+        </is>
+      </c>
       <c r="G660" t="inlineStr">
         <is>
           <t>When Leaders Use Self-Uncertainty Strategically: Consequences for Intergroup Leadership and Identity Confirmation Dynamics By Alison Young Claremont Graduate University: 2023 Framed by the social identity theory of leadership, one question that is beginning to receive attention is how intergroup leaders can lead across distinct subgroups and improve intersubgroup relations without provoking social identity-related concerns (e.g., subgroup identity distinctiveness threat). Past studies have found that leaders can use their rhetoric and boundary spanning behavior to meet their members’ identity needs and garner support. In addition, the self-uncertainty literature has suggested that leaders can strategically elevate and resolve members’ self-uncertainty through their rhetoric. The current research proposed that members who felt uncertain about their subgroup’s identity would have more favorable evaluations of the intergroup leader and perceptions of the out-subgroup if the leader confirmed their subgroup identity and/or was a blended boundary spanner. Members’ identity-uncertainty and subgroup identity validation have yet to be jointly examined in the context of intergroup leadership. Study 1 (N = 214) showed that those with high identity centrality had more positive leader evaluations and out-subgroup perceptions. Study 2 (N = 248) showed that those with greater subgroup identity-uncertainty who received a message from their leader that confirmed their subgroup identity had more positive out-subgroup perceptions; however, a person’s level of subgroup identity-uncertainty led to differential perceptions depending on the leader’s boundary spanning behavior. Implications and future directions are discussed.</t>
@@ -33589,7 +33893,11 @@
       <c r="K660" t="n">
         <v>2023</v>
       </c>
-      <c r="P660" s="8" t="n"/>
+      <c r="P660" s="8" t="inlineStr">
+        <is>
+          <t>The paper does not measure individual-level boundary spanning behavior. Instead, it manipulates boundary spanning as a characteristic of a hypothetical leader in an experimental vignette.. Verbatim Evidence: "There were three independent variables, all manipulated: subgroup identity-uncertainty (low vs. high), leader rhetoric (confirm subgroup identity vs. remain neutral) and boundary spanning leader behavior (discrete vs. blended)."</t>
+        </is>
+      </c>
     </row>
     <row r="661" ht="18" customHeight="1" s="10">
       <c r="A661" t="inlineStr">
@@ -33602,6 +33910,16 @@
           <t>BSMA0658</t>
         </is>
       </c>
+      <c r="E661" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F661" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G661" t="inlineStr">
         <is>
           <t>This study examines how deans and associate deans of a group from similar universities use networking. Specifically, we consider whether the deans, traditionally considered to perform boundary-spanning functions, make more use of external networking than do the associate deans, who are their subordinates. We examine the relationship between accuracy in perceiving a network and influence in the network. Finally, we consider the relationship between reports of networking outside the sample and influence within the sample. We find support for our first two propositions and raise several issues related to our final one.</t>
@@ -33625,7 +33943,11 @@
       <c r="K661" t="n">
         <v>2001</v>
       </c>
-      <c r="P661" s="8" t="n"/>
+      <c r="P661" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures individual-level boundary spanning behaviors (external contacts of deans) and contains a zero-order Pearson correlation matrix (Table IV) reporting relationships among importance, accuracy, and external contacts.. Verbatim Evidence: "Table IV provides the correlation matrix showing the relationships among importance ratings, accuracy ratings, and reports of external contacts"</t>
+        </is>
+      </c>
     </row>
     <row r="662" ht="18" customHeight="1" s="10">
       <c r="A662" t="inlineStr">
@@ -33638,6 +33960,16 @@
           <t>BSMA0659</t>
         </is>
       </c>
+      <c r="E662" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F662" t="inlineStr">
+        <is>
+          <t>Retracted Article / Firm Level</t>
+        </is>
+      </c>
       <c r="G662" t="inlineStr">
         <is>
           <t>This research paper investigates the vital role of boundary-spanning knowledge search and absorptive capacity in shaping the cooperative innovation performance of noncore firms operating in the context of sustainable development. The dynamic nature of technological innovation, exacerbated by market flattening and the challenges posed by the COVID-19 pandemic, has compelled small and medium-sized enterprises (SMEs) to seek innovative breakthroughs. Cooperative innovation emerges as a strategic avenue for SMEs to mitigate risks and enhance their willingness to innovate. However, non-core firms often encounter technological and market disadvantages, hindering innovation efforts. This study explores how boundary-spanning knowledge search, which bridges the gap between non-core firms and the external environment, influences cooperative innovation. Furthermore, the research delves into the mediating role of both potential and actual absorptive capacity in the relationship between boundaryspanning knowledge search and cooperative innovation performance. Empirical findings indicate that boundary-spanning knowledge searches positively impact cooperative innovation, with technological and market knowledge searches yield significant results. Moreover, absorptive capacity exhibits a dual mechanism, directly influencing cooperative innovation and mediating the relationship between knowledge search and performance. This paper extends existing research by focusing on non-core firms within the sustainable development context, offering valuable insights for SMEs seeking innovative strategies. It also highlights the diverse pathways through which boundary-spanning knowledge search affects cooperative innovation. These findings offer practical implications for enhancing non-core firms’ innovation capabilities, including encouraging proactive knowledge search and developing absorptive capacity-inducing mechanisms through employee training and information platforms.</t>
@@ -33661,7 +33993,11 @@
       <c r="K662" t="n">
         <v>2024</v>
       </c>
-      <c r="P662" s="8" t="n"/>
+      <c r="P662" s="8" t="inlineStr">
+        <is>
+          <t>The study was conducted at the firm level, examining non-core firms, rather than individual-level boundary spanning. Furthermore, the PDF is stamped as a RETRACTED ARTICLE on every page.. Verbatim Evidence: "This research paper investigates the vital role of boundary-spanning knowledge search and absorptive capacity in shaping the cooperative innovation performance of non-core firms"</t>
+        </is>
+      </c>
     </row>
     <row r="663" ht="18" customHeight="1" s="10">
       <c r="A663" t="inlineStr">
@@ -33674,6 +34010,16 @@
           <t>BSMA0660</t>
         </is>
       </c>
+      <c r="E663" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F663" t="inlineStr">
+        <is>
+          <t>Not Individual Level</t>
+        </is>
+      </c>
       <c r="G663" t="inlineStr">
         <is>
           <t>This paper examines the influence of boundary-spanning knowledge search on cooperative innovation performance and explores the moderating role of innovation passion in Chinese firms. We collected 229 valid responses from Chinese firms participating in collaborative innovation projects and applied confirmatory factor analysis to test the reliability and validity of the constructs, multiple stepwise regressions to verify the direct effect, and the PROCESS macro to test the moderating effect. The results show that all three dimensions of boundary-spanning knowledge search (i.e. network capability, IT capability, and absorptive capacity) positively affect cooperative innovation performance. Harmonious innovation passion positively moderates the relationship between network capability and cooperative innovation performance. In contrast, compulsive innovation passion plays a negative moderating role in the relationship between absorptive capacity and cooperative innovation performance. This study further enriches and extends the theoretical framework of cooperative innovation performance by emphasizing the impact of the three dimensions of boundary-spanning knowledge search.</t>
@@ -33697,7 +34043,11 @@
       <c r="K663" t="n">
         <v>2025</v>
       </c>
-      <c r="P663" s="8" t="n"/>
+      <c r="P663" s="8" t="inlineStr">
+        <is>
+          <t>The study focuses on boundary-spanning knowledge search at the enterprise/firm level, not the individual level.. Verbatim Evidence: "We collected 229 valid responses from Chinese firms participating in collaborative innovation projects..."</t>
+        </is>
+      </c>
     </row>
     <row r="664" ht="18" customHeight="1" s="10">
       <c r="A664" t="inlineStr">
@@ -33710,6 +34060,16 @@
           <t>BSMA0661</t>
         </is>
       </c>
+      <c r="E664" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F664" t="inlineStr">
+        <is>
+          <t>EXCL_TEAM_LEVEL</t>
+        </is>
+      </c>
       <c r="G664" t="inlineStr">
         <is>
           <t>Based on upper echelons, paradox, and social capital theory, this study extends the association of CEO vision articulation and feedback-seeking behavior with ﬁrm sustainability by identifying the mediating role of eco-innovation and top management team (TMT) boundary-spanning behavior as a moderator. By analyzing the data of mid-sized to large Chinese ﬁrms using hierarchical regression and bootstrapping-based moderated path analysis, we found that product and process eco-innovation mediates the link between CEO vision articulation and ﬁrm sustainability while CEO feedbackseeking behavior enhances ﬁrm’s sustainability through product eco-innovation only. Finally, conditional indirect effects show the vital role of TMT boundary-spanning behavior in facilitating CEOs to improve the ﬁrm’s long-term sustainability through eco-innovation.</t>
@@ -33733,7 +34093,11 @@
       <c r="K664" t="n">
         <v>2022</v>
       </c>
-      <c r="P664" s="8" t="n"/>
+      <c r="P664" s="8" t="inlineStr">
+        <is>
+          <t>The paper focuses on Top Management Team (TMT) boundary-spanning behavior rather than individual-level behaviors, and aggregates individual responses to the organizational level.. Verbatim Evidence: "We measured TMT boundary-spanning behavior through the modified scale of Yan et al. (2020)... After validating the fitness of our measurements, we proceed with the aggregation of individual responses to the organizational level due to the hierarchical structure of our data."</t>
+        </is>
+      </c>
     </row>
     <row r="665" ht="18" customHeight="1" s="10">
       <c r="A665" t="inlineStr">
@@ -33746,6 +34110,16 @@
           <t>BSMA0662</t>
         </is>
       </c>
+      <c r="E665" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F665" t="inlineStr">
+        <is>
+          <t>No Correlation Matrix</t>
+        </is>
+      </c>
       <c r="G665" t="inlineStr">
         <is>
           <t>Local government or better known as the local authority vested with the power to plan, develop, and regulate businesses in the area within its jurisdiction plays a significant role in creating a conducive environment for businesses to grow and flourish. In playing this role, employees in local authority must possess a certain degree of innovative work behavior. This paper reports on a study that investigated innovative work behavior orientation among employees of the local government. A total of 100 employees of a local city council responded to a self-administered questionnaire on innovative work behavior. The results revealed that respondents scored a moderate high orientation on the innovative work behavior scale.</t>
@@ -33769,7 +34143,11 @@
       <c r="K665" t="n">
         <v>2014</v>
       </c>
-      <c r="P665" s="8" t="n"/>
+      <c r="P665" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures innovative work behavior but does not report a zero-order correlation matrix, only reporting means and standard deviations across demographic groups.. Verbatim Evidence: "Table 1: Respondents’ innovative work behavior mean score according to demographic factors (N=100)"</t>
+        </is>
+      </c>
     </row>
     <row r="666" ht="18" customHeight="1" s="10">
       <c r="A666" t="inlineStr">
@@ -33782,6 +34160,16 @@
           <t>BSMA0663</t>
         </is>
       </c>
+      <c r="E666" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F666" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G666" t="inlineStr">
         <is>
           <t>This study investigates the role of green strategic intent in facilitating the adoption of circular economy practices within public sector organizations. Using the dynamic capability view, we proposed that green strategic intent leads to circular economy practices. We also proposed that artificial intelligence (AI) capability and green learning ambidexterity act as significant underlying mechanisms and leader boundary-spanning behavior as a moderator. Data were collected from 228 managers of various public sector departments in United Arab Emirates (UAE) using a time-lagged design. Our results supported that there is a positive relationship between green strategic intent and circular economy practices. Further, green strategic intent positively influences circular economy practices through AI capability and green learning ambidexterity that act as serial mediators of the green strategic intent-circular economy practices link. Finally, leader boundary-spanning behavior significantly moderates the effects of green strategic intent on AI capability. Our findings offer important insights that can enable public sector organizations to implement circular economy practices.</t>
@@ -33805,7 +34193,11 @@
       <c r="K666" t="n">
         <v>2025</v>
       </c>
-      <c r="P666" s="8" t="n"/>
+      <c r="P666" s="8" t="inlineStr">
+        <is>
+          <t>The study measures individual-level leader boundary-spanning behavior and reports a valid raw zero-order correlation matrix in Table 1.. Verbatim Evidence: "Leader boundary-spanning behavior was assessed by adapting a six-item scale (α = 0.92) from Marrone et al. (2007). “I reach out to individuals outside of our organization that can offer expertise or ideas about the task at hand” was a sample item."</t>
+        </is>
+      </c>
     </row>
     <row r="667" ht="18" customHeight="1" s="10">
       <c r="A667" t="inlineStr">
@@ -33818,6 +34210,16 @@
           <t>BSMA0664</t>
         </is>
       </c>
+      <c r="E667" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F667" t="inlineStr">
+        <is>
+          <t>No Correlation Matrix</t>
+        </is>
+      </c>
       <c r="G667" t="inlineStr">
         <is>
           <t>This paper examines organizational learning through a multilevel network lens. We assess how interpersonal knowledge transfer is sustained by the organizational structure of interunit work-ﬂow ties and by the level of specialism of the connected units.</t>
@@ -33841,7 +34243,11 @@
       <c r="K667" t="n">
         <v>2016</v>
       </c>
-      <c r="P667" s="8" t="n"/>
+      <c r="P667" s="8" t="inlineStr">
+        <is>
+          <t>The paper does not report a zero-order correlation matrix. It only reports network descriptive statistics and ERGM/MERGM estimates.. Verbatim Evidence: "Table 4 ERGM and MERGM estimates."</t>
+        </is>
+      </c>
     </row>
     <row r="668" ht="18" customHeight="1" s="10">
       <c r="A668" t="inlineStr">
@@ -33854,6 +34260,16 @@
           <t>BSMA0665</t>
         </is>
       </c>
+      <c r="E668" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F668" t="inlineStr">
+        <is>
+          <t>EXCL_FIRM_LEVEL</t>
+        </is>
+      </c>
       <c r="G668" t="inlineStr">
         <is>
           <t>Innovation is a key driver for organizations to survive and thrive in increasingly hyper-competitive markets. This study investigates the effects of boundary-spanning search on innovation capability. Speciﬁcally, it examines the mediating and moderating effects of network ties and absorptive capacity on boundary-spanning search and innovation in Chinese companies. We constructed a theoretical model of an organization’s boundary-spanning search and innovation capability and distributed a survey questionnaire to a sample of speciﬁc industries with upstream and downstream relations in Sichuan Province in China for their responses. Results from the study reveal that boundary-spanning search has a positive and signiﬁcant impact on innovation capability as well as a positive moderating effect on absorptive capacity and innovation capability. This paper shows that enterprises need to continuously focus on exploring networking opportunities in direct and indirect ways to get access to effective ﬂow and diffusion of resources, which in turn can enhance innovation capability.</t>
@@ -33877,7 +34293,11 @@
       <c r="K668" t="n">
         <v>2018</v>
       </c>
-      <c r="P668" s="8" t="n"/>
+      <c r="P668" s="8" t="inlineStr">
+        <is>
+          <t>The study measures boundary-spanning at the organizational (firm) level, not at the individual level. Additionally, the correlation matrix reports latent construct intercorrelations used for discriminant validity.. Verbatim Evidence: "First, the population of the study consisted of high-tech industries operating in Sichuan Province in China as of June 2017. Second, we selected 450 firms possessing upstream and downstream relationships"</t>
+        </is>
+      </c>
     </row>
     <row r="669" ht="18" customHeight="1" s="10">
       <c r="A669" t="inlineStr">
@@ -33890,6 +34310,16 @@
           <t>BSMA0666</t>
         </is>
       </c>
+      <c r="E669" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F669" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
+      </c>
       <c r="G669" t="inlineStr">
         <is>
           <t>Due to their complexity and high social impact, urban infrastructure projects often face challenges in managing the design decision-making processes across disparate disciplinary and knowledge domain boundaries. This paper introduces the notion of design boundary dynamics to describe the various cross-boundary coordination phenomena associated with organising the design of infrastructure projects. Taking a practice-based theoretical stance, the paper presents findings of qualitative research on the nature and genesis of design boundaries and their relation to the strategic decision-making on a transportation infrastructure project. Findings illustrate the entangled processes, through which the disciplinary, knowledge-domain and stage-based design boundaries emerged as a result of unfolding project practices. Paper identifies the key role of resource allocation constraints, path dependency of project decisions, and problem-solving nature of design and concludes with strategic recommendations for upstream operational integration to mitigate the impact of design boundary dynamics on infrastructure projects.</t>
@@ -33913,7 +34343,11 @@
       <c r="K669" t="n">
         <v>2015</v>
       </c>
-      <c r="P669" s="8" t="n"/>
+      <c r="P669" s="8" t="inlineStr">
+        <is>
+          <t>The paper is a qualitative case study based on interviews and project documentation; it does not measure individual-level boundary spanning behaviors quantitatively and lacks a correlation matrix.. Verbatim Evidence: "The empirical basis for this paper is qualitative research I conducted in the setting of a major transport infrastructure project."</t>
+        </is>
+      </c>
     </row>
     <row r="670" ht="18" customHeight="1" s="10">
       <c r="A670" t="inlineStr">
@@ -33926,6 +34360,16 @@
           <t>BSMA0667</t>
         </is>
       </c>
+      <c r="E670" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F670" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G670" t="inlineStr">
         <is>
           <t>Innovations transform our research traditions and become the driving force to advance individual, group, and social creativity. Meanwhile, interdisciplinary research is increasingly being promoted as a route to advance the complex challenges we face as a society. In this paper, we use Latent Dirichlet Allocation (LDA) citation as a proxy context for the diffusion of an innovation. With an analysis of topic evolution, we divide the diffusion process into five stages: testing and evaluation, implementation, improvement, extending, and fading. Through a correlation analysis of topic and subject, we show the application of LDA in different subjects. We also reveal the cross‐boundary diffusion between different subjects based on the analysis of the interdisciplinary studies. The results show that as LDA is transferred into different areas, the adoption of each subject is relatively adjacent to those with similar research interests. Our findings further support researchers' understanding of the impact formation of innovation.</t>
@@ -33949,7 +34393,11 @@
       <c r="K670" t="n">
         <v>2018</v>
       </c>
-      <c r="P670" s="8" t="n"/>
+      <c r="P670" s="8" t="inlineStr">
+        <is>
+          <t>The paper conducts a citation analysis of the Latent Dirichlet Allocation (LDA) algorithm. It does not measure individual-level boundary spanning behaviors nor does it contain a raw, zero-order correlation matrix.. Verbatim Evidence: "In this paper, we quantitatively measure the diffusion of a particular innovation, building on previous work that defines the trail of progress in terms of citations. With a case study of the evolution of LDA, we demonstrate the sequence and progress of the growth of innovation..."</t>
+        </is>
+      </c>
     </row>
     <row r="671" ht="18" customHeight="1" s="10">
       <c r="A671" t="inlineStr">
@@ -33962,6 +34410,16 @@
           <t>BSMA0668</t>
         </is>
       </c>
+      <c r="E671" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F671" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G671" t="inlineStr">
         <is>
           <t>This study examines how individual purchasing agents function as boundary spanners with suppliers to inﬂuence trust development in themselves and the buying ﬁrms that employ them. Building upon boundary theory and supply chain cooperation research, we identify three boundary spanning capabilities of purchasing agents and empirically test how these capabilities shape buyer–supplier trust development. Using two samples of data collected from suppliers in the automotive industry and food industry, we found that a purchasing agent’s effectiveness in strategic communication with suppliers affects a supplier’s trust in the buying ﬁrm, while an agent’s professional knowledge and ability to reach compromises with suppliers affect a supplier’s trust in the purchasing agent representing the ﬁrm. Trust in the purchasing agent in turn affects trust in the buying ﬁrm. Theoretical and managerial implications are discussed.</t>
@@ -33985,7 +34443,11 @@
       <c r="K671" t="n">
         <v>2011</v>
       </c>
-      <c r="P671" s="8" t="n"/>
+      <c r="P671" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures individual-level boundary spanning behaviors (purchasing agent capabilities) and provides a raw, zero-order correlation matrix.. Verbatim Evidence: "Table 2 Correlation matrix of variables analyzed."</t>
+        </is>
+      </c>
     </row>
     <row r="672" ht="18" customHeight="1" s="10">
       <c r="A672" t="inlineStr">
@@ -33998,6 +34460,16 @@
           <t>BSMA0669</t>
         </is>
       </c>
+      <c r="E672" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F672" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G672" t="inlineStr">
         <is>
           <t>Despite growing recognition of the importance of boundary spanners at managing inter-organizational relationships, the process by which capabilities residing in boundary spanning individuals are leveraged to encourage partner firm investment remains unclear. In addressing this gap, we find that a boundary spanner's capabilities in strategic communication and job expertise enhance a customer firm's communication with a supplier firm, which increases a supplier's willingness to make future-oriented investment both directly as well as indirectly through increasing customer firm trustworthiness. Data collected from two samples of suppliers in the U.S. and other Western industrialized countries provide empirical support for our propositions. Furthermore, we found that the process of how boundary spanning capabilities influence supplier willingness to invest differs significantly between the two regions in ways that affect managerial decisions on resource allocation.</t>
@@ -34021,7 +34493,11 @@
       <c r="K672" t="n">
         <v>2015</v>
       </c>
-      <c r="P672" s="8" t="n"/>
+      <c r="P672" s="8" t="inlineStr">
+        <is>
+          <t>The study measures individual-level boundary spanning behaviors of purchasing managers (strategic communication and job expertise) and provides a raw, zero-order correlation matrix based on composite scores.. Verbatim Evidence: "composite scores of each construct were used to test a structural model. ... Table 2 presents the correlation matrix."</t>
+        </is>
+      </c>
     </row>
     <row r="673" ht="18" customHeight="1" s="10">
       <c r="A673" t="inlineStr">
@@ -34034,6 +34510,16 @@
           <t>BSMA0670</t>
         </is>
       </c>
+      <c r="E673" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F673" t="inlineStr">
+        <is>
+          <t>Non-Individual Anchors</t>
+        </is>
+      </c>
       <c r="G673" t="inlineStr">
         <is>
           <t>Purpose – This study extends the concept of managerial efficacy to include managerial means efficacy (MME) attributed to the utility and quality of means external to managers for performing a task. Focusing on its antecedents, the authors theorize and empirically test MME sourced from the organization (MMEO) and situate the examination under extreme events.</t>
@@ -34057,7 +34543,11 @@
       <c r="K673" t="n">
         <v>2022</v>
       </c>
-      <c r="P673" s="8" t="n"/>
+      <c r="P673" s="8" t="inlineStr">
+        <is>
+          <t>The boundary spanning variables (Horizontal and Vertical Relationship Management) are measured at the organizational level (agency), not the individual level.. Verbatim Evidence: "How effective is your agency in managing its relationship with each of the following groups?"</t>
+        </is>
+      </c>
     </row>
     <row r="674" ht="18" customHeight="1" s="10">
       <c r="A674" t="inlineStr">
@@ -34070,6 +34560,16 @@
           <t>BSMA0671</t>
         </is>
       </c>
+      <c r="E674" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F674" t="inlineStr">
+        <is>
+          <t>Level of Analysis / No Correlation Matrix</t>
+        </is>
+      </c>
       <c r="G674" t="inlineStr">
         <is>
           <t>In order to reveal the impact of boundary-spanning activities of cooperative innovation teams on team innovation performance, this paper takes the panel data of 71 cooperative innovation teams from January to November 2022 as the research sample. It introduces intermediary variables (teamwork crafting and individual work crafting) to analyze the impact mechanism of boundaryspanning activities of teams on innovation performance, 71 teams were divided into 41 experimental groups and 30 control groups, and a quasi-natural experiment was conducted on the innovation performance of team boundary-spanning activities using the Double Difference Model (DID).Research has shown that boundary-spanning activities of collaborative innovation teams can promote team innovation performance. Team job crafting has a mediating effect on team innovation performance in boundary-spanning activities of collaborative innovation teams. Team job crafting and individual job crafting mediate between the boundary-spanning activities of collaborative innovation teams and team innovation performance. Further analysis using the double difference model found that compared to teams without boundary-spanning activities, teams with boundary-spanning activities can directly improve team innovation performance. When team reflection is vital, and task interdependence is high, it will promote team innovation performance. This research enriches the research on the effects of boundary-spanning activities of collaborative innovation teams, explores solutions based on quasi-nature, and provides a reference for improving the team innovation performance of collaborative innovation teams.</t>
@@ -34093,7 +34593,11 @@
       <c r="K674" t="n">
         <v>2023</v>
       </c>
-      <c r="P674" s="8" t="n"/>
+      <c r="P674" s="8" t="inlineStr">
+        <is>
+          <t>The study focuses on firm-level joint-patent networks (patent-intensive enterprises) rather than individual-level boundary spanning behaviors. Furthermore, the paper does not report any correlation matrix.. Verbatim Evidence: "This paper focuses on PI enterprises in China and examines their co-innovation position advantage and technological innovation performance using DEA and SNA. The sample consists of 103 listed firms with more than 500 invention patents and a 5-year R&amp;D history."</t>
+        </is>
+      </c>
     </row>
     <row r="675" ht="18" customHeight="1" s="10">
       <c r="A675" t="inlineStr">
@@ -34106,6 +34610,16 @@
           <t>BSMA0672</t>
         </is>
       </c>
+      <c r="E675" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F675" t="inlineStr">
+        <is>
+          <t>Latent Matrix</t>
+        </is>
+      </c>
       <c r="G675" t="inlineStr">
         <is>
           <t>Purpose – In the field of innovation, there is growing interest in exploring the factors that determine the extent to which firms can learn from external sources. However, most previous studies neglect the role of human factors. Little is known about which employee behaviors are desirable for boundary-spanning learning activities and which human resource management (HRM) practices are appropriate to respond to external knowledge transfer across boundaries. To fill this gap, the authors investigate the role of empowermentfocused HRM in interfirm learning and explore the integration of external inputs from the perspective of employees.</t>
@@ -34129,7 +34643,11 @@
       <c r="K675" t="n">
         <v>2021</v>
       </c>
-      <c r="P675" s="8" t="n"/>
+      <c r="P675" s="8" t="inlineStr">
+        <is>
+          <t>The correlation matrix in Table 3 is explicitly labeled 'Discriminant validity' and contains the square roots of AVEs on the diagonal, indicating it reports latent correlations rather than raw zero-order correlations. Additionally, the study measures variables at the organizational/plant level (N=288 manufacturing plants) rather than individual-level boundary spanning behaviors.. Verbatim Evidence: "Our results showed that all correlations were lower than the square roots of AVEs (Table 3). Thus, discriminant validity of the constructs was acceptable. [...] Table 3. Discriminant validity"</t>
+        </is>
+      </c>
     </row>
     <row r="676" ht="18" customHeight="1" s="10">
       <c r="A676" t="inlineStr">
@@ -34142,6 +34660,16 @@
           <t>BSMA0673</t>
         </is>
       </c>
+      <c r="E676" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F676" t="inlineStr">
+        <is>
+          <t>EXC_LATENT_CORR</t>
+        </is>
+      </c>
       <c r="G676" t="inlineStr">
         <is>
           <t>Enterprise social media (ESM) provides convenient channels for employees to access enterprise-wide work resources but also exposes employees to potential distractions. Prior studies have confirmed this “two-sided” role of ESM usage on employee work performance. Ongoing studies are exploring possible methods to alleviate side effects of ESM usage. Drawing on boundary management literature and information processing theory, we propose the concept of individual boundary spanning to capture employees’ information-obtaining behaviors via ESM and identify two mediating mechanisms—mindfulness and information overload—through which an individual’s boundary spanning affects work performance. We also propose the concept of individual boundary buffering to capture protective actions by individuals that prevent them from becoming disturbed or overloaded with ESM requests. We further investigate the interaction effects of these two boundary activities in the ESM context. We conducted a survey and collected data from 202 ESM users from a research and development enterprise in China. The results suggest that individual boundary spanning triggers mindfulness in individuals that benefits their work performance but also increases information overload, harming work performance. Individual boundary buffering can enhance the positive relationship between individual boundary spanning and mindfulness, and mitigate the positive relationship between spanning activity and information overload.</t>
@@ -34165,7 +34693,11 @@
       <c r="K676" t="n">
         <v>2022</v>
       </c>
-      <c r="P676" s="8" t="n"/>
+      <c r="P676" s="8" t="inlineStr">
+        <is>
+          <t>The paper only provides a latent construct correlation matrix with square roots of AVEs on the diagonal for discriminant validity, rather than a raw zero-order correlation matrix with 1.00 or Cronbach's alpha on the diagonal.. Verbatim Evidence: "Table 5. The correlation matrix of constructs. ... Notes: The bolded elements on diagonal are the square roots of AVEs, and off-diagonal elements are correlations between constructs."</t>
+        </is>
+      </c>
     </row>
     <row r="677" ht="18" customHeight="1" s="10">
       <c r="A677" t="inlineStr">
@@ -34178,6 +34710,16 @@
           <t>BSMA0674</t>
         </is>
       </c>
+      <c r="E677" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F677" t="inlineStr">
+        <is>
+          <t>Firm-Level Analysis</t>
+        </is>
+      </c>
       <c r="G677" t="inlineStr">
         <is>
           <t>Research Summary: This study elucidates the previously underexplored structural heterogeneity inherent in multinational corporations' (MNCs) internal linkages by examining the concentration of cross-border collaborations among inventors within host countries. Building on the boundary spanning literature, we develop a two-stage framework identifying the knowledge distortion mechanism arising from this concentration: information overload in the cross-country knowledge absorption stage and long transmission paths and knowledge hoarding in the within-country diffusion stage. Both hinder local knowledge creation. We further propose that cross-country and withincountry network structures serve as contingencies moderating this relationship. The negative effects of collaboration concentration are exacerbated by structural holes in cross-country networks but attenuated by the reach and density of within-country networks. Empirical results based on American pharmaceutical MNCs from 1980 to 2008 support our hypotheses.</t>
@@ -34201,7 +34743,11 @@
       <c r="K677" t="n">
         <v>2026</v>
       </c>
-      <c r="P677" s="8" t="n"/>
+      <c r="P677" s="8" t="inlineStr">
+        <is>
+          <t>The study measures variables at the macro firm level (MNC-country-year) rather than measuring individual-level boundary spanning behaviors. Furthermore, the correlation matrix is not provided in the paper (it is in a supplementary appendix).. Verbatim Evidence: "We used an unbalanced panel of 1954 MNC-country-year observations for our regression analyses."</t>
+        </is>
+      </c>
     </row>
     <row r="678" ht="18" customHeight="1" s="10">
       <c r="A678" t="inlineStr">
@@ -34214,6 +34760,16 @@
           <t>BSMA0675</t>
         </is>
       </c>
+      <c r="E678" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F678" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G678" t="inlineStr">
         <is>
           <t>Technology transfer is an essential source of technological innovation for enterprises, which is conducive to the market transformation of patent achievements and the commercial application of new technologies. Building upon social capital theory, all data analyses were performed using SPSS 22.0 and Amos software with the multiple linear regression method. The study explores the mechanism of policy perception to obtain the technical resources needed for enterprise development through boundary-spanning behavior, with a moderating effect of inter-organizational trust and technological potential gap. The study uses survey data from 125 enterprise teams of 42 technology-based enterprises in China. The results show that policy perceived usefulness and usability significantly promote technology transfer performance and boundary-spanning behavior plays a mediating role between them. Speaking of the influencing factors of technology transfer, technological potential gap significantly moderates the relationship between boundary-spanning and technology transfer performance. In contrast, inter-organizational trust positively moderates the relationship between boundary-spanning and technology transfer performance. The research provides theoretical reference and guidance for enterprises on using policy perception better to improve technology transfer performance in the institutional environment. It also helps inspire enterprises to better deal with the cooperative relationship between relevant stakeholders and achieve win-win cooperation.</t>
@@ -34237,7 +34793,11 @@
       <c r="K678" t="n">
         <v>2022</v>
       </c>
-      <c r="P678" s="8" t="n"/>
+      <c r="P678" s="8" t="inlineStr">
+        <is>
+          <t>The boundary spanning construct is measured at the team/enterprise level rather than the individual level.. Verbatim Evidence: "In this study, boundary-spanning behavior refers to the interactive actions between the enterprise technology transfer team and external members of the enterprises"</t>
+        </is>
+      </c>
     </row>
     <row r="679" ht="18" customHeight="1" s="10">
       <c r="A679" t="inlineStr">

</xml_diff>

<commit_message>
chore: completed Batch 18 extraction (final)
</commit_message>
<xml_diff>
--- a/BSMA_AI_Run_V2.xlsx
+++ b/BSMA_AI_Run_V2.xlsx
@@ -34810,6 +34810,16 @@
           <t>BSMA0676</t>
         </is>
       </c>
+      <c r="E679" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F679" t="inlineStr">
+        <is>
+          <t>Wrong Level of Analysis</t>
+        </is>
+      </c>
       <c r="G679" t="inlineStr">
         <is>
           <t>In this dissertation, I attempt to study the antecedents, processes, and
@@ -34851,7 +34861,11 @@
       <c r="K679" t="n">
         <v>2019</v>
       </c>
-      <c r="P679" s="8" t="n"/>
+      <c r="P679" s="8" t="inlineStr">
+        <is>
+          <t>The dissertation conducts firm-level and dyad-level analyses focusing on organizational boundary-spanning, R&amp;D centralization, and firm-level inventor mobility using patent and alliance data. It does not measure individual-level boundary spanning behaviors.. Verbatim Evidence: "We employ a firm-year fixed effects negative binomial framework for our regression of inventor mobility because of the count nature and over dispersion of mobility events."</t>
+        </is>
+      </c>
     </row>
     <row r="680" ht="18" customHeight="1" s="10">
       <c r="A680" t="inlineStr">
@@ -34864,6 +34878,16 @@
           <t>BSMA0677</t>
         </is>
       </c>
+      <c r="E680" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F680" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G680" t="inlineStr">
         <is>
           <t>Purpose – The complex and changeable working environment makes individual cross-boundary activities inevitable. Yet, how employee’s boundary-spanning behavior (BSB) stimulates innovation performance remains to be further explored. This study aims to analyze the intermediary mechanism and boundary conditions between employee’s BSB and innovation performance based on knowledge integration theory.</t>
@@ -34887,7 +34911,11 @@
       <c r="K680" t="n">
         <v>2021</v>
       </c>
-      <c r="P680" s="8" t="n"/>
+      <c r="P680" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures employee boundary-spanning behavior (BSB) at the individual level and provides a valid zero-order correlation matrix of all key variables.. Verbatim Evidence: "Table 1. Means, standard deviations and correlations at the individual level... (7) BSB"</t>
+        </is>
+      </c>
     </row>
     <row r="681" ht="18" customHeight="1" s="10">
       <c r="A681" t="inlineStr">
@@ -34900,6 +34928,16 @@
           <t>BSMA0678</t>
         </is>
       </c>
+      <c r="E681" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F681" t="inlineStr">
+        <is>
+          <t>Firm-level</t>
+        </is>
+      </c>
       <c r="G681" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this paper is to explore how boundary-spanning demand-side search (BSDSS) fuels radical technological innovations as well as how innovation appropriability moderates this relationship. In particular, based on Teece’s (1986) argument regarding the appropriability of innovation, the authors divide factors to influence innovation appropriability into two types: external institution related and internal capability related.</t>
@@ -34923,7 +34961,11 @@
       <c r="K681" t="n">
         <v>2017</v>
       </c>
-      <c r="P681" s="8" t="n"/>
+      <c r="P681" s="8" t="inlineStr">
+        <is>
+          <t>The study measures boundary spanning at the firm level (Boundary-spanning demand-side search) rather than the individual level.. Verbatim Evidence: "we collected a sample of high-tech manufacturing firms in the China-Singapore Suzhou Industrial Park."</t>
+        </is>
+      </c>
     </row>
     <row r="682" ht="18" customHeight="1" s="10">
       <c r="A682" t="inlineStr">
@@ -34936,6 +34978,16 @@
           <t>BSMA0679</t>
         </is>
       </c>
+      <c r="E682" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F682" t="inlineStr">
+        <is>
+          <t>No Correlation Matrix</t>
+        </is>
+      </c>
       <c r="G682" t="inlineStr">
         <is>
           <t>Virtual teamwork has become a prevalent mode of collaboration. However, scant empirical attention has been given to the impact of virtual teamwork on individual members’ performance beyond the team setting. In this paper, we fill this gap by studying virtual teams in the context of online medical consultation (OMC) platforms. Specifically, we collect data from two OMC platforms during a time period when both platforms offered individual consultations (i.e., one patient connected with one physician) but only one offered team consultations (i.e., one patient connected with a team of physicians). Using a difference-in-difference-in-differences approach, we find that team participation has a robust, positive effect on physicians’ performance in individual consultations. We further explore the potential mechanisms through which team participation improves physicians’ performance. The empirical results indicate that the observed performance improvement is likely driven by peer effects in team settings. In particular, we find that physicians exert more effort in individual consultations after joining a team, and that performance improvement is stronger when (1) a physician can easily observe the performance of his teammates (peers), (2) a physician has teammates (peers) who performs well in individual consultations, (3) a physician has teammates (peers) from the same hospital or the same city, or (4) a physician has a lower performance prior to joining in a team. Our findings shed new light on the boundary-spanning roles of virtual teams and provide timely insights into the ongoing development of OMC platforms.</t>
@@ -34959,7 +35011,11 @@
       <c r="K682" t="n">
         <v>2025</v>
       </c>
-      <c r="P682" s="8" t="n"/>
+      <c r="P682" s="8" t="inlineStr">
+        <is>
+          <t>The study relies on econometric panel data (DDD) and does not provide a zero-order correlation matrix. Furthermore, it does not measure individual-level boundary spanning behaviors.. Verbatim Evidence: "Our findings shed new light on the boundary-spanning roles of virtual teams... [No correlation matrix is reported in the paper]"</t>
+        </is>
+      </c>
     </row>
     <row r="683" ht="18" customHeight="1" s="10">
       <c r="A683" t="inlineStr">
@@ -34972,6 +35028,16 @@
           <t>BSMA0680</t>
         </is>
       </c>
+      <c r="E683" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F683" t="inlineStr">
+        <is>
+          <t>Latent Construct Intercorrelations</t>
+        </is>
+      </c>
       <c r="G683" t="inlineStr">
         <is>
           <t>Purpose – Although enterprise social media (ESM) offers new opportunities for developing radical creativity, limited research has been conducted on how to foster such creativity in ESM contexts. Based on the approachinhibition theory of power (AITP), this study examines how supervisor-subordinate instrumental and expressive ties on ESM promote radical creativity through sense of power. Furthermore, it further investigates how boundary buffering moderates the influence of these supervisor-subordinate ties on sense of power.</t>
@@ -34995,7 +35061,11 @@
       <c r="K683" t="n">
         <v>2025</v>
       </c>
-      <c r="P683" s="8" t="n"/>
+      <c r="P683" s="8" t="inlineStr">
+        <is>
+          <t>The study does not report a raw zero-order correlation matrix with Means and SDs. Table 3 presents latent inter-construct correlations from a PLS-SEM model, with the square root of AVE on the diagonal to demonstrate discriminant validity.. Verbatim Evidence: "the square root of each construct’s AVE was greater than its inter-construct correlations, supporting discriminant validity."</t>
+        </is>
+      </c>
     </row>
     <row r="684" ht="18" customHeight="1" s="10">
       <c r="A684" t="inlineStr">
@@ -35008,6 +35078,16 @@
           <t>BSMA0681</t>
         </is>
       </c>
+      <c r="E684" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F684" t="inlineStr">
+        <is>
+          <t>Non-Individual Anchors</t>
+        </is>
+      </c>
       <c r="G684" t="inlineStr">
         <is>
           <t>Conﬂict among teams is inevitable in a multiteam system. Drawing on the theory of co-operation and competition, we proposed and tested a model linking the approaches teams adopt to conﬂict, inter-team co-ordination, and multiteam system performance. Data collected from 123 operation teams in 44 subway stations in Shanghai revealed that co-operative conﬂict management positively related to inter-team co-ordination, which in turn positively related to performance of the multiteam system. The relationship between competitive conﬂict management and inter-team co-ordination was insigniﬁcant and was moderated by co-operative conﬂict management. When co-operative conﬂict management was at a low level, competitive conﬂict management negatively related to inter-team co-ordination.</t>
@@ -35031,7 +35111,11 @@
       <c r="K684" t="n">
         <v>2019</v>
       </c>
-      <c r="P684" s="8" t="n"/>
+      <c r="P684" s="8" t="inlineStr">
+        <is>
+          <t>Boundary spanning behaviors (inter-team co-ordination and conflict management) are conceptualized and measured at the team/station level rather than the individual level.. Verbatim Evidence: "Because the level of analysis was at the station level, we retained a station in the sample only when it had responses from no fewer than two team leaders as well as no fewer than two shift teams."</t>
+        </is>
+      </c>
     </row>
     <row r="685" ht="18" customHeight="1" s="10">
       <c r="A685" t="inlineStr">
@@ -35044,6 +35128,16 @@
           <t>BSMA0682</t>
         </is>
       </c>
+      <c r="E685" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F685" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G685" t="inlineStr">
         <is>
           <t>This article draws on status characteristics theory to explore the mechanisms of individual-level boundaryspanning behavior on employee creative performance, as well as the mediating role of informal status and the moderating role of Zhongyong thinking. The results of a two-wave questionnaire survey of 202 employees show that boundary-spanning behavior has a significant positive relationship with employees’ creative performance, informal status mediates the link between boundary-spanning behavior and creative performance of this employee, Zhongyong thinking plays a moderating role between employees’ boundary-spanning behavior and their informal status, and Zhongyong thinking also moderates the mediating role of informal status between boundary-spanning behavior and employee creative performance. In this paper, a moderated mediation model is established to enhance the understanding of the effects and mechanisms of individual boundary-spanning behavior, as well as to provide some constructive insight into how boundary-spanning behavior can be effectively employed in management practice within the Chinese context.</t>
@@ -35067,7 +35161,11 @@
       <c r="K685" t="n">
         <v>2024</v>
       </c>
-      <c r="P685" s="8" t="n"/>
+      <c r="P685" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures individual-level boundary spanning behaviors and provides a valid zero-order correlation matrix.. Verbatim Evidence: "Table 2 Means, Standard deviations and Correlation among variables"</t>
+        </is>
+      </c>
     </row>
     <row r="686" ht="18" customHeight="1" s="10">
       <c r="A686" t="inlineStr">
@@ -35080,6 +35178,16 @@
           <t>BSMA0683</t>
         </is>
       </c>
+      <c r="E686" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F686" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G686" t="inlineStr">
         <is>
           <t>With the increasing uncertainty of the environment and the complexity of team tasks, it’s now common practice to encourage employees to implement boundary spanning behaviors. In spite of the fact that a few studies have explored the relationship between boundary spanning behavior and employee creative performance, little is known about the mechanism behind this association. Drawing on the conservation of resource theory (COR), this paper examines the mediating role of meaning of work and the moderating role of team Chaxu climate to reveal the internal process and boundary condition regarding the effect of boundary spanning behavior on employee creative performance. A sample of 211 supervisorsubordinate dyads from six companies located in China is collected in this study, and a hierarchical linear model is used to test the hypotheses. The results show that boundary spanning behavior has a positive effect on employee creative performance, meaning of work mediates the link between them, and team Chaxu climate negatively moderates the relationship between boundary spanning behavior and meaning of work. This research provides a new insight into the linkage between boundary spanning behavior and employee creative performance, as well as further answers the question “how and when boundary spanning behavior influences employee creative performance”.</t>
@@ -35103,7 +35211,11 @@
       <c r="K686" t="n">
         <v>2024</v>
       </c>
-      <c r="P686" s="8" t="n"/>
+      <c r="P686" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures individual-level employee boundary-spanning behavior and provides a raw, zero-order correlation matrix.. Verbatim Evidence: "This article draws on status characteristics theory to explore the mechanisms of individual-level boundary-spanning behavior on employee creative performance"</t>
+        </is>
+      </c>
     </row>
     <row r="687" ht="18" customHeight="1" s="10">
       <c r="A687" t="inlineStr">
@@ -35116,6 +35228,16 @@
           <t>BSMA0684</t>
         </is>
       </c>
+      <c r="E687" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F687" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G687" t="inlineStr">
         <is>
           <t>In the context of encouraging collaborative innovation, employee boundary spanning has become a source of organizational innovation. However, existing research has mainly explored the impact of employee boundary spanning on themselves from an actor-centered perspective, little is known about whether employee boundary spanning can influence supervisor support. Drawing on the perspective of positive interpersonal interaction, the current study employed a scenario experiment (Study 1) and a multi-wave and multi-source questionnaire survey (Study 2) to explore when and how employee boundary spanning affects supervisor support. Results from Study 1 (N= 220) indicated that when upward advice seeking is high, supervisors develop stronger cognitive trust and affective trust towards boundary spanning employees, leading to higher levels of supervisor support. Study 2 (N= 406) further confirmed that upward advice seeking positively moderates the direct effect of employee boundary spanning on supervisor affective trust as well as the indirect effect of employee boundary spanning on supervisor support via affective trust. However, it did not support the moderating effect of upward advice seeking on the supervisor cognitive trust path. These findings contribute to a comprehensive understanding of the impact of employee boundary spanning on supervisor support, providing decision-making references for organizations to manage employee boundary spanning to maintain harmonious supervisor-subordinate relationships.</t>
@@ -35139,7 +35261,11 @@
       <c r="K687" t="n">
         <v>2024</v>
       </c>
-      <c r="P687" s="8" t="n"/>
+      <c r="P687" s="8" t="inlineStr">
+        <is>
+          <t>The paper includes a field survey (Study 2) that measures individual-level employee boundary spanning behavior and reports a valid raw, zero-order correlation matrix (Table 6) alongside means and standard deviations.. Verbatim Evidence: "表 6 显示研究 2 各变量平均值、标准差及相关系数"</t>
+        </is>
+      </c>
     </row>
     <row r="688" ht="18" customHeight="1" s="10">
       <c r="A688" t="inlineStr">
@@ -35152,6 +35278,16 @@
           <t>BSMA0685</t>
         </is>
       </c>
+      <c r="E688" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F688" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G688" t="inlineStr">
         <is>
           <t>To comprehend the mechanism of decent work’s impact on employee boundaryspanning behaviour, this paper constructs a research framework that includes promotion focus and a supportive organizational climate as a mediating factor and moderating variable. A two-stage survey is used to examine these assumptions with data collected from 346 frontline employees. The ﬁndings reveal that decent work has a signiﬁcant positive impact on employee boundary-spanning behaviour and promotion focus has a partial mediating eﬀect on this relationship. A supportive organizational climate plays a positive moderating role in the relationship between decent work and promotion focus.</t>
@@ -35175,7 +35311,11 @@
       <c r="K688" t="n">
         <v>2023</v>
       </c>
-      <c r="P688" s="8" t="n"/>
+      <c r="P688" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures individual-level boundary spanning behaviors among expatriates and provides a valid zero-order correlation matrix.. Verbatim Evidence: "Table 1 Descriptive statistics and correlations... Alpha coefficients are presented on the diagonal"</t>
+        </is>
+      </c>
     </row>
     <row r="689" ht="18" customHeight="1" s="10">
       <c r="A689" t="inlineStr">
@@ -35188,6 +35328,16 @@
           <t>BSMA0686</t>
         </is>
       </c>
+      <c r="E689" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F689" t="inlineStr">
+        <is>
+          <t>Firm-Level</t>
+        </is>
+      </c>
       <c r="G689" t="inlineStr">
         <is>
           <t>Digital transformation promotes the cross-organizational flow of knowledge to provide a new impetus and a new engine for corporate innovation. This study uses dynamic capability theory to demonstrate the intrinsic linkages between digital transformation, open innovation, absorptive capacity and innovation performance. The study utilizes data from Chinese A-share listed manufacturing enterprises from 2016 to 2022. The results show that there is a significant positive correlation between digital transformation and enterprise innovation performance, and the results are still valid after robustness test. The findings of the mediating mechanism indicate that digital transformation can facilitate open innovation activities and enhance the absorptive capacity of enterprises, which leads to improved innovation performance. Starting from the knowledge flow perspective, this paper provides essential theoretical and empirical support for clarifying the mechanism of digital transformation in manufacturing and its impact on innovation performance. The study has significant implications for the long-term development of China's manufacturing industry in the digital economy environment.</t>
@@ -35211,7 +35361,11 @@
       <c r="K689" t="n">
         <v>2024</v>
       </c>
-      <c r="P689" s="8" t="n"/>
+      <c r="P689" s="8" t="inlineStr">
+        <is>
+          <t>The study conducts a firm-level analysis of listed manufacturing companies rather than measuring individual-level boundary spanning behaviors.. Verbatim Evidence: "This paper focuses on the period from 2016 to 2022 and examines the manufacturing companies listed on China's A-share market in Shanghai and Shenzhen as the research subject."</t>
+        </is>
+      </c>
     </row>
     <row r="690" ht="18" customHeight="1" s="10">
       <c r="A690" t="inlineStr">
@@ -35224,6 +35378,16 @@
           <t>BSMA0687</t>
         </is>
       </c>
+      <c r="E690" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F690" t="inlineStr">
+        <is>
+          <t>No Boundary Spanning</t>
+        </is>
+      </c>
       <c r="G690" t="inlineStr">
         <is>
           <t>Purpose – The purpose of this paper is to examine optimism and how facets of subordinates’ psychological characteristics, such as their attitudes and personalities, are similar to their direct supervisors’ (as person-supervisor deep-level similarity or P-S deep-level similarity) in order to understand their interactions with job insecurity in predicting employee job satisfaction.</t>
@@ -35247,7 +35411,11 @@
       <c r="K690" t="n">
         <v>2014</v>
       </c>
-      <c r="P690" s="8" t="n"/>
+      <c r="P690" s="8" t="inlineStr">
+        <is>
+          <t>The study does not measure individual-level boundary spanning behaviors. The variables analyzed include job insecurity, job satisfaction, optimism, P-S deep-level similarity, and P-S guanxi.. Verbatim Evidence: "Participants reported job insecurity, optimism, and job satisfaction. In order to diminish the possibility of common method biases, we used participants’ dyad supervisors to rate P-S deep-level similarity and P-S guanxi."</t>
+        </is>
+      </c>
     </row>
     <row r="691" ht="18" customHeight="1" s="10">
       <c r="A691" t="inlineStr">
@@ -35260,6 +35428,16 @@
           <t>BSMA0688</t>
         </is>
       </c>
+      <c r="E691" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F691" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G691" t="inlineStr">
         <is>
           <t>Purpose – This paper examined the mediating role of boundary spanning behavior and the moderating effects of traditionality linking humble leadership and employee creative performance from the perspective of Social Exchange Theory (SET) to reveal the behavioral mechanism and boundary condition regarding the influence of humble leadership on creative performance.</t>
@@ -35283,7 +35461,11 @@
       <c r="K691" t="n">
         <v>2024</v>
       </c>
-      <c r="P691" s="8" t="n"/>
+      <c r="P691" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures individual-level boundary spanning behavior and provides a raw zero-order correlation matrix with Means and SDs.. Verbatim Evidence: "Table 2 presents the means, standard deviations and correlations of all variables. [...] We measured boundary spanning behavior using Marrone et al. (2007) 4-item scale."</t>
+        </is>
+      </c>
     </row>
     <row r="692" ht="18" customHeight="1" s="10">
       <c r="A692" t="inlineStr">
@@ -35296,6 +35478,16 @@
           <t>BSMA0689</t>
         </is>
       </c>
+      <c r="E692" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F692" t="inlineStr">
+        <is>
+          <t>2 = No boundary spanning measure</t>
+        </is>
+      </c>
       <c r="G692" t="inlineStr">
         <is>
           <t>Integrating boundary spanning and organizational identification theories, we posit that a boundary spanner’s organizational identification (i.e., the sense of oneness with an organization) is an important factor shaping inter-organizational relationships. We examined CEOs of international joint ventures (IJVs) as the boundary spanners in the Asia Pacific region by sampling 185 Chinabased IJVs. We found that organizational identification of an IJV’s CEO with a parent firm is positively related to cooperation between the venture and that parent, and this relationship is stronger when the level of goal differences between parents is higher. The cooperation between the foreign (but not local) parent and the IJV is in turn positively related to the IJV’s performance. This study extends extant research by revealing the role of a boundary spanner’s organizational identification in inter-organizational collaboration as well as inter-firm goal differences as a boundary condition for this role.</t>
@@ -35319,7 +35511,11 @@
       <c r="K692" t="n">
         <v>2023</v>
       </c>
-      <c r="P692" s="8" t="n"/>
+      <c r="P692" s="8" t="inlineStr">
+        <is>
+          <t>The study conceptualizes IJV CEOs as boundary spanners but only measures their organizational identification and inter-firm cooperation, rather than individual-level boundary spanning behaviors.. Verbatim Evidence: "We collected data on the IJV CEO’s identification with the parent firms and IJV performance from two informants in each IJV (i.e., an IJV CEO and an IJV senior vice president)... IJV CEOs also reported the cooperation between parent firms and IJVs"</t>
+        </is>
+      </c>
     </row>
     <row r="693" ht="18" customHeight="1" s="10">
       <c r="A693" t="inlineStr">
@@ -35332,6 +35528,16 @@
           <t>BSMA0690</t>
         </is>
       </c>
+      <c r="E693" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F693" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G693" t="inlineStr">
         <is>
           <t>Purpose – Drawing on conservation of resources (COR) theory, this study develops a theoretical model to explain how and under what conditions resource-based faultlines influence employee creativity, emphasizing the mediating role of employee boundary-spanning behavior and the moderating role of team motivational climate.</t>
@@ -35355,7 +35561,11 @@
       <c r="K693" t="n">
         <v>2026</v>
       </c>
-      <c r="P693" s="8" t="n"/>
+      <c r="P693" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures individual-level employee boundary-spanning behavior and provides a valid zero-order correlation matrix.. Verbatim Evidence: "Table 2 presents the variables’ means, standard deviations, and correlations. As anticipated, the findings indicated that, at the individual level, employee boundary-spanning behavior was positively related to employee creativity (r = 0.51, p &lt; 0.01)."</t>
+        </is>
+      </c>
     </row>
     <row r="694" ht="18" customHeight="1" s="10">
       <c r="A694" t="inlineStr">
@@ -35368,6 +35578,16 @@
           <t>BSMA0691</t>
         </is>
       </c>
+      <c r="E694" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F694" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G694" t="inlineStr">
         <is>
           <t>Purpose – This study aimed to investigate the underlying boundary conditions under which boundaryspanning behaviour has a positive or negative effect on innovative behaviour. Design/methodology/approach – A multi-wave and multi-source research design was adopted to collect data. Data were analysed using the multilevel structural equation modelling and latent moderated structural equation approach.</t>
@@ -35391,7 +35611,11 @@
       <c r="K694" t="n">
         <v>2025</v>
       </c>
-      <c r="P694" s="8" t="n"/>
+      <c r="P694" s="8" t="inlineStr">
+        <is>
+          <t>The paper provides a zero-order correlation matrix that includes individual-level boundary-spanning behaviour and other individual-level variables like innovative behaviour.. Verbatim Evidence: "Table 3. Means, standard deviations and correlations ... Individual level ... 6 Boundary-spanning behaviour"</t>
+        </is>
+      </c>
     </row>
     <row r="695" ht="18" customHeight="1" s="10">
       <c r="A695" t="inlineStr">
@@ -35404,6 +35628,16 @@
           <t>BSMA0692</t>
         </is>
       </c>
+      <c r="E695" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F695" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G695" t="inlineStr">
         <is>
           <t>Boundary-spanning behavior has attracted considerable interest in recent years. Studies on this type of behavior have focused on its positive outcomes from the perspective of social networks. For decades, research has consistently demonstrated that the boundary-spanning behavior produces a wide array of positive results for teams and organizations. However, scholars have found that such behavior has negative outcomes for individuals. Using the conservation of resources theory (COR), we examined the double-edged-sword effect of boundary- spanning behavior on creativity at different levels, as well as its mediating mechanism and boundary conditions.</t>
@@ -35427,7 +35661,11 @@
       <c r="K695" t="n">
         <v>2020</v>
       </c>
-      <c r="P695" s="8" t="n"/>
+      <c r="P695" s="8" t="inlineStr">
+        <is>
+          <t>The paper measures individual-level boundary spanning behavior and provides a valid zero-order correlation matrix with raw Pearson correlations at the individual level.. Verbatim Evidence: "At the individual level, there was a significant positive correlation between employees’ boundary-spanning behavior and role stress (r = 0.15, p &lt; 0.001)"</t>
+        </is>
+      </c>
     </row>
     <row r="696" ht="18" customHeight="1" s="10">
       <c r="A696" t="inlineStr">
@@ -35440,6 +35678,16 @@
           <t>BSMA0693</t>
         </is>
       </c>
+      <c r="E696" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F696" t="inlineStr">
+        <is>
+          <t>Wrong Level of Analysis</t>
+        </is>
+      </c>
       <c r="G696" t="inlineStr">
         <is>
           <t>Purpose – Business model innovation (BMI) is an important channel of enterprise innovation, and BMI’s antecedents have attracted extensive attention. The purpose of this paper is to address a substantial gap in the extant literature by developing a moderate model to explain the effects of boundary-spanning search on BMI as well as whether and how innovative cognitive imprinting (ICI) and environmental dynamics (ED) affect the above relationship.</t>
@@ -35463,7 +35711,11 @@
       <c r="K696" t="n">
         <v>2024</v>
       </c>
-      <c r="P696" s="8" t="n"/>
+      <c r="P696" s="8" t="inlineStr">
+        <is>
+          <t>The study focuses on boundary-spanning search at the firm level rather than the individual level.. Verbatim Evidence: "A total of 239 usable questionnaires from different enterprises in China were collected to obtain firm-level data."</t>
+        </is>
+      </c>
     </row>
     <row r="697" ht="18" customHeight="1" s="10">
       <c r="A697" t="inlineStr">
@@ -35476,6 +35728,16 @@
           <t>BSMA0694</t>
         </is>
       </c>
+      <c r="E697" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F697" t="inlineStr">
+        <is>
+          <t>Non-Individual Anchors</t>
+        </is>
+      </c>
       <c r="G697" t="inlineStr">
         <is>
           <t>Based on organizational learning theory, the influence of the transactive memory system of the top management team on business model innovation is discussed, as is the impact of different dimensions of boundary-spanning search on different business model innovation attributes when attention distribution is taken into account. Meanwhile, the moderating effects of environmental dynamism are considered. Regression and bootstrap analysis are used to test hypotheses. The results based on empirical research show that the transactive memory system has a positive effect on the dual attributes of business model innovation; acute boundary-spanning search and concentrated boundary-spanning search affect novelty-centered business model innovation and efficiencycentered business model innovation, respectively, and play mediating roles. Meanwhile, environmental dynamism positively moderates the relationship between acute boundary-spanning search and novelty-centered business model innovation, but negatively moderates the relationship between concentrated boundaryspanning and business efficiency-centered model innovation efficiency.</t>
@@ -35499,7 +35761,11 @@
       <c r="K697" t="n">
         <v>2023</v>
       </c>
-      <c r="P697" s="8" t="n"/>
+      <c r="P697" s="8" t="inlineStr">
+        <is>
+          <t>The study measures boundary-spanning search at the team (TMT) level rather than the individual level.. Verbatim Evidence: "Since the transactive memory system is at the team level, the data collected needs to be aggregated. Mediating Variable: Boundary-spanning searches... this study used 4 items to measure acute boundary-spanning search (AS): "We are able to develop a variety of partners and build relationships""</t>
+        </is>
+      </c>
     </row>
     <row r="698" ht="18" customHeight="1" s="10">
       <c r="A698" t="inlineStr">
@@ -35512,6 +35778,16 @@
           <t>BSMA0695</t>
         </is>
       </c>
+      <c r="E698" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F698" t="inlineStr">
+        <is>
+          <t>Wrong Level of Analysis</t>
+        </is>
+      </c>
       <c r="G698" t="inlineStr">
         <is>
           <t>Due to their distinctive features, multiteam systems (MTSs) face significant coordination challenges—both within component teams and across the larger system. Despite the benefits of informal mechanisms of coordination for knowledge-based work, there is considerable ambiguity regarding their effects in MTSs. To resolve this ambiguity, we build and test theory about how interpersonal interactions among MTS members serve as an informal coordination mechanism that facilitates team and system functioning. Integrating MTS research with insights from the team boundary spanning literature, we argue that the degree to which MTS members balance their interactions with members of their own component team (i.e., intrateam interactions) and with the members of other teams in the system (i.e., interteam interactions) shapes team- and system-level performance. The findings of a multimethod study of 44 MTSs composed of 295 teams and 930 members show that as interteam interactions exceed intrateam interactions, team conflict arises and detracts from component team performance. At the system level, a balance between intrateam and interteam interactions enhances system success. Our findings advance understanding of MTSs by highlighting how informal coordination mechanisms enable MTSs to overcome their coordination challenges and address the unique performance tension between component teams and the larger system.</t>
@@ -35535,7 +35811,11 @@
       <c r="K698" t="n">
         <v>2022</v>
       </c>
-      <c r="P698" s="8" t="n"/>
+      <c r="P698" s="8" t="inlineStr">
+        <is>
+          <t>The study measures and reports intercorrelations for interpersonal interactions (boundary spanning) at the team and system levels, rather than at the individual level.. Verbatim Evidence: "Tables 1 and 2 provide descriptive statistics for and intercorrelations among study variables at the team level and the system level, respectively."</t>
+        </is>
+      </c>
     </row>
     <row r="699" ht="18" customHeight="1" s="10">
       <c r="A699" t="inlineStr">
@@ -35548,6 +35828,16 @@
           <t>BSMA0696</t>
         </is>
       </c>
+      <c r="E699" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F699" t="inlineStr">
+        <is>
+          <t>Latent Correlations</t>
+        </is>
+      </c>
       <c r="G699" t="inlineStr">
         <is>
           <t>Although the information‐seeking literature has tended to focus upon the selection and use of inanimate objects as information sources, this research follows the more recent trend of investigating how individuals evaluate and use interpersonal information sources. By drawing from the structural, relational, and cognitive elements of social capital theory to inform antecedents to information quality and source accessibility, a research model is developed and tested. For interpersonal information sources, information quality is the key determinant of source use. Perceptions of information quality and accessibility of an interpersonal source are shown to be influenced by boundary spanning, transactive memory, and content type. Implications and prescriptions for future research are discussed.</t>
@@ -35571,7 +35861,11 @@
       <c r="K699" t="n">
         <v>2017</v>
       </c>
-      <c r="P699" s="8" t="n"/>
+      <c r="P699" s="8" t="inlineStr">
+        <is>
+          <t>The paper does not provide a raw, zero-order correlation matrix with means and standard deviations. The only correlation matrix (Table 3) reports latent construct intercorrelations used for assessing discriminant validity, with the square root of AVE on the diagonal.. Verbatim Evidence: "Evaluating convergent and discriminant validity was performed in three ways. First, the correlations among the constructs were compared to the square root of the AVE... The square root of the AVE is shown on the diagonal in Table 3"</t>
+        </is>
+      </c>
     </row>
     <row r="700" ht="18" customHeight="1" s="10">
       <c r="A700" t="inlineStr">
@@ -35584,6 +35878,16 @@
           <t>BSMA0697</t>
         </is>
       </c>
+      <c r="E700" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F700" t="inlineStr">
+        <is>
+          <t>No Correlation Matrix</t>
+        </is>
+      </c>
       <c r="G700" t="inlineStr">
         <is>
           <t>This study adopts a temporal perspective to investigate how boundary spanners can increase the inflow of external knowledge by engaging with both external and internal parties. We add to prior work on knowledge transfer by shifting the focus from engagement levels to investigating engagement dynamics, especially the degree of switching between external and internal engagement across consecutive time periods. Drawing from a cognitive perspective, we argue that switching strongly between engagement types is associated with a segmented knowledge structure that enables quick and efficient categorical processing when knowledge can simply be “channeled” from source to recipient units. In contrast, weak or no switching is associated with a blended knowledge structure and more reflective processing, which is particularly helpful when knowledge transfer requires more translation and transformation. Correspondingly, we adopt a contingency perspective and theorize that the cognitive advantages associated with stronger versus weaker switching weigh differently, contingent on the stickiness of knowledge to be transferred and the nature of boundary-spanning activities that vary in importance over time. Fixed effects models of eight waves of original survey data reveal that, in line with our theorizing, the association between switching and knowledge transfer becomes increasingly negative (1) the more boundary spanners access knowledge that is transspecialist in nature, (2) the greater the organizational distance between source and recipient units, and (3) in later phases of the boundary-spanning process.</t>
@@ -35607,7 +35911,11 @@
       <c r="K700" t="n">
         <v>2024</v>
       </c>
-      <c r="P700" s="8" t="n"/>
+      <c r="P700" s="8" t="inlineStr">
+        <is>
+          <t>The paper does not contain a correlation matrix in the main text. The authors indicate that the correlation table is located in an online appendix, which is not included in the provided PDF.. Verbatim Evidence: "Details on all measures and descriptive statistics can be found in the online appendix (Tables A1–A3 and Figures A1 and A2). The correlation table and an estimation of variance inflation factors indicate that our estimations are not subject to multicollinearity issues."</t>
+        </is>
+      </c>
     </row>
     <row r="701" ht="18" customHeight="1" s="10">
       <c r="A701" t="inlineStr">
@@ -35620,6 +35928,16 @@
           <t>BSMA0698</t>
         </is>
       </c>
+      <c r="E701" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F701" t="inlineStr">
+        <is>
+          <t>Latent Construct Matrix</t>
+        </is>
+      </c>
       <c r="G701" t="inlineStr">
         <is>
           <t>While digital product innovation offers unprecedented opportunities for incumbent firms to create competitive advantages, its fluid and iterative nature presents distinctive cognitive challenges. There is limited empirical literature explaining the role of constructive cognitive characteristics of executives in differentiating the successful pursuit of digital product innovation. Drawing on upper echelons theory and the attention-based view, we examine how chief executive officer (CEO) cognitive flexibility enables incumbent firms to pursue digital product innovation. Through a mixed-methods approach combining a field survey of 178 machine-building firms and a scenario-based experiment with 134 participants, we demonstrate that CEOs with higher cognitive flexibility achieve superior digital product innovation outcomes by facilitating insightful information acquisition and processing. This relationship is strengthened when CEOs engage in more boundary spanning activities and when firms possess greater social capital. Our study contributes to strategic leadership research by demonstrating how CEO cognitive flexibility enables incumbent firms to navigate the cognitive demands of digital product innovation, while enriching our understanding of how adaptive attention patterns shape strategic adaptation in increasingly digitized environments.</t>
@@ -35643,7 +35961,11 @@
       <c r="K701" t="n">
         <v>2026</v>
       </c>
-      <c r="P701" s="8" t="n"/>
+      <c r="P701" s="8" t="inlineStr">
+        <is>
+          <t>The correlation matrix (Table 3) has the square root of AVE on the diagonal and is explicitly used for Fornell-Larcker discriminant validity testing, violating the rule to only extract from matrices where the diagonal is 1.00 or alpha.. Verbatim Evidence: "Furthermore, all pairs of constructs were subjected to Fornell and Larcker’s (1981) discriminant validity test. The findings reveal that the AVE’s square roots for each construct exceed the inter-scale correlations (see Table 3), providing strong evidence for discriminant validity of our core constructs."</t>
+        </is>
+      </c>
     </row>
     <row r="702" ht="18" customHeight="1" s="10">
       <c r="A702" t="inlineStr">
@@ -35656,6 +35978,16 @@
           <t>BSMA0699</t>
         </is>
       </c>
+      <c r="E702" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F702" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
       <c r="G702" t="inlineStr">
         <is>
           <t>We focus on the design of an organization’s set of boundary-spanning transactions—business model design—and ask how business model design affects the performance of entrepreneurial firms. By extending and integrating theoretical perspectives that inform the study of boundary-spanning organization design, we propose hypotheses about the impact of efficiency-centered and novelty-centered business model design on the performance of entrepreneurial firms. To test these hypotheses, we developed and analyzed a unique data set of 190 entrepreneurial firms that were publicly listed on U.S. and European stock exchanges. The empirical results show that novelty-centered business model design matters to the performance of entrepreneurial firms. Our analysis also shows that this positive relationship is remarkably stable across time, even under varying environmental regimes. Additionally, we find indications of potential diseconomies of scope in design; that is, entrepreneurs’ attempts to incorporate both efficiency- and novelty-centered design elements into their business models may be counterproductive.</t>
@@ -35679,7 +36011,11 @@
       <c r="K702" t="n">
         <v>2007</v>
       </c>
-      <c r="P702" s="8" t="n"/>
+      <c r="P702" s="8" t="inlineStr">
+        <is>
+          <t>The paper focuses on business model design and boundary-spanning transactions at the firm level, analyzing a sample of 190 entrepreneurial firms, rather than individual-level behaviors.. Verbatim Evidence: "we developed and analyzed a unique data set of 190 entrepreneurial ﬁrms"</t>
+        </is>
+      </c>
     </row>
     <row r="703" ht="18" customHeight="1" s="10">
       <c r="A703" t="inlineStr">
@@ -35692,6 +36028,16 @@
           <t>BSMA0700</t>
         </is>
       </c>
+      <c r="E703" t="inlineStr">
+        <is>
+          <t>1 = Include</t>
+        </is>
+      </c>
+      <c r="F703" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="G703" t="inlineStr">
         <is>
           <t>We propose and test a framework that describes the relationship between network structures and job performance. We provide an integration of the current conceptualizations of social capital as they pertain to job performance outcomes by taking a multi-dimensional view of job performance. We break down job performance into creativity, decision-making, task execution, and teamwork, and distinguish the effect of structural holes within and across the organizational boundary on these four job performance domains. In an analysis of 318 managers, we ﬁnd that networks rich in structural holes that cross the organizational boundary had a positive association with creativity and decision-making, whereas networks with few structural holes within the organization had a positive association with task execution and teamwork. We discuss the theoretical implications for integrating the social capital, boundary spanning, and network structure literatures, as well as the practical beneﬁts of giving much more precise advice to managers and employees regarding how to use networks to improve performance at work.</t>
@@ -35715,7 +36061,11 @@
       <c r="K703" t="n">
         <v>2013</v>
       </c>
-      <c r="P703" s="8" t="n"/>
+      <c r="P703" s="8" t="inlineStr">
+        <is>
+          <t>The study measures individual-level boundary spanning structural ties (No. of Contact Outside Organization) and provides a raw, zero-order correlation matrix.. Verbatim Evidence: "Table 4 Means, standard deviations, and correlations."</t>
+        </is>
+      </c>
     </row>
     <row r="704" ht="18" customHeight="1" s="10">
       <c r="A704" t="inlineStr">
@@ -35728,6 +36078,16 @@
           <t>BSMA0701</t>
         </is>
       </c>
+      <c r="E704" t="inlineStr">
+        <is>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F704" t="inlineStr">
+        <is>
+          <t>002_No_Quantitative_Data</t>
+        </is>
+      </c>
       <c r="G704" t="inlineStr">
         <is>
           <t>This investigation extends normative conceptions of an organizations public relations roles and communication through an examination of the communicative aspects of boundary spanning processes. The study reconceptualizes the organizational environmental interfaces to identify the public relations processes at the interactional and institutional levels. The research objective aims to develop a structurationist perspective of public relations by employing Giddens'(1979, 1984, 1990, 1991, 1993) structuration framework and a political orientation (Deetz, 1992, 1995; Mumby, 1987, 1989). A structurationist perspective of public relations illuminates how members negotiate ideological frames in back regions which, in turn, influence an organization's public communication efforts, more specifically, an organization's communicative role. Thus, the communicative role evolves from the dominant and resistant ideologies that sustain dominance relations in organizations.</t>
@@ -35751,7 +36111,11 @@
       <c r="K704" t="n">
         <v>2001</v>
       </c>
-      <c r="P704" s="8" t="n"/>
+      <c r="P704" s="8" t="inlineStr">
+        <is>
+          <t>. Verbatim Evidence: ""</t>
+        </is>
+      </c>
     </row>
     <row r="705" ht="18" customHeight="1" s="10">
       <c r="P705" s="8" t="n"/>

</xml_diff>